<commit_message>
Mon Feb 23 03:57:28 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{073FDCE8-6881-4BAC-9F86-031D2BEA0EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{9B650938-22C8-4B29-8C5A-5CBEA6C791C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-11220" windowWidth="29040" windowHeight="17520" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -708,16 +708,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G65"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.3984375"/>
-    <col min="3" max="3" width="18.265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125"/>
+    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="6.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
@@ -728,7 +728,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -737,7 +737,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -748,7 +748,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -759,7 +759,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -768,7 +768,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
         <v>3</v>
       </c>
@@ -779,7 +779,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -800,133 +800,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>158.09</v>
+        <v>160.16</v>
       </c>
       <c r="E8" s="10">
-        <v>147.71</v>
+        <v>149.9</v>
       </c>
       <c r="F8" s="10">
-        <v>157.71</v>
+        <v>159.9</v>
       </c>
       <c r="G8" s="10">
-        <v>147.6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+        <v>149.79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>158.09</v>
+        <v>160.16</v>
       </c>
       <c r="E9" s="13">
-        <v>147.71</v>
+        <v>149.9</v>
       </c>
       <c r="F9" s="13">
-        <v>157.71</v>
+        <v>159.9</v>
       </c>
       <c r="G9" s="13">
-        <v>147.6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+        <v>149.79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>159.72</v>
+        <v>161.68</v>
       </c>
       <c r="E10" s="10">
-        <v>150.41</v>
+        <v>152.51</v>
       </c>
       <c r="F10" s="10">
-        <v>160.41</v>
+        <v>162.51</v>
       </c>
       <c r="G10" s="10">
-        <v>150.65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+        <v>152.75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>157.41</v>
+        <v>158.09</v>
       </c>
       <c r="E11" s="13">
-        <v>147.24</v>
+        <v>147.71</v>
       </c>
       <c r="F11" s="13">
-        <v>157.25</v>
+        <v>157.71</v>
       </c>
       <c r="G11" s="13">
-        <v>147.13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+        <v>147.6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>157.41</v>
+        <v>158.09</v>
       </c>
       <c r="E12" s="10">
-        <v>147.24</v>
+        <v>147.71</v>
       </c>
       <c r="F12" s="10">
-        <v>157.25</v>
+        <v>157.71</v>
       </c>
       <c r="G12" s="10">
-        <v>147.13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+        <v>147.6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>158.87</v>
+        <v>159.72</v>
       </c>
       <c r="E13" s="13">
-        <v>149.97999999999999</v>
+        <v>150.41</v>
       </c>
       <c r="F13" s="13">
-        <v>159.97999999999999</v>
+        <v>160.41</v>
       </c>
       <c r="G13" s="13">
-        <v>150.22</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+        <v>150.65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -935,7 +935,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
         <v>13</v>
       </c>
@@ -946,7 +946,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -965,45 +965,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>164.13</v>
+        <v>166.1</v>
       </c>
       <c r="E17" s="10">
-        <v>153.99</v>
+        <v>156.1</v>
       </c>
       <c r="F17" s="10">
-        <v>163.99</v>
+        <v>166.1</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>163.27000000000001</v>
+        <v>164.13</v>
       </c>
       <c r="E18" s="13">
-        <v>153.55000000000001</v>
+        <v>153.99</v>
       </c>
       <c r="F18" s="13">
-        <v>163.55000000000001</v>
+        <v>163.99</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1012,7 +1012,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
         <v>15</v>
       </c>
@@ -1023,7 +1023,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1044,217 +1044,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>159.49</v>
+        <v>161.55000000000001</v>
       </c>
       <c r="E22" s="10">
-        <v>150.06</v>
+        <v>152.24</v>
       </c>
       <c r="F22" s="10">
-        <v>159.66</v>
+        <v>161.84</v>
       </c>
       <c r="G22" s="10">
-        <v>151.81</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+        <v>153.99</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>164.69</v>
+        <v>166.64</v>
       </c>
       <c r="E23" s="13">
-        <v>156.11000000000001</v>
+        <v>158.21</v>
       </c>
       <c r="F23" s="13">
-        <v>166.11</v>
+        <v>168.21</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>164.88</v>
+        <v>166.84</v>
       </c>
       <c r="E24" s="10">
-        <v>156.63</v>
+        <v>158.72999999999999</v>
       </c>
       <c r="F24" s="10">
-        <v>166.63</v>
+        <v>168.73</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>164.88</v>
+        <v>166.84</v>
       </c>
       <c r="E25" s="13">
-        <v>156.13999999999999</v>
+        <v>158.24</v>
       </c>
       <c r="F25" s="13">
-        <v>166.14</v>
+        <v>168.24</v>
       </c>
       <c r="G25" s="13">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+        <v>159.09</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>164.52</v>
+        <v>166.49</v>
       </c>
       <c r="E26" s="10">
-        <v>157.72</v>
+        <v>159.83000000000001</v>
       </c>
       <c r="F26" s="10">
-        <v>167.72</v>
+        <v>169.83</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>158.59</v>
+        <v>159.49</v>
       </c>
       <c r="E27" s="13">
-        <v>149.59</v>
+        <v>150.06</v>
       </c>
       <c r="F27" s="13">
-        <v>159.19</v>
+        <v>159.66</v>
       </c>
       <c r="G27" s="13">
-        <v>151.34</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+        <v>151.81</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>163.83000000000001</v>
+        <v>164.69</v>
       </c>
       <c r="E28" s="22">
-        <v>155.68</v>
+        <v>156.11000000000001</v>
       </c>
       <c r="F28" s="22">
-        <v>165.68</v>
+        <v>166.11</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>164.03</v>
+        <v>164.88</v>
       </c>
       <c r="E29" s="13">
-        <v>156.21</v>
+        <v>156.63</v>
       </c>
       <c r="F29" s="13">
-        <v>166.21</v>
+        <v>166.63</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>164.03</v>
+        <v>164.88</v>
       </c>
       <c r="E30" s="22">
-        <v>155.71</v>
+        <v>156.13999999999999</v>
       </c>
       <c r="F30" s="22">
-        <v>165.71</v>
+        <v>166.14</v>
       </c>
       <c r="G30" s="22">
-        <v>156.57</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>163.66999999999999</v>
+        <v>164.52</v>
       </c>
       <c r="E31" s="13">
-        <v>157.29</v>
+        <v>157.72</v>
       </c>
       <c r="F31" s="13">
-        <v>167.29</v>
+        <v>167.72</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1263,7 +1263,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="27" t="s">
         <v>22</v>
       </c>
@@ -1274,7 +1274,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1293,45 +1293,45 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>158.11000000000001</v>
+        <v>160.07</v>
       </c>
       <c r="E35" s="10">
-        <v>148.11000000000001</v>
+        <v>150.19999999999999</v>
       </c>
       <c r="F35" s="10">
-        <v>157.11000000000001</v>
+        <v>159.19999999999999</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>157.37</v>
+        <v>158.11000000000001</v>
       </c>
       <c r="E36" s="13">
-        <v>147.68</v>
+        <v>148.11000000000001</v>
       </c>
       <c r="F36" s="13">
-        <v>156.68</v>
+        <v>157.11000000000001</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="14"/>
       <c r="B37" s="14"/>
       <c r="C37" s="15"/>
@@ -1340,7 +1340,7 @@
       <c r="F37" s="16"/>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A38" s="27" t="s">
         <v>24</v>
       </c>
@@ -1351,7 +1351,7 @@
       <c r="F38" s="17"/>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="23" t="s">
         <v>4</v>
       </c>
@@ -1370,83 +1370,83 @@
       </c>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>164.39</v>
+        <v>166.34</v>
       </c>
       <c r="E40" s="10">
-        <v>155.28</v>
+        <v>157.35</v>
       </c>
       <c r="F40" s="10">
-        <v>165.28</v>
+        <v>167.35</v>
       </c>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>164.11</v>
+        <v>166.06</v>
       </c>
       <c r="E41" s="13">
-        <v>155.69999999999999</v>
+        <v>157.77000000000001</v>
       </c>
       <c r="F41" s="13">
-        <v>165.7</v>
+        <v>167.77</v>
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>163.54</v>
+        <v>164.39</v>
       </c>
       <c r="E42" s="10">
-        <v>154.75</v>
+        <v>155.28</v>
       </c>
       <c r="F42" s="10">
-        <v>164.75</v>
+        <v>165.28</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>163.26</v>
+        <v>164.11</v>
       </c>
       <c r="E43" s="13">
-        <v>155.16999999999999</v>
+        <v>155.69999999999999</v>
       </c>
       <c r="F43" s="13">
-        <v>165.17</v>
+        <v>165.7</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="14"/>
       <c r="B44" s="24"/>
       <c r="C44" s="15"/>
@@ -1455,7 +1455,7 @@
       <c r="F44" s="16"/>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="25" t="s">
         <v>27</v>
       </c>
@@ -1466,7 +1466,7 @@
       <c r="F45" s="17"/>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="23" t="s">
         <v>4</v>
       </c>
@@ -1485,83 +1485,83 @@
       </c>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>158.59</v>
+        <v>159.36000000000001</v>
       </c>
       <c r="E47" s="10">
-        <v>150.31</v>
+        <v>150.86000000000001</v>
       </c>
       <c r="F47" s="10">
-        <v>160.31</v>
+        <v>160.86000000000001</v>
       </c>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>158.30000000000001</v>
+        <v>159.08000000000001</v>
       </c>
       <c r="E48" s="13">
-        <v>150.30000000000001</v>
+        <v>150.85</v>
       </c>
       <c r="F48" s="13">
-        <v>160.30000000000001</v>
+        <v>160.85</v>
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>158.43</v>
+        <v>158.59</v>
       </c>
       <c r="E49" s="10">
-        <v>150.37</v>
+        <v>150.31</v>
       </c>
       <c r="F49" s="10">
-        <v>160.37</v>
+        <v>160.31</v>
       </c>
       <c r="G49" s="17"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>158.13999999999999</v>
+        <v>158.30000000000001</v>
       </c>
       <c r="E50" s="13">
-        <v>150.36000000000001</v>
+        <v>150.30000000000001</v>
       </c>
       <c r="F50" s="13">
-        <v>160.36000000000001</v>
+        <v>160.30000000000001</v>
       </c>
       <c r="G50" s="17"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="14"/>
       <c r="B51" s="14"/>
       <c r="C51" s="15"/>
@@ -1570,7 +1570,7 @@
       <c r="F51" s="16"/>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A52" s="27" t="s">
         <v>30</v>
       </c>
@@ -1581,7 +1581,7 @@
       <c r="F52" s="17"/>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="23" t="s">
         <v>4</v>
       </c>
@@ -1600,54 +1600,54 @@
       </c>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>173.62</v>
+        <v>175.6</v>
       </c>
       <c r="E54" s="10">
-        <v>162.86000000000001</v>
+        <v>164.89</v>
       </c>
       <c r="F54" s="10">
-        <v>172.86</v>
+        <v>174.89</v>
       </c>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>162.97</v>
+        <v>164.93</v>
       </c>
       <c r="E55" s="13">
-        <v>162.04</v>
+        <v>164.14</v>
       </c>
       <c r="F55" s="13">
-        <v>172.04</v>
+        <v>174.14</v>
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>162.61000000000001</v>
+        <v>164.68</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1657,111 +1657,111 @@
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>163.55000000000001</v>
+        <v>165.63</v>
       </c>
       <c r="E57" s="13">
-        <v>156.46</v>
+        <v>158.56</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>159.32</v>
+        <v>161.4</v>
       </c>
       <c r="E58" s="10">
-        <v>152.36000000000001</v>
+        <v>154.46</v>
       </c>
       <c r="F58" s="10">
-        <v>162.36000000000001</v>
+        <v>164.46</v>
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>166.57</v>
+        <v>168.54</v>
       </c>
       <c r="E59" s="13">
-        <v>161.46</v>
+        <v>163.54</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>172.75</v>
+        <v>173.62</v>
       </c>
       <c r="E60" s="10">
-        <v>162.47</v>
+        <v>162.86000000000001</v>
       </c>
       <c r="F60" s="10">
-        <v>172.47</v>
+        <v>172.86</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>162.11000000000001</v>
+        <v>162.97</v>
       </c>
       <c r="E61" s="13">
-        <v>161.71</v>
+        <v>162.04</v>
       </c>
       <c r="F61" s="13">
-        <v>171.71</v>
+        <v>172.04</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>161.97999999999999</v>
+        <v>162.61000000000001</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1771,57 +1771,57 @@
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>162.91</v>
+        <v>163.55000000000001</v>
       </c>
       <c r="E63" s="13">
-        <v>156.13</v>
+        <v>156.46</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>158.68</v>
+        <v>159.32</v>
       </c>
       <c r="E64" s="10">
-        <v>152.03</v>
+        <v>152.36000000000001</v>
       </c>
       <c r="F64" s="10">
-        <v>162.03</v>
+        <v>162.36000000000001</v>
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>165.71</v>
+        <v>166.57</v>
       </c>
       <c r="E65" s="13">
-        <v>161.05000000000001</v>
+        <v>161.46</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,6 +1850,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2109,42 +2129,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2168,9 +2156,21 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Tue Feb 24 03:45:38 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{9B650938-22C8-4B29-8C5A-5CBEA6C791C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{EA6C9416-E1E3-4351-A64C-913DBFB2DAEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>160.16</v>
+        <v>161.63999999999999</v>
       </c>
       <c r="E8" s="10">
-        <v>149.9</v>
+        <v>151.96</v>
       </c>
       <c r="F8" s="10">
-        <v>159.9</v>
+        <v>161.96</v>
       </c>
       <c r="G8" s="10">
-        <v>149.79</v>
+        <v>151.85</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>160.16</v>
+        <v>161.63999999999999</v>
       </c>
       <c r="E9" s="13">
-        <v>149.9</v>
+        <v>151.96</v>
       </c>
       <c r="F9" s="13">
-        <v>159.9</v>
+        <v>161.96</v>
       </c>
       <c r="G9" s="13">
-        <v>149.79</v>
+        <v>151.85</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>161.68</v>
+        <v>163.34</v>
       </c>
       <c r="E10" s="10">
-        <v>152.51</v>
+        <v>154.54</v>
       </c>
       <c r="F10" s="10">
-        <v>162.51</v>
+        <v>164.54</v>
       </c>
       <c r="G10" s="10">
-        <v>152.75</v>
+        <v>154.78</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>158.09</v>
+        <v>160.16</v>
       </c>
       <c r="E11" s="13">
-        <v>147.71</v>
+        <v>149.9</v>
       </c>
       <c r="F11" s="13">
-        <v>157.71</v>
+        <v>159.9</v>
       </c>
       <c r="G11" s="13">
-        <v>147.6</v>
+        <v>149.79</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>158.09</v>
+        <v>160.16</v>
       </c>
       <c r="E12" s="10">
-        <v>147.71</v>
+        <v>149.9</v>
       </c>
       <c r="F12" s="10">
-        <v>157.71</v>
+        <v>159.9</v>
       </c>
       <c r="G12" s="10">
-        <v>147.6</v>
+        <v>149.79</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>159.72</v>
+        <v>161.68</v>
       </c>
       <c r="E13" s="13">
-        <v>150.41</v>
+        <v>152.51</v>
       </c>
       <c r="F13" s="13">
-        <v>160.41</v>
+        <v>162.51</v>
       </c>
       <c r="G13" s="13">
-        <v>150.65</v>
+        <v>152.75</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>166.1</v>
+        <v>167.74</v>
       </c>
       <c r="E17" s="10">
-        <v>156.1</v>
+        <v>158.12</v>
       </c>
       <c r="F17" s="10">
-        <v>166.1</v>
+        <v>168.12</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>164.13</v>
+        <v>166.1</v>
       </c>
       <c r="E18" s="13">
-        <v>153.99</v>
+        <v>156.1</v>
       </c>
       <c r="F18" s="13">
-        <v>163.99</v>
+        <v>166.1</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>161.55000000000001</v>
+        <v>162.81</v>
       </c>
       <c r="E22" s="10">
-        <v>152.24</v>
+        <v>154.30000000000001</v>
       </c>
       <c r="F22" s="10">
-        <v>161.84</v>
+        <v>163.9</v>
       </c>
       <c r="G22" s="10">
-        <v>153.99</v>
+        <v>156.05000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>166.64</v>
+        <v>168.31</v>
       </c>
       <c r="E23" s="13">
-        <v>158.21</v>
+        <v>160.25</v>
       </c>
       <c r="F23" s="13">
-        <v>168.21</v>
+        <v>170.25</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>166.84</v>
+        <v>168.5</v>
       </c>
       <c r="E24" s="10">
-        <v>158.72999999999999</v>
+        <v>160.76</v>
       </c>
       <c r="F24" s="10">
-        <v>168.73</v>
+        <v>170.76</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>166.84</v>
+        <v>168.5</v>
       </c>
       <c r="E25" s="13">
-        <v>158.24</v>
+        <v>160.28</v>
       </c>
       <c r="F25" s="13">
-        <v>168.24</v>
+        <v>170.28</v>
       </c>
       <c r="G25" s="13">
-        <v>159.09</v>
+        <v>161.13</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>166.49</v>
+        <v>168.15</v>
       </c>
       <c r="E26" s="10">
-        <v>159.83000000000001</v>
+        <v>161.88999999999999</v>
       </c>
       <c r="F26" s="10">
-        <v>169.83</v>
+        <v>171.89</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>159.49</v>
+        <v>161.55000000000001</v>
       </c>
       <c r="E27" s="13">
-        <v>150.06</v>
+        <v>152.24</v>
       </c>
       <c r="F27" s="13">
-        <v>159.66</v>
+        <v>161.84</v>
       </c>
       <c r="G27" s="13">
-        <v>151.81</v>
+        <v>153.99</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>164.69</v>
+        <v>166.64</v>
       </c>
       <c r="E28" s="22">
-        <v>156.11000000000001</v>
+        <v>158.21</v>
       </c>
       <c r="F28" s="22">
-        <v>166.11</v>
+        <v>168.21</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>164.88</v>
+        <v>166.84</v>
       </c>
       <c r="E29" s="13">
-        <v>156.63</v>
+        <v>158.72999999999999</v>
       </c>
       <c r="F29" s="13">
-        <v>166.63</v>
+        <v>168.73</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>164.88</v>
+        <v>166.84</v>
       </c>
       <c r="E30" s="22">
-        <v>156.13999999999999</v>
+        <v>158.24</v>
       </c>
       <c r="F30" s="22">
-        <v>166.14</v>
+        <v>168.24</v>
       </c>
       <c r="G30" s="22">
-        <v>157</v>
+        <v>159.09</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>164.52</v>
+        <v>166.49</v>
       </c>
       <c r="E31" s="13">
-        <v>157.72</v>
+        <v>159.83000000000001</v>
       </c>
       <c r="F31" s="13">
-        <v>167.72</v>
+        <v>169.83</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>160.07</v>
+        <v>161.72999999999999</v>
       </c>
       <c r="E35" s="10">
-        <v>150.19999999999999</v>
+        <v>152.22</v>
       </c>
       <c r="F35" s="10">
-        <v>159.19999999999999</v>
+        <v>161.22</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>158.11000000000001</v>
+        <v>160.07</v>
       </c>
       <c r="E36" s="13">
-        <v>148.11000000000001</v>
+        <v>150.19999999999999</v>
       </c>
       <c r="F36" s="13">
-        <v>157.11000000000001</v>
+        <v>159.19999999999999</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>166.34</v>
+        <v>168.02</v>
       </c>
       <c r="E40" s="10">
-        <v>157.35</v>
+        <v>159.28</v>
       </c>
       <c r="F40" s="10">
-        <v>167.35</v>
+        <v>169.28</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>166.06</v>
+        <v>167.73</v>
       </c>
       <c r="E41" s="13">
-        <v>157.77000000000001</v>
+        <v>159.69999999999999</v>
       </c>
       <c r="F41" s="13">
-        <v>167.77</v>
+        <v>169.7</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>164.39</v>
+        <v>166.34</v>
       </c>
       <c r="E42" s="10">
-        <v>155.28</v>
+        <v>157.35</v>
       </c>
       <c r="F42" s="10">
-        <v>165.28</v>
+        <v>167.35</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>164.11</v>
+        <v>166.06</v>
       </c>
       <c r="E43" s="13">
-        <v>155.69999999999999</v>
+        <v>157.77000000000001</v>
       </c>
       <c r="F43" s="13">
-        <v>165.7</v>
+        <v>167.77</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>159.36000000000001</v>
+        <v>160.09</v>
       </c>
       <c r="E47" s="10">
-        <v>150.86000000000001</v>
+        <v>151.44999999999999</v>
       </c>
       <c r="F47" s="10">
-        <v>160.86000000000001</v>
+        <v>161.44999999999999</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>159.08000000000001</v>
+        <v>159.81</v>
       </c>
       <c r="E48" s="13">
-        <v>150.85</v>
+        <v>151.44</v>
       </c>
       <c r="F48" s="13">
-        <v>160.85</v>
+        <v>161.44</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>158.59</v>
+        <v>159.36000000000001</v>
       </c>
       <c r="E49" s="10">
-        <v>150.31</v>
+        <v>150.86000000000001</v>
       </c>
       <c r="F49" s="10">
-        <v>160.31</v>
+        <v>160.86000000000001</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>158.30000000000001</v>
+        <v>159.08000000000001</v>
       </c>
       <c r="E50" s="13">
-        <v>150.30000000000001</v>
+        <v>150.85</v>
       </c>
       <c r="F50" s="13">
-        <v>160.30000000000001</v>
+        <v>160.85</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>175.6</v>
+        <v>177.26</v>
       </c>
       <c r="E54" s="10">
-        <v>164.89</v>
+        <v>166.98</v>
       </c>
       <c r="F54" s="10">
-        <v>174.89</v>
+        <v>176.98</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>164.93</v>
+        <v>166.6</v>
       </c>
       <c r="E55" s="13">
-        <v>164.14</v>
+        <v>166.15</v>
       </c>
       <c r="F55" s="13">
-        <v>174.14</v>
+        <v>176.15</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>164.68</v>
+        <v>166.23</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>165.63</v>
+        <v>167.16</v>
       </c>
       <c r="E57" s="13">
-        <v>158.56</v>
+        <v>160.57</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>161.4</v>
+        <v>162.93</v>
       </c>
       <c r="E58" s="10">
-        <v>154.46</v>
+        <v>156.47</v>
       </c>
       <c r="F58" s="10">
-        <v>164.46</v>
+        <v>166.47</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>168.54</v>
+        <v>170.18</v>
       </c>
       <c r="E59" s="13">
-        <v>163.54</v>
+        <v>165.6</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>173.62</v>
+        <v>175.6</v>
       </c>
       <c r="E60" s="10">
-        <v>162.86000000000001</v>
+        <v>164.89</v>
       </c>
       <c r="F60" s="10">
-        <v>172.86</v>
+        <v>174.89</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>162.97</v>
+        <v>164.93</v>
       </c>
       <c r="E61" s="13">
-        <v>162.04</v>
+        <v>164.14</v>
       </c>
       <c r="F61" s="13">
-        <v>172.04</v>
+        <v>174.14</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>162.61000000000001</v>
+        <v>164.68</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>163.55000000000001</v>
+        <v>165.63</v>
       </c>
       <c r="E63" s="13">
-        <v>156.46</v>
+        <v>158.56</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>159.32</v>
+        <v>161.4</v>
       </c>
       <c r="E64" s="10">
-        <v>152.36000000000001</v>
+        <v>154.46</v>
       </c>
       <c r="F64" s="10">
-        <v>162.36000000000001</v>
+        <v>164.46</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46074</v>
+        <v>46077</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>166.57</v>
+        <v>168.54</v>
       </c>
       <c r="E65" s="13">
-        <v>161.46</v>
+        <v>163.54</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,15 +1850,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -1867,6 +1858,15 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2130,14 +2130,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -2151,6 +2143,14 @@
     <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
     <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Wed Feb 25 03:53:48 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{EA6C9416-E1E3-4351-A64C-913DBFB2DAEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{69F80480-3060-428F-B060-CDDE647A1BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>161.63999999999999</v>
+        <v>161.47</v>
       </c>
       <c r="E8" s="10">
-        <v>151.96</v>
+        <v>152.55000000000001</v>
       </c>
       <c r="F8" s="10">
-        <v>161.96</v>
+        <v>162.55000000000001</v>
       </c>
       <c r="G8" s="10">
-        <v>151.85</v>
+        <v>152.44</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>161.63999999999999</v>
+        <v>161.47</v>
       </c>
       <c r="E9" s="13">
-        <v>151.96</v>
+        <v>152.55000000000001</v>
       </c>
       <c r="F9" s="13">
-        <v>161.96</v>
+        <v>162.55000000000001</v>
       </c>
       <c r="G9" s="13">
-        <v>151.85</v>
+        <v>152.44</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>163.34</v>
+        <v>163.26</v>
       </c>
       <c r="E10" s="10">
-        <v>154.54</v>
+        <v>154.88999999999999</v>
       </c>
       <c r="F10" s="10">
-        <v>164.54</v>
+        <v>164.89</v>
       </c>
       <c r="G10" s="10">
-        <v>154.78</v>
+        <v>155.13999999999999</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>160.16</v>
+        <v>161.63999999999999</v>
       </c>
       <c r="E11" s="13">
-        <v>149.9</v>
+        <v>151.96</v>
       </c>
       <c r="F11" s="13">
-        <v>159.9</v>
+        <v>161.96</v>
       </c>
       <c r="G11" s="13">
-        <v>149.79</v>
+        <v>151.85</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>160.16</v>
+        <v>161.63999999999999</v>
       </c>
       <c r="E12" s="10">
-        <v>149.9</v>
+        <v>151.96</v>
       </c>
       <c r="F12" s="10">
-        <v>159.9</v>
+        <v>161.96</v>
       </c>
       <c r="G12" s="10">
-        <v>149.79</v>
+        <v>151.85</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>161.68</v>
+        <v>163.34</v>
       </c>
       <c r="E13" s="13">
-        <v>152.51</v>
+        <v>154.54</v>
       </c>
       <c r="F13" s="13">
-        <v>162.51</v>
+        <v>164.54</v>
       </c>
       <c r="G13" s="13">
-        <v>152.75</v>
+        <v>154.78</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>167.74</v>
+        <v>167.87</v>
       </c>
       <c r="E17" s="10">
-        <v>158.12</v>
+        <v>158.69</v>
       </c>
       <c r="F17" s="10">
-        <v>168.12</v>
+        <v>168.69</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>166.1</v>
+        <v>167.74</v>
       </c>
       <c r="E18" s="13">
-        <v>156.1</v>
+        <v>158.12</v>
       </c>
       <c r="F18" s="13">
-        <v>166.1</v>
+        <v>168.12</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>162.81</v>
+        <v>162.97</v>
       </c>
       <c r="E22" s="10">
-        <v>154.30000000000001</v>
+        <v>154.35</v>
       </c>
       <c r="F22" s="10">
-        <v>163.9</v>
+        <v>163.95</v>
       </c>
       <c r="G22" s="10">
-        <v>156.05000000000001</v>
+        <v>156.1</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>168.31</v>
+        <v>168.13</v>
       </c>
       <c r="E23" s="13">
-        <v>160.25</v>
+        <v>160.6</v>
       </c>
       <c r="F23" s="13">
-        <v>170.25</v>
+        <v>170.6</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>168.5</v>
+        <v>168.32</v>
       </c>
       <c r="E24" s="10">
-        <v>160.76</v>
+        <v>161.13</v>
       </c>
       <c r="F24" s="10">
-        <v>170.76</v>
+        <v>171.13</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>168.5</v>
+        <v>168.32</v>
       </c>
       <c r="E25" s="13">
-        <v>160.28</v>
+        <v>160.63999999999999</v>
       </c>
       <c r="F25" s="13">
-        <v>170.28</v>
+        <v>170.64</v>
       </c>
       <c r="G25" s="13">
-        <v>161.13</v>
+        <v>161.5</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>168.15</v>
+        <v>167.96</v>
       </c>
       <c r="E26" s="10">
-        <v>161.88999999999999</v>
+        <v>162.26</v>
       </c>
       <c r="F26" s="10">
-        <v>171.89</v>
+        <v>172.26</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>161.55000000000001</v>
+        <v>162.81</v>
       </c>
       <c r="E27" s="13">
-        <v>152.24</v>
+        <v>154.30000000000001</v>
       </c>
       <c r="F27" s="13">
-        <v>161.84</v>
+        <v>163.9</v>
       </c>
       <c r="G27" s="13">
-        <v>153.99</v>
+        <v>156.05000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>166.64</v>
+        <v>168.31</v>
       </c>
       <c r="E28" s="22">
-        <v>158.21</v>
+        <v>160.25</v>
       </c>
       <c r="F28" s="22">
-        <v>168.21</v>
+        <v>170.25</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>166.84</v>
+        <v>168.5</v>
       </c>
       <c r="E29" s="13">
-        <v>158.72999999999999</v>
+        <v>160.76</v>
       </c>
       <c r="F29" s="13">
-        <v>168.73</v>
+        <v>170.76</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>166.84</v>
+        <v>168.5</v>
       </c>
       <c r="E30" s="22">
-        <v>158.24</v>
+        <v>160.28</v>
       </c>
       <c r="F30" s="22">
-        <v>168.24</v>
+        <v>170.28</v>
       </c>
       <c r="G30" s="22">
-        <v>159.09</v>
+        <v>161.13</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>166.49</v>
+        <v>168.15</v>
       </c>
       <c r="E31" s="13">
-        <v>159.83000000000001</v>
+        <v>161.88999999999999</v>
       </c>
       <c r="F31" s="13">
-        <v>169.83</v>
+        <v>171.89</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>161.72999999999999</v>
+        <v>161.76</v>
       </c>
       <c r="E35" s="10">
-        <v>152.22</v>
+        <v>152.80000000000001</v>
       </c>
       <c r="F35" s="10">
-        <v>161.22</v>
+        <v>161.80000000000001</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>160.07</v>
+        <v>161.72999999999999</v>
       </c>
       <c r="E36" s="13">
-        <v>150.19999999999999</v>
+        <v>152.22</v>
       </c>
       <c r="F36" s="13">
-        <v>159.19999999999999</v>
+        <v>161.22</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>168.02</v>
+        <v>168.17</v>
       </c>
       <c r="E40" s="10">
-        <v>159.28</v>
+        <v>159.81</v>
       </c>
       <c r="F40" s="10">
-        <v>169.28</v>
+        <v>169.81</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>167.73</v>
+        <v>167.89</v>
       </c>
       <c r="E41" s="13">
-        <v>159.69999999999999</v>
+        <v>160.22999999999999</v>
       </c>
       <c r="F41" s="13">
-        <v>169.7</v>
+        <v>170.23</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>166.34</v>
+        <v>168.02</v>
       </c>
       <c r="E42" s="10">
-        <v>157.35</v>
+        <v>159.28</v>
       </c>
       <c r="F42" s="10">
-        <v>167.35</v>
+        <v>169.28</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>166.06</v>
+        <v>167.73</v>
       </c>
       <c r="E43" s="13">
-        <v>157.77000000000001</v>
+        <v>159.69999999999999</v>
       </c>
       <c r="F43" s="13">
-        <v>167.77</v>
+        <v>169.7</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>160.09</v>
+        <v>161.41</v>
       </c>
       <c r="E47" s="10">
-        <v>151.44999999999999</v>
+        <v>153</v>
       </c>
       <c r="F47" s="10">
-        <v>161.44999999999999</v>
+        <v>163</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>159.81</v>
+        <v>161.12</v>
       </c>
       <c r="E48" s="13">
-        <v>151.44</v>
+        <v>152.99</v>
       </c>
       <c r="F48" s="13">
-        <v>161.44</v>
+        <v>162.99</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>159.36000000000001</v>
+        <v>160.09</v>
       </c>
       <c r="E49" s="10">
-        <v>150.86000000000001</v>
+        <v>151.44999999999999</v>
       </c>
       <c r="F49" s="10">
-        <v>160.86000000000001</v>
+        <v>161.44999999999999</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>159.08000000000001</v>
+        <v>159.81</v>
       </c>
       <c r="E50" s="13">
-        <v>150.85</v>
+        <v>151.44</v>
       </c>
       <c r="F50" s="13">
-        <v>160.85</v>
+        <v>161.44</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,33 +1602,33 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>177.26</v>
+        <v>177.4</v>
       </c>
       <c r="E54" s="10">
-        <v>166.98</v>
+        <v>167.63</v>
       </c>
       <c r="F54" s="10">
-        <v>176.98</v>
+        <v>177.63</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>166.6</v>
+        <v>166.74</v>
       </c>
       <c r="E55" s="13">
         <v>166.15</v>
@@ -1640,14 +1640,14 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>166.23</v>
+        <v>166.38</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,14 +1659,14 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>167.16</v>
+        <v>167.28</v>
       </c>
       <c r="E57" s="13">
         <v>160.57</v>
@@ -1678,14 +1678,14 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>162.93</v>
+        <v>163.06</v>
       </c>
       <c r="E58" s="10">
         <v>156.47</v>
@@ -1697,17 +1697,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>170.18</v>
+        <v>170.3</v>
       </c>
       <c r="E59" s="13">
-        <v>165.6</v>
+        <v>166.22</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>175.6</v>
+        <v>177.26</v>
       </c>
       <c r="E60" s="10">
-        <v>164.89</v>
+        <v>166.98</v>
       </c>
       <c r="F60" s="10">
-        <v>174.89</v>
+        <v>176.98</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>164.93</v>
+        <v>166.6</v>
       </c>
       <c r="E61" s="13">
-        <v>164.14</v>
+        <v>166.15</v>
       </c>
       <c r="F61" s="13">
-        <v>174.14</v>
+        <v>176.15</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>164.68</v>
+        <v>166.23</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>165.63</v>
+        <v>167.16</v>
       </c>
       <c r="E63" s="13">
-        <v>158.56</v>
+        <v>160.57</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>161.4</v>
+        <v>162.93</v>
       </c>
       <c r="E64" s="10">
-        <v>154.46</v>
+        <v>156.47</v>
       </c>
       <c r="F64" s="10">
-        <v>164.46</v>
+        <v>166.47</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>168.54</v>
+        <v>170.18</v>
       </c>
       <c r="E65" s="13">
-        <v>163.54</v>
+        <v>165.6</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,26 +1850,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2129,33 +2109,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2175,6 +2149,32 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Thu Feb 26 03:43:06 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{69F80480-3060-428F-B060-CDDE647A1BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{2F1CD274-9519-44B5-9F09-6E4891027120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>161.47</v>
+        <v>161.43</v>
       </c>
       <c r="E8" s="10">
-        <v>152.55000000000001</v>
+        <v>152.84</v>
       </c>
       <c r="F8" s="10">
-        <v>162.55000000000001</v>
+        <v>162.84</v>
       </c>
       <c r="G8" s="10">
-        <v>152.44</v>
+        <v>152.72999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>161.47</v>
+        <v>161.43</v>
       </c>
       <c r="E9" s="13">
-        <v>152.55000000000001</v>
+        <v>152.84</v>
       </c>
       <c r="F9" s="13">
-        <v>162.55000000000001</v>
+        <v>162.84</v>
       </c>
       <c r="G9" s="13">
-        <v>152.44</v>
+        <v>152.72999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>163.26</v>
+        <v>163.19999999999999</v>
       </c>
       <c r="E10" s="10">
-        <v>154.88999999999999</v>
+        <v>155.15</v>
       </c>
       <c r="F10" s="10">
-        <v>164.89</v>
+        <v>165.15</v>
       </c>
       <c r="G10" s="10">
-        <v>155.13999999999999</v>
+        <v>155.4</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>161.63999999999999</v>
+        <v>161.47</v>
       </c>
       <c r="E11" s="13">
-        <v>151.96</v>
+        <v>152.55000000000001</v>
       </c>
       <c r="F11" s="13">
-        <v>161.96</v>
+        <v>162.55000000000001</v>
       </c>
       <c r="G11" s="13">
-        <v>151.85</v>
+        <v>152.44</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>161.63999999999999</v>
+        <v>161.47</v>
       </c>
       <c r="E12" s="10">
-        <v>151.96</v>
+        <v>152.55000000000001</v>
       </c>
       <c r="F12" s="10">
-        <v>161.96</v>
+        <v>162.55000000000001</v>
       </c>
       <c r="G12" s="10">
-        <v>151.85</v>
+        <v>152.44</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>163.34</v>
+        <v>163.26</v>
       </c>
       <c r="E13" s="13">
-        <v>154.54</v>
+        <v>154.88999999999999</v>
       </c>
       <c r="F13" s="13">
-        <v>164.54</v>
+        <v>164.89</v>
       </c>
       <c r="G13" s="13">
-        <v>154.78</v>
+        <v>155.13999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>167.87</v>
+        <v>167.8</v>
       </c>
       <c r="E17" s="10">
-        <v>158.69</v>
+        <v>158.94</v>
       </c>
       <c r="F17" s="10">
-        <v>168.69</v>
+        <v>168.94</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>167.74</v>
+        <v>167.87</v>
       </c>
       <c r="E18" s="13">
-        <v>158.12</v>
+        <v>158.69</v>
       </c>
       <c r="F18" s="13">
-        <v>168.12</v>
+        <v>168.69</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>162.97</v>
+        <v>162.93</v>
       </c>
       <c r="E22" s="10">
-        <v>154.35</v>
+        <v>154.63</v>
       </c>
       <c r="F22" s="10">
-        <v>163.95</v>
+        <v>164.23</v>
       </c>
       <c r="G22" s="10">
-        <v>156.1</v>
+        <v>156.38</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>168.13</v>
+        <v>168.06</v>
       </c>
       <c r="E23" s="13">
-        <v>160.6</v>
+        <v>160.86000000000001</v>
       </c>
       <c r="F23" s="13">
-        <v>170.6</v>
+        <v>170.86</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>168.32</v>
+        <v>168.25</v>
       </c>
       <c r="E24" s="10">
-        <v>161.13</v>
+        <v>161.38999999999999</v>
       </c>
       <c r="F24" s="10">
-        <v>171.13</v>
+        <v>171.39</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>168.32</v>
+        <v>168.25</v>
       </c>
       <c r="E25" s="13">
-        <v>160.63999999999999</v>
+        <v>160.91</v>
       </c>
       <c r="F25" s="13">
-        <v>170.64</v>
+        <v>170.91</v>
       </c>
       <c r="G25" s="13">
-        <v>161.5</v>
+        <v>161.76</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>167.96</v>
+        <v>167.89</v>
       </c>
       <c r="E26" s="10">
-        <v>162.26</v>
+        <v>162.52000000000001</v>
       </c>
       <c r="F26" s="10">
-        <v>172.26</v>
+        <v>172.52</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>162.81</v>
+        <v>162.97</v>
       </c>
       <c r="E27" s="13">
-        <v>154.30000000000001</v>
+        <v>154.35</v>
       </c>
       <c r="F27" s="13">
-        <v>163.9</v>
+        <v>163.95</v>
       </c>
       <c r="G27" s="13">
-        <v>156.05000000000001</v>
+        <v>156.1</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>168.31</v>
+        <v>168.13</v>
       </c>
       <c r="E28" s="22">
-        <v>160.25</v>
+        <v>160.6</v>
       </c>
       <c r="F28" s="22">
-        <v>170.25</v>
+        <v>170.6</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>168.5</v>
+        <v>168.32</v>
       </c>
       <c r="E29" s="13">
-        <v>160.76</v>
+        <v>161.13</v>
       </c>
       <c r="F29" s="13">
-        <v>170.76</v>
+        <v>171.13</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>168.5</v>
+        <v>168.32</v>
       </c>
       <c r="E30" s="22">
-        <v>160.28</v>
+        <v>160.63999999999999</v>
       </c>
       <c r="F30" s="22">
-        <v>170.28</v>
+        <v>170.64</v>
       </c>
       <c r="G30" s="22">
-        <v>161.13</v>
+        <v>161.5</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>168.15</v>
+        <v>167.96</v>
       </c>
       <c r="E31" s="13">
-        <v>161.88999999999999</v>
+        <v>162.26</v>
       </c>
       <c r="F31" s="13">
-        <v>171.89</v>
+        <v>172.26</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>161.76</v>
+        <v>161.69</v>
       </c>
       <c r="E35" s="10">
-        <v>152.80000000000001</v>
+        <v>153.06</v>
       </c>
       <c r="F35" s="10">
-        <v>161.80000000000001</v>
+        <v>162.06</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>161.72999999999999</v>
+        <v>161.76</v>
       </c>
       <c r="E36" s="13">
-        <v>152.22</v>
+        <v>152.80000000000001</v>
       </c>
       <c r="F36" s="13">
-        <v>161.22</v>
+        <v>161.80000000000001</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>168.17</v>
+        <v>168.11</v>
       </c>
       <c r="E40" s="10">
-        <v>159.81</v>
+        <v>160.05000000000001</v>
       </c>
       <c r="F40" s="10">
-        <v>169.81</v>
+        <v>170.05</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>167.89</v>
+        <v>167.82</v>
       </c>
       <c r="E41" s="13">
-        <v>160.22999999999999</v>
+        <v>160.47</v>
       </c>
       <c r="F41" s="13">
-        <v>170.23</v>
+        <v>170.47</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>168.02</v>
+        <v>168.17</v>
       </c>
       <c r="E42" s="10">
-        <v>159.28</v>
+        <v>159.81</v>
       </c>
       <c r="F42" s="10">
-        <v>169.28</v>
+        <v>169.81</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>167.73</v>
+        <v>167.89</v>
       </c>
       <c r="E43" s="13">
-        <v>159.69999999999999</v>
+        <v>160.22999999999999</v>
       </c>
       <c r="F43" s="13">
-        <v>169.7</v>
+        <v>170.23</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>161.41</v>
+        <v>162.01</v>
       </c>
       <c r="E47" s="10">
-        <v>153</v>
+        <v>154.5</v>
       </c>
       <c r="F47" s="10">
-        <v>163</v>
+        <v>164.5</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>161.12</v>
+        <v>161.72999999999999</v>
       </c>
       <c r="E48" s="13">
-        <v>152.99</v>
+        <v>154.49</v>
       </c>
       <c r="F48" s="13">
-        <v>162.99</v>
+        <v>164.49</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>160.09</v>
+        <v>161.41</v>
       </c>
       <c r="E49" s="10">
-        <v>151.44999999999999</v>
+        <v>153</v>
       </c>
       <c r="F49" s="10">
-        <v>161.44999999999999</v>
+        <v>163</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>159.81</v>
+        <v>161.12</v>
       </c>
       <c r="E50" s="13">
-        <v>151.44</v>
+        <v>152.99</v>
       </c>
       <c r="F50" s="13">
-        <v>161.44</v>
+        <v>162.99</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>177.4</v>
+        <v>177.32</v>
       </c>
       <c r="E54" s="10">
-        <v>167.63</v>
+        <v>167.92</v>
       </c>
       <c r="F54" s="10">
-        <v>177.63</v>
+        <v>177.92</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>166.74</v>
+        <v>166.67</v>
       </c>
       <c r="E55" s="13">
-        <v>166.15</v>
+        <v>166.4</v>
       </c>
       <c r="F55" s="13">
-        <v>176.15</v>
+        <v>176.4</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>166.38</v>
+        <v>166.31</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>167.28</v>
+        <v>167.21</v>
       </c>
       <c r="E57" s="13">
-        <v>160.57</v>
+        <v>160.83000000000001</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>163.06</v>
+        <v>162.97999999999999</v>
       </c>
       <c r="E58" s="10">
-        <v>156.47</v>
+        <v>156.72</v>
       </c>
       <c r="F58" s="10">
-        <v>166.47</v>
+        <v>166.72</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>170.3</v>
+        <v>170.23</v>
       </c>
       <c r="E59" s="13">
-        <v>166.22</v>
+        <v>166.5</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,33 +1716,33 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>177.26</v>
+        <v>177.4</v>
       </c>
       <c r="E60" s="10">
-        <v>166.98</v>
+        <v>167.63</v>
       </c>
       <c r="F60" s="10">
-        <v>176.98</v>
+        <v>177.63</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>166.6</v>
+        <v>166.74</v>
       </c>
       <c r="E61" s="13">
         <v>166.15</v>
@@ -1754,14 +1754,14 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>166.23</v>
+        <v>166.38</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,14 +1773,14 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>167.16</v>
+        <v>167.28</v>
       </c>
       <c r="E63" s="13">
         <v>160.57</v>
@@ -1792,14 +1792,14 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>162.93</v>
+        <v>163.06</v>
       </c>
       <c r="E64" s="10">
         <v>156.47</v>
@@ -1811,17 +1811,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46078</v>
+        <v>46079</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>170.18</v>
+        <v>170.3</v>
       </c>
       <c r="E65" s="13">
-        <v>165.6</v>
+        <v>166.22</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,6 +1850,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2109,15 +2118,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2130,6 +2130,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2145,14 +2153,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Fri Feb 27 03:39:34 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{2F1CD274-9519-44B5-9F09-6E4891027120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{032270A5-D7EB-4795-BB6B-F5366089E1DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>161.43</v>
+        <v>161.9</v>
       </c>
       <c r="E8" s="10">
-        <v>152.84</v>
+        <v>153.44999999999999</v>
       </c>
       <c r="F8" s="10">
-        <v>162.84</v>
+        <v>163.44999999999999</v>
       </c>
       <c r="G8" s="10">
-        <v>152.72999999999999</v>
+        <v>153.34</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>161.43</v>
+        <v>161.9</v>
       </c>
       <c r="E9" s="13">
-        <v>152.84</v>
+        <v>153.44999999999999</v>
       </c>
       <c r="F9" s="13">
-        <v>162.84</v>
+        <v>163.44999999999999</v>
       </c>
       <c r="G9" s="13">
-        <v>152.72999999999999</v>
+        <v>153.34</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>163.19999999999999</v>
+        <v>163.22999999999999</v>
       </c>
       <c r="E10" s="10">
-        <v>155.15</v>
+        <v>155.77000000000001</v>
       </c>
       <c r="F10" s="10">
-        <v>165.15</v>
+        <v>165.77</v>
       </c>
       <c r="G10" s="10">
-        <v>155.4</v>
+        <v>156.01</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>161.47</v>
+        <v>161.43</v>
       </c>
       <c r="E11" s="13">
-        <v>152.55000000000001</v>
+        <v>152.84</v>
       </c>
       <c r="F11" s="13">
-        <v>162.55000000000001</v>
+        <v>162.84</v>
       </c>
       <c r="G11" s="13">
-        <v>152.44</v>
+        <v>152.72999999999999</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>161.47</v>
+        <v>161.43</v>
       </c>
       <c r="E12" s="10">
-        <v>152.55000000000001</v>
+        <v>152.84</v>
       </c>
       <c r="F12" s="10">
-        <v>162.55000000000001</v>
+        <v>162.84</v>
       </c>
       <c r="G12" s="10">
-        <v>152.44</v>
+        <v>152.72999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>163.26</v>
+        <v>163.19999999999999</v>
       </c>
       <c r="E13" s="13">
-        <v>154.88999999999999</v>
+        <v>155.15</v>
       </c>
       <c r="F13" s="13">
-        <v>164.89</v>
+        <v>165.15</v>
       </c>
       <c r="G13" s="13">
-        <v>155.13999999999999</v>
+        <v>155.4</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,7 +967,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
@@ -977,29 +977,29 @@
         <v>167.8</v>
       </c>
       <c r="E17" s="10">
-        <v>158.94</v>
+        <v>159.53</v>
       </c>
       <c r="F17" s="10">
-        <v>168.94</v>
+        <v>169.53</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>167.87</v>
+        <v>167.8</v>
       </c>
       <c r="E18" s="13">
-        <v>158.69</v>
+        <v>158.94</v>
       </c>
       <c r="F18" s="13">
-        <v>168.69</v>
+        <v>168.94</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>162.93</v>
+        <v>162.97</v>
       </c>
       <c r="E22" s="10">
-        <v>154.63</v>
+        <v>155.24</v>
       </c>
       <c r="F22" s="10">
-        <v>164.23</v>
+        <v>164.84</v>
       </c>
       <c r="G22" s="10">
-        <v>156.38</v>
+        <v>156.99</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>168.06</v>
+        <v>168.1</v>
       </c>
       <c r="E23" s="13">
-        <v>160.86000000000001</v>
+        <v>161.47999999999999</v>
       </c>
       <c r="F23" s="13">
-        <v>170.86</v>
+        <v>171.48</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>168.25</v>
+        <v>168.28</v>
       </c>
       <c r="E24" s="10">
-        <v>161.38999999999999</v>
+        <v>162.01</v>
       </c>
       <c r="F24" s="10">
-        <v>171.39</v>
+        <v>172.01</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>168.25</v>
+        <v>168.29</v>
       </c>
       <c r="E25" s="13">
-        <v>160.91</v>
+        <v>161.54</v>
       </c>
       <c r="F25" s="13">
-        <v>170.91</v>
+        <v>171.54</v>
       </c>
       <c r="G25" s="13">
-        <v>161.76</v>
+        <v>162.38999999999999</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>167.89</v>
+        <v>167.91</v>
       </c>
       <c r="E26" s="10">
-        <v>162.52000000000001</v>
+        <v>163.16</v>
       </c>
       <c r="F26" s="10">
-        <v>172.52</v>
+        <v>173.16</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>162.97</v>
+        <v>162.93</v>
       </c>
       <c r="E27" s="13">
-        <v>154.35</v>
+        <v>154.63</v>
       </c>
       <c r="F27" s="13">
-        <v>163.95</v>
+        <v>164.23</v>
       </c>
       <c r="G27" s="13">
-        <v>156.1</v>
+        <v>156.38</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>168.13</v>
+        <v>168.06</v>
       </c>
       <c r="E28" s="22">
-        <v>160.6</v>
+        <v>160.86000000000001</v>
       </c>
       <c r="F28" s="22">
-        <v>170.6</v>
+        <v>170.86</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>168.32</v>
+        <v>168.25</v>
       </c>
       <c r="E29" s="13">
-        <v>161.13</v>
+        <v>161.38999999999999</v>
       </c>
       <c r="F29" s="13">
-        <v>171.13</v>
+        <v>171.39</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>168.32</v>
+        <v>168.25</v>
       </c>
       <c r="E30" s="22">
-        <v>160.63999999999999</v>
+        <v>160.91</v>
       </c>
       <c r="F30" s="22">
-        <v>170.64</v>
+        <v>170.91</v>
       </c>
       <c r="G30" s="22">
-        <v>161.5</v>
+        <v>161.76</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>167.96</v>
+        <v>167.89</v>
       </c>
       <c r="E31" s="13">
-        <v>162.26</v>
+        <v>162.52000000000001</v>
       </c>
       <c r="F31" s="13">
-        <v>172.26</v>
+        <v>172.52</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>161.69</v>
+        <v>161.94999999999999</v>
       </c>
       <c r="E35" s="10">
-        <v>153.06</v>
+        <v>153.66999999999999</v>
       </c>
       <c r="F35" s="10">
-        <v>162.06</v>
+        <v>162.66999999999999</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>161.76</v>
+        <v>161.69</v>
       </c>
       <c r="E36" s="13">
-        <v>152.80000000000001</v>
+        <v>153.06</v>
       </c>
       <c r="F36" s="13">
-        <v>161.80000000000001</v>
+        <v>162.06</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>168.11</v>
+        <v>168.17</v>
       </c>
       <c r="E40" s="10">
-        <v>160.05000000000001</v>
+        <v>160.6</v>
       </c>
       <c r="F40" s="10">
-        <v>170.05</v>
+        <v>170.6</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>167.82</v>
+        <v>167.88</v>
       </c>
       <c r="E41" s="13">
-        <v>160.47</v>
+        <v>161.02000000000001</v>
       </c>
       <c r="F41" s="13">
-        <v>170.47</v>
+        <v>171.02</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>168.17</v>
+        <v>168.11</v>
       </c>
       <c r="E42" s="10">
-        <v>159.81</v>
+        <v>160.05000000000001</v>
       </c>
       <c r="F42" s="10">
-        <v>169.81</v>
+        <v>170.05</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>167.89</v>
+        <v>167.82</v>
       </c>
       <c r="E43" s="13">
-        <v>160.22999999999999</v>
+        <v>160.47</v>
       </c>
       <c r="F43" s="13">
-        <v>170.23</v>
+        <v>170.47</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>162.01</v>
+        <v>162.12</v>
       </c>
       <c r="E47" s="10">
-        <v>154.5</v>
+        <v>154.72</v>
       </c>
       <c r="F47" s="10">
-        <v>164.5</v>
+        <v>164.72</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>161.72999999999999</v>
+        <v>161.83000000000001</v>
       </c>
       <c r="E48" s="13">
-        <v>154.49</v>
+        <v>154.71</v>
       </c>
       <c r="F48" s="13">
-        <v>164.49</v>
+        <v>164.71</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>161.41</v>
+        <v>162.01</v>
       </c>
       <c r="E49" s="10">
-        <v>153</v>
+        <v>154.5</v>
       </c>
       <c r="F49" s="10">
-        <v>163</v>
+        <v>164.5</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>161.12</v>
+        <v>161.72999999999999</v>
       </c>
       <c r="E50" s="13">
-        <v>152.99</v>
+        <v>154.49</v>
       </c>
       <c r="F50" s="13">
-        <v>162.99</v>
+        <v>164.49</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>177.32</v>
+        <v>177.34</v>
       </c>
       <c r="E54" s="10">
-        <v>167.92</v>
+        <v>168.68</v>
       </c>
       <c r="F54" s="10">
-        <v>177.92</v>
+        <v>178.68</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>166.67</v>
+        <v>166.71</v>
       </c>
       <c r="E55" s="13">
-        <v>166.4</v>
+        <v>166.98</v>
       </c>
       <c r="F55" s="13">
-        <v>176.4</v>
+        <v>176.98</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>166.31</v>
+        <v>166.47</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>167.21</v>
+        <v>167.31</v>
       </c>
       <c r="E57" s="13">
-        <v>160.83000000000001</v>
+        <v>161.4</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,26 +1678,26 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>162.97999999999999</v>
+        <v>163.08000000000001</v>
       </c>
       <c r="E58" s="10">
-        <v>156.72</v>
+        <v>157.30000000000001</v>
       </c>
       <c r="F58" s="10">
-        <v>166.72</v>
+        <v>167.3</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
@@ -1707,7 +1707,7 @@
         <v>170.23</v>
       </c>
       <c r="E59" s="13">
-        <v>166.5</v>
+        <v>167.19</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>177.4</v>
+        <v>177.32</v>
       </c>
       <c r="E60" s="10">
-        <v>167.63</v>
+        <v>167.92</v>
       </c>
       <c r="F60" s="10">
-        <v>177.63</v>
+        <v>177.92</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>166.74</v>
+        <v>166.67</v>
       </c>
       <c r="E61" s="13">
-        <v>166.15</v>
+        <v>166.4</v>
       </c>
       <c r="F61" s="13">
-        <v>176.15</v>
+        <v>176.4</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>166.38</v>
+        <v>166.31</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>167.28</v>
+        <v>167.21</v>
       </c>
       <c r="E63" s="13">
-        <v>160.57</v>
+        <v>160.83000000000001</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>163.06</v>
+        <v>162.97999999999999</v>
       </c>
       <c r="E64" s="10">
-        <v>156.47</v>
+        <v>156.72</v>
       </c>
       <c r="F64" s="10">
-        <v>166.47</v>
+        <v>166.72</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46079</v>
+        <v>46080</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>170.3</v>
+        <v>170.23</v>
       </c>
       <c r="E65" s="13">
-        <v>166.22</v>
+        <v>166.5</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1859,6 +1859,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2118,17 +2129,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
@@ -2138,6 +2138,24 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2157,24 +2175,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Mon Mar  2 03:39:12 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{032270A5-D7EB-4795-BB6B-F5366089E1DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{E280D55F-C107-41DA-9B29-39BAD72E1A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>161.9</v>
+        <v>161.79</v>
       </c>
       <c r="E8" s="10">
-        <v>153.44999999999999</v>
+        <v>153.80000000000001</v>
       </c>
       <c r="F8" s="10">
-        <v>163.44999999999999</v>
+        <v>163.80000000000001</v>
       </c>
       <c r="G8" s="10">
-        <v>153.34</v>
+        <v>153.69</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>161.9</v>
+        <v>161.79</v>
       </c>
       <c r="E9" s="13">
-        <v>153.44999999999999</v>
+        <v>153.80000000000001</v>
       </c>
       <c r="F9" s="13">
-        <v>163.44999999999999</v>
+        <v>163.80000000000001</v>
       </c>
       <c r="G9" s="13">
-        <v>153.34</v>
+        <v>153.69</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>163.22999999999999</v>
+        <v>163.27000000000001</v>
       </c>
       <c r="E10" s="10">
-        <v>155.77000000000001</v>
+        <v>156.28</v>
       </c>
       <c r="F10" s="10">
-        <v>165.77</v>
+        <v>166.28</v>
       </c>
       <c r="G10" s="10">
-        <v>156.01</v>
+        <v>156.52000000000001</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>161.43</v>
+        <v>161.9</v>
       </c>
       <c r="E11" s="13">
-        <v>152.84</v>
+        <v>153.44999999999999</v>
       </c>
       <c r="F11" s="13">
-        <v>162.84</v>
+        <v>163.44999999999999</v>
       </c>
       <c r="G11" s="13">
-        <v>152.72999999999999</v>
+        <v>153.34</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>161.43</v>
+        <v>161.9</v>
       </c>
       <c r="E12" s="10">
-        <v>152.84</v>
+        <v>153.44999999999999</v>
       </c>
       <c r="F12" s="10">
-        <v>162.84</v>
+        <v>163.44999999999999</v>
       </c>
       <c r="G12" s="10">
-        <v>152.72999999999999</v>
+        <v>153.34</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>163.19999999999999</v>
+        <v>163.22999999999999</v>
       </c>
       <c r="E13" s="13">
-        <v>155.15</v>
+        <v>155.77000000000001</v>
       </c>
       <c r="F13" s="13">
-        <v>165.15</v>
+        <v>165.77</v>
       </c>
       <c r="G13" s="13">
-        <v>155.4</v>
+        <v>156.01</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,26 +967,26 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>167.8</v>
+        <v>167.58</v>
       </c>
       <c r="E17" s="10">
-        <v>159.53</v>
+        <v>159.79</v>
       </c>
       <c r="F17" s="10">
-        <v>169.53</v>
+        <v>169.79</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
@@ -996,10 +996,10 @@
         <v>167.8</v>
       </c>
       <c r="E18" s="13">
-        <v>158.94</v>
+        <v>159.53</v>
       </c>
       <c r="F18" s="13">
-        <v>168.94</v>
+        <v>169.53</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>162.97</v>
+        <v>162.96</v>
       </c>
       <c r="E22" s="10">
-        <v>155.24</v>
+        <v>155.93</v>
       </c>
       <c r="F22" s="10">
-        <v>164.84</v>
+        <v>165.52</v>
       </c>
       <c r="G22" s="10">
-        <v>156.99</v>
+        <v>157.66999999999999</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>168.1</v>
+        <v>167.92</v>
       </c>
       <c r="E23" s="13">
-        <v>161.47999999999999</v>
+        <v>161.77000000000001</v>
       </c>
       <c r="F23" s="13">
-        <v>171.48</v>
+        <v>171.77</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>168.28</v>
+        <v>168.1</v>
       </c>
       <c r="E24" s="10">
-        <v>162.01</v>
+        <v>162.33000000000001</v>
       </c>
       <c r="F24" s="10">
-        <v>172.01</v>
+        <v>172.33</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>168.29</v>
+        <v>168.11</v>
       </c>
       <c r="E25" s="13">
-        <v>161.54</v>
+        <v>161.85</v>
       </c>
       <c r="F25" s="13">
-        <v>171.54</v>
+        <v>171.85</v>
       </c>
       <c r="G25" s="13">
-        <v>162.38999999999999</v>
+        <v>162.69999999999999</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>167.91</v>
+        <v>167.72</v>
       </c>
       <c r="E26" s="10">
-        <v>163.16</v>
+        <v>163.47999999999999</v>
       </c>
       <c r="F26" s="10">
-        <v>173.16</v>
+        <v>173.48</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>162.93</v>
+        <v>162.97</v>
       </c>
       <c r="E27" s="13">
-        <v>154.63</v>
+        <v>155.24</v>
       </c>
       <c r="F27" s="13">
-        <v>164.23</v>
+        <v>164.84</v>
       </c>
       <c r="G27" s="13">
-        <v>156.38</v>
+        <v>156.99</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>168.06</v>
+        <v>168.1</v>
       </c>
       <c r="E28" s="22">
-        <v>160.86000000000001</v>
+        <v>161.47999999999999</v>
       </c>
       <c r="F28" s="22">
-        <v>170.86</v>
+        <v>171.48</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>168.25</v>
+        <v>168.28</v>
       </c>
       <c r="E29" s="13">
-        <v>161.38999999999999</v>
+        <v>162.01</v>
       </c>
       <c r="F29" s="13">
-        <v>171.39</v>
+        <v>172.01</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>168.25</v>
+        <v>168.29</v>
       </c>
       <c r="E30" s="22">
-        <v>160.91</v>
+        <v>161.54</v>
       </c>
       <c r="F30" s="22">
-        <v>170.91</v>
+        <v>171.54</v>
       </c>
       <c r="G30" s="22">
-        <v>161.76</v>
+        <v>162.38999999999999</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>167.89</v>
+        <v>167.91</v>
       </c>
       <c r="E31" s="13">
-        <v>162.52000000000001</v>
+        <v>163.16</v>
       </c>
       <c r="F31" s="13">
-        <v>172.52</v>
+        <v>173.16</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>161.94999999999999</v>
+        <v>161.78</v>
       </c>
       <c r="E35" s="10">
-        <v>153.66999999999999</v>
+        <v>153.97999999999999</v>
       </c>
       <c r="F35" s="10">
-        <v>162.66999999999999</v>
+        <v>162.97999999999999</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>161.69</v>
+        <v>161.94999999999999</v>
       </c>
       <c r="E36" s="13">
-        <v>153.06</v>
+        <v>153.66999999999999</v>
       </c>
       <c r="F36" s="13">
-        <v>162.06</v>
+        <v>162.66999999999999</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>168.17</v>
+        <v>168.02</v>
       </c>
       <c r="E40" s="10">
-        <v>160.6</v>
+        <v>160.91</v>
       </c>
       <c r="F40" s="10">
-        <v>170.6</v>
+        <v>170.91</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>167.88</v>
+        <v>167.74</v>
       </c>
       <c r="E41" s="13">
-        <v>161.02000000000001</v>
+        <v>161.33000000000001</v>
       </c>
       <c r="F41" s="13">
-        <v>171.02</v>
+        <v>171.33</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>168.11</v>
+        <v>168.17</v>
       </c>
       <c r="E42" s="10">
-        <v>160.05000000000001</v>
+        <v>160.6</v>
       </c>
       <c r="F42" s="10">
-        <v>170.05</v>
+        <v>170.6</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>167.82</v>
+        <v>167.88</v>
       </c>
       <c r="E43" s="13">
-        <v>160.47</v>
+        <v>161.02000000000001</v>
       </c>
       <c r="F43" s="13">
-        <v>170.47</v>
+        <v>171.02</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>162.12</v>
+        <v>162.46</v>
       </c>
       <c r="E47" s="10">
-        <v>154.72</v>
+        <v>154.91</v>
       </c>
       <c r="F47" s="10">
-        <v>164.72</v>
+        <v>164.91</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>161.83000000000001</v>
+        <v>162.16</v>
       </c>
       <c r="E48" s="13">
-        <v>154.71</v>
+        <v>154.9</v>
       </c>
       <c r="F48" s="13">
-        <v>164.71</v>
+        <v>164.9</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>162.01</v>
+        <v>162.12</v>
       </c>
       <c r="E49" s="10">
-        <v>154.5</v>
+        <v>154.72</v>
       </c>
       <c r="F49" s="10">
-        <v>164.5</v>
+        <v>164.72</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>161.72999999999999</v>
+        <v>161.83000000000001</v>
       </c>
       <c r="E50" s="13">
-        <v>154.49</v>
+        <v>154.71</v>
       </c>
       <c r="F50" s="13">
-        <v>164.49</v>
+        <v>164.71</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>177.34</v>
+        <v>177.13</v>
       </c>
       <c r="E54" s="10">
-        <v>168.68</v>
+        <v>169.17</v>
       </c>
       <c r="F54" s="10">
-        <v>178.68</v>
+        <v>179.17</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>166.71</v>
+        <v>166.52</v>
       </c>
       <c r="E55" s="13">
-        <v>166.98</v>
+        <v>167.45</v>
       </c>
       <c r="F55" s="13">
-        <v>176.98</v>
+        <v>177.45</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>166.47</v>
+        <v>166.3</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>167.31</v>
+        <v>167.08</v>
       </c>
       <c r="E57" s="13">
-        <v>161.4</v>
+        <v>161.87</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>163.08000000000001</v>
+        <v>162.85</v>
       </c>
       <c r="E58" s="10">
-        <v>157.30000000000001</v>
+        <v>157.77000000000001</v>
       </c>
       <c r="F58" s="10">
-        <v>167.3</v>
+        <v>167.77</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>170.23</v>
+        <v>170</v>
       </c>
       <c r="E59" s="13">
-        <v>167.19</v>
+        <v>167.59</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>177.32</v>
+        <v>177.34</v>
       </c>
       <c r="E60" s="10">
-        <v>167.92</v>
+        <v>168.68</v>
       </c>
       <c r="F60" s="10">
-        <v>177.92</v>
+        <v>178.68</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>166.67</v>
+        <v>166.71</v>
       </c>
       <c r="E61" s="13">
-        <v>166.4</v>
+        <v>166.98</v>
       </c>
       <c r="F61" s="13">
-        <v>176.4</v>
+        <v>176.98</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>166.31</v>
+        <v>166.47</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>167.21</v>
+        <v>167.31</v>
       </c>
       <c r="E63" s="13">
-        <v>160.83000000000001</v>
+        <v>161.4</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,26 +1792,26 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>162.97999999999999</v>
+        <v>163.08000000000001</v>
       </c>
       <c r="E64" s="10">
-        <v>156.72</v>
+        <v>157.30000000000001</v>
       </c>
       <c r="F64" s="10">
-        <v>166.72</v>
+        <v>167.3</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46080</v>
+        <v>46081</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
@@ -1821,7 +1821,7 @@
         <v>170.23</v>
       </c>
       <c r="E65" s="13">
-        <v>166.5</v>
+        <v>167.19</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,26 +1850,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2129,10 +2109,42 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2156,21 +2168,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Tue Mar  3 03:42:26 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{E280D55F-C107-41DA-9B29-39BAD72E1A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{6A66887F-5BF0-47F8-B44B-D76163ABF89E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>161.79</v>
+        <v>166.72</v>
       </c>
       <c r="E8" s="10">
-        <v>153.80000000000001</v>
+        <v>156.69999999999999</v>
       </c>
       <c r="F8" s="10">
-        <v>163.80000000000001</v>
+        <v>166.7</v>
       </c>
       <c r="G8" s="10">
-        <v>153.69</v>
+        <v>156.59</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>161.79</v>
+        <v>166.72</v>
       </c>
       <c r="E9" s="13">
-        <v>153.80000000000001</v>
+        <v>156.69999999999999</v>
       </c>
       <c r="F9" s="13">
-        <v>163.80000000000001</v>
+        <v>166.7</v>
       </c>
       <c r="G9" s="13">
-        <v>153.69</v>
+        <v>156.59</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>163.27000000000001</v>
+        <v>167.85</v>
       </c>
       <c r="E10" s="10">
-        <v>156.28</v>
+        <v>158.41999999999999</v>
       </c>
       <c r="F10" s="10">
-        <v>166.28</v>
+        <v>168.42</v>
       </c>
       <c r="G10" s="10">
-        <v>156.52000000000001</v>
+        <v>158.66</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>161.9</v>
+        <v>161.79</v>
       </c>
       <c r="E11" s="13">
-        <v>153.44999999999999</v>
+        <v>153.80000000000001</v>
       </c>
       <c r="F11" s="13">
-        <v>163.44999999999999</v>
+        <v>163.80000000000001</v>
       </c>
       <c r="G11" s="13">
-        <v>153.34</v>
+        <v>153.69</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>161.9</v>
+        <v>161.79</v>
       </c>
       <c r="E12" s="10">
-        <v>153.44999999999999</v>
+        <v>153.80000000000001</v>
       </c>
       <c r="F12" s="10">
-        <v>163.44999999999999</v>
+        <v>163.80000000000001</v>
       </c>
       <c r="G12" s="10">
-        <v>153.34</v>
+        <v>153.69</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>163.22999999999999</v>
+        <v>163.27000000000001</v>
       </c>
       <c r="E13" s="13">
-        <v>155.77000000000001</v>
+        <v>156.28</v>
       </c>
       <c r="F13" s="13">
-        <v>165.77</v>
+        <v>166.28</v>
       </c>
       <c r="G13" s="13">
-        <v>156.01</v>
+        <v>156.52000000000001</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>167.58</v>
+        <v>172.13</v>
       </c>
       <c r="E17" s="10">
-        <v>159.79</v>
+        <v>162.35</v>
       </c>
       <c r="F17" s="10">
-        <v>169.79</v>
+        <v>172.35</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>167.8</v>
+        <v>167.58</v>
       </c>
       <c r="E18" s="13">
-        <v>159.53</v>
+        <v>159.79</v>
       </c>
       <c r="F18" s="13">
-        <v>169.53</v>
+        <v>169.79</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>162.96</v>
+        <v>167.67</v>
       </c>
       <c r="E22" s="10">
-        <v>155.93</v>
+        <v>158.27000000000001</v>
       </c>
       <c r="F22" s="10">
-        <v>165.52</v>
+        <v>167.87</v>
       </c>
       <c r="G22" s="10">
-        <v>157.66999999999999</v>
+        <v>160.02000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>167.92</v>
+        <v>172.51</v>
       </c>
       <c r="E23" s="13">
-        <v>161.77000000000001</v>
+        <v>164.36</v>
       </c>
       <c r="F23" s="13">
-        <v>171.77</v>
+        <v>174.36</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>168.1</v>
+        <v>172.69</v>
       </c>
       <c r="E24" s="10">
-        <v>162.33000000000001</v>
+        <v>164.92</v>
       </c>
       <c r="F24" s="10">
-        <v>172.33</v>
+        <v>174.92</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>168.11</v>
+        <v>172.69</v>
       </c>
       <c r="E25" s="13">
-        <v>161.85</v>
+        <v>164.45</v>
       </c>
       <c r="F25" s="13">
-        <v>171.85</v>
+        <v>174.45</v>
       </c>
       <c r="G25" s="13">
-        <v>162.69999999999999</v>
+        <v>165.3</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>167.72</v>
+        <v>172.3</v>
       </c>
       <c r="E26" s="10">
-        <v>163.47999999999999</v>
+        <v>166.09</v>
       </c>
       <c r="F26" s="10">
-        <v>173.48</v>
+        <v>176.09</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>162.97</v>
+        <v>162.96</v>
       </c>
       <c r="E27" s="13">
-        <v>155.24</v>
+        <v>155.93</v>
       </c>
       <c r="F27" s="13">
-        <v>164.84</v>
+        <v>165.52</v>
       </c>
       <c r="G27" s="13">
-        <v>156.99</v>
+        <v>157.66999999999999</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>168.1</v>
+        <v>167.92</v>
       </c>
       <c r="E28" s="22">
-        <v>161.47999999999999</v>
+        <v>161.77000000000001</v>
       </c>
       <c r="F28" s="22">
-        <v>171.48</v>
+        <v>171.77</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>168.28</v>
+        <v>168.1</v>
       </c>
       <c r="E29" s="13">
-        <v>162.01</v>
+        <v>162.33000000000001</v>
       </c>
       <c r="F29" s="13">
-        <v>172.01</v>
+        <v>172.33</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>168.29</v>
+        <v>168.11</v>
       </c>
       <c r="E30" s="22">
-        <v>161.54</v>
+        <v>161.85</v>
       </c>
       <c r="F30" s="22">
-        <v>171.54</v>
+        <v>171.85</v>
       </c>
       <c r="G30" s="22">
-        <v>162.38999999999999</v>
+        <v>162.69999999999999</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>167.91</v>
+        <v>167.72</v>
       </c>
       <c r="E31" s="13">
-        <v>163.16</v>
+        <v>163.47999999999999</v>
       </c>
       <c r="F31" s="13">
-        <v>173.16</v>
+        <v>173.48</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>161.78</v>
+        <v>166.36</v>
       </c>
       <c r="E35" s="10">
-        <v>153.97999999999999</v>
+        <v>156.55000000000001</v>
       </c>
       <c r="F35" s="10">
-        <v>162.97999999999999</v>
+        <v>165.55</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>161.94999999999999</v>
+        <v>161.78</v>
       </c>
       <c r="E36" s="13">
-        <v>153.66999999999999</v>
+        <v>153.97999999999999</v>
       </c>
       <c r="F36" s="13">
-        <v>162.66999999999999</v>
+        <v>162.97999999999999</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>168.02</v>
+        <v>172.63</v>
       </c>
       <c r="E40" s="10">
-        <v>160.91</v>
+        <v>163.49</v>
       </c>
       <c r="F40" s="10">
-        <v>170.91</v>
+        <v>173.49</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>167.74</v>
+        <v>172.34</v>
       </c>
       <c r="E41" s="13">
-        <v>161.33000000000001</v>
+        <v>163.91</v>
       </c>
       <c r="F41" s="13">
-        <v>171.33</v>
+        <v>173.91</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>168.17</v>
+        <v>168.02</v>
       </c>
       <c r="E42" s="10">
-        <v>160.6</v>
+        <v>160.91</v>
       </c>
       <c r="F42" s="10">
-        <v>170.6</v>
+        <v>170.91</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>167.88</v>
+        <v>167.74</v>
       </c>
       <c r="E43" s="13">
-        <v>161.02000000000001</v>
+        <v>161.33000000000001</v>
       </c>
       <c r="F43" s="13">
-        <v>171.02</v>
+        <v>171.33</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>162.46</v>
+        <v>165.49</v>
       </c>
       <c r="E47" s="10">
-        <v>154.91</v>
+        <v>156.96</v>
       </c>
       <c r="F47" s="10">
-        <v>164.91</v>
+        <v>166.96</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>162.16</v>
+        <v>165.18</v>
       </c>
       <c r="E48" s="13">
-        <v>154.9</v>
+        <v>156.94999999999999</v>
       </c>
       <c r="F48" s="13">
-        <v>164.9</v>
+        <v>166.95</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>162.12</v>
+        <v>162.46</v>
       </c>
       <c r="E49" s="10">
-        <v>154.72</v>
+        <v>154.91</v>
       </c>
       <c r="F49" s="10">
-        <v>164.72</v>
+        <v>164.91</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>161.83000000000001</v>
+        <v>162.16</v>
       </c>
       <c r="E50" s="13">
-        <v>154.71</v>
+        <v>154.9</v>
       </c>
       <c r="F50" s="13">
-        <v>164.71</v>
+        <v>164.9</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>177.13</v>
+        <v>181.71</v>
       </c>
       <c r="E54" s="10">
-        <v>169.17</v>
+        <v>171.88</v>
       </c>
       <c r="F54" s="10">
-        <v>179.17</v>
+        <v>181.89</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>166.52</v>
+        <v>171.11</v>
       </c>
       <c r="E55" s="13">
-        <v>167.45</v>
+        <v>169.44</v>
       </c>
       <c r="F55" s="13">
-        <v>177.45</v>
+        <v>179.44</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>166.3</v>
+        <v>170.88</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>167.08</v>
+        <v>171.61</v>
       </c>
       <c r="E57" s="13">
-        <v>161.87</v>
+        <v>163.86</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>162.85</v>
+        <v>167.39</v>
       </c>
       <c r="E58" s="10">
-        <v>157.77000000000001</v>
+        <v>159.76</v>
       </c>
       <c r="F58" s="10">
-        <v>167.77</v>
+        <v>169.76</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>170</v>
+        <v>174.54</v>
       </c>
       <c r="E59" s="13">
-        <v>167.59</v>
+        <v>170.25</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>177.34</v>
+        <v>177.13</v>
       </c>
       <c r="E60" s="10">
-        <v>168.68</v>
+        <v>169.17</v>
       </c>
       <c r="F60" s="10">
-        <v>178.68</v>
+        <v>179.17</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>166.71</v>
+        <v>166.52</v>
       </c>
       <c r="E61" s="13">
-        <v>166.98</v>
+        <v>167.45</v>
       </c>
       <c r="F61" s="13">
-        <v>176.98</v>
+        <v>177.45</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>166.47</v>
+        <v>166.3</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>167.31</v>
+        <v>167.08</v>
       </c>
       <c r="E63" s="13">
-        <v>161.4</v>
+        <v>161.87</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>163.08000000000001</v>
+        <v>162.85</v>
       </c>
       <c r="E64" s="10">
-        <v>157.30000000000001</v>
+        <v>157.77000000000001</v>
       </c>
       <c r="F64" s="10">
-        <v>167.3</v>
+        <v>167.77</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46081</v>
+        <v>46084</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>170.23</v>
+        <v>170</v>
       </c>
       <c r="E65" s="13">
-        <v>167.19</v>
+        <v>167.59</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,6 +1850,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2109,42 +2129,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2168,9 +2156,21 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Wed Mar  4 03:34:31 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{6A66887F-5BF0-47F8-B44B-D76163ABF89E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{812D32C0-291C-4ADC-9FFA-76150638A439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>166.72</v>
+        <v>173.96</v>
       </c>
       <c r="E8" s="10">
-        <v>156.69999999999999</v>
+        <v>161.30000000000001</v>
       </c>
       <c r="F8" s="10">
-        <v>166.7</v>
+        <v>171.3</v>
       </c>
       <c r="G8" s="10">
-        <v>156.59</v>
+        <v>161.18</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>166.72</v>
+        <v>173.96</v>
       </c>
       <c r="E9" s="13">
-        <v>156.69999999999999</v>
+        <v>161.30000000000001</v>
       </c>
       <c r="F9" s="13">
-        <v>166.7</v>
+        <v>171.3</v>
       </c>
       <c r="G9" s="13">
-        <v>156.59</v>
+        <v>161.18</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>167.85</v>
+        <v>174.94</v>
       </c>
       <c r="E10" s="10">
-        <v>158.41999999999999</v>
+        <v>162.4</v>
       </c>
       <c r="F10" s="10">
-        <v>168.42</v>
+        <v>172.4</v>
       </c>
       <c r="G10" s="10">
-        <v>158.66</v>
+        <v>162.63999999999999</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>161.79</v>
+        <v>166.72</v>
       </c>
       <c r="E11" s="13">
-        <v>153.80000000000001</v>
+        <v>156.69999999999999</v>
       </c>
       <c r="F11" s="13">
-        <v>163.80000000000001</v>
+        <v>166.7</v>
       </c>
       <c r="G11" s="13">
-        <v>153.69</v>
+        <v>156.59</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>161.79</v>
+        <v>166.72</v>
       </c>
       <c r="E12" s="10">
-        <v>153.80000000000001</v>
+        <v>156.69999999999999</v>
       </c>
       <c r="F12" s="10">
-        <v>163.80000000000001</v>
+        <v>166.7</v>
       </c>
       <c r="G12" s="10">
-        <v>153.69</v>
+        <v>156.59</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>163.27000000000001</v>
+        <v>167.85</v>
       </c>
       <c r="E13" s="13">
-        <v>156.28</v>
+        <v>158.41999999999999</v>
       </c>
       <c r="F13" s="13">
-        <v>166.28</v>
+        <v>168.42</v>
       </c>
       <c r="G13" s="13">
-        <v>156.52000000000001</v>
+        <v>158.66</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>172.13</v>
+        <v>178.61</v>
       </c>
       <c r="E17" s="10">
-        <v>162.35</v>
+        <v>165.73</v>
       </c>
       <c r="F17" s="10">
-        <v>172.35</v>
+        <v>175.73</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>167.58</v>
+        <v>172.13</v>
       </c>
       <c r="E18" s="13">
-        <v>159.79</v>
+        <v>162.35</v>
       </c>
       <c r="F18" s="13">
-        <v>169.79</v>
+        <v>172.35</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>167.67</v>
+        <v>174.8</v>
       </c>
       <c r="E22" s="10">
-        <v>158.27000000000001</v>
+        <v>162.31</v>
       </c>
       <c r="F22" s="10">
-        <v>167.87</v>
+        <v>171.91</v>
       </c>
       <c r="G22" s="10">
-        <v>160.02000000000001</v>
+        <v>164.06</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>172.51</v>
+        <v>179.61</v>
       </c>
       <c r="E23" s="13">
-        <v>164.36</v>
+        <v>168.12</v>
       </c>
       <c r="F23" s="13">
-        <v>174.36</v>
+        <v>178.12</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>172.69</v>
+        <v>179.78</v>
       </c>
       <c r="E24" s="10">
-        <v>164.92</v>
+        <v>168.7</v>
       </c>
       <c r="F24" s="10">
-        <v>174.92</v>
+        <v>178.7</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>172.69</v>
+        <v>179.78</v>
       </c>
       <c r="E25" s="13">
-        <v>164.45</v>
+        <v>168.25</v>
       </c>
       <c r="F25" s="13">
-        <v>174.45</v>
+        <v>178.25</v>
       </c>
       <c r="G25" s="13">
-        <v>165.3</v>
+        <v>169.09</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>172.3</v>
+        <v>179.37</v>
       </c>
       <c r="E26" s="10">
-        <v>166.09</v>
+        <v>169.91</v>
       </c>
       <c r="F26" s="10">
-        <v>176.09</v>
+        <v>179.91</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>162.96</v>
+        <v>167.67</v>
       </c>
       <c r="E27" s="13">
-        <v>155.93</v>
+        <v>158.27000000000001</v>
       </c>
       <c r="F27" s="13">
-        <v>165.52</v>
+        <v>167.87</v>
       </c>
       <c r="G27" s="13">
-        <v>157.66999999999999</v>
+        <v>160.02000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>167.92</v>
+        <v>172.51</v>
       </c>
       <c r="E28" s="22">
-        <v>161.77000000000001</v>
+        <v>164.36</v>
       </c>
       <c r="F28" s="22">
-        <v>171.77</v>
+        <v>174.36</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>168.1</v>
+        <v>172.69</v>
       </c>
       <c r="E29" s="13">
-        <v>162.33000000000001</v>
+        <v>164.92</v>
       </c>
       <c r="F29" s="13">
-        <v>172.33</v>
+        <v>174.92</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>168.11</v>
+        <v>172.69</v>
       </c>
       <c r="E30" s="22">
-        <v>161.85</v>
+        <v>164.45</v>
       </c>
       <c r="F30" s="22">
-        <v>171.85</v>
+        <v>174.45</v>
       </c>
       <c r="G30" s="22">
-        <v>162.69999999999999</v>
+        <v>165.3</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>167.72</v>
+        <v>172.3</v>
       </c>
       <c r="E31" s="13">
-        <v>163.47999999999999</v>
+        <v>166.09</v>
       </c>
       <c r="F31" s="13">
-        <v>173.48</v>
+        <v>176.09</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>166.36</v>
+        <v>172.57</v>
       </c>
       <c r="E35" s="10">
-        <v>156.55000000000001</v>
+        <v>159.97999999999999</v>
       </c>
       <c r="F35" s="10">
-        <v>165.55</v>
+        <v>168.98</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>161.78</v>
+        <v>166.36</v>
       </c>
       <c r="E36" s="13">
-        <v>153.97999999999999</v>
+        <v>156.55000000000001</v>
       </c>
       <c r="F36" s="13">
-        <v>162.97999999999999</v>
+        <v>165.55</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>172.63</v>
+        <v>179.23</v>
       </c>
       <c r="E40" s="10">
-        <v>163.49</v>
+        <v>166.85</v>
       </c>
       <c r="F40" s="10">
-        <v>173.49</v>
+        <v>176.85</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>172.34</v>
+        <v>178.93</v>
       </c>
       <c r="E41" s="13">
-        <v>163.91</v>
+        <v>167.27</v>
       </c>
       <c r="F41" s="13">
-        <v>173.91</v>
+        <v>177.27</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>168.02</v>
+        <v>172.63</v>
       </c>
       <c r="E42" s="10">
-        <v>160.91</v>
+        <v>163.49</v>
       </c>
       <c r="F42" s="10">
-        <v>170.91</v>
+        <v>173.49</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>167.74</v>
+        <v>172.34</v>
       </c>
       <c r="E43" s="13">
-        <v>161.33000000000001</v>
+        <v>163.91</v>
       </c>
       <c r="F43" s="13">
-        <v>171.33</v>
+        <v>173.91</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>165.49</v>
+        <v>169.85</v>
       </c>
       <c r="E47" s="10">
-        <v>156.96</v>
+        <v>159.80000000000001</v>
       </c>
       <c r="F47" s="10">
-        <v>166.96</v>
+        <v>169.8</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>165.18</v>
+        <v>169.54</v>
       </c>
       <c r="E48" s="13">
-        <v>156.94999999999999</v>
+        <v>159.79</v>
       </c>
       <c r="F48" s="13">
-        <v>166.95</v>
+        <v>169.79</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>162.46</v>
+        <v>165.49</v>
       </c>
       <c r="E49" s="10">
-        <v>154.91</v>
+        <v>156.96</v>
       </c>
       <c r="F49" s="10">
-        <v>164.91</v>
+        <v>166.96</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>162.16</v>
+        <v>165.18</v>
       </c>
       <c r="E50" s="13">
-        <v>154.9</v>
+        <v>156.94999999999999</v>
       </c>
       <c r="F50" s="13">
-        <v>164.9</v>
+        <v>166.95</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>181.71</v>
+        <v>188.24</v>
       </c>
       <c r="E54" s="10">
-        <v>171.88</v>
+        <v>175.57</v>
       </c>
       <c r="F54" s="10">
-        <v>181.89</v>
+        <v>185.57</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>171.11</v>
+        <v>177.66</v>
       </c>
       <c r="E55" s="13">
-        <v>169.44</v>
+        <v>173.34</v>
       </c>
       <c r="F55" s="13">
-        <v>179.44</v>
+        <v>183.34</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>170.88</v>
+        <v>177.66</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>171.61</v>
+        <v>178.28</v>
       </c>
       <c r="E57" s="13">
-        <v>163.86</v>
+        <v>167.75</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>167.39</v>
+        <v>174.06</v>
       </c>
       <c r="E58" s="10">
-        <v>159.76</v>
+        <v>163.66</v>
       </c>
       <c r="F58" s="10">
-        <v>169.76</v>
+        <v>173.66</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>174.54</v>
+        <v>181.01</v>
       </c>
       <c r="E59" s="13">
-        <v>170.25</v>
+        <v>173.83</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>177.13</v>
+        <v>181.71</v>
       </c>
       <c r="E60" s="10">
-        <v>169.17</v>
+        <v>171.88</v>
       </c>
       <c r="F60" s="10">
-        <v>179.17</v>
+        <v>181.89</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>166.52</v>
+        <v>171.11</v>
       </c>
       <c r="E61" s="13">
-        <v>167.45</v>
+        <v>169.44</v>
       </c>
       <c r="F61" s="13">
-        <v>177.45</v>
+        <v>179.44</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>166.3</v>
+        <v>170.88</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>167.08</v>
+        <v>171.61</v>
       </c>
       <c r="E63" s="13">
-        <v>161.87</v>
+        <v>163.86</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>162.85</v>
+        <v>167.39</v>
       </c>
       <c r="E64" s="10">
-        <v>157.77000000000001</v>
+        <v>159.76</v>
       </c>
       <c r="F64" s="10">
-        <v>167.77</v>
+        <v>169.76</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>170</v>
+        <v>174.54</v>
       </c>
       <c r="E65" s="13">
-        <v>167.59</v>
+        <v>170.25</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1859,17 +1859,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2129,6 +2118,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
@@ -2138,24 +2138,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2175,6 +2157,24 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Thu Mar  5 03:38:02 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{812D32C0-291C-4ADC-9FFA-76150638A439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{5EABC69B-65C2-4DF9-AD34-FC9F7A30FA7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>173.96</v>
+        <v>188.78</v>
       </c>
       <c r="E8" s="10">
-        <v>161.30000000000001</v>
+        <v>167.95</v>
       </c>
       <c r="F8" s="10">
-        <v>171.3</v>
+        <v>177.95</v>
       </c>
       <c r="G8" s="10">
-        <v>161.18</v>
+        <v>167.84</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>173.96</v>
+        <v>188.78</v>
       </c>
       <c r="E9" s="13">
-        <v>161.30000000000001</v>
+        <v>167.95</v>
       </c>
       <c r="F9" s="13">
-        <v>171.3</v>
+        <v>177.95</v>
       </c>
       <c r="G9" s="13">
-        <v>161.18</v>
+        <v>167.84</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>174.94</v>
+        <v>185.8</v>
       </c>
       <c r="E10" s="10">
-        <v>162.4</v>
+        <v>167.37</v>
       </c>
       <c r="F10" s="10">
-        <v>172.4</v>
+        <v>177.37</v>
       </c>
       <c r="G10" s="10">
-        <v>162.63999999999999</v>
+        <v>167.61</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>166.72</v>
+        <v>173.96</v>
       </c>
       <c r="E11" s="13">
-        <v>156.69999999999999</v>
+        <v>161.30000000000001</v>
       </c>
       <c r="F11" s="13">
-        <v>166.7</v>
+        <v>171.3</v>
       </c>
       <c r="G11" s="13">
-        <v>156.59</v>
+        <v>161.18</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>166.72</v>
+        <v>173.96</v>
       </c>
       <c r="E12" s="10">
-        <v>156.69999999999999</v>
+        <v>161.30000000000001</v>
       </c>
       <c r="F12" s="10">
-        <v>166.7</v>
+        <v>171.3</v>
       </c>
       <c r="G12" s="10">
-        <v>156.59</v>
+        <v>161.18</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>167.85</v>
+        <v>174.94</v>
       </c>
       <c r="E13" s="13">
-        <v>158.41999999999999</v>
+        <v>162.4</v>
       </c>
       <c r="F13" s="13">
-        <v>168.42</v>
+        <v>172.4</v>
       </c>
       <c r="G13" s="13">
-        <v>158.66</v>
+        <v>162.63999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>178.61</v>
+        <v>189.39</v>
       </c>
       <c r="E17" s="10">
-        <v>165.73</v>
+        <v>170.65</v>
       </c>
       <c r="F17" s="10">
-        <v>175.73</v>
+        <v>180.65</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>172.13</v>
+        <v>178.61</v>
       </c>
       <c r="E18" s="13">
-        <v>162.35</v>
+        <v>165.73</v>
       </c>
       <c r="F18" s="13">
-        <v>172.35</v>
+        <v>175.73</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>174.8</v>
+        <v>186.31</v>
       </c>
       <c r="E22" s="10">
-        <v>162.31</v>
+        <v>167.87</v>
       </c>
       <c r="F22" s="10">
-        <v>171.91</v>
+        <v>177.47</v>
       </c>
       <c r="G22" s="10">
-        <v>164.06</v>
+        <v>169.62</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>179.61</v>
+        <v>190.48</v>
       </c>
       <c r="E23" s="13">
-        <v>168.12</v>
+        <v>173.09</v>
       </c>
       <c r="F23" s="13">
-        <v>178.12</v>
+        <v>183.09</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>179.78</v>
+        <v>190.64</v>
       </c>
       <c r="E24" s="10">
-        <v>168.7</v>
+        <v>173.7</v>
       </c>
       <c r="F24" s="10">
-        <v>178.7</v>
+        <v>183.7</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>179.78</v>
+        <v>190.64</v>
       </c>
       <c r="E25" s="13">
-        <v>168.25</v>
+        <v>173.26</v>
       </c>
       <c r="F25" s="13">
-        <v>178.25</v>
+        <v>183.26</v>
       </c>
       <c r="G25" s="13">
-        <v>169.09</v>
+        <v>174.11</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>179.37</v>
+        <v>190.22</v>
       </c>
       <c r="E26" s="10">
-        <v>169.91</v>
+        <v>174.97</v>
       </c>
       <c r="F26" s="10">
-        <v>179.91</v>
+        <v>184.97</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>167.67</v>
+        <v>174.8</v>
       </c>
       <c r="E27" s="13">
-        <v>158.27000000000001</v>
+        <v>162.31</v>
       </c>
       <c r="F27" s="13">
-        <v>167.87</v>
+        <v>171.91</v>
       </c>
       <c r="G27" s="13">
-        <v>160.02000000000001</v>
+        <v>164.06</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>172.51</v>
+        <v>179.61</v>
       </c>
       <c r="E28" s="22">
-        <v>164.36</v>
+        <v>168.12</v>
       </c>
       <c r="F28" s="22">
-        <v>174.36</v>
+        <v>178.12</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>172.69</v>
+        <v>179.78</v>
       </c>
       <c r="E29" s="13">
-        <v>164.92</v>
+        <v>168.7</v>
       </c>
       <c r="F29" s="13">
-        <v>174.92</v>
+        <v>178.7</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>172.69</v>
+        <v>179.78</v>
       </c>
       <c r="E30" s="22">
-        <v>164.45</v>
+        <v>168.25</v>
       </c>
       <c r="F30" s="22">
-        <v>174.45</v>
+        <v>178.25</v>
       </c>
       <c r="G30" s="22">
-        <v>165.3</v>
+        <v>169.09</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>172.3</v>
+        <v>179.37</v>
       </c>
       <c r="E31" s="13">
-        <v>166.09</v>
+        <v>169.91</v>
       </c>
       <c r="F31" s="13">
-        <v>176.09</v>
+        <v>179.91</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>172.57</v>
+        <v>183.42</v>
       </c>
       <c r="E35" s="10">
-        <v>159.97999999999999</v>
+        <v>164.94</v>
       </c>
       <c r="F35" s="10">
-        <v>168.98</v>
+        <v>173.94</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>166.36</v>
+        <v>172.57</v>
       </c>
       <c r="E36" s="13">
-        <v>156.55000000000001</v>
+        <v>159.97999999999999</v>
       </c>
       <c r="F36" s="13">
-        <v>165.55</v>
+        <v>168.98</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>179.23</v>
+        <v>190.15</v>
       </c>
       <c r="E40" s="10">
-        <v>166.85</v>
+        <v>171.45</v>
       </c>
       <c r="F40" s="10">
-        <v>176.85</v>
+        <v>181.45</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>178.93</v>
+        <v>189.84</v>
       </c>
       <c r="E41" s="13">
-        <v>167.27</v>
+        <v>171.87</v>
       </c>
       <c r="F41" s="13">
-        <v>177.27</v>
+        <v>181.87</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>172.63</v>
+        <v>179.23</v>
       </c>
       <c r="E42" s="10">
-        <v>163.49</v>
+        <v>166.85</v>
       </c>
       <c r="F42" s="10">
-        <v>173.49</v>
+        <v>176.85</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>172.34</v>
+        <v>178.93</v>
       </c>
       <c r="E43" s="13">
-        <v>163.91</v>
+        <v>167.27</v>
       </c>
       <c r="F43" s="13">
-        <v>173.91</v>
+        <v>177.27</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>169.85</v>
+        <v>180.9</v>
       </c>
       <c r="E47" s="10">
-        <v>159.80000000000001</v>
+        <v>165.17</v>
       </c>
       <c r="F47" s="10">
-        <v>169.8</v>
+        <v>175.17</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>169.54</v>
+        <v>180.57</v>
       </c>
       <c r="E48" s="13">
-        <v>159.79</v>
+        <v>165.15</v>
       </c>
       <c r="F48" s="13">
-        <v>169.79</v>
+        <v>175.15</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>165.49</v>
+        <v>169.85</v>
       </c>
       <c r="E49" s="10">
-        <v>156.96</v>
+        <v>159.80000000000001</v>
       </c>
       <c r="F49" s="10">
-        <v>166.96</v>
+        <v>169.8</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>165.18</v>
+        <v>169.54</v>
       </c>
       <c r="E50" s="13">
-        <v>156.94999999999999</v>
+        <v>159.79</v>
       </c>
       <c r="F50" s="13">
-        <v>166.95</v>
+        <v>169.79</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>188.24</v>
+        <v>199.12</v>
       </c>
       <c r="E54" s="10">
-        <v>175.57</v>
+        <v>180.85</v>
       </c>
       <c r="F54" s="10">
-        <v>185.57</v>
+        <v>190.85</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>177.66</v>
+        <v>188.53</v>
       </c>
       <c r="E55" s="13">
-        <v>173.34</v>
+        <v>179.31</v>
       </c>
       <c r="F55" s="13">
-        <v>183.34</v>
+        <v>189.31</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>177.66</v>
+        <v>189.62</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>178.28</v>
+        <v>190.12</v>
       </c>
       <c r="E57" s="13">
-        <v>167.75</v>
+        <v>173.72</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>174.06</v>
+        <v>185.9</v>
       </c>
       <c r="E58" s="10">
-        <v>163.66</v>
+        <v>169.63</v>
       </c>
       <c r="F58" s="10">
-        <v>173.66</v>
+        <v>179.63</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>181.01</v>
+        <v>191.76</v>
       </c>
       <c r="E59" s="13">
-        <v>173.83</v>
+        <v>178.98</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>181.71</v>
+        <v>188.24</v>
       </c>
       <c r="E60" s="10">
-        <v>171.88</v>
+        <v>175.57</v>
       </c>
       <c r="F60" s="10">
-        <v>181.89</v>
+        <v>185.57</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>171.11</v>
+        <v>177.66</v>
       </c>
       <c r="E61" s="13">
-        <v>169.44</v>
+        <v>173.34</v>
       </c>
       <c r="F61" s="13">
-        <v>179.44</v>
+        <v>183.34</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>170.88</v>
+        <v>177.66</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>171.61</v>
+        <v>178.28</v>
       </c>
       <c r="E63" s="13">
-        <v>163.86</v>
+        <v>167.75</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>167.39</v>
+        <v>174.06</v>
       </c>
       <c r="E64" s="10">
-        <v>159.76</v>
+        <v>163.66</v>
       </c>
       <c r="F64" s="10">
-        <v>169.76</v>
+        <v>173.66</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>174.54</v>
+        <v>181.01</v>
       </c>
       <c r="E65" s="13">
-        <v>170.25</v>
+        <v>173.83</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,12 +1850,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2119,20 +2121,28 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2158,19 +2168,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Fri Mar  6 03:37:08 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{5EABC69B-65C2-4DF9-AD34-FC9F7A30FA7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{FA2B5EEA-648C-4B56-AF8C-4917C82CE112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -708,16 +708,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G65"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125"/>
-    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.3984375"/>
+    <col min="3" max="3" width="18.265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.86328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="6.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
       <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
@@ -728,7 +728,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -737,7 +737,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -748,7 +748,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -759,7 +759,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -768,7 +768,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A6" s="27" t="s">
         <v>3</v>
       </c>
@@ -779,7 +779,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -800,133 +800,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>188.78</v>
+        <v>201.59</v>
       </c>
       <c r="E8" s="10">
-        <v>167.95</v>
+        <v>174.51</v>
       </c>
       <c r="F8" s="10">
-        <v>177.95</v>
+        <v>184.51</v>
       </c>
       <c r="G8" s="10">
-        <v>167.84</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>174.39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>188.78</v>
+        <v>201.59</v>
       </c>
       <c r="E9" s="13">
-        <v>167.95</v>
+        <v>174.51</v>
       </c>
       <c r="F9" s="13">
-        <v>177.95</v>
+        <v>184.51</v>
       </c>
       <c r="G9" s="13">
-        <v>167.84</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>174.39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>185.8</v>
+        <v>198.03</v>
       </c>
       <c r="E10" s="10">
-        <v>167.37</v>
+        <v>173.97</v>
       </c>
       <c r="F10" s="10">
-        <v>177.37</v>
+        <v>183.97</v>
       </c>
       <c r="G10" s="10">
-        <v>167.61</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>174.21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>173.96</v>
+        <v>188.78</v>
       </c>
       <c r="E11" s="13">
-        <v>161.30000000000001</v>
+        <v>167.95</v>
       </c>
       <c r="F11" s="13">
-        <v>171.3</v>
+        <v>177.95</v>
       </c>
       <c r="G11" s="13">
-        <v>161.18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>167.84</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>173.96</v>
+        <v>188.78</v>
       </c>
       <c r="E12" s="10">
-        <v>161.30000000000001</v>
+        <v>167.95</v>
       </c>
       <c r="F12" s="10">
-        <v>171.3</v>
+        <v>177.95</v>
       </c>
       <c r="G12" s="10">
-        <v>161.18</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>167.84</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>174.94</v>
+        <v>185.8</v>
       </c>
       <c r="E13" s="13">
-        <v>162.4</v>
+        <v>167.37</v>
       </c>
       <c r="F13" s="13">
-        <v>172.4</v>
+        <v>177.37</v>
       </c>
       <c r="G13" s="13">
-        <v>162.63999999999999</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>167.61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -935,7 +935,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A15" s="27" t="s">
         <v>13</v>
       </c>
@@ -946,7 +946,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -965,45 +965,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>189.39</v>
+        <v>201.59</v>
       </c>
       <c r="E17" s="10">
-        <v>170.65</v>
+        <v>176.69</v>
       </c>
       <c r="F17" s="10">
-        <v>180.65</v>
+        <v>186.69</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>178.61</v>
+        <v>189.39</v>
       </c>
       <c r="E18" s="13">
-        <v>165.73</v>
+        <v>170.65</v>
       </c>
       <c r="F18" s="13">
-        <v>175.73</v>
+        <v>180.65</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1012,7 +1012,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A20" s="27" t="s">
         <v>15</v>
       </c>
@@ -1023,7 +1023,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1044,217 +1044,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>186.31</v>
+        <v>199.11</v>
       </c>
       <c r="E22" s="10">
-        <v>167.87</v>
+        <v>174.42</v>
       </c>
       <c r="F22" s="10">
-        <v>177.47</v>
+        <v>184.02</v>
       </c>
       <c r="G22" s="10">
-        <v>169.62</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>176.17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>190.48</v>
+        <v>203.28</v>
       </c>
       <c r="E23" s="13">
-        <v>173.09</v>
+        <v>179.71</v>
       </c>
       <c r="F23" s="13">
-        <v>183.09</v>
+        <v>189.71</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>190.64</v>
+        <v>203.43</v>
       </c>
       <c r="E24" s="10">
-        <v>173.7</v>
+        <v>180.32</v>
       </c>
       <c r="F24" s="10">
-        <v>183.7</v>
+        <v>190.32</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>190.64</v>
+        <v>203.42</v>
       </c>
       <c r="E25" s="13">
-        <v>173.26</v>
+        <v>179.9</v>
       </c>
       <c r="F25" s="13">
-        <v>183.26</v>
+        <v>189.9</v>
       </c>
       <c r="G25" s="13">
-        <v>174.11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>180.75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>190.22</v>
+        <v>203.01</v>
       </c>
       <c r="E26" s="10">
-        <v>174.97</v>
+        <v>181.65</v>
       </c>
       <c r="F26" s="10">
-        <v>184.97</v>
+        <v>191.65</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>174.8</v>
+        <v>186.31</v>
       </c>
       <c r="E27" s="13">
-        <v>162.31</v>
+        <v>167.87</v>
       </c>
       <c r="F27" s="13">
-        <v>171.91</v>
+        <v>177.47</v>
       </c>
       <c r="G27" s="13">
-        <v>164.06</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>169.62</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>179.61</v>
+        <v>190.48</v>
       </c>
       <c r="E28" s="22">
-        <v>168.12</v>
+        <v>173.09</v>
       </c>
       <c r="F28" s="22">
-        <v>178.12</v>
+        <v>183.09</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>179.78</v>
+        <v>190.64</v>
       </c>
       <c r="E29" s="13">
-        <v>168.7</v>
+        <v>173.7</v>
       </c>
       <c r="F29" s="13">
-        <v>178.7</v>
+        <v>183.7</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>179.78</v>
+        <v>190.64</v>
       </c>
       <c r="E30" s="22">
-        <v>168.25</v>
+        <v>173.26</v>
       </c>
       <c r="F30" s="22">
-        <v>178.25</v>
+        <v>183.26</v>
       </c>
       <c r="G30" s="22">
-        <v>169.09</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>174.11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>179.37</v>
+        <v>190.22</v>
       </c>
       <c r="E31" s="13">
-        <v>169.91</v>
+        <v>174.97</v>
       </c>
       <c r="F31" s="13">
-        <v>179.91</v>
+        <v>184.97</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1263,7 +1263,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A33" s="27" t="s">
         <v>22</v>
       </c>
@@ -1274,7 +1274,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1293,45 +1293,45 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>183.42</v>
+        <v>195.65</v>
       </c>
       <c r="E35" s="10">
-        <v>164.94</v>
+        <v>170.98</v>
       </c>
       <c r="F35" s="10">
-        <v>173.94</v>
+        <v>179.98</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>172.57</v>
+        <v>183.42</v>
       </c>
       <c r="E36" s="13">
-        <v>159.97999999999999</v>
+        <v>164.94</v>
       </c>
       <c r="F36" s="13">
-        <v>168.98</v>
+        <v>173.94</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="14"/>
       <c r="B37" s="14"/>
       <c r="C37" s="15"/>
@@ -1340,7 +1340,7 @@
       <c r="F37" s="16"/>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A38" s="27" t="s">
         <v>24</v>
       </c>
@@ -1351,7 +1351,7 @@
       <c r="F38" s="17"/>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" s="23" t="s">
         <v>4</v>
       </c>
@@ -1370,83 +1370,83 @@
       </c>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A40" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>190.15</v>
+        <v>202.43</v>
       </c>
       <c r="E40" s="10">
-        <v>171.45</v>
+        <v>177.09</v>
       </c>
       <c r="F40" s="10">
-        <v>181.45</v>
+        <v>187.09</v>
       </c>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>189.84</v>
+        <v>202.11</v>
       </c>
       <c r="E41" s="13">
-        <v>171.87</v>
+        <v>177.51</v>
       </c>
       <c r="F41" s="13">
-        <v>181.87</v>
+        <v>187.51</v>
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>179.23</v>
+        <v>190.15</v>
       </c>
       <c r="E42" s="10">
-        <v>166.85</v>
+        <v>171.45</v>
       </c>
       <c r="F42" s="10">
-        <v>176.85</v>
+        <v>181.45</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>178.93</v>
+        <v>189.84</v>
       </c>
       <c r="E43" s="13">
-        <v>167.27</v>
+        <v>171.87</v>
       </c>
       <c r="F43" s="13">
-        <v>177.27</v>
+        <v>181.87</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="14"/>
       <c r="B44" s="24"/>
       <c r="C44" s="15"/>
@@ -1455,7 +1455,7 @@
       <c r="F44" s="16"/>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="25" t="s">
         <v>27</v>
       </c>
@@ -1466,7 +1466,7 @@
       <c r="F45" s="17"/>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46" s="23" t="s">
         <v>4</v>
       </c>
@@ -1485,83 +1485,83 @@
       </c>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A47" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>180.9</v>
+        <v>189.49</v>
       </c>
       <c r="E47" s="10">
-        <v>165.17</v>
+        <v>171.62</v>
       </c>
       <c r="F47" s="10">
-        <v>175.17</v>
+        <v>181.62</v>
       </c>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A48" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>180.57</v>
+        <v>189.17</v>
       </c>
       <c r="E48" s="13">
-        <v>165.15</v>
+        <v>171.6</v>
       </c>
       <c r="F48" s="13">
-        <v>175.15</v>
+        <v>181.6</v>
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>169.85</v>
+        <v>180.9</v>
       </c>
       <c r="E49" s="10">
-        <v>159.80000000000001</v>
+        <v>165.17</v>
       </c>
       <c r="F49" s="10">
-        <v>169.8</v>
+        <v>175.17</v>
       </c>
       <c r="G49" s="17"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>169.54</v>
+        <v>180.57</v>
       </c>
       <c r="E50" s="13">
-        <v>159.79</v>
+        <v>165.15</v>
       </c>
       <c r="F50" s="13">
-        <v>169.79</v>
+        <v>175.15</v>
       </c>
       <c r="G50" s="17"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="14"/>
       <c r="B51" s="14"/>
       <c r="C51" s="15"/>
@@ -1570,7 +1570,7 @@
       <c r="F51" s="16"/>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A52" s="27" t="s">
         <v>30</v>
       </c>
@@ -1581,7 +1581,7 @@
       <c r="F52" s="17"/>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A53" s="23" t="s">
         <v>4</v>
       </c>
@@ -1600,54 +1600,54 @@
       </c>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A54" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>199.12</v>
+        <v>211.39</v>
       </c>
       <c r="E54" s="10">
-        <v>180.85</v>
+        <v>187.06</v>
       </c>
       <c r="F54" s="10">
-        <v>190.85</v>
+        <v>197.06</v>
       </c>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A55" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>188.53</v>
+        <v>200.79</v>
       </c>
       <c r="E55" s="13">
-        <v>179.31</v>
+        <v>185.3</v>
       </c>
       <c r="F55" s="13">
-        <v>189.31</v>
+        <v>195.3</v>
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>189.62</v>
+        <v>201.87</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1657,111 +1657,111 @@
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>190.12</v>
+        <v>202.28</v>
       </c>
       <c r="E57" s="13">
-        <v>173.72</v>
+        <v>179.71</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>185.9</v>
+        <v>198.07</v>
       </c>
       <c r="E58" s="10">
-        <v>169.63</v>
+        <v>175.62</v>
       </c>
       <c r="F58" s="10">
-        <v>179.63</v>
+        <v>185.62</v>
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>191.76</v>
+        <v>203.95</v>
       </c>
       <c r="E59" s="13">
-        <v>178.98</v>
+        <v>185.14</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>188.24</v>
+        <v>199.12</v>
       </c>
       <c r="E60" s="10">
-        <v>175.57</v>
+        <v>180.85</v>
       </c>
       <c r="F60" s="10">
-        <v>185.57</v>
+        <v>190.85</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>177.66</v>
+        <v>188.53</v>
       </c>
       <c r="E61" s="13">
-        <v>173.34</v>
+        <v>179.31</v>
       </c>
       <c r="F61" s="13">
-        <v>183.34</v>
+        <v>189.31</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>177.66</v>
+        <v>189.62</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1771,57 +1771,57 @@
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>178.28</v>
+        <v>190.12</v>
       </c>
       <c r="E63" s="13">
-        <v>167.75</v>
+        <v>173.72</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>174.06</v>
+        <v>185.9</v>
       </c>
       <c r="E64" s="10">
-        <v>163.66</v>
+        <v>169.63</v>
       </c>
       <c r="F64" s="10">
-        <v>173.66</v>
+        <v>179.63</v>
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>181.01</v>
+        <v>191.76</v>
       </c>
       <c r="E65" s="13">
-        <v>173.83</v>
+        <v>178.98</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,17 +1850,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2120,6 +2109,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2130,24 +2130,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2167,6 +2149,24 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Mon Mar  9 03:42:54 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{FA2B5EEA-648C-4B56-AF8C-4917C82CE112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{E06B1640-5FDE-4F0C-A562-91B3DEB5F92B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -708,16 +708,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G65"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.3984375"/>
-    <col min="3" max="3" width="18.265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125"/>
+    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="6.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
@@ -728,7 +728,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -737,7 +737,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -748,7 +748,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -759,7 +759,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -768,7 +768,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
         <v>3</v>
       </c>
@@ -779,7 +779,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -800,133 +800,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>201.59</v>
+        <v>216.89</v>
       </c>
       <c r="E8" s="10">
-        <v>174.51</v>
+        <v>183.97</v>
       </c>
       <c r="F8" s="10">
-        <v>184.51</v>
+        <v>193.97</v>
       </c>
       <c r="G8" s="10">
-        <v>174.39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+        <v>183.86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>201.59</v>
+        <v>216.89</v>
       </c>
       <c r="E9" s="13">
-        <v>174.51</v>
+        <v>183.97</v>
       </c>
       <c r="F9" s="13">
-        <v>184.51</v>
+        <v>193.97</v>
       </c>
       <c r="G9" s="13">
-        <v>174.39</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+        <v>183.86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>198.03</v>
+        <v>218.54</v>
       </c>
       <c r="E10" s="10">
-        <v>173.97</v>
+        <v>186.49</v>
       </c>
       <c r="F10" s="10">
-        <v>183.97</v>
+        <v>196.49</v>
       </c>
       <c r="G10" s="10">
-        <v>174.21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+        <v>186.73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>188.78</v>
+        <v>201.59</v>
       </c>
       <c r="E11" s="13">
-        <v>167.95</v>
+        <v>174.51</v>
       </c>
       <c r="F11" s="13">
-        <v>177.95</v>
+        <v>184.51</v>
       </c>
       <c r="G11" s="13">
-        <v>167.84</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+        <v>174.39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>188.78</v>
+        <v>201.59</v>
       </c>
       <c r="E12" s="10">
-        <v>167.95</v>
+        <v>174.51</v>
       </c>
       <c r="F12" s="10">
-        <v>177.95</v>
+        <v>184.51</v>
       </c>
       <c r="G12" s="10">
-        <v>167.84</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+        <v>174.39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>185.8</v>
+        <v>198.03</v>
       </c>
       <c r="E13" s="13">
-        <v>167.37</v>
+        <v>173.97</v>
       </c>
       <c r="F13" s="13">
-        <v>177.37</v>
+        <v>183.97</v>
       </c>
       <c r="G13" s="13">
-        <v>167.61</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+        <v>174.21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -935,7 +935,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
         <v>13</v>
       </c>
@@ -946,7 +946,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -965,45 +965,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>201.59</v>
+        <v>220.96</v>
       </c>
       <c r="E17" s="10">
-        <v>176.69</v>
+        <v>188.09</v>
       </c>
       <c r="F17" s="10">
-        <v>186.69</v>
+        <v>198.09</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>189.39</v>
+        <v>201.59</v>
       </c>
       <c r="E18" s="13">
-        <v>170.65</v>
+        <v>176.69</v>
       </c>
       <c r="F18" s="13">
-        <v>180.65</v>
+        <v>186.69</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1012,7 +1012,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
         <v>15</v>
       </c>
@@ -1023,7 +1023,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1044,217 +1044,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>199.11</v>
+        <v>216.6</v>
       </c>
       <c r="E22" s="10">
-        <v>174.42</v>
+        <v>186.08</v>
       </c>
       <c r="F22" s="10">
-        <v>184.02</v>
+        <v>195.68</v>
       </c>
       <c r="G22" s="10">
-        <v>176.17</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+        <v>187.83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>203.28</v>
+        <v>223.8</v>
       </c>
       <c r="E23" s="13">
-        <v>179.71</v>
+        <v>192.24</v>
       </c>
       <c r="F23" s="13">
-        <v>189.71</v>
+        <v>202.24</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>203.43</v>
+        <v>223.94</v>
       </c>
       <c r="E24" s="10">
-        <v>180.32</v>
+        <v>192.84</v>
       </c>
       <c r="F24" s="10">
-        <v>190.32</v>
+        <v>202.84</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>203.42</v>
+        <v>223.93</v>
       </c>
       <c r="E25" s="13">
-        <v>179.9</v>
+        <v>192.44</v>
       </c>
       <c r="F25" s="13">
-        <v>189.9</v>
+        <v>202.44</v>
       </c>
       <c r="G25" s="13">
-        <v>180.75</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+        <v>193.29</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>203.01</v>
+        <v>223.52</v>
       </c>
       <c r="E26" s="10">
-        <v>181.65</v>
+        <v>194.26</v>
       </c>
       <c r="F26" s="10">
-        <v>191.65</v>
+        <v>204.26</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>186.31</v>
+        <v>199.11</v>
       </c>
       <c r="E27" s="13">
-        <v>167.87</v>
+        <v>174.42</v>
       </c>
       <c r="F27" s="13">
-        <v>177.47</v>
+        <v>184.02</v>
       </c>
       <c r="G27" s="13">
-        <v>169.62</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+        <v>176.17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>190.48</v>
+        <v>203.28</v>
       </c>
       <c r="E28" s="22">
-        <v>173.09</v>
+        <v>179.71</v>
       </c>
       <c r="F28" s="22">
-        <v>183.09</v>
+        <v>189.71</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>190.64</v>
+        <v>203.43</v>
       </c>
       <c r="E29" s="13">
-        <v>173.7</v>
+        <v>180.32</v>
       </c>
       <c r="F29" s="13">
-        <v>183.7</v>
+        <v>190.32</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>190.64</v>
+        <v>203.42</v>
       </c>
       <c r="E30" s="22">
-        <v>173.26</v>
+        <v>179.9</v>
       </c>
       <c r="F30" s="22">
-        <v>183.26</v>
+        <v>189.9</v>
       </c>
       <c r="G30" s="22">
-        <v>174.11</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+        <v>180.75</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>190.22</v>
+        <v>203.01</v>
       </c>
       <c r="E31" s="13">
-        <v>174.97</v>
+        <v>181.65</v>
       </c>
       <c r="F31" s="13">
-        <v>184.97</v>
+        <v>191.65</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1263,7 +1263,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="27" t="s">
         <v>22</v>
       </c>
@@ -1274,7 +1274,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1293,45 +1293,45 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>195.65</v>
+        <v>216.14</v>
       </c>
       <c r="E35" s="10">
-        <v>170.98</v>
+        <v>184.58</v>
       </c>
       <c r="F35" s="10">
-        <v>179.98</v>
+        <v>193.58</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>183.42</v>
+        <v>195.65</v>
       </c>
       <c r="E36" s="13">
-        <v>164.94</v>
+        <v>170.98</v>
       </c>
       <c r="F36" s="13">
-        <v>173.94</v>
+        <v>179.98</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="14"/>
       <c r="B37" s="14"/>
       <c r="C37" s="15"/>
@@ -1340,7 +1340,7 @@
       <c r="F37" s="16"/>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A38" s="27" t="s">
         <v>24</v>
       </c>
@@ -1351,7 +1351,7 @@
       <c r="F38" s="17"/>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="23" t="s">
         <v>4</v>
       </c>
@@ -1370,83 +1370,83 @@
       </c>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>202.43</v>
+        <v>218.58</v>
       </c>
       <c r="E40" s="10">
-        <v>177.09</v>
+        <v>187.39</v>
       </c>
       <c r="F40" s="10">
-        <v>187.09</v>
+        <v>197.39</v>
       </c>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>202.11</v>
+        <v>218.24</v>
       </c>
       <c r="E41" s="13">
-        <v>177.51</v>
+        <v>187.81</v>
       </c>
       <c r="F41" s="13">
-        <v>187.51</v>
+        <v>197.81</v>
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>190.15</v>
+        <v>202.43</v>
       </c>
       <c r="E42" s="10">
-        <v>171.45</v>
+        <v>177.09</v>
       </c>
       <c r="F42" s="10">
-        <v>181.45</v>
+        <v>187.09</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>189.84</v>
+        <v>202.11</v>
       </c>
       <c r="E43" s="13">
-        <v>171.87</v>
+        <v>177.51</v>
       </c>
       <c r="F43" s="13">
-        <v>181.87</v>
+        <v>187.51</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="14"/>
       <c r="B44" s="24"/>
       <c r="C44" s="15"/>
@@ -1455,7 +1455,7 @@
       <c r="F44" s="16"/>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="25" t="s">
         <v>27</v>
       </c>
@@ -1466,7 +1466,7 @@
       <c r="F45" s="17"/>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="23" t="s">
         <v>4</v>
       </c>
@@ -1485,83 +1485,83 @@
       </c>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>189.49</v>
+        <v>207.43</v>
       </c>
       <c r="E47" s="10">
-        <v>171.62</v>
+        <v>180.77</v>
       </c>
       <c r="F47" s="10">
-        <v>181.62</v>
+        <v>190.77</v>
       </c>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>189.17</v>
+        <v>207.11</v>
       </c>
       <c r="E48" s="13">
-        <v>171.6</v>
+        <v>180.75</v>
       </c>
       <c r="F48" s="13">
-        <v>181.6</v>
+        <v>190.75</v>
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>180.9</v>
+        <v>189.49</v>
       </c>
       <c r="E49" s="10">
-        <v>165.17</v>
+        <v>171.62</v>
       </c>
       <c r="F49" s="10">
-        <v>175.17</v>
+        <v>181.62</v>
       </c>
       <c r="G49" s="17"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>180.57</v>
+        <v>189.17</v>
       </c>
       <c r="E50" s="13">
-        <v>165.15</v>
+        <v>171.6</v>
       </c>
       <c r="F50" s="13">
-        <v>175.15</v>
+        <v>181.6</v>
       </c>
       <c r="G50" s="17"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="14"/>
       <c r="B51" s="14"/>
       <c r="C51" s="15"/>
@@ -1570,7 +1570,7 @@
       <c r="F51" s="16"/>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A52" s="27" t="s">
         <v>30</v>
       </c>
@@ -1581,7 +1581,7 @@
       <c r="F52" s="17"/>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="23" t="s">
         <v>4</v>
       </c>
@@ -1600,54 +1600,54 @@
       </c>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>211.39</v>
+        <v>227.54</v>
       </c>
       <c r="E54" s="10">
-        <v>187.06</v>
+        <v>195.31</v>
       </c>
       <c r="F54" s="10">
-        <v>197.06</v>
+        <v>205.31</v>
       </c>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>200.79</v>
+        <v>220.21</v>
       </c>
       <c r="E55" s="13">
-        <v>185.3</v>
+        <v>197.75</v>
       </c>
       <c r="F55" s="13">
-        <v>195.3</v>
+        <v>207.75</v>
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>201.87</v>
+        <v>221.27</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1657,111 +1657,111 @@
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>202.28</v>
+        <v>221.61</v>
       </c>
       <c r="E57" s="13">
-        <v>179.71</v>
+        <v>192.15</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
+        <v>217.41</v>
+      </c>
+      <c r="E58" s="10">
+        <v>188.07</v>
+      </c>
+      <c r="F58" s="10">
         <v>198.07</v>
       </c>
-      <c r="E58" s="10">
-        <v>175.62</v>
-      </c>
-      <c r="F58" s="10">
-        <v>185.62</v>
-      </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>203.95</v>
+        <v>220.01</v>
       </c>
       <c r="E59" s="13">
-        <v>185.14</v>
+        <v>193.34</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>199.12</v>
+        <v>211.39</v>
       </c>
       <c r="E60" s="10">
-        <v>180.85</v>
+        <v>187.06</v>
       </c>
       <c r="F60" s="10">
-        <v>190.85</v>
+        <v>197.06</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>188.53</v>
+        <v>200.79</v>
       </c>
       <c r="E61" s="13">
-        <v>179.31</v>
+        <v>185.3</v>
       </c>
       <c r="F61" s="13">
-        <v>189.31</v>
+        <v>195.3</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>189.62</v>
+        <v>201.87</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1771,57 +1771,57 @@
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>190.12</v>
+        <v>202.28</v>
       </c>
       <c r="E63" s="13">
-        <v>173.72</v>
+        <v>179.71</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>185.9</v>
+        <v>198.07</v>
       </c>
       <c r="E64" s="10">
-        <v>169.63</v>
+        <v>175.62</v>
       </c>
       <c r="F64" s="10">
-        <v>179.63</v>
+        <v>185.62</v>
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46087</v>
+        <v>46088</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>191.76</v>
+        <v>203.95</v>
       </c>
       <c r="E65" s="13">
-        <v>178.98</v>
+        <v>185.14</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,6 +1850,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2109,17 +2120,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2130,6 +2130,24 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2149,24 +2167,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Tue Mar 10 03:35:17 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{E06B1640-5FDE-4F0C-A562-91B3DEB5F92B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{401276B8-8257-4CAC-829F-29368610B0D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" concurrentManualCount="20"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>216.89</v>
+        <v>231.38</v>
       </c>
       <c r="E8" s="10">
-        <v>183.97</v>
+        <v>195.3</v>
       </c>
       <c r="F8" s="10">
-        <v>193.97</v>
+        <v>205.3</v>
       </c>
       <c r="G8" s="10">
-        <v>183.86</v>
+        <v>195.19</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>216.89</v>
+        <v>231.38</v>
       </c>
       <c r="E9" s="13">
-        <v>183.97</v>
+        <v>195.3</v>
       </c>
       <c r="F9" s="13">
-        <v>193.97</v>
+        <v>205.3</v>
       </c>
       <c r="G9" s="13">
-        <v>183.86</v>
+        <v>195.19</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>218.54</v>
+        <v>232.89</v>
       </c>
       <c r="E10" s="10">
-        <v>186.49</v>
+        <v>197.71</v>
       </c>
       <c r="F10" s="10">
-        <v>196.49</v>
+        <v>207.71</v>
       </c>
       <c r="G10" s="10">
-        <v>186.73</v>
+        <v>197.95</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>201.59</v>
+        <v>216.89</v>
       </c>
       <c r="E11" s="13">
-        <v>174.51</v>
+        <v>183.97</v>
       </c>
       <c r="F11" s="13">
-        <v>184.51</v>
+        <v>193.97</v>
       </c>
       <c r="G11" s="13">
-        <v>174.39</v>
+        <v>183.86</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>201.59</v>
+        <v>216.89</v>
       </c>
       <c r="E12" s="10">
-        <v>174.51</v>
+        <v>183.97</v>
       </c>
       <c r="F12" s="10">
-        <v>184.51</v>
+        <v>193.97</v>
       </c>
       <c r="G12" s="10">
-        <v>174.39</v>
+        <v>183.86</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>198.03</v>
+        <v>218.54</v>
       </c>
       <c r="E13" s="13">
-        <v>173.97</v>
+        <v>186.49</v>
       </c>
       <c r="F13" s="13">
-        <v>183.97</v>
+        <v>196.49</v>
       </c>
       <c r="G13" s="13">
-        <v>174.21</v>
+        <v>186.73</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>220.96</v>
+        <v>235.29</v>
       </c>
       <c r="E17" s="10">
-        <v>188.09</v>
+        <v>199.32</v>
       </c>
       <c r="F17" s="10">
-        <v>198.09</v>
+        <v>209.32</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>201.59</v>
+        <v>220.96</v>
       </c>
       <c r="E18" s="13">
-        <v>176.69</v>
+        <v>188.09</v>
       </c>
       <c r="F18" s="13">
-        <v>186.69</v>
+        <v>198.09</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>216.6</v>
+        <v>231.08</v>
       </c>
       <c r="E22" s="10">
-        <v>186.08</v>
+        <v>197.41</v>
       </c>
       <c r="F22" s="10">
-        <v>195.68</v>
+        <v>207.01</v>
       </c>
       <c r="G22" s="10">
-        <v>187.83</v>
+        <v>199.16</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>223.8</v>
+        <v>238.16</v>
       </c>
       <c r="E23" s="13">
-        <v>192.24</v>
+        <v>203.49</v>
       </c>
       <c r="F23" s="13">
-        <v>202.24</v>
+        <v>213.49</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>223.94</v>
+        <v>238.3</v>
       </c>
       <c r="E24" s="10">
-        <v>192.84</v>
+        <v>204.08</v>
       </c>
       <c r="F24" s="10">
-        <v>202.84</v>
+        <v>214.08</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>223.93</v>
+        <v>238.28</v>
       </c>
       <c r="E25" s="13">
-        <v>192.44</v>
+        <v>203.71</v>
       </c>
       <c r="F25" s="13">
-        <v>202.44</v>
+        <v>213.71</v>
       </c>
       <c r="G25" s="13">
-        <v>193.29</v>
+        <v>204.56</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>223.52</v>
+        <v>237.87</v>
       </c>
       <c r="E26" s="10">
-        <v>194.26</v>
+        <v>205.61</v>
       </c>
       <c r="F26" s="10">
-        <v>204.26</v>
+        <v>215.61</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>199.11</v>
+        <v>216.6</v>
       </c>
       <c r="E27" s="13">
-        <v>174.42</v>
+        <v>186.08</v>
       </c>
       <c r="F27" s="13">
-        <v>184.02</v>
+        <v>195.68</v>
       </c>
       <c r="G27" s="13">
-        <v>176.17</v>
+        <v>187.83</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>203.28</v>
+        <v>223.8</v>
       </c>
       <c r="E28" s="22">
-        <v>179.71</v>
+        <v>192.24</v>
       </c>
       <c r="F28" s="22">
-        <v>189.71</v>
+        <v>202.24</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>203.43</v>
+        <v>223.94</v>
       </c>
       <c r="E29" s="13">
-        <v>180.32</v>
+        <v>192.84</v>
       </c>
       <c r="F29" s="13">
-        <v>190.32</v>
+        <v>202.84</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>203.42</v>
+        <v>223.93</v>
       </c>
       <c r="E30" s="22">
-        <v>179.9</v>
+        <v>192.44</v>
       </c>
       <c r="F30" s="22">
-        <v>189.9</v>
+        <v>202.44</v>
       </c>
       <c r="G30" s="22">
-        <v>180.75</v>
+        <v>193.29</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>203.01</v>
+        <v>223.52</v>
       </c>
       <c r="E31" s="13">
-        <v>181.65</v>
+        <v>194.26</v>
       </c>
       <c r="F31" s="13">
-        <v>191.65</v>
+        <v>204.26</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>216.14</v>
+        <v>230.48</v>
       </c>
       <c r="E35" s="10">
-        <v>184.58</v>
+        <v>195.78</v>
       </c>
       <c r="F35" s="10">
-        <v>193.58</v>
+        <v>204.78</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>195.65</v>
+        <v>216.14</v>
       </c>
       <c r="E36" s="13">
-        <v>170.98</v>
+        <v>184.58</v>
       </c>
       <c r="F36" s="13">
-        <v>179.98</v>
+        <v>193.58</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>218.58</v>
+        <v>232.96</v>
       </c>
       <c r="E40" s="10">
-        <v>187.39</v>
+        <v>197.49</v>
       </c>
       <c r="F40" s="10">
-        <v>197.39</v>
+        <v>207.49</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>218.24</v>
+        <v>232.61</v>
       </c>
       <c r="E41" s="13">
-        <v>187.81</v>
+        <v>197.91</v>
       </c>
       <c r="F41" s="13">
-        <v>197.81</v>
+        <v>207.91</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>202.43</v>
+        <v>218.58</v>
       </c>
       <c r="E42" s="10">
-        <v>177.09</v>
+        <v>187.39</v>
       </c>
       <c r="F42" s="10">
-        <v>187.09</v>
+        <v>197.39</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>202.11</v>
+        <v>218.24</v>
       </c>
       <c r="E43" s="13">
-        <v>177.51</v>
+        <v>187.81</v>
       </c>
       <c r="F43" s="13">
-        <v>187.51</v>
+        <v>197.81</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>207.43</v>
+        <v>227.46</v>
       </c>
       <c r="E47" s="10">
-        <v>180.77</v>
+        <v>192.55</v>
       </c>
       <c r="F47" s="10">
-        <v>190.77</v>
+        <v>202.55</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>207.11</v>
+        <v>227.15</v>
       </c>
       <c r="E48" s="13">
-        <v>180.75</v>
+        <v>192.54</v>
       </c>
       <c r="F48" s="13">
-        <v>190.75</v>
+        <v>202.54</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>189.49</v>
+        <v>207.43</v>
       </c>
       <c r="E49" s="10">
-        <v>171.62</v>
+        <v>180.77</v>
       </c>
       <c r="F49" s="10">
-        <v>181.62</v>
+        <v>190.77</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>189.17</v>
+        <v>207.11</v>
       </c>
       <c r="E50" s="13">
-        <v>171.6</v>
+        <v>180.75</v>
       </c>
       <c r="F50" s="13">
-        <v>181.6</v>
+        <v>190.75</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>227.54</v>
+        <v>244.13</v>
       </c>
       <c r="E54" s="10">
-        <v>195.31</v>
+        <v>206.64</v>
       </c>
       <c r="F54" s="10">
-        <v>205.31</v>
+        <v>216.64</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>220.21</v>
+        <v>234.58</v>
       </c>
       <c r="E55" s="13">
-        <v>197.75</v>
+        <v>208.91</v>
       </c>
       <c r="F55" s="13">
-        <v>207.75</v>
+        <v>218.91</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>221.27</v>
+        <v>235.62</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>221.61</v>
+        <v>235.89</v>
       </c>
       <c r="E57" s="13">
-        <v>192.15</v>
+        <v>203.3</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>217.41</v>
+        <v>231.7</v>
       </c>
       <c r="E58" s="10">
-        <v>188.07</v>
+        <v>199.23</v>
       </c>
       <c r="F58" s="10">
-        <v>198.07</v>
+        <v>209.23</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>220.01</v>
+        <v>236.51</v>
       </c>
       <c r="E59" s="13">
-        <v>193.34</v>
+        <v>204.66</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>211.39</v>
+        <v>227.54</v>
       </c>
       <c r="E60" s="10">
-        <v>187.06</v>
+        <v>195.31</v>
       </c>
       <c r="F60" s="10">
-        <v>197.06</v>
+        <v>205.31</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>200.79</v>
+        <v>220.21</v>
       </c>
       <c r="E61" s="13">
-        <v>185.3</v>
+        <v>197.75</v>
       </c>
       <c r="F61" s="13">
-        <v>195.3</v>
+        <v>207.75</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>201.87</v>
+        <v>221.27</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>202.28</v>
+        <v>221.61</v>
       </c>
       <c r="E63" s="13">
-        <v>179.71</v>
+        <v>192.15</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
+        <v>217.41</v>
+      </c>
+      <c r="E64" s="10">
+        <v>188.07</v>
+      </c>
+      <c r="F64" s="10">
         <v>198.07</v>
-      </c>
-      <c r="E64" s="10">
-        <v>175.62</v>
-      </c>
-      <c r="F64" s="10">
-        <v>185.62</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46088</v>
+        <v>46091</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>203.95</v>
+        <v>220.01</v>
       </c>
       <c r="E65" s="13">
-        <v>185.14</v>
+        <v>193.34</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,6 +1850,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -1860,7 +1869,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2120,16 +2129,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -2147,7 +2155,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2167,14 +2175,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Wed Mar 11 03:34:39 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{401276B8-8257-4CAC-829F-29368610B0D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{78192765-3791-473F-A909-D89D3FD3A97A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentManualCount="20"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>231.38</v>
+        <v>238.32</v>
       </c>
       <c r="E8" s="10">
-        <v>195.3</v>
+        <v>200.91</v>
       </c>
       <c r="F8" s="10">
-        <v>205.3</v>
+        <v>210.91</v>
       </c>
       <c r="G8" s="10">
-        <v>195.19</v>
+        <v>200.79</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>231.38</v>
+        <v>238.32</v>
       </c>
       <c r="E9" s="13">
-        <v>195.3</v>
+        <v>200.91</v>
       </c>
       <c r="F9" s="13">
-        <v>205.3</v>
+        <v>210.91</v>
       </c>
       <c r="G9" s="13">
-        <v>195.19</v>
+        <v>200.79</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>232.89</v>
+        <v>240.07</v>
       </c>
       <c r="E10" s="10">
-        <v>197.71</v>
+        <v>203.54</v>
       </c>
       <c r="F10" s="10">
-        <v>207.71</v>
+        <v>213.54</v>
       </c>
       <c r="G10" s="10">
-        <v>197.95</v>
+        <v>203.78</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>216.89</v>
+        <v>231.38</v>
       </c>
       <c r="E11" s="13">
-        <v>183.97</v>
+        <v>195.3</v>
       </c>
       <c r="F11" s="13">
-        <v>193.97</v>
+        <v>205.3</v>
       </c>
       <c r="G11" s="13">
-        <v>183.86</v>
+        <v>195.19</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>216.89</v>
+        <v>231.38</v>
       </c>
       <c r="E12" s="10">
-        <v>183.97</v>
+        <v>195.3</v>
       </c>
       <c r="F12" s="10">
-        <v>193.97</v>
+        <v>205.3</v>
       </c>
       <c r="G12" s="10">
-        <v>183.86</v>
+        <v>195.19</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>218.54</v>
+        <v>232.89</v>
       </c>
       <c r="E13" s="13">
-        <v>186.49</v>
+        <v>197.71</v>
       </c>
       <c r="F13" s="13">
-        <v>196.49</v>
+        <v>207.71</v>
       </c>
       <c r="G13" s="13">
-        <v>186.73</v>
+        <v>197.95</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>235.29</v>
+        <v>242.48</v>
       </c>
       <c r="E17" s="10">
-        <v>199.32</v>
+        <v>205.18</v>
       </c>
       <c r="F17" s="10">
-        <v>209.32</v>
+        <v>215.18</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>220.96</v>
+        <v>235.29</v>
       </c>
       <c r="E18" s="13">
-        <v>188.09</v>
+        <v>199.32</v>
       </c>
       <c r="F18" s="13">
-        <v>198.09</v>
+        <v>209.32</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>231.08</v>
+        <v>238.02</v>
       </c>
       <c r="E22" s="10">
-        <v>197.41</v>
+        <v>203.01</v>
       </c>
       <c r="F22" s="10">
-        <v>207.01</v>
+        <v>212.61</v>
       </c>
       <c r="G22" s="10">
-        <v>199.16</v>
+        <v>204.76</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>238.16</v>
+        <v>245.34</v>
       </c>
       <c r="E23" s="13">
-        <v>203.49</v>
+        <v>209.34</v>
       </c>
       <c r="F23" s="13">
-        <v>213.49</v>
+        <v>219.34</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>238.3</v>
+        <v>245.48</v>
       </c>
       <c r="E24" s="10">
-        <v>204.08</v>
+        <v>209.91</v>
       </c>
       <c r="F24" s="10">
-        <v>214.08</v>
+        <v>219.91</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>238.28</v>
+        <v>245.46</v>
       </c>
       <c r="E25" s="13">
-        <v>203.71</v>
+        <v>209.54</v>
       </c>
       <c r="F25" s="13">
-        <v>213.71</v>
+        <v>219.54</v>
       </c>
       <c r="G25" s="13">
-        <v>204.56</v>
+        <v>210.39</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>237.87</v>
+        <v>245.06</v>
       </c>
       <c r="E26" s="10">
-        <v>205.61</v>
+        <v>211.49</v>
       </c>
       <c r="F26" s="10">
-        <v>215.61</v>
+        <v>221.49</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>216.6</v>
+        <v>231.08</v>
       </c>
       <c r="E27" s="13">
-        <v>186.08</v>
+        <v>197.41</v>
       </c>
       <c r="F27" s="13">
-        <v>195.68</v>
+        <v>207.01</v>
       </c>
       <c r="G27" s="13">
-        <v>187.83</v>
+        <v>199.16</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>223.8</v>
+        <v>238.16</v>
       </c>
       <c r="E28" s="22">
-        <v>192.24</v>
+        <v>203.49</v>
       </c>
       <c r="F28" s="22">
-        <v>202.24</v>
+        <v>213.49</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>223.94</v>
+        <v>238.3</v>
       </c>
       <c r="E29" s="13">
-        <v>192.84</v>
+        <v>204.08</v>
       </c>
       <c r="F29" s="13">
-        <v>202.84</v>
+        <v>214.08</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>223.93</v>
+        <v>238.28</v>
       </c>
       <c r="E30" s="22">
-        <v>192.44</v>
+        <v>203.71</v>
       </c>
       <c r="F30" s="22">
-        <v>202.44</v>
+        <v>213.71</v>
       </c>
       <c r="G30" s="22">
-        <v>193.29</v>
+        <v>204.56</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>223.52</v>
+        <v>237.87</v>
       </c>
       <c r="E31" s="13">
-        <v>194.26</v>
+        <v>205.61</v>
       </c>
       <c r="F31" s="13">
-        <v>204.26</v>
+        <v>215.61</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>230.48</v>
+        <v>237.66</v>
       </c>
       <c r="E35" s="10">
-        <v>195.78</v>
+        <v>201.6</v>
       </c>
       <c r="F35" s="10">
-        <v>204.78</v>
+        <v>210.6</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>216.14</v>
+        <v>230.48</v>
       </c>
       <c r="E36" s="13">
-        <v>184.58</v>
+        <v>195.78</v>
       </c>
       <c r="F36" s="13">
-        <v>193.58</v>
+        <v>204.78</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>232.96</v>
+        <v>240.15</v>
       </c>
       <c r="E40" s="10">
-        <v>197.49</v>
+        <v>202.3</v>
       </c>
       <c r="F40" s="10">
-        <v>207.49</v>
+        <v>212.3</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>232.61</v>
+        <v>239.78</v>
       </c>
       <c r="E41" s="13">
-        <v>197.91</v>
+        <v>202.71</v>
       </c>
       <c r="F41" s="13">
-        <v>207.91</v>
+        <v>212.71</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>218.58</v>
+        <v>232.96</v>
       </c>
       <c r="E42" s="10">
-        <v>187.39</v>
+        <v>197.49</v>
       </c>
       <c r="F42" s="10">
-        <v>197.39</v>
+        <v>207.49</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>218.24</v>
+        <v>232.61</v>
       </c>
       <c r="E43" s="13">
-        <v>187.81</v>
+        <v>197.91</v>
       </c>
       <c r="F43" s="13">
-        <v>197.81</v>
+        <v>207.91</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>227.46</v>
+        <v>237.32</v>
       </c>
       <c r="E47" s="10">
-        <v>192.55</v>
+        <v>199.12</v>
       </c>
       <c r="F47" s="10">
-        <v>202.55</v>
+        <v>209.12</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>227.15</v>
+        <v>237.02</v>
       </c>
       <c r="E48" s="13">
-        <v>192.54</v>
+        <v>199.12</v>
       </c>
       <c r="F48" s="13">
-        <v>202.54</v>
+        <v>209.12</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>207.43</v>
+        <v>227.46</v>
       </c>
       <c r="E49" s="10">
-        <v>180.77</v>
+        <v>192.55</v>
       </c>
       <c r="F49" s="10">
-        <v>190.77</v>
+        <v>202.55</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>207.11</v>
+        <v>227.15</v>
       </c>
       <c r="E50" s="13">
-        <v>180.75</v>
+        <v>192.54</v>
       </c>
       <c r="F50" s="13">
-        <v>190.75</v>
+        <v>202.54</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>244.13</v>
+        <v>251.34</v>
       </c>
       <c r="E54" s="10">
-        <v>206.64</v>
+        <v>212.44</v>
       </c>
       <c r="F54" s="10">
-        <v>216.64</v>
+        <v>222.44</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>234.58</v>
+        <v>241.77</v>
       </c>
       <c r="E55" s="13">
-        <v>208.91</v>
+        <v>214.72</v>
       </c>
       <c r="F55" s="13">
-        <v>218.91</v>
+        <v>224.72</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>235.62</v>
+        <v>242.8</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>235.89</v>
+        <v>243.06</v>
       </c>
       <c r="E57" s="13">
-        <v>203.3</v>
+        <v>209.11</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>231.7</v>
+        <v>238.87</v>
       </c>
       <c r="E58" s="10">
-        <v>199.23</v>
+        <v>205.04</v>
       </c>
       <c r="F58" s="10">
-        <v>209.23</v>
+        <v>215.04</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>236.51</v>
+        <v>243.7</v>
       </c>
       <c r="E59" s="13">
-        <v>204.66</v>
+        <v>210.48</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>227.54</v>
+        <v>244.13</v>
       </c>
       <c r="E60" s="10">
-        <v>195.31</v>
+        <v>206.64</v>
       </c>
       <c r="F60" s="10">
-        <v>205.31</v>
+        <v>216.64</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>220.21</v>
+        <v>234.58</v>
       </c>
       <c r="E61" s="13">
-        <v>197.75</v>
+        <v>208.91</v>
       </c>
       <c r="F61" s="13">
-        <v>207.75</v>
+        <v>218.91</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>221.27</v>
+        <v>235.62</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>221.61</v>
+        <v>235.89</v>
       </c>
       <c r="E63" s="13">
-        <v>192.15</v>
+        <v>203.3</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>217.41</v>
+        <v>231.7</v>
       </c>
       <c r="E64" s="10">
-        <v>188.07</v>
+        <v>199.23</v>
       </c>
       <c r="F64" s="10">
-        <v>198.07</v>
+        <v>209.23</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>220.01</v>
+        <v>236.51</v>
       </c>
       <c r="E65" s="13">
-        <v>193.34</v>
+        <v>204.66</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,26 +1850,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2129,33 +2109,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2175,6 +2149,32 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Thu Mar 12 03:40:49 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{78192765-3791-473F-A909-D89D3FD3A97A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{E675D79E-4876-43A3-AD43-8FFA1F2CD8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>238.32</v>
+        <v>240.85</v>
       </c>
       <c r="E8" s="10">
-        <v>200.91</v>
+        <v>204.73</v>
       </c>
       <c r="F8" s="10">
-        <v>210.91</v>
+        <v>214.73</v>
       </c>
       <c r="G8" s="10">
-        <v>200.79</v>
+        <v>204.61</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>238.32</v>
+        <v>240.85</v>
       </c>
       <c r="E9" s="13">
-        <v>200.91</v>
+        <v>204.73</v>
       </c>
       <c r="F9" s="13">
-        <v>210.91</v>
+        <v>214.73</v>
       </c>
       <c r="G9" s="13">
-        <v>200.79</v>
+        <v>204.61</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>240.07</v>
+        <v>242.97</v>
       </c>
       <c r="E10" s="10">
-        <v>203.54</v>
+        <v>207.71</v>
       </c>
       <c r="F10" s="10">
-        <v>213.54</v>
+        <v>217.71</v>
       </c>
       <c r="G10" s="10">
-        <v>203.78</v>
+        <v>207.95</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>231.38</v>
+        <v>238.32</v>
       </c>
       <c r="E11" s="13">
-        <v>195.3</v>
+        <v>200.91</v>
       </c>
       <c r="F11" s="13">
-        <v>205.3</v>
+        <v>210.91</v>
       </c>
       <c r="G11" s="13">
-        <v>195.19</v>
+        <v>200.79</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>231.38</v>
+        <v>238.32</v>
       </c>
       <c r="E12" s="10">
-        <v>195.3</v>
+        <v>200.91</v>
       </c>
       <c r="F12" s="10">
-        <v>205.3</v>
+        <v>210.91</v>
       </c>
       <c r="G12" s="10">
-        <v>195.19</v>
+        <v>200.79</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>232.89</v>
+        <v>240.07</v>
       </c>
       <c r="E13" s="13">
-        <v>197.71</v>
+        <v>203.54</v>
       </c>
       <c r="F13" s="13">
-        <v>207.71</v>
+        <v>213.54</v>
       </c>
       <c r="G13" s="13">
-        <v>197.95</v>
+        <v>203.78</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>242.48</v>
+        <v>245.41</v>
       </c>
       <c r="E17" s="10">
-        <v>205.18</v>
+        <v>209.38</v>
       </c>
       <c r="F17" s="10">
-        <v>215.18</v>
+        <v>219.38</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>235.29</v>
+        <v>242.48</v>
       </c>
       <c r="E18" s="13">
-        <v>199.32</v>
+        <v>205.18</v>
       </c>
       <c r="F18" s="13">
-        <v>209.32</v>
+        <v>215.18</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>238.02</v>
+        <v>240.54</v>
       </c>
       <c r="E22" s="10">
-        <v>203.01</v>
+        <v>206.83</v>
       </c>
       <c r="F22" s="10">
-        <v>212.61</v>
+        <v>216.43</v>
       </c>
       <c r="G22" s="10">
-        <v>204.76</v>
+        <v>208.58</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>245.34</v>
+        <v>248.25</v>
       </c>
       <c r="E23" s="13">
-        <v>209.34</v>
+        <v>213.51</v>
       </c>
       <c r="F23" s="13">
-        <v>219.34</v>
+        <v>223.51</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>245.48</v>
+        <v>248.39</v>
       </c>
       <c r="E24" s="10">
-        <v>209.91</v>
+        <v>214.07</v>
       </c>
       <c r="F24" s="10">
-        <v>219.91</v>
+        <v>224.07</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>245.46</v>
+        <v>248.37</v>
       </c>
       <c r="E25" s="13">
-        <v>209.54</v>
+        <v>213.71</v>
       </c>
       <c r="F25" s="13">
-        <v>219.54</v>
+        <v>223.71</v>
       </c>
       <c r="G25" s="13">
-        <v>210.39</v>
+        <v>214.56</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>245.06</v>
+        <v>247.97</v>
       </c>
       <c r="E26" s="10">
-        <v>211.49</v>
+        <v>215.68</v>
       </c>
       <c r="F26" s="10">
-        <v>221.49</v>
+        <v>225.68</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>231.08</v>
+        <v>238.02</v>
       </c>
       <c r="E27" s="13">
-        <v>197.41</v>
+        <v>203.01</v>
       </c>
       <c r="F27" s="13">
-        <v>207.01</v>
+        <v>212.61</v>
       </c>
       <c r="G27" s="13">
-        <v>199.16</v>
+        <v>204.76</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>238.16</v>
+        <v>245.34</v>
       </c>
       <c r="E28" s="22">
-        <v>203.49</v>
+        <v>209.34</v>
       </c>
       <c r="F28" s="22">
-        <v>213.49</v>
+        <v>219.34</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>238.3</v>
+        <v>245.48</v>
       </c>
       <c r="E29" s="13">
-        <v>204.08</v>
+        <v>209.91</v>
       </c>
       <c r="F29" s="13">
-        <v>214.08</v>
+        <v>219.91</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>238.28</v>
+        <v>245.46</v>
       </c>
       <c r="E30" s="22">
-        <v>203.71</v>
+        <v>209.54</v>
       </c>
       <c r="F30" s="22">
-        <v>213.71</v>
+        <v>219.54</v>
       </c>
       <c r="G30" s="22">
-        <v>204.56</v>
+        <v>210.39</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>237.87</v>
+        <v>245.06</v>
       </c>
       <c r="E31" s="13">
-        <v>205.61</v>
+        <v>211.49</v>
       </c>
       <c r="F31" s="13">
-        <v>215.61</v>
+        <v>221.49</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>237.66</v>
+        <v>240.57</v>
       </c>
       <c r="E35" s="10">
-        <v>201.6</v>
+        <v>205.76</v>
       </c>
       <c r="F35" s="10">
-        <v>210.6</v>
+        <v>214.76</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>230.48</v>
+        <v>237.66</v>
       </c>
       <c r="E36" s="13">
-        <v>195.78</v>
+        <v>201.6</v>
       </c>
       <c r="F36" s="13">
-        <v>204.78</v>
+        <v>210.6</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>240.15</v>
+        <v>243.04</v>
       </c>
       <c r="E40" s="10">
-        <v>202.3</v>
+        <v>204.94</v>
       </c>
       <c r="F40" s="10">
-        <v>212.3</v>
+        <v>214.94</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>239.78</v>
+        <v>242.67</v>
       </c>
       <c r="E41" s="13">
-        <v>202.71</v>
+        <v>205.36</v>
       </c>
       <c r="F41" s="13">
-        <v>212.71</v>
+        <v>215.36</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>232.96</v>
+        <v>240.15</v>
       </c>
       <c r="E42" s="10">
-        <v>197.49</v>
+        <v>202.3</v>
       </c>
       <c r="F42" s="10">
-        <v>207.49</v>
+        <v>212.3</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>232.61</v>
+        <v>239.78</v>
       </c>
       <c r="E43" s="13">
-        <v>197.91</v>
+        <v>202.71</v>
       </c>
       <c r="F43" s="13">
-        <v>207.91</v>
+        <v>212.71</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>237.32</v>
+        <v>244.02</v>
       </c>
       <c r="E47" s="10">
-        <v>199.12</v>
+        <v>204.06</v>
       </c>
       <c r="F47" s="10">
-        <v>209.12</v>
+        <v>214.06</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>237.02</v>
+        <v>243.73</v>
       </c>
       <c r="E48" s="13">
-        <v>199.12</v>
+        <v>204.06</v>
       </c>
       <c r="F48" s="13">
-        <v>209.12</v>
+        <v>214.06</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>227.46</v>
+        <v>237.32</v>
       </c>
       <c r="E49" s="10">
-        <v>192.55</v>
+        <v>199.12</v>
       </c>
       <c r="F49" s="10">
-        <v>202.55</v>
+        <v>209.12</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>227.15</v>
+        <v>237.02</v>
       </c>
       <c r="E50" s="13">
-        <v>192.54</v>
+        <v>199.12</v>
       </c>
       <c r="F50" s="13">
-        <v>202.54</v>
+        <v>209.12</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>251.34</v>
+        <v>254.24</v>
       </c>
       <c r="E54" s="10">
-        <v>212.44</v>
+        <v>216.52</v>
       </c>
       <c r="F54" s="10">
-        <v>222.44</v>
+        <v>226.52</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>241.77</v>
+        <v>244.67</v>
       </c>
       <c r="E55" s="13">
-        <v>214.72</v>
+        <v>218.89</v>
       </c>
       <c r="F55" s="13">
-        <v>224.72</v>
+        <v>228.89</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>242.8</v>
+        <v>245.7</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>243.06</v>
+        <v>245.99</v>
       </c>
       <c r="E57" s="13">
-        <v>209.11</v>
+        <v>213.28</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>238.87</v>
+        <v>241.8</v>
       </c>
       <c r="E58" s="10">
-        <v>205.04</v>
+        <v>209.21</v>
       </c>
       <c r="F58" s="10">
-        <v>215.04</v>
+        <v>219.21</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>243.7</v>
+        <v>246.64</v>
       </c>
       <c r="E59" s="13">
-        <v>210.48</v>
+        <v>214.6</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>244.13</v>
+        <v>251.34</v>
       </c>
       <c r="E60" s="10">
-        <v>206.64</v>
+        <v>212.44</v>
       </c>
       <c r="F60" s="10">
-        <v>216.64</v>
+        <v>222.44</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>234.58</v>
+        <v>241.77</v>
       </c>
       <c r="E61" s="13">
-        <v>208.91</v>
+        <v>214.72</v>
       </c>
       <c r="F61" s="13">
-        <v>218.91</v>
+        <v>224.72</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>235.62</v>
+        <v>242.8</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>235.89</v>
+        <v>243.06</v>
       </c>
       <c r="E63" s="13">
-        <v>203.3</v>
+        <v>209.11</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>231.7</v>
+        <v>238.87</v>
       </c>
       <c r="E64" s="10">
-        <v>199.23</v>
+        <v>205.04</v>
       </c>
       <c r="F64" s="10">
-        <v>209.23</v>
+        <v>215.04</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>236.51</v>
+        <v>243.7</v>
       </c>
       <c r="E65" s="13">
-        <v>204.66</v>
+        <v>210.48</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,6 +1850,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2109,7 +2120,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2118,18 +2129,25 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2149,28 +2167,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Fri Mar 13 03:38:07 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{E675D79E-4876-43A3-AD43-8FFA1F2CD8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{05764E49-E093-4905-BD8F-22A14921E1FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>240.85</v>
+        <v>259.35000000000002</v>
       </c>
       <c r="E8" s="10">
-        <v>204.73</v>
+        <v>216.1</v>
       </c>
       <c r="F8" s="10">
-        <v>214.73</v>
+        <v>226.11</v>
       </c>
       <c r="G8" s="10">
-        <v>204.61</v>
+        <v>215.99</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>240.85</v>
+        <v>259.35000000000002</v>
       </c>
       <c r="E9" s="13">
-        <v>204.73</v>
+        <v>216.1</v>
       </c>
       <c r="F9" s="13">
-        <v>214.73</v>
+        <v>226.11</v>
       </c>
       <c r="G9" s="13">
-        <v>204.61</v>
+        <v>215.99</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>242.97</v>
+        <v>260.38</v>
       </c>
       <c r="E10" s="10">
-        <v>207.71</v>
+        <v>218.42</v>
       </c>
       <c r="F10" s="10">
-        <v>217.71</v>
+        <v>228.42</v>
       </c>
       <c r="G10" s="10">
-        <v>207.95</v>
+        <v>218.67</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>238.32</v>
+        <v>240.85</v>
       </c>
       <c r="E11" s="13">
-        <v>200.91</v>
+        <v>204.73</v>
       </c>
       <c r="F11" s="13">
-        <v>210.91</v>
+        <v>214.73</v>
       </c>
       <c r="G11" s="13">
-        <v>200.79</v>
+        <v>204.61</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>238.32</v>
+        <v>240.85</v>
       </c>
       <c r="E12" s="10">
-        <v>200.91</v>
+        <v>204.73</v>
       </c>
       <c r="F12" s="10">
-        <v>210.91</v>
+        <v>214.73</v>
       </c>
       <c r="G12" s="10">
-        <v>200.79</v>
+        <v>204.61</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>240.07</v>
+        <v>242.97</v>
       </c>
       <c r="E13" s="13">
-        <v>203.54</v>
+        <v>207.71</v>
       </c>
       <c r="F13" s="13">
-        <v>213.54</v>
+        <v>217.71</v>
       </c>
       <c r="G13" s="13">
-        <v>203.78</v>
+        <v>207.95</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>245.41</v>
+        <v>256.45999999999998</v>
       </c>
       <c r="E17" s="10">
-        <v>209.38</v>
+        <v>217.71</v>
       </c>
       <c r="F17" s="10">
-        <v>219.38</v>
+        <v>227.71</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>242.48</v>
+        <v>245.41</v>
       </c>
       <c r="E18" s="13">
-        <v>205.18</v>
+        <v>209.38</v>
       </c>
       <c r="F18" s="13">
-        <v>215.18</v>
+        <v>219.38</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>240.54</v>
+        <v>259.04000000000002</v>
       </c>
       <c r="E22" s="10">
-        <v>206.83</v>
+        <v>218.2</v>
       </c>
       <c r="F22" s="10">
-        <v>216.43</v>
+        <v>227.8</v>
       </c>
       <c r="G22" s="10">
-        <v>208.58</v>
+        <v>219.95</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>248.25</v>
+        <v>266.98</v>
       </c>
       <c r="E23" s="13">
-        <v>213.51</v>
+        <v>225.13</v>
       </c>
       <c r="F23" s="13">
-        <v>223.51</v>
+        <v>235.13</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>248.39</v>
+        <v>267.13</v>
       </c>
       <c r="E24" s="10">
-        <v>214.07</v>
+        <v>225.66</v>
       </c>
       <c r="F24" s="10">
-        <v>224.07</v>
+        <v>235.66</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>248.37</v>
+        <v>267.11</v>
       </c>
       <c r="E25" s="13">
-        <v>213.71</v>
+        <v>225.31</v>
       </c>
       <c r="F25" s="13">
-        <v>223.71</v>
+        <v>235.31</v>
       </c>
       <c r="G25" s="13">
-        <v>214.56</v>
+        <v>226.16</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>247.97</v>
+        <v>266.70999999999998</v>
       </c>
       <c r="E26" s="10">
-        <v>215.68</v>
+        <v>227.33</v>
       </c>
       <c r="F26" s="10">
-        <v>225.68</v>
+        <v>237.33</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>238.02</v>
+        <v>240.54</v>
       </c>
       <c r="E27" s="13">
-        <v>203.01</v>
+        <v>206.83</v>
       </c>
       <c r="F27" s="13">
-        <v>212.61</v>
+        <v>216.43</v>
       </c>
       <c r="G27" s="13">
-        <v>204.76</v>
+        <v>208.58</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>245.34</v>
+        <v>248.25</v>
       </c>
       <c r="E28" s="22">
-        <v>209.34</v>
+        <v>213.51</v>
       </c>
       <c r="F28" s="22">
-        <v>219.34</v>
+        <v>223.51</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>245.48</v>
+        <v>248.39</v>
       </c>
       <c r="E29" s="13">
-        <v>209.91</v>
+        <v>214.07</v>
       </c>
       <c r="F29" s="13">
-        <v>219.91</v>
+        <v>224.07</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>245.46</v>
+        <v>248.37</v>
       </c>
       <c r="E30" s="22">
-        <v>209.54</v>
+        <v>213.71</v>
       </c>
       <c r="F30" s="22">
-        <v>219.54</v>
+        <v>223.71</v>
       </c>
       <c r="G30" s="22">
-        <v>210.39</v>
+        <v>214.56</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>245.06</v>
+        <v>247.97</v>
       </c>
       <c r="E31" s="13">
-        <v>211.49</v>
+        <v>215.68</v>
       </c>
       <c r="F31" s="13">
-        <v>221.49</v>
+        <v>225.68</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>240.57</v>
+        <v>259.3</v>
       </c>
       <c r="E35" s="10">
-        <v>205.76</v>
+        <v>217.35</v>
       </c>
       <c r="F35" s="10">
-        <v>214.76</v>
+        <v>226.35</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>237.66</v>
+        <v>240.57</v>
       </c>
       <c r="E36" s="13">
-        <v>201.6</v>
+        <v>205.76</v>
       </c>
       <c r="F36" s="13">
-        <v>210.6</v>
+        <v>214.76</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>243.04</v>
+        <v>258.47000000000003</v>
       </c>
       <c r="E40" s="10">
-        <v>204.94</v>
+        <v>217.04</v>
       </c>
       <c r="F40" s="10">
-        <v>214.94</v>
+        <v>227.04</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>242.67</v>
+        <v>258.10000000000002</v>
       </c>
       <c r="E41" s="13">
-        <v>205.36</v>
+        <v>217.45</v>
       </c>
       <c r="F41" s="13">
-        <v>215.36</v>
+        <v>227.45</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>240.15</v>
+        <v>243.04</v>
       </c>
       <c r="E42" s="10">
-        <v>202.3</v>
+        <v>204.94</v>
       </c>
       <c r="F42" s="10">
-        <v>212.3</v>
+        <v>214.94</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>239.78</v>
+        <v>242.67</v>
       </c>
       <c r="E43" s="13">
-        <v>202.71</v>
+        <v>205.36</v>
       </c>
       <c r="F43" s="13">
-        <v>212.71</v>
+        <v>215.36</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>244.02</v>
+        <v>260.14</v>
       </c>
       <c r="E47" s="10">
-        <v>204.06</v>
+        <v>215.76</v>
       </c>
       <c r="F47" s="10">
-        <v>214.06</v>
+        <v>225.76</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>243.73</v>
+        <v>259.87</v>
       </c>
       <c r="E48" s="13">
-        <v>204.06</v>
+        <v>215.78</v>
       </c>
       <c r="F48" s="13">
-        <v>214.06</v>
+        <v>225.78</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>237.32</v>
+        <v>244.02</v>
       </c>
       <c r="E49" s="10">
-        <v>199.12</v>
+        <v>204.06</v>
       </c>
       <c r="F49" s="10">
-        <v>209.12</v>
+        <v>214.06</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>237.02</v>
+        <v>243.73</v>
       </c>
       <c r="E50" s="13">
-        <v>199.12</v>
+        <v>204.06</v>
       </c>
       <c r="F50" s="13">
-        <v>209.12</v>
+        <v>214.06</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>254.24</v>
+        <v>272.99</v>
       </c>
       <c r="E54" s="10">
-        <v>216.52</v>
+        <v>228.09</v>
       </c>
       <c r="F54" s="10">
-        <v>226.52</v>
+        <v>238.09</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>244.67</v>
+        <v>261.20999999999998</v>
       </c>
       <c r="E55" s="13">
-        <v>218.89</v>
+        <v>230.47</v>
       </c>
       <c r="F55" s="13">
-        <v>228.89</v>
+        <v>240.47</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>245.7</v>
+        <v>265.52999999999997</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>245.99</v>
+        <v>265.81</v>
       </c>
       <c r="E57" s="13">
-        <v>213.28</v>
+        <v>224.86</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>241.8</v>
+        <v>261.63</v>
       </c>
       <c r="E58" s="10">
-        <v>209.21</v>
+        <v>220.79</v>
       </c>
       <c r="F58" s="10">
-        <v>219.21</v>
+        <v>230.79</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>246.64</v>
+        <v>265.38</v>
       </c>
       <c r="E59" s="13">
-        <v>214.6</v>
+        <v>226.18</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>251.34</v>
+        <v>254.24</v>
       </c>
       <c r="E60" s="10">
-        <v>212.44</v>
+        <v>216.52</v>
       </c>
       <c r="F60" s="10">
-        <v>222.44</v>
+        <v>226.52</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>241.77</v>
+        <v>244.67</v>
       </c>
       <c r="E61" s="13">
-        <v>214.72</v>
+        <v>218.89</v>
       </c>
       <c r="F61" s="13">
-        <v>224.72</v>
+        <v>228.89</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>242.8</v>
+        <v>245.7</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>243.06</v>
+        <v>245.99</v>
       </c>
       <c r="E63" s="13">
-        <v>209.11</v>
+        <v>213.28</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>238.87</v>
+        <v>241.8</v>
       </c>
       <c r="E64" s="10">
-        <v>205.04</v>
+        <v>209.21</v>
       </c>
       <c r="F64" s="10">
-        <v>215.04</v>
+        <v>219.21</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>243.7</v>
+        <v>246.64</v>
       </c>
       <c r="E65" s="13">
-        <v>210.48</v>
+        <v>214.6</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,14 +1850,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2121,28 +2119,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2168,9 +2158,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Mon Mar 16 04:13:21 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{05764E49-E093-4905-BD8F-22A14921E1FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{7F3733D1-6B5E-49F9-8107-B24FCB0E8960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>259.35000000000002</v>
+        <v>263</v>
       </c>
       <c r="E8" s="10">
-        <v>216.1</v>
+        <v>221.47</v>
       </c>
       <c r="F8" s="10">
-        <v>226.11</v>
+        <v>231.47</v>
       </c>
       <c r="G8" s="10">
-        <v>215.99</v>
+        <v>221.36</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>259.35000000000002</v>
+        <v>263</v>
       </c>
       <c r="E9" s="13">
-        <v>216.1</v>
+        <v>221.47</v>
       </c>
       <c r="F9" s="13">
-        <v>226.11</v>
+        <v>231.47</v>
       </c>
       <c r="G9" s="13">
-        <v>215.99</v>
+        <v>221.36</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>260.38</v>
+        <v>266.32</v>
       </c>
       <c r="E10" s="10">
-        <v>218.42</v>
+        <v>223.33</v>
       </c>
       <c r="F10" s="10">
-        <v>228.42</v>
+        <v>233.33</v>
       </c>
       <c r="G10" s="10">
-        <v>218.67</v>
+        <v>223.57</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>240.85</v>
+        <v>259.35000000000002</v>
       </c>
       <c r="E11" s="13">
-        <v>204.73</v>
+        <v>216.1</v>
       </c>
       <c r="F11" s="13">
-        <v>214.73</v>
+        <v>226.11</v>
       </c>
       <c r="G11" s="13">
-        <v>204.61</v>
+        <v>215.99</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>240.85</v>
+        <v>259.35000000000002</v>
       </c>
       <c r="E12" s="10">
-        <v>204.73</v>
+        <v>216.1</v>
       </c>
       <c r="F12" s="10">
-        <v>214.73</v>
+        <v>226.11</v>
       </c>
       <c r="G12" s="10">
-        <v>204.61</v>
+        <v>215.99</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>242.97</v>
+        <v>260.38</v>
       </c>
       <c r="E13" s="13">
-        <v>207.71</v>
+        <v>218.42</v>
       </c>
       <c r="F13" s="13">
-        <v>217.71</v>
+        <v>228.42</v>
       </c>
       <c r="G13" s="13">
-        <v>207.95</v>
+        <v>218.67</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>256.45999999999998</v>
+        <v>263.5</v>
       </c>
       <c r="E17" s="10">
-        <v>217.71</v>
+        <v>223.18</v>
       </c>
       <c r="F17" s="10">
-        <v>227.71</v>
+        <v>233.18</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>245.41</v>
+        <v>256.45999999999998</v>
       </c>
       <c r="E18" s="13">
-        <v>209.38</v>
+        <v>217.71</v>
       </c>
       <c r="F18" s="13">
-        <v>219.38</v>
+        <v>227.71</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>259.04000000000002</v>
+        <v>262.68</v>
       </c>
       <c r="E22" s="10">
-        <v>218.2</v>
+        <v>223.57</v>
       </c>
       <c r="F22" s="10">
-        <v>227.8</v>
+        <v>233.17</v>
       </c>
       <c r="G22" s="10">
-        <v>219.95</v>
+        <v>225.32</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>266.98</v>
+        <v>271.27999999999997</v>
       </c>
       <c r="E23" s="13">
-        <v>225.13</v>
+        <v>228.95</v>
       </c>
       <c r="F23" s="13">
-        <v>235.13</v>
+        <v>238.95</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>267.13</v>
+        <v>271.42</v>
       </c>
       <c r="E24" s="10">
-        <v>225.66</v>
+        <v>229.47</v>
       </c>
       <c r="F24" s="10">
-        <v>235.66</v>
+        <v>239.47</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>267.11</v>
+        <v>271.39999999999998</v>
       </c>
       <c r="E25" s="13">
-        <v>225.31</v>
+        <v>229.13</v>
       </c>
       <c r="F25" s="13">
-        <v>235.31</v>
+        <v>239.13</v>
       </c>
       <c r="G25" s="13">
-        <v>226.16</v>
+        <v>229.98</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>266.70999999999998</v>
+        <v>271</v>
       </c>
       <c r="E26" s="10">
-        <v>227.33</v>
+        <v>231.19</v>
       </c>
       <c r="F26" s="10">
-        <v>237.33</v>
+        <v>241.19</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>240.54</v>
+        <v>259.04000000000002</v>
       </c>
       <c r="E27" s="13">
-        <v>206.83</v>
+        <v>218.2</v>
       </c>
       <c r="F27" s="13">
-        <v>216.43</v>
+        <v>227.8</v>
       </c>
       <c r="G27" s="13">
-        <v>208.58</v>
+        <v>219.95</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>248.25</v>
+        <v>266.98</v>
       </c>
       <c r="E28" s="22">
-        <v>213.51</v>
+        <v>225.13</v>
       </c>
       <c r="F28" s="22">
-        <v>223.51</v>
+        <v>235.13</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>248.39</v>
+        <v>267.13</v>
       </c>
       <c r="E29" s="13">
-        <v>214.07</v>
+        <v>225.66</v>
       </c>
       <c r="F29" s="13">
-        <v>224.07</v>
+        <v>235.66</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>248.37</v>
+        <v>267.11</v>
       </c>
       <c r="E30" s="22">
-        <v>213.71</v>
+        <v>225.31</v>
       </c>
       <c r="F30" s="22">
-        <v>223.71</v>
+        <v>235.31</v>
       </c>
       <c r="G30" s="22">
-        <v>214.56</v>
+        <v>226.16</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>247.97</v>
+        <v>266.70999999999998</v>
       </c>
       <c r="E31" s="13">
-        <v>215.68</v>
+        <v>227.33</v>
       </c>
       <c r="F31" s="13">
-        <v>225.68</v>
+        <v>237.33</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>259.3</v>
+        <v>266.33</v>
       </c>
       <c r="E35" s="10">
-        <v>217.35</v>
+        <v>222.8</v>
       </c>
       <c r="F35" s="10">
-        <v>226.35</v>
+        <v>231.8</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>240.57</v>
+        <v>259.3</v>
       </c>
       <c r="E36" s="13">
-        <v>205.76</v>
+        <v>217.35</v>
       </c>
       <c r="F36" s="13">
-        <v>214.76</v>
+        <v>226.35</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>258.47000000000003</v>
+        <v>265.51</v>
       </c>
       <c r="E40" s="10">
-        <v>217.04</v>
+        <v>221.49</v>
       </c>
       <c r="F40" s="10">
-        <v>227.04</v>
+        <v>231.49</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>258.10000000000002</v>
+        <v>265.13</v>
       </c>
       <c r="E41" s="13">
-        <v>217.45</v>
+        <v>221.91</v>
       </c>
       <c r="F41" s="13">
-        <v>227.45</v>
+        <v>231.91</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>243.04</v>
+        <v>258.47000000000003</v>
       </c>
       <c r="E42" s="10">
-        <v>204.94</v>
+        <v>217.04</v>
       </c>
       <c r="F42" s="10">
-        <v>214.94</v>
+        <v>227.04</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>242.67</v>
+        <v>258.10000000000002</v>
       </c>
       <c r="E43" s="13">
-        <v>205.36</v>
+        <v>217.45</v>
       </c>
       <c r="F43" s="13">
-        <v>215.36</v>
+        <v>227.45</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>260.14</v>
+        <v>262.11</v>
       </c>
       <c r="E47" s="10">
-        <v>215.76</v>
+        <v>221.92</v>
       </c>
       <c r="F47" s="10">
-        <v>225.76</v>
+        <v>231.92</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>259.87</v>
+        <v>261.85000000000002</v>
       </c>
       <c r="E48" s="13">
-        <v>215.78</v>
+        <v>221.95</v>
       </c>
       <c r="F48" s="13">
-        <v>225.78</v>
+        <v>231.95</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>244.02</v>
+        <v>260.14</v>
       </c>
       <c r="E49" s="10">
-        <v>204.06</v>
+        <v>215.76</v>
       </c>
       <c r="F49" s="10">
-        <v>214.06</v>
+        <v>225.76</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>243.73</v>
+        <v>259.87</v>
       </c>
       <c r="E50" s="13">
-        <v>204.06</v>
+        <v>215.78</v>
       </c>
       <c r="F50" s="13">
-        <v>214.06</v>
+        <v>225.78</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>272.99</v>
+        <v>275.64999999999998</v>
       </c>
       <c r="E54" s="10">
-        <v>228.09</v>
+        <v>233.55</v>
       </c>
       <c r="F54" s="10">
-        <v>238.09</v>
+        <v>243.55</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>261.20999999999998</v>
+        <v>268.25</v>
       </c>
       <c r="E55" s="13">
-        <v>230.47</v>
+        <v>233.71</v>
       </c>
       <c r="F55" s="13">
-        <v>240.47</v>
+        <v>243.71</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>265.52999999999997</v>
+        <v>268.17</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>265.81</v>
+        <v>268.43</v>
       </c>
       <c r="E57" s="13">
-        <v>224.86</v>
+        <v>228.09</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>261.63</v>
+        <v>264.26</v>
       </c>
       <c r="E58" s="10">
-        <v>220.79</v>
+        <v>224.03</v>
       </c>
       <c r="F58" s="10">
-        <v>230.79</v>
+        <v>234.03</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>265.38</v>
+        <v>268.02</v>
       </c>
       <c r="E59" s="13">
-        <v>226.18</v>
+        <v>231.65</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>254.24</v>
+        <v>272.99</v>
       </c>
       <c r="E60" s="10">
-        <v>216.52</v>
+        <v>228.09</v>
       </c>
       <c r="F60" s="10">
-        <v>226.52</v>
+        <v>238.09</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>244.67</v>
+        <v>261.20999999999998</v>
       </c>
       <c r="E61" s="13">
-        <v>218.89</v>
+        <v>230.47</v>
       </c>
       <c r="F61" s="13">
-        <v>228.89</v>
+        <v>240.47</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>245.7</v>
+        <v>265.52999999999997</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>245.99</v>
+        <v>265.81</v>
       </c>
       <c r="E63" s="13">
-        <v>213.28</v>
+        <v>224.86</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>241.8</v>
+        <v>261.63</v>
       </c>
       <c r="E64" s="10">
-        <v>209.21</v>
+        <v>220.79</v>
       </c>
       <c r="F64" s="10">
-        <v>219.21</v>
+        <v>230.79</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46094</v>
+        <v>46095</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>246.64</v>
+        <v>265.38</v>
       </c>
       <c r="E65" s="13">
-        <v>214.6</v>
+        <v>226.18</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,15 +1850,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2118,6 +2109,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2130,14 +2130,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2153,6 +2145,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Tue Mar 17 03:43:17 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{7F3733D1-6B5E-49F9-8107-B24FCB0E8960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{E40C9ED2-AFB6-448F-9830-88ABEA6FDC4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>263</v>
+        <v>262.17</v>
       </c>
       <c r="E8" s="10">
-        <v>221.47</v>
+        <v>222.42</v>
       </c>
       <c r="F8" s="10">
-        <v>231.47</v>
+        <v>232.42</v>
       </c>
       <c r="G8" s="10">
-        <v>221.36</v>
+        <v>222.31</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>263</v>
+        <v>262.17</v>
       </c>
       <c r="E9" s="13">
-        <v>221.47</v>
+        <v>222.42</v>
       </c>
       <c r="F9" s="13">
-        <v>231.47</v>
+        <v>232.42</v>
       </c>
       <c r="G9" s="13">
-        <v>221.36</v>
+        <v>222.31</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>266.32</v>
+        <v>265.67</v>
       </c>
       <c r="E10" s="10">
-        <v>223.33</v>
+        <v>224.44</v>
       </c>
       <c r="F10" s="10">
-        <v>233.33</v>
+        <v>234.44</v>
       </c>
       <c r="G10" s="10">
-        <v>223.57</v>
+        <v>224.68</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>259.35000000000002</v>
+        <v>263</v>
       </c>
       <c r="E11" s="13">
-        <v>216.1</v>
+        <v>221.47</v>
       </c>
       <c r="F11" s="13">
-        <v>226.11</v>
+        <v>231.47</v>
       </c>
       <c r="G11" s="13">
-        <v>215.99</v>
+        <v>221.36</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>259.35000000000002</v>
+        <v>263</v>
       </c>
       <c r="E12" s="10">
-        <v>216.1</v>
+        <v>221.47</v>
       </c>
       <c r="F12" s="10">
-        <v>226.11</v>
+        <v>231.47</v>
       </c>
       <c r="G12" s="10">
-        <v>215.99</v>
+        <v>221.36</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>260.38</v>
+        <v>266.32</v>
       </c>
       <c r="E13" s="13">
-        <v>218.42</v>
+        <v>223.33</v>
       </c>
       <c r="F13" s="13">
-        <v>228.42</v>
+        <v>233.33</v>
       </c>
       <c r="G13" s="13">
-        <v>218.67</v>
+        <v>223.57</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>263.5</v>
+        <v>262.85000000000002</v>
       </c>
       <c r="E17" s="10">
-        <v>223.18</v>
+        <v>224.29</v>
       </c>
       <c r="F17" s="10">
-        <v>233.18</v>
+        <v>234.29</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>256.45999999999998</v>
+        <v>263.5</v>
       </c>
       <c r="E18" s="13">
-        <v>217.71</v>
+        <v>223.18</v>
       </c>
       <c r="F18" s="13">
-        <v>227.71</v>
+        <v>233.18</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>262.68</v>
+        <v>261.85000000000002</v>
       </c>
       <c r="E22" s="10">
-        <v>223.57</v>
+        <v>224.52</v>
       </c>
       <c r="F22" s="10">
-        <v>233.17</v>
+        <v>234.12</v>
       </c>
       <c r="G22" s="10">
-        <v>225.32</v>
+        <v>226.27</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>271.27999999999997</v>
+        <v>270.62</v>
       </c>
       <c r="E23" s="13">
-        <v>228.95</v>
+        <v>230.06</v>
       </c>
       <c r="F23" s="13">
-        <v>238.95</v>
+        <v>240.06</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>271.42</v>
+        <v>270.76</v>
       </c>
       <c r="E24" s="10">
-        <v>229.47</v>
+        <v>230.57</v>
       </c>
       <c r="F24" s="10">
-        <v>239.47</v>
+        <v>240.57</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>271.39999999999998</v>
+        <v>270.74</v>
       </c>
       <c r="E25" s="13">
-        <v>229.13</v>
+        <v>230.24</v>
       </c>
       <c r="F25" s="13">
-        <v>239.13</v>
+        <v>240.24</v>
       </c>
       <c r="G25" s="13">
-        <v>229.98</v>
+        <v>231.09</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>271</v>
+        <v>270.35000000000002</v>
       </c>
       <c r="E26" s="10">
-        <v>231.19</v>
+        <v>232.3</v>
       </c>
       <c r="F26" s="10">
-        <v>241.19</v>
+        <v>242.3</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>259.04000000000002</v>
+        <v>262.68</v>
       </c>
       <c r="E27" s="13">
-        <v>218.2</v>
+        <v>223.57</v>
       </c>
       <c r="F27" s="13">
-        <v>227.8</v>
+        <v>233.17</v>
       </c>
       <c r="G27" s="13">
-        <v>219.95</v>
+        <v>225.32</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>266.98</v>
+        <v>271.27999999999997</v>
       </c>
       <c r="E28" s="22">
-        <v>225.13</v>
+        <v>228.95</v>
       </c>
       <c r="F28" s="22">
-        <v>235.13</v>
+        <v>238.95</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>267.13</v>
+        <v>271.42</v>
       </c>
       <c r="E29" s="13">
-        <v>225.66</v>
+        <v>229.47</v>
       </c>
       <c r="F29" s="13">
-        <v>235.66</v>
+        <v>239.47</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>267.11</v>
+        <v>271.39999999999998</v>
       </c>
       <c r="E30" s="22">
-        <v>225.31</v>
+        <v>229.13</v>
       </c>
       <c r="F30" s="22">
-        <v>235.31</v>
+        <v>239.13</v>
       </c>
       <c r="G30" s="22">
-        <v>226.16</v>
+        <v>229.98</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>266.70999999999998</v>
+        <v>271</v>
       </c>
       <c r="E31" s="13">
-        <v>227.33</v>
+        <v>231.19</v>
       </c>
       <c r="F31" s="13">
-        <v>237.33</v>
+        <v>241.19</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>266.33</v>
+        <v>265.67</v>
       </c>
       <c r="E35" s="10">
-        <v>222.8</v>
+        <v>223.9</v>
       </c>
       <c r="F35" s="10">
-        <v>231.8</v>
+        <v>232.9</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>259.3</v>
+        <v>266.33</v>
       </c>
       <c r="E36" s="13">
-        <v>217.35</v>
+        <v>222.8</v>
       </c>
       <c r="F36" s="13">
-        <v>226.35</v>
+        <v>231.8</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>265.51</v>
+        <v>264.85000000000002</v>
       </c>
       <c r="E40" s="10">
-        <v>221.49</v>
+        <v>221.59</v>
       </c>
       <c r="F40" s="10">
-        <v>231.49</v>
+        <v>231.59</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>265.13</v>
+        <v>264.48</v>
       </c>
       <c r="E41" s="13">
-        <v>221.91</v>
+        <v>222.01</v>
       </c>
       <c r="F41" s="13">
-        <v>231.91</v>
+        <v>232.01</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>258.47000000000003</v>
+        <v>265.51</v>
       </c>
       <c r="E42" s="10">
-        <v>217.04</v>
+        <v>221.49</v>
       </c>
       <c r="F42" s="10">
-        <v>227.04</v>
+        <v>231.49</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>258.10000000000002</v>
+        <v>265.13</v>
       </c>
       <c r="E43" s="13">
-        <v>217.45</v>
+        <v>221.91</v>
       </c>
       <c r="F43" s="13">
-        <v>227.45</v>
+        <v>231.91</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>262.11</v>
+        <v>265.89</v>
       </c>
       <c r="E47" s="10">
-        <v>221.92</v>
+        <v>227.99</v>
       </c>
       <c r="F47" s="10">
-        <v>231.92</v>
+        <v>237.99</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>261.85000000000002</v>
+        <v>265.64</v>
       </c>
       <c r="E48" s="13">
-        <v>221.95</v>
+        <v>228.04</v>
       </c>
       <c r="F48" s="13">
-        <v>231.95</v>
+        <v>238.04</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>260.14</v>
+        <v>262.11</v>
       </c>
       <c r="E49" s="10">
-        <v>215.76</v>
+        <v>221.92</v>
       </c>
       <c r="F49" s="10">
-        <v>225.76</v>
+        <v>231.92</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>259.87</v>
+        <v>261.85000000000002</v>
       </c>
       <c r="E50" s="13">
-        <v>215.78</v>
+        <v>221.95</v>
       </c>
       <c r="F50" s="13">
-        <v>225.78</v>
+        <v>231.95</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>275.64999999999998</v>
+        <v>275</v>
       </c>
       <c r="E54" s="10">
-        <v>233.55</v>
+        <v>234.63</v>
       </c>
       <c r="F54" s="10">
-        <v>243.55</v>
+        <v>244.63</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>268.25</v>
+        <v>267.58999999999997</v>
       </c>
       <c r="E55" s="13">
-        <v>233.71</v>
+        <v>234.82</v>
       </c>
       <c r="F55" s="13">
-        <v>243.71</v>
+        <v>244.82</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>268.17</v>
+        <v>267.51</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>268.43</v>
+        <v>267.77999999999997</v>
       </c>
       <c r="E57" s="13">
-        <v>228.09</v>
+        <v>229.2</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>264.26</v>
+        <v>263.61</v>
       </c>
       <c r="E58" s="10">
-        <v>224.03</v>
+        <v>225.14</v>
       </c>
       <c r="F58" s="10">
-        <v>234.03</v>
+        <v>235.14</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>268.02</v>
+        <v>267.37</v>
       </c>
       <c r="E59" s="13">
-        <v>231.65</v>
+        <v>232.75</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>272.99</v>
+        <v>275.64999999999998</v>
       </c>
       <c r="E60" s="10">
-        <v>228.09</v>
+        <v>233.55</v>
       </c>
       <c r="F60" s="10">
-        <v>238.09</v>
+        <v>243.55</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>261.20999999999998</v>
+        <v>268.25</v>
       </c>
       <c r="E61" s="13">
-        <v>230.47</v>
+        <v>233.71</v>
       </c>
       <c r="F61" s="13">
-        <v>240.47</v>
+        <v>243.71</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>265.52999999999997</v>
+        <v>268.17</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>265.81</v>
+        <v>268.43</v>
       </c>
       <c r="E63" s="13">
-        <v>224.86</v>
+        <v>228.09</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>261.63</v>
+        <v>264.26</v>
       </c>
       <c r="E64" s="10">
-        <v>220.79</v>
+        <v>224.03</v>
       </c>
       <c r="F64" s="10">
-        <v>230.79</v>
+        <v>234.03</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46095</v>
+        <v>46098</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>265.38</v>
+        <v>268.02</v>
       </c>
       <c r="E65" s="13">
-        <v>226.18</v>
+        <v>231.65</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -2110,15 +2110,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -2127,6 +2118,15 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2150,14 +2150,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -2175,6 +2167,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Wed Mar 18 03:57:54 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{E40C9ED2-AFB6-448F-9830-88ABEA6FDC4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{EC2449D1-AF70-4B2E-B002-233089EC5BFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>262.17</v>
+        <v>269.24</v>
       </c>
       <c r="E8" s="10">
-        <v>222.42</v>
+        <v>225.51</v>
       </c>
       <c r="F8" s="10">
-        <v>232.42</v>
+        <v>235.51</v>
       </c>
       <c r="G8" s="10">
-        <v>222.31</v>
+        <v>225.4</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>262.17</v>
+        <v>269.24</v>
       </c>
       <c r="E9" s="13">
-        <v>222.42</v>
+        <v>225.51</v>
       </c>
       <c r="F9" s="13">
-        <v>232.42</v>
+        <v>235.51</v>
       </c>
       <c r="G9" s="13">
-        <v>222.31</v>
+        <v>225.4</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>265.67</v>
+        <v>272.81</v>
       </c>
       <c r="E10" s="10">
-        <v>224.44</v>
+        <v>227.6</v>
       </c>
       <c r="F10" s="10">
-        <v>234.44</v>
+        <v>237.6</v>
       </c>
       <c r="G10" s="10">
-        <v>224.68</v>
+        <v>227.84</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>263</v>
+        <v>262.17</v>
       </c>
       <c r="E11" s="13">
-        <v>221.47</v>
+        <v>222.42</v>
       </c>
       <c r="F11" s="13">
-        <v>231.47</v>
+        <v>232.42</v>
       </c>
       <c r="G11" s="13">
-        <v>221.36</v>
+        <v>222.31</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>263</v>
+        <v>262.17</v>
       </c>
       <c r="E12" s="10">
-        <v>221.47</v>
+        <v>222.42</v>
       </c>
       <c r="F12" s="10">
-        <v>231.47</v>
+        <v>232.42</v>
       </c>
       <c r="G12" s="10">
-        <v>221.36</v>
+        <v>222.31</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>266.32</v>
+        <v>265.67</v>
       </c>
       <c r="E13" s="13">
-        <v>223.33</v>
+        <v>224.44</v>
       </c>
       <c r="F13" s="13">
-        <v>233.33</v>
+        <v>234.44</v>
       </c>
       <c r="G13" s="13">
-        <v>223.57</v>
+        <v>224.68</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>262.85000000000002</v>
+        <v>270</v>
       </c>
       <c r="E17" s="10">
-        <v>224.29</v>
+        <v>227.48</v>
       </c>
       <c r="F17" s="10">
-        <v>234.29</v>
+        <v>237.48</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>263.5</v>
+        <v>262.85000000000002</v>
       </c>
       <c r="E18" s="13">
-        <v>223.18</v>
+        <v>224.29</v>
       </c>
       <c r="F18" s="13">
-        <v>233.18</v>
+        <v>234.29</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>261.85000000000002</v>
+        <v>268.92</v>
       </c>
       <c r="E22" s="10">
-        <v>224.52</v>
+        <v>227.61</v>
       </c>
       <c r="F22" s="10">
-        <v>234.12</v>
+        <v>237.21</v>
       </c>
       <c r="G22" s="10">
-        <v>226.27</v>
+        <v>229.36</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>270.62</v>
+        <v>277.77</v>
       </c>
       <c r="E23" s="13">
-        <v>230.06</v>
+        <v>233.23</v>
       </c>
       <c r="F23" s="13">
-        <v>240.06</v>
+        <v>243.23</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>270.76</v>
+        <v>277.91000000000003</v>
       </c>
       <c r="E24" s="10">
-        <v>230.57</v>
+        <v>233.74</v>
       </c>
       <c r="F24" s="10">
-        <v>240.57</v>
+        <v>243.74</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>270.74</v>
+        <v>277.89</v>
       </c>
       <c r="E25" s="13">
-        <v>230.24</v>
+        <v>233.41</v>
       </c>
       <c r="F25" s="13">
-        <v>240.24</v>
+        <v>243.41</v>
       </c>
       <c r="G25" s="13">
-        <v>231.09</v>
+        <v>234.26</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>270.35000000000002</v>
+        <v>277.51</v>
       </c>
       <c r="E26" s="10">
-        <v>232.3</v>
+        <v>235.52</v>
       </c>
       <c r="F26" s="10">
-        <v>242.3</v>
+        <v>245.52</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>262.68</v>
+        <v>261.85000000000002</v>
       </c>
       <c r="E27" s="13">
-        <v>223.57</v>
+        <v>224.52</v>
       </c>
       <c r="F27" s="13">
-        <v>233.17</v>
+        <v>234.12</v>
       </c>
       <c r="G27" s="13">
-        <v>225.32</v>
+        <v>226.27</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>271.27999999999997</v>
+        <v>270.62</v>
       </c>
       <c r="E28" s="22">
-        <v>228.95</v>
+        <v>230.06</v>
       </c>
       <c r="F28" s="22">
-        <v>238.95</v>
+        <v>240.06</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>271.42</v>
+        <v>270.76</v>
       </c>
       <c r="E29" s="13">
-        <v>229.47</v>
+        <v>230.57</v>
       </c>
       <c r="F29" s="13">
-        <v>239.47</v>
+        <v>240.57</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>271.39999999999998</v>
+        <v>270.74</v>
       </c>
       <c r="E30" s="22">
-        <v>229.13</v>
+        <v>230.24</v>
       </c>
       <c r="F30" s="22">
-        <v>239.13</v>
+        <v>240.24</v>
       </c>
       <c r="G30" s="22">
-        <v>229.98</v>
+        <v>231.09</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>271</v>
+        <v>270.35000000000002</v>
       </c>
       <c r="E31" s="13">
-        <v>231.19</v>
+        <v>232.3</v>
       </c>
       <c r="F31" s="13">
-        <v>241.19</v>
+        <v>242.3</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>265.67</v>
+        <v>271.72000000000003</v>
       </c>
       <c r="E35" s="10">
-        <v>223.9</v>
+        <v>227.06</v>
       </c>
       <c r="F35" s="10">
-        <v>232.9</v>
+        <v>236.06</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>266.33</v>
+        <v>265.67</v>
       </c>
       <c r="E36" s="13">
-        <v>222.8</v>
+        <v>223.9</v>
       </c>
       <c r="F36" s="13">
-        <v>231.8</v>
+        <v>232.9</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>264.85000000000002</v>
+        <v>272.01</v>
       </c>
       <c r="E40" s="10">
-        <v>221.59</v>
+        <v>223.75</v>
       </c>
       <c r="F40" s="10">
-        <v>231.59</v>
+        <v>233.75</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>264.48</v>
+        <v>271.62</v>
       </c>
       <c r="E41" s="13">
-        <v>222.01</v>
+        <v>224.17</v>
       </c>
       <c r="F41" s="13">
-        <v>232.01</v>
+        <v>234.17</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>265.51</v>
+        <v>264.85000000000002</v>
       </c>
       <c r="E42" s="10">
-        <v>221.49</v>
+        <v>221.59</v>
       </c>
       <c r="F42" s="10">
-        <v>231.49</v>
+        <v>231.59</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>265.13</v>
+        <v>264.48</v>
       </c>
       <c r="E43" s="13">
-        <v>221.91</v>
+        <v>222.01</v>
       </c>
       <c r="F43" s="13">
-        <v>231.91</v>
+        <v>232.01</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>265.89</v>
+        <v>268.37</v>
       </c>
       <c r="E47" s="10">
-        <v>227.99</v>
+        <v>231.07</v>
       </c>
       <c r="F47" s="10">
-        <v>237.99</v>
+        <v>241.07</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>265.64</v>
+        <v>268.13</v>
       </c>
       <c r="E48" s="13">
-        <v>228.04</v>
+        <v>231.13</v>
       </c>
       <c r="F48" s="13">
-        <v>238.04</v>
+        <v>241.13</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>262.11</v>
+        <v>265.89</v>
       </c>
       <c r="E49" s="10">
-        <v>221.92</v>
+        <v>227.99</v>
       </c>
       <c r="F49" s="10">
-        <v>231.92</v>
+        <v>237.99</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>261.85000000000002</v>
+        <v>265.64</v>
       </c>
       <c r="E50" s="13">
-        <v>221.95</v>
+        <v>228.04</v>
       </c>
       <c r="F50" s="13">
-        <v>231.95</v>
+        <v>238.04</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>275</v>
+        <v>282.17</v>
       </c>
       <c r="E54" s="10">
-        <v>234.63</v>
+        <v>237.79</v>
       </c>
       <c r="F54" s="10">
-        <v>244.63</v>
+        <v>247.79</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>267.58999999999997</v>
+        <v>274.75</v>
       </c>
       <c r="E55" s="13">
-        <v>234.82</v>
+        <v>237.97</v>
       </c>
       <c r="F55" s="13">
-        <v>244.82</v>
+        <v>247.97</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>267.51</v>
+        <v>274.64999999999998</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>267.77999999999997</v>
+        <v>274.91000000000003</v>
       </c>
       <c r="E57" s="13">
-        <v>229.2</v>
+        <v>232.35</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>263.61</v>
+        <v>270.74</v>
       </c>
       <c r="E58" s="10">
-        <v>225.14</v>
+        <v>228.29</v>
       </c>
       <c r="F58" s="10">
-        <v>235.14</v>
+        <v>238.29</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>267.37</v>
+        <v>274.52</v>
       </c>
       <c r="E59" s="13">
-        <v>232.75</v>
+        <v>235.92</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>275.64999999999998</v>
+        <v>275</v>
       </c>
       <c r="E60" s="10">
-        <v>233.55</v>
+        <v>234.63</v>
       </c>
       <c r="F60" s="10">
-        <v>243.55</v>
+        <v>244.63</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>268.25</v>
+        <v>267.58999999999997</v>
       </c>
       <c r="E61" s="13">
-        <v>233.71</v>
+        <v>234.82</v>
       </c>
       <c r="F61" s="13">
-        <v>243.71</v>
+        <v>244.82</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>268.17</v>
+        <v>267.51</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>268.43</v>
+        <v>267.77999999999997</v>
       </c>
       <c r="E63" s="13">
-        <v>228.09</v>
+        <v>229.2</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>264.26</v>
+        <v>263.61</v>
       </c>
       <c r="E64" s="10">
-        <v>224.03</v>
+        <v>225.14</v>
       </c>
       <c r="F64" s="10">
-        <v>234.03</v>
+        <v>235.14</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46098</v>
+        <v>46099</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>268.02</v>
+        <v>267.37</v>
       </c>
       <c r="E65" s="13">
-        <v>231.65</v>
+        <v>232.75</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,6 +1850,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2109,42 +2129,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2168,9 +2156,21 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Thu Mar 19 03:57:29 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{EC2449D1-AF70-4B2E-B002-233089EC5BFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{19B93D3E-F551-48E6-9543-9EF9961054AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-345" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -708,16 +708,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G65"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125"/>
-    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.3984375"/>
+    <col min="3" max="3" width="18.265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.86328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="6.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
       <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
@@ -728,7 +728,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -737,7 +737,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -748,7 +748,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -759,7 +759,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -768,7 +768,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A6" s="27" t="s">
         <v>3</v>
       </c>
@@ -779,7 +779,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -800,133 +800,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>269.24</v>
+        <v>279.64</v>
       </c>
       <c r="E8" s="10">
-        <v>225.51</v>
+        <v>230.51</v>
       </c>
       <c r="F8" s="10">
-        <v>235.51</v>
+        <v>240.51</v>
       </c>
       <c r="G8" s="10">
-        <v>225.4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>230.39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>269.24</v>
+        <v>279.64</v>
       </c>
       <c r="E9" s="13">
-        <v>225.51</v>
+        <v>230.51</v>
       </c>
       <c r="F9" s="13">
-        <v>235.51</v>
+        <v>240.51</v>
       </c>
       <c r="G9" s="13">
-        <v>225.4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>230.39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>272.81</v>
+        <v>283.2</v>
       </c>
       <c r="E10" s="10">
-        <v>227.6</v>
+        <v>232.6</v>
       </c>
       <c r="F10" s="10">
-        <v>237.6</v>
+        <v>242.6</v>
       </c>
       <c r="G10" s="10">
-        <v>227.84</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>232.84</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>262.17</v>
+        <v>269.24</v>
       </c>
       <c r="E11" s="13">
-        <v>222.42</v>
+        <v>225.51</v>
       </c>
       <c r="F11" s="13">
-        <v>232.42</v>
+        <v>235.51</v>
       </c>
       <c r="G11" s="13">
-        <v>222.31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>225.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>262.17</v>
+        <v>269.24</v>
       </c>
       <c r="E12" s="10">
-        <v>222.42</v>
+        <v>225.51</v>
       </c>
       <c r="F12" s="10">
-        <v>232.42</v>
+        <v>235.51</v>
       </c>
       <c r="G12" s="10">
-        <v>222.31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>225.4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>265.67</v>
+        <v>272.81</v>
       </c>
       <c r="E13" s="13">
-        <v>224.44</v>
+        <v>227.6</v>
       </c>
       <c r="F13" s="13">
-        <v>234.44</v>
+        <v>237.6</v>
       </c>
       <c r="G13" s="13">
-        <v>224.68</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>227.84</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -935,7 +935,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A15" s="27" t="s">
         <v>13</v>
       </c>
@@ -946,7 +946,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -965,45 +965,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>270</v>
+        <v>280.38</v>
       </c>
       <c r="E17" s="10">
-        <v>227.48</v>
+        <v>232.49</v>
       </c>
       <c r="F17" s="10">
-        <v>237.48</v>
+        <v>242.49</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>262.85000000000002</v>
+        <v>270</v>
       </c>
       <c r="E18" s="13">
-        <v>224.29</v>
+        <v>227.48</v>
       </c>
       <c r="F18" s="13">
-        <v>234.29</v>
+        <v>237.48</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1012,7 +1012,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A20" s="27" t="s">
         <v>15</v>
       </c>
@@ -1023,7 +1023,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1044,217 +1044,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>268.92</v>
+        <v>279.31</v>
       </c>
       <c r="E22" s="10">
-        <v>227.61</v>
+        <v>232.6</v>
       </c>
       <c r="F22" s="10">
-        <v>237.21</v>
+        <v>242.2</v>
       </c>
       <c r="G22" s="10">
-        <v>229.36</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>234.35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>277.77</v>
+        <v>284.87</v>
       </c>
       <c r="E23" s="13">
-        <v>233.23</v>
+        <v>238.24</v>
       </c>
       <c r="F23" s="13">
-        <v>243.23</v>
+        <v>248.24</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>277.91000000000003</v>
+        <v>285</v>
       </c>
       <c r="E24" s="10">
-        <v>233.74</v>
+        <v>238.74</v>
       </c>
       <c r="F24" s="10">
-        <v>243.74</v>
+        <v>248.74</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>277.89</v>
+        <v>284.98</v>
       </c>
       <c r="E25" s="13">
-        <v>233.41</v>
+        <v>238.42</v>
       </c>
       <c r="F25" s="13">
-        <v>243.41</v>
+        <v>248.42</v>
       </c>
       <c r="G25" s="13">
-        <v>234.26</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>239.27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>277.51</v>
+        <v>284.60000000000002</v>
       </c>
       <c r="E26" s="10">
-        <v>235.52</v>
+        <v>240.56</v>
       </c>
       <c r="F26" s="10">
-        <v>245.52</v>
+        <v>250.56</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>261.85000000000002</v>
+        <v>268.92</v>
       </c>
       <c r="E27" s="13">
-        <v>224.52</v>
+        <v>227.61</v>
       </c>
       <c r="F27" s="13">
-        <v>234.12</v>
+        <v>237.21</v>
       </c>
       <c r="G27" s="13">
-        <v>226.27</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>229.36</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>270.62</v>
+        <v>277.77</v>
       </c>
       <c r="E28" s="22">
-        <v>230.06</v>
+        <v>233.23</v>
       </c>
       <c r="F28" s="22">
-        <v>240.06</v>
+        <v>243.23</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>270.76</v>
+        <v>277.91000000000003</v>
       </c>
       <c r="E29" s="13">
-        <v>230.57</v>
+        <v>233.74</v>
       </c>
       <c r="F29" s="13">
-        <v>240.57</v>
+        <v>243.74</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>270.74</v>
+        <v>277.89</v>
       </c>
       <c r="E30" s="22">
-        <v>230.24</v>
+        <v>233.41</v>
       </c>
       <c r="F30" s="22">
-        <v>240.24</v>
+        <v>243.41</v>
       </c>
       <c r="G30" s="22">
-        <v>231.09</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>234.26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>270.35000000000002</v>
+        <v>277.51</v>
       </c>
       <c r="E31" s="13">
-        <v>232.3</v>
+        <v>235.52</v>
       </c>
       <c r="F31" s="13">
-        <v>242.3</v>
+        <v>245.52</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1263,7 +1263,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A33" s="27" t="s">
         <v>22</v>
       </c>
@@ -1274,7 +1274,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1293,45 +1293,45 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>271.72000000000003</v>
+        <v>278.8</v>
       </c>
       <c r="E35" s="10">
-        <v>227.06</v>
+        <v>232.05</v>
       </c>
       <c r="F35" s="10">
-        <v>236.06</v>
+        <v>241.05</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>265.67</v>
+        <v>271.72000000000003</v>
       </c>
       <c r="E36" s="13">
-        <v>223.9</v>
+        <v>227.06</v>
       </c>
       <c r="F36" s="13">
-        <v>232.9</v>
+        <v>236.06</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="14"/>
       <c r="B37" s="14"/>
       <c r="C37" s="15"/>
@@ -1340,7 +1340,7 @@
       <c r="F37" s="16"/>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A38" s="27" t="s">
         <v>24</v>
       </c>
@@ -1351,7 +1351,7 @@
       <c r="F38" s="17"/>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" s="23" t="s">
         <v>4</v>
       </c>
@@ -1370,83 +1370,83 @@
       </c>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A40" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>272.01</v>
+        <v>282.39999999999998</v>
       </c>
       <c r="E40" s="10">
-        <v>223.75</v>
+        <v>228.54</v>
       </c>
       <c r="F40" s="10">
-        <v>233.75</v>
+        <v>238.54</v>
       </c>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>271.62</v>
+        <v>282</v>
       </c>
       <c r="E41" s="13">
-        <v>224.17</v>
+        <v>228.96</v>
       </c>
       <c r="F41" s="13">
-        <v>234.17</v>
+        <v>238.96</v>
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>264.85000000000002</v>
+        <v>272.01</v>
       </c>
       <c r="E42" s="10">
-        <v>221.59</v>
+        <v>223.75</v>
       </c>
       <c r="F42" s="10">
-        <v>231.59</v>
+        <v>233.75</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>264.48</v>
+        <v>271.62</v>
       </c>
       <c r="E43" s="13">
-        <v>222.01</v>
+        <v>224.17</v>
       </c>
       <c r="F43" s="13">
-        <v>232.01</v>
+        <v>234.17</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="14"/>
       <c r="B44" s="24"/>
       <c r="C44" s="15"/>
@@ -1455,7 +1455,7 @@
       <c r="F44" s="16"/>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="25" t="s">
         <v>27</v>
       </c>
@@ -1466,7 +1466,7 @@
       <c r="F45" s="17"/>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46" s="23" t="s">
         <v>4</v>
       </c>
@@ -1485,83 +1485,83 @@
       </c>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A47" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>268.37</v>
+        <v>273.08</v>
       </c>
       <c r="E47" s="10">
-        <v>231.07</v>
+        <v>231.49</v>
       </c>
       <c r="F47" s="10">
-        <v>241.07</v>
+        <v>241.49</v>
       </c>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A48" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>268.13</v>
+        <v>272.83999999999997</v>
       </c>
       <c r="E48" s="13">
-        <v>231.13</v>
+        <v>231.54</v>
       </c>
       <c r="F48" s="13">
-        <v>241.13</v>
+        <v>241.54</v>
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>265.89</v>
+        <v>268.37</v>
       </c>
       <c r="E49" s="10">
-        <v>227.99</v>
+        <v>231.07</v>
       </c>
       <c r="F49" s="10">
-        <v>237.99</v>
+        <v>241.07</v>
       </c>
       <c r="G49" s="17"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>265.64</v>
+        <v>268.13</v>
       </c>
       <c r="E50" s="13">
-        <v>228.04</v>
+        <v>231.13</v>
       </c>
       <c r="F50" s="13">
-        <v>238.04</v>
+        <v>241.13</v>
       </c>
       <c r="G50" s="17"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="14"/>
       <c r="B51" s="14"/>
       <c r="C51" s="15"/>
@@ -1570,7 +1570,7 @@
       <c r="F51" s="16"/>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A52" s="27" t="s">
         <v>30</v>
       </c>
@@ -1581,7 +1581,7 @@
       <c r="F52" s="17"/>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A53" s="23" t="s">
         <v>4</v>
       </c>
@@ -1600,54 +1600,54 @@
       </c>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A54" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>282.17</v>
+        <v>292.58</v>
       </c>
       <c r="E54" s="10">
-        <v>237.79</v>
+        <v>242.78</v>
       </c>
       <c r="F54" s="10">
-        <v>247.79</v>
+        <v>252.78</v>
       </c>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A55" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>274.75</v>
+        <v>285.14</v>
       </c>
       <c r="E55" s="13">
-        <v>237.97</v>
+        <v>242.95</v>
       </c>
       <c r="F55" s="13">
-        <v>247.97</v>
+        <v>252.95</v>
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>274.64999999999998</v>
+        <v>285.02999999999997</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1657,111 +1657,111 @@
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>274.91000000000003</v>
+        <v>285.27999999999997</v>
       </c>
       <c r="E57" s="13">
-        <v>232.35</v>
+        <v>237.33</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>270.74</v>
+        <v>281.11</v>
       </c>
       <c r="E58" s="10">
-        <v>228.29</v>
+        <v>233.27</v>
       </c>
       <c r="F58" s="10">
-        <v>238.29</v>
+        <v>243.27</v>
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>274.52</v>
+        <v>284.89999999999998</v>
       </c>
       <c r="E59" s="13">
-        <v>235.92</v>
+        <v>240.92</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>275</v>
+        <v>282.17</v>
       </c>
       <c r="E60" s="10">
-        <v>234.63</v>
+        <v>237.79</v>
       </c>
       <c r="F60" s="10">
-        <v>244.63</v>
+        <v>247.79</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>267.58999999999997</v>
+        <v>274.75</v>
       </c>
       <c r="E61" s="13">
-        <v>234.82</v>
+        <v>237.97</v>
       </c>
       <c r="F61" s="13">
-        <v>244.82</v>
+        <v>247.97</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>267.51</v>
+        <v>274.64999999999998</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1771,57 +1771,57 @@
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>267.77999999999997</v>
+        <v>274.91000000000003</v>
       </c>
       <c r="E63" s="13">
-        <v>229.2</v>
+        <v>232.35</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>263.61</v>
+        <v>270.74</v>
       </c>
       <c r="E64" s="10">
-        <v>225.14</v>
+        <v>228.29</v>
       </c>
       <c r="F64" s="10">
-        <v>235.14</v>
+        <v>238.29</v>
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>267.37</v>
+        <v>274.52</v>
       </c>
       <c r="E65" s="13">
-        <v>232.75</v>
+        <v>235.92</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,26 +1850,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2129,10 +2109,42 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2156,21 +2168,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Fri Mar 20 03:39:28 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{19B93D3E-F551-48E6-9543-9EF9961054AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{8B9EEE63-8B11-444D-BFC4-D54AF79E7C48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-345" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -708,16 +708,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G65"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.3984375"/>
-    <col min="3" max="3" width="18.265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125"/>
+    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="6.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
@@ -728,7 +728,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -737,7 +737,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -748,7 +748,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -759,7 +759,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -768,7 +768,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A6" s="27" t="s">
         <v>3</v>
       </c>
@@ -779,7 +779,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -800,133 +800,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>279.64</v>
+        <v>289.3</v>
       </c>
       <c r="E8" s="10">
-        <v>230.51</v>
+        <v>236.27</v>
       </c>
       <c r="F8" s="10">
-        <v>240.51</v>
+        <v>246.27</v>
       </c>
       <c r="G8" s="10">
-        <v>230.39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+        <v>236.15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>279.64</v>
+        <v>289.3</v>
       </c>
       <c r="E9" s="13">
-        <v>230.51</v>
+        <v>236.27</v>
       </c>
       <c r="F9" s="13">
-        <v>240.51</v>
+        <v>246.27</v>
       </c>
       <c r="G9" s="13">
-        <v>230.39</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+        <v>236.15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>283.2</v>
+        <v>292.93</v>
       </c>
       <c r="E10" s="10">
-        <v>232.6</v>
+        <v>238.44</v>
       </c>
       <c r="F10" s="10">
-        <v>242.6</v>
+        <v>248.44</v>
       </c>
       <c r="G10" s="10">
-        <v>232.84</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+        <v>238.68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>269.24</v>
+        <v>279.64</v>
       </c>
       <c r="E11" s="13">
-        <v>225.51</v>
+        <v>230.51</v>
       </c>
       <c r="F11" s="13">
-        <v>235.51</v>
+        <v>240.51</v>
       </c>
       <c r="G11" s="13">
-        <v>225.4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+        <v>230.39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>269.24</v>
+        <v>279.64</v>
       </c>
       <c r="E12" s="10">
-        <v>225.51</v>
+        <v>230.51</v>
       </c>
       <c r="F12" s="10">
-        <v>235.51</v>
+        <v>240.51</v>
       </c>
       <c r="G12" s="10">
-        <v>225.4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+        <v>230.39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>272.81</v>
+        <v>283.2</v>
       </c>
       <c r="E13" s="13">
-        <v>227.6</v>
+        <v>232.6</v>
       </c>
       <c r="F13" s="13">
-        <v>237.6</v>
+        <v>242.6</v>
       </c>
       <c r="G13" s="13">
-        <v>227.84</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+        <v>232.84</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -935,7 +935,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A15" s="27" t="s">
         <v>13</v>
       </c>
@@ -946,7 +946,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -965,45 +965,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>280.38</v>
+        <v>286.8</v>
       </c>
       <c r="E17" s="10">
-        <v>232.49</v>
+        <v>237.22</v>
       </c>
       <c r="F17" s="10">
-        <v>242.49</v>
+        <v>247.22</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>270</v>
+        <v>280.38</v>
       </c>
       <c r="E18" s="13">
-        <v>227.48</v>
+        <v>232.49</v>
       </c>
       <c r="F18" s="13">
-        <v>237.48</v>
+        <v>242.49</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1012,7 +1012,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
         <v>15</v>
       </c>
@@ -1023,7 +1023,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1044,217 +1044,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>279.31</v>
+        <v>288.95999999999998</v>
       </c>
       <c r="E22" s="10">
-        <v>232.6</v>
+        <v>238.91</v>
       </c>
       <c r="F22" s="10">
-        <v>242.2</v>
+        <v>248.51</v>
       </c>
       <c r="G22" s="10">
-        <v>234.35</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+        <v>240.66</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>284.87</v>
+        <v>291.31</v>
       </c>
       <c r="E23" s="13">
-        <v>238.24</v>
+        <v>242.99</v>
       </c>
       <c r="F23" s="13">
-        <v>248.24</v>
+        <v>252.99</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>285</v>
+        <v>291.44</v>
       </c>
       <c r="E24" s="10">
-        <v>238.74</v>
+        <v>243.48</v>
       </c>
       <c r="F24" s="10">
-        <v>248.74</v>
+        <v>253.48</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>284.98</v>
+        <v>291.41000000000003</v>
       </c>
       <c r="E25" s="13">
-        <v>238.42</v>
+        <v>243.18</v>
       </c>
       <c r="F25" s="13">
-        <v>248.42</v>
+        <v>253.18</v>
       </c>
       <c r="G25" s="13">
-        <v>239.27</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+        <v>244.03</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>284.60000000000002</v>
+        <v>291.04000000000002</v>
       </c>
       <c r="E26" s="10">
-        <v>240.56</v>
+        <v>245.36</v>
       </c>
       <c r="F26" s="10">
-        <v>250.56</v>
+        <v>255.36</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>268.92</v>
+        <v>279.31</v>
       </c>
       <c r="E27" s="13">
-        <v>227.61</v>
+        <v>232.6</v>
       </c>
       <c r="F27" s="13">
-        <v>237.21</v>
+        <v>242.2</v>
       </c>
       <c r="G27" s="13">
-        <v>229.36</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+        <v>234.35</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>277.77</v>
+        <v>284.87</v>
       </c>
       <c r="E28" s="22">
-        <v>233.23</v>
+        <v>238.24</v>
       </c>
       <c r="F28" s="22">
-        <v>243.23</v>
+        <v>248.24</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>277.91000000000003</v>
+        <v>285</v>
       </c>
       <c r="E29" s="13">
-        <v>233.74</v>
+        <v>238.74</v>
       </c>
       <c r="F29" s="13">
-        <v>243.74</v>
+        <v>248.74</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>277.89</v>
+        <v>284.98</v>
       </c>
       <c r="E30" s="22">
-        <v>233.41</v>
+        <v>238.42</v>
       </c>
       <c r="F30" s="22">
-        <v>243.41</v>
+        <v>248.42</v>
       </c>
       <c r="G30" s="22">
-        <v>234.26</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+        <v>239.27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>277.51</v>
+        <v>284.60000000000002</v>
       </c>
       <c r="E31" s="13">
-        <v>235.52</v>
+        <v>240.56</v>
       </c>
       <c r="F31" s="13">
-        <v>245.52</v>
+        <v>250.56</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1263,7 +1263,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="27" t="s">
         <v>22</v>
       </c>
@@ -1274,7 +1274,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1293,45 +1293,45 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>278.8</v>
+        <v>285.23</v>
       </c>
       <c r="E35" s="10">
-        <v>232.05</v>
+        <v>236.77</v>
       </c>
       <c r="F35" s="10">
-        <v>241.05</v>
+        <v>245.77</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>271.72000000000003</v>
+        <v>278.8</v>
       </c>
       <c r="E36" s="13">
-        <v>227.06</v>
+        <v>232.05</v>
       </c>
       <c r="F36" s="13">
-        <v>236.06</v>
+        <v>241.05</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="14"/>
       <c r="B37" s="14"/>
       <c r="C37" s="15"/>
@@ -1340,7 +1340,7 @@
       <c r="F37" s="16"/>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A38" s="27" t="s">
         <v>24</v>
       </c>
@@ -1351,7 +1351,7 @@
       <c r="F38" s="17"/>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="23" t="s">
         <v>4</v>
       </c>
@@ -1370,83 +1370,83 @@
       </c>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>282.39999999999998</v>
+        <v>288.85000000000002</v>
       </c>
       <c r="E40" s="10">
-        <v>228.54</v>
+        <v>233.27</v>
       </c>
       <c r="F40" s="10">
-        <v>238.54</v>
+        <v>243.27</v>
       </c>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>282</v>
+        <v>288.45</v>
       </c>
       <c r="E41" s="13">
-        <v>228.96</v>
+        <v>233.68</v>
       </c>
       <c r="F41" s="13">
-        <v>238.96</v>
+        <v>243.68</v>
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>272.01</v>
+        <v>282.39999999999998</v>
       </c>
       <c r="E42" s="10">
-        <v>223.75</v>
+        <v>228.54</v>
       </c>
       <c r="F42" s="10">
-        <v>233.75</v>
+        <v>238.54</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>271.62</v>
+        <v>282</v>
       </c>
       <c r="E43" s="13">
-        <v>224.17</v>
+        <v>228.96</v>
       </c>
       <c r="F43" s="13">
-        <v>234.17</v>
+        <v>238.96</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="14"/>
       <c r="B44" s="24"/>
       <c r="C44" s="15"/>
@@ -1455,7 +1455,7 @@
       <c r="F44" s="16"/>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="25" t="s">
         <v>27</v>
       </c>
@@ -1466,7 +1466,7 @@
       <c r="F45" s="17"/>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="23" t="s">
         <v>4</v>
       </c>
@@ -1485,83 +1485,83 @@
       </c>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>273.08</v>
+        <v>286.41000000000003</v>
       </c>
       <c r="E47" s="10">
-        <v>231.49</v>
+        <v>237.98</v>
       </c>
       <c r="F47" s="10">
-        <v>241.49</v>
+        <v>247.98</v>
       </c>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>272.83999999999997</v>
+        <v>286.19</v>
       </c>
       <c r="E48" s="13">
-        <v>231.54</v>
+        <v>238.04</v>
       </c>
       <c r="F48" s="13">
-        <v>241.54</v>
+        <v>248.04</v>
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>268.37</v>
+        <v>273.08</v>
       </c>
       <c r="E49" s="10">
-        <v>231.07</v>
+        <v>231.49</v>
       </c>
       <c r="F49" s="10">
-        <v>241.07</v>
+        <v>241.49</v>
       </c>
       <c r="G49" s="17"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>268.13</v>
+        <v>272.83999999999997</v>
       </c>
       <c r="E50" s="13">
-        <v>231.13</v>
+        <v>231.54</v>
       </c>
       <c r="F50" s="13">
-        <v>241.13</v>
+        <v>241.54</v>
       </c>
       <c r="G50" s="17"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="14"/>
       <c r="B51" s="14"/>
       <c r="C51" s="15"/>
@@ -1570,7 +1570,7 @@
       <c r="F51" s="16"/>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A52" s="27" t="s">
         <v>30</v>
       </c>
@@ -1581,7 +1581,7 @@
       <c r="F52" s="17"/>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="23" t="s">
         <v>4</v>
       </c>
@@ -1600,54 +1600,54 @@
       </c>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>292.58</v>
+        <v>299.04000000000002</v>
       </c>
       <c r="E54" s="10">
-        <v>242.78</v>
+        <v>247.59</v>
       </c>
       <c r="F54" s="10">
-        <v>252.78</v>
+        <v>257.58999999999997</v>
       </c>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>285.14</v>
+        <v>291.58999999999997</v>
       </c>
       <c r="E55" s="13">
-        <v>242.95</v>
+        <v>247.65</v>
       </c>
       <c r="F55" s="13">
-        <v>252.95</v>
+        <v>257.64999999999998</v>
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>285.02999999999997</v>
+        <v>291.47000000000003</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1657,111 +1657,111 @@
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>285.27999999999997</v>
+        <v>291.67</v>
       </c>
       <c r="E57" s="13">
-        <v>237.33</v>
+        <v>242.02</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>281.11</v>
+        <v>287.51</v>
       </c>
       <c r="E58" s="10">
-        <v>233.27</v>
+        <v>237.97</v>
       </c>
       <c r="F58" s="10">
-        <v>243.27</v>
+        <v>247.97</v>
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>284.89999999999998</v>
+        <v>291.3</v>
       </c>
       <c r="E59" s="13">
-        <v>240.92</v>
+        <v>245.71</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>282.17</v>
+        <v>292.58</v>
       </c>
       <c r="E60" s="10">
-        <v>237.79</v>
+        <v>242.78</v>
       </c>
       <c r="F60" s="10">
-        <v>247.79</v>
+        <v>252.78</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>274.75</v>
+        <v>285.14</v>
       </c>
       <c r="E61" s="13">
-        <v>237.97</v>
+        <v>242.95</v>
       </c>
       <c r="F61" s="13">
-        <v>247.97</v>
+        <v>252.95</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>274.64999999999998</v>
+        <v>285.02999999999997</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1771,57 +1771,57 @@
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>274.91000000000003</v>
+        <v>285.27999999999997</v>
       </c>
       <c r="E63" s="13">
-        <v>232.35</v>
+        <v>237.33</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>270.74</v>
+        <v>281.11</v>
       </c>
       <c r="E64" s="10">
-        <v>228.29</v>
+        <v>233.27</v>
       </c>
       <c r="F64" s="10">
-        <v>238.29</v>
+        <v>243.27</v>
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>274.52</v>
+        <v>284.89999999999998</v>
       </c>
       <c r="E65" s="13">
-        <v>235.92</v>
+        <v>240.92</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -2110,6 +2110,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -2118,15 +2127,6 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2150,6 +2150,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -2167,14 +2175,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Mon Mar 23 04:01:12 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{8B9EEE63-8B11-444D-BFC4-D54AF79E7C48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{16F99B7B-74EC-401F-89D9-1044ADB80638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>289.3</v>
+        <v>293.08999999999997</v>
       </c>
       <c r="E8" s="10">
-        <v>236.27</v>
+        <v>236.87</v>
       </c>
       <c r="F8" s="10">
-        <v>246.27</v>
+        <v>246.87</v>
       </c>
       <c r="G8" s="10">
-        <v>236.15</v>
+        <v>236.75</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>289.3</v>
+        <v>293.08999999999997</v>
       </c>
       <c r="E9" s="13">
-        <v>236.27</v>
+        <v>236.87</v>
       </c>
       <c r="F9" s="13">
-        <v>246.27</v>
+        <v>246.87</v>
       </c>
       <c r="G9" s="13">
-        <v>236.15</v>
+        <v>236.75</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>292.93</v>
+        <v>293.52</v>
       </c>
       <c r="E10" s="10">
-        <v>238.44</v>
+        <v>241.32</v>
       </c>
       <c r="F10" s="10">
-        <v>248.44</v>
+        <v>251.32</v>
       </c>
       <c r="G10" s="10">
-        <v>238.68</v>
+        <v>241.56</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>279.64</v>
+        <v>289.3</v>
       </c>
       <c r="E11" s="13">
-        <v>230.51</v>
+        <v>236.27</v>
       </c>
       <c r="F11" s="13">
-        <v>240.51</v>
+        <v>246.27</v>
       </c>
       <c r="G11" s="13">
-        <v>230.39</v>
+        <v>236.15</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>279.64</v>
+        <v>289.3</v>
       </c>
       <c r="E12" s="10">
-        <v>230.51</v>
+        <v>236.27</v>
       </c>
       <c r="F12" s="10">
-        <v>240.51</v>
+        <v>246.27</v>
       </c>
       <c r="G12" s="10">
-        <v>230.39</v>
+        <v>236.15</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>283.2</v>
+        <v>292.93</v>
       </c>
       <c r="E13" s="13">
-        <v>232.6</v>
+        <v>238.44</v>
       </c>
       <c r="F13" s="13">
-        <v>242.6</v>
+        <v>248.44</v>
       </c>
       <c r="G13" s="13">
-        <v>232.84</v>
+        <v>238.68</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>286.8</v>
+        <v>292.8</v>
       </c>
       <c r="E17" s="10">
-        <v>237.22</v>
+        <v>240.04</v>
       </c>
       <c r="F17" s="10">
-        <v>247.22</v>
+        <v>250.04</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>280.38</v>
+        <v>286.8</v>
       </c>
       <c r="E18" s="13">
-        <v>232.49</v>
+        <v>237.22</v>
       </c>
       <c r="F18" s="13">
-        <v>242.49</v>
+        <v>247.22</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>288.95999999999998</v>
+        <v>292.75</v>
       </c>
       <c r="E22" s="10">
-        <v>238.91</v>
+        <v>240.06</v>
       </c>
       <c r="F22" s="10">
-        <v>248.51</v>
+        <v>249.66</v>
       </c>
       <c r="G22" s="10">
-        <v>240.66</v>
+        <v>241.81</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>291.31</v>
+        <v>295.20999999999998</v>
       </c>
       <c r="E23" s="13">
-        <v>242.99</v>
+        <v>245.88</v>
       </c>
       <c r="F23" s="13">
-        <v>252.99</v>
+        <v>255.88</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>291.44</v>
+        <v>295.33</v>
       </c>
       <c r="E24" s="10">
-        <v>243.48</v>
+        <v>246.4</v>
       </c>
       <c r="F24" s="10">
-        <v>253.48</v>
+        <v>256.39999999999998</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>291.41000000000003</v>
+        <v>295.3</v>
       </c>
       <c r="E25" s="13">
-        <v>243.18</v>
+        <v>246.11</v>
       </c>
       <c r="F25" s="13">
-        <v>253.18</v>
+        <v>256.11</v>
       </c>
       <c r="G25" s="13">
-        <v>244.03</v>
+        <v>246.96</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>291.04000000000002</v>
+        <v>294.91000000000003</v>
       </c>
       <c r="E26" s="10">
-        <v>245.36</v>
+        <v>248.31</v>
       </c>
       <c r="F26" s="10">
-        <v>255.36</v>
+        <v>258.31</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>279.31</v>
+        <v>288.95999999999998</v>
       </c>
       <c r="E27" s="13">
-        <v>232.6</v>
+        <v>238.91</v>
       </c>
       <c r="F27" s="13">
-        <v>242.2</v>
+        <v>248.51</v>
       </c>
       <c r="G27" s="13">
-        <v>234.35</v>
+        <v>240.66</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>284.87</v>
+        <v>291.31</v>
       </c>
       <c r="E28" s="22">
-        <v>238.24</v>
+        <v>242.99</v>
       </c>
       <c r="F28" s="22">
-        <v>248.24</v>
+        <v>252.99</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>285</v>
+        <v>291.44</v>
       </c>
       <c r="E29" s="13">
-        <v>238.74</v>
+        <v>243.48</v>
       </c>
       <c r="F29" s="13">
-        <v>248.74</v>
+        <v>253.48</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>284.98</v>
+        <v>291.41000000000003</v>
       </c>
       <c r="E30" s="22">
-        <v>238.42</v>
+        <v>243.18</v>
       </c>
       <c r="F30" s="22">
-        <v>248.42</v>
+        <v>253.18</v>
       </c>
       <c r="G30" s="22">
-        <v>239.27</v>
+        <v>244.03</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>284.60000000000002</v>
+        <v>291.04000000000002</v>
       </c>
       <c r="E31" s="13">
-        <v>240.56</v>
+        <v>245.36</v>
       </c>
       <c r="F31" s="13">
-        <v>250.56</v>
+        <v>255.36</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>285.23</v>
+        <v>289.12</v>
       </c>
       <c r="E35" s="10">
-        <v>236.77</v>
+        <v>239.66</v>
       </c>
       <c r="F35" s="10">
-        <v>245.77</v>
+        <v>248.66</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>278.8</v>
+        <v>285.23</v>
       </c>
       <c r="E36" s="13">
-        <v>232.05</v>
+        <v>236.77</v>
       </c>
       <c r="F36" s="13">
-        <v>241.05</v>
+        <v>245.77</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>288.85000000000002</v>
+        <v>295.01</v>
       </c>
       <c r="E40" s="10">
-        <v>233.27</v>
+        <v>236.23</v>
       </c>
       <c r="F40" s="10">
-        <v>243.27</v>
+        <v>246.23</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>288.45</v>
+        <v>294.60000000000002</v>
       </c>
       <c r="E41" s="13">
-        <v>233.68</v>
+        <v>236.65</v>
       </c>
       <c r="F41" s="13">
-        <v>243.68</v>
+        <v>246.65</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>282.39999999999998</v>
+        <v>288.85000000000002</v>
       </c>
       <c r="E42" s="10">
-        <v>228.54</v>
+        <v>233.27</v>
       </c>
       <c r="F42" s="10">
-        <v>238.54</v>
+        <v>243.27</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>282</v>
+        <v>288.45</v>
       </c>
       <c r="E43" s="13">
-        <v>228.96</v>
+        <v>233.68</v>
       </c>
       <c r="F43" s="13">
-        <v>238.96</v>
+        <v>243.68</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>286.41000000000003</v>
+        <v>292.94</v>
       </c>
       <c r="E47" s="10">
-        <v>237.98</v>
+        <v>240.34</v>
       </c>
       <c r="F47" s="10">
-        <v>247.98</v>
+        <v>250.34</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>286.19</v>
+        <v>292.7</v>
       </c>
       <c r="E48" s="13">
-        <v>238.04</v>
+        <v>240.39</v>
       </c>
       <c r="F48" s="13">
-        <v>248.04</v>
+        <v>250.39</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>273.08</v>
+        <v>286.41000000000003</v>
       </c>
       <c r="E49" s="10">
-        <v>231.49</v>
+        <v>237.98</v>
       </c>
       <c r="F49" s="10">
-        <v>241.49</v>
+        <v>247.98</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>272.83999999999997</v>
+        <v>286.19</v>
       </c>
       <c r="E50" s="13">
-        <v>231.54</v>
+        <v>238.04</v>
       </c>
       <c r="F50" s="13">
-        <v>241.54</v>
+        <v>248.04</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>299.04000000000002</v>
+        <v>302.91000000000003</v>
       </c>
       <c r="E54" s="10">
-        <v>247.59</v>
+        <v>250.83</v>
       </c>
       <c r="F54" s="10">
-        <v>257.58999999999997</v>
+        <v>260.83</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>291.58999999999997</v>
+        <v>295.49</v>
       </c>
       <c r="E55" s="13">
-        <v>247.65</v>
+        <v>250.43</v>
       </c>
       <c r="F55" s="13">
-        <v>257.64999999999998</v>
+        <v>260.43</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>291.47000000000003</v>
+        <v>295.38</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>291.67</v>
+        <v>295.44</v>
       </c>
       <c r="E57" s="13">
-        <v>242.02</v>
+        <v>244.8</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>287.51</v>
+        <v>291.29000000000002</v>
       </c>
       <c r="E58" s="10">
-        <v>237.97</v>
+        <v>240.75</v>
       </c>
       <c r="F58" s="10">
-        <v>247.97</v>
+        <v>250.75</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>291.3</v>
+        <v>295.08999999999997</v>
       </c>
       <c r="E59" s="13">
-        <v>245.71</v>
+        <v>248.8</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>292.58</v>
+        <v>299.04000000000002</v>
       </c>
       <c r="E60" s="10">
-        <v>242.78</v>
+        <v>247.59</v>
       </c>
       <c r="F60" s="10">
-        <v>252.78</v>
+        <v>257.58999999999997</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>285.14</v>
+        <v>291.58999999999997</v>
       </c>
       <c r="E61" s="13">
-        <v>242.95</v>
+        <v>247.65</v>
       </c>
       <c r="F61" s="13">
-        <v>252.95</v>
+        <v>257.64999999999998</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>285.02999999999997</v>
+        <v>291.47000000000003</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>285.27999999999997</v>
+        <v>291.67</v>
       </c>
       <c r="E63" s="13">
-        <v>237.33</v>
+        <v>242.02</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>281.11</v>
+        <v>287.51</v>
       </c>
       <c r="E64" s="10">
-        <v>233.27</v>
+        <v>237.97</v>
       </c>
       <c r="F64" s="10">
-        <v>243.27</v>
+        <v>247.97</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46101</v>
+        <v>46102</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>284.89999999999998</v>
+        <v>291.3</v>
       </c>
       <c r="E65" s="13">
-        <v>240.92</v>
+        <v>245.71</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,6 +1850,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2109,27 +2129,33 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2149,32 +2175,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Tue Mar 24 03:43:45 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{16F99B7B-74EC-401F-89D9-1044ADB80638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{6E8DBC87-0E7F-485F-ACAC-9CA1E74B784A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>293.08999999999997</v>
+        <v>299.25</v>
       </c>
       <c r="E8" s="10">
-        <v>236.87</v>
+        <v>240.5</v>
       </c>
       <c r="F8" s="10">
-        <v>246.87</v>
+        <v>250.5</v>
       </c>
       <c r="G8" s="10">
-        <v>236.75</v>
+        <v>240.39</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>293.08999999999997</v>
+        <v>299.25</v>
       </c>
       <c r="E9" s="13">
-        <v>236.87</v>
+        <v>240.5</v>
       </c>
       <c r="F9" s="13">
-        <v>246.87</v>
+        <v>250.5</v>
       </c>
       <c r="G9" s="13">
-        <v>236.75</v>
+        <v>240.39</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>293.52</v>
+        <v>300.89999999999998</v>
       </c>
       <c r="E10" s="10">
-        <v>241.32</v>
+        <v>242.87</v>
       </c>
       <c r="F10" s="10">
-        <v>251.32</v>
+        <v>252.87</v>
       </c>
       <c r="G10" s="10">
-        <v>241.56</v>
+        <v>243.11</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>289.3</v>
+        <v>293.08999999999997</v>
       </c>
       <c r="E11" s="13">
-        <v>236.27</v>
+        <v>236.87</v>
       </c>
       <c r="F11" s="13">
-        <v>246.27</v>
+        <v>246.87</v>
       </c>
       <c r="G11" s="13">
-        <v>236.15</v>
+        <v>236.75</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>289.3</v>
+        <v>293.08999999999997</v>
       </c>
       <c r="E12" s="10">
-        <v>236.27</v>
+        <v>236.87</v>
       </c>
       <c r="F12" s="10">
-        <v>246.27</v>
+        <v>246.87</v>
       </c>
       <c r="G12" s="10">
-        <v>236.15</v>
+        <v>236.75</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>292.93</v>
+        <v>293.52</v>
       </c>
       <c r="E13" s="13">
-        <v>238.44</v>
+        <v>241.32</v>
       </c>
       <c r="F13" s="13">
-        <v>248.44</v>
+        <v>251.32</v>
       </c>
       <c r="G13" s="13">
-        <v>238.68</v>
+        <v>241.56</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>292.8</v>
+        <v>301.27999999999997</v>
       </c>
       <c r="E17" s="10">
-        <v>240.04</v>
+        <v>243.7</v>
       </c>
       <c r="F17" s="10">
-        <v>250.04</v>
+        <v>253.7</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>286.8</v>
+        <v>292.8</v>
       </c>
       <c r="E18" s="13">
-        <v>237.22</v>
+        <v>240.04</v>
       </c>
       <c r="F18" s="13">
-        <v>247.22</v>
+        <v>250.04</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>292.75</v>
+        <v>300</v>
       </c>
       <c r="E22" s="10">
-        <v>240.06</v>
+        <v>243.69</v>
       </c>
       <c r="F22" s="10">
-        <v>249.66</v>
+        <v>253.29</v>
       </c>
       <c r="G22" s="10">
-        <v>241.81</v>
+        <v>245.44</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>295.20999999999998</v>
+        <v>302.60000000000002</v>
       </c>
       <c r="E23" s="13">
-        <v>245.88</v>
+        <v>249.62</v>
       </c>
       <c r="F23" s="13">
-        <v>255.88</v>
+        <v>259.62</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>295.33</v>
+        <v>302.70999999999998</v>
       </c>
       <c r="E24" s="10">
-        <v>246.4</v>
+        <v>250.19</v>
       </c>
       <c r="F24" s="10">
-        <v>256.39999999999998</v>
+        <v>260.19</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>295.3</v>
+        <v>302.68</v>
       </c>
       <c r="E25" s="13">
-        <v>246.11</v>
+        <v>249.91</v>
       </c>
       <c r="F25" s="13">
-        <v>256.11</v>
+        <v>259.91000000000003</v>
       </c>
       <c r="G25" s="13">
-        <v>246.96</v>
+        <v>250.76</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>294.91000000000003</v>
+        <v>302.26</v>
       </c>
       <c r="E26" s="10">
-        <v>248.31</v>
+        <v>250.49</v>
       </c>
       <c r="F26" s="10">
-        <v>258.31</v>
+        <v>260.49</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>288.95999999999998</v>
+        <v>292.75</v>
       </c>
       <c r="E27" s="13">
-        <v>238.91</v>
+        <v>240.06</v>
       </c>
       <c r="F27" s="13">
-        <v>248.51</v>
+        <v>249.66</v>
       </c>
       <c r="G27" s="13">
-        <v>240.66</v>
+        <v>241.81</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>291.31</v>
+        <v>295.20999999999998</v>
       </c>
       <c r="E28" s="22">
-        <v>242.99</v>
+        <v>245.88</v>
       </c>
       <c r="F28" s="22">
-        <v>252.99</v>
+        <v>255.88</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>291.44</v>
+        <v>295.33</v>
       </c>
       <c r="E29" s="13">
-        <v>243.48</v>
+        <v>246.4</v>
       </c>
       <c r="F29" s="13">
-        <v>253.48</v>
+        <v>256.39999999999998</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>291.41000000000003</v>
+        <v>295.3</v>
       </c>
       <c r="E30" s="22">
-        <v>243.18</v>
+        <v>246.11</v>
       </c>
       <c r="F30" s="22">
-        <v>253.18</v>
+        <v>256.11</v>
       </c>
       <c r="G30" s="22">
-        <v>244.03</v>
+        <v>246.96</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>291.04000000000002</v>
+        <v>294.91000000000003</v>
       </c>
       <c r="E31" s="13">
-        <v>245.36</v>
+        <v>248.31</v>
       </c>
       <c r="F31" s="13">
-        <v>255.36</v>
+        <v>258.31</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>289.12</v>
+        <v>296.49</v>
       </c>
       <c r="E35" s="10">
-        <v>239.66</v>
+        <v>243.4</v>
       </c>
       <c r="F35" s="10">
-        <v>248.66</v>
+        <v>252.4</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>285.23</v>
+        <v>289.12</v>
       </c>
       <c r="E36" s="13">
-        <v>236.77</v>
+        <v>239.66</v>
       </c>
       <c r="F36" s="13">
-        <v>245.77</v>
+        <v>248.66</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>295.01</v>
+        <v>302.48</v>
       </c>
       <c r="E40" s="10">
-        <v>236.23</v>
+        <v>240.06</v>
       </c>
       <c r="F40" s="10">
-        <v>246.23</v>
+        <v>250.06</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>294.60000000000002</v>
+        <v>302.06</v>
       </c>
       <c r="E41" s="13">
-        <v>236.65</v>
+        <v>240.48</v>
       </c>
       <c r="F41" s="13">
-        <v>246.65</v>
+        <v>250.48</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>288.85000000000002</v>
+        <v>295.01</v>
       </c>
       <c r="E42" s="10">
-        <v>233.27</v>
+        <v>236.23</v>
       </c>
       <c r="F42" s="10">
-        <v>243.27</v>
+        <v>246.23</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>288.45</v>
+        <v>294.60000000000002</v>
       </c>
       <c r="E43" s="13">
-        <v>233.68</v>
+        <v>236.65</v>
       </c>
       <c r="F43" s="13">
-        <v>243.68</v>
+        <v>246.65</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>292.94</v>
+        <v>297.24</v>
       </c>
       <c r="E47" s="10">
-        <v>240.34</v>
+        <v>244.8</v>
       </c>
       <c r="F47" s="10">
-        <v>250.34</v>
+        <v>254.8</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>292.7</v>
+        <v>296.99</v>
       </c>
       <c r="E48" s="13">
-        <v>240.39</v>
+        <v>244.85</v>
       </c>
       <c r="F48" s="13">
-        <v>250.39</v>
+        <v>254.85</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>286.41000000000003</v>
+        <v>292.94</v>
       </c>
       <c r="E49" s="10">
-        <v>237.98</v>
+        <v>240.34</v>
       </c>
       <c r="F49" s="10">
-        <v>247.98</v>
+        <v>250.34</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>286.19</v>
+        <v>292.7</v>
       </c>
       <c r="E50" s="13">
-        <v>238.04</v>
+        <v>240.39</v>
       </c>
       <c r="F50" s="13">
-        <v>248.04</v>
+        <v>250.39</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>302.91000000000003</v>
+        <v>311.49</v>
       </c>
       <c r="E54" s="10">
-        <v>250.83</v>
+        <v>255.03</v>
       </c>
       <c r="F54" s="10">
-        <v>260.83</v>
+        <v>265.02999999999997</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>295.49</v>
+        <v>304.08999999999997</v>
       </c>
       <c r="E55" s="13">
-        <v>250.43</v>
+        <v>254.05</v>
       </c>
       <c r="F55" s="13">
-        <v>260.43</v>
+        <v>264.05</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>295.38</v>
+        <v>303.98</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>295.44</v>
+        <v>303.87</v>
       </c>
       <c r="E57" s="13">
-        <v>244.8</v>
+        <v>248.42</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>291.29000000000002</v>
+        <v>299.72000000000003</v>
       </c>
       <c r="E58" s="10">
-        <v>240.75</v>
+        <v>244.37</v>
       </c>
       <c r="F58" s="10">
-        <v>250.75</v>
+        <v>254.37</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>295.08999999999997</v>
+        <v>303.54000000000002</v>
       </c>
       <c r="E59" s="13">
-        <v>248.8</v>
+        <v>252.8</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>299.04000000000002</v>
+        <v>302.91000000000003</v>
       </c>
       <c r="E60" s="10">
-        <v>247.59</v>
+        <v>250.83</v>
       </c>
       <c r="F60" s="10">
-        <v>257.58999999999997</v>
+        <v>260.83</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>291.58999999999997</v>
+        <v>295.49</v>
       </c>
       <c r="E61" s="13">
-        <v>247.65</v>
+        <v>250.43</v>
       </c>
       <c r="F61" s="13">
-        <v>257.64999999999998</v>
+        <v>260.43</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>291.47000000000003</v>
+        <v>295.38</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>291.67</v>
+        <v>295.44</v>
       </c>
       <c r="E63" s="13">
-        <v>242.02</v>
+        <v>244.8</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>287.51</v>
+        <v>291.29000000000002</v>
       </c>
       <c r="E64" s="10">
-        <v>237.97</v>
+        <v>240.75</v>
       </c>
       <c r="F64" s="10">
-        <v>247.97</v>
+        <v>250.75</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46102</v>
+        <v>46105</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>291.3</v>
+        <v>295.08999999999997</v>
       </c>
       <c r="E65" s="13">
-        <v>245.71</v>
+        <v>248.8</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,6 +1850,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -1858,15 +1867,6 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2130,6 +2130,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -2143,14 +2151,6 @@
     <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
     <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Wed Mar 25 03:54:17 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{6E8DBC87-0E7F-485F-ACAC-9CA1E74B784A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{F21BA19B-ACC8-4ABD-978C-F8695E10E534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>299.25</v>
+        <v>298.77</v>
       </c>
       <c r="E8" s="10">
-        <v>240.5</v>
+        <v>239.93</v>
       </c>
       <c r="F8" s="10">
-        <v>250.5</v>
+        <v>249.93</v>
       </c>
       <c r="G8" s="10">
-        <v>240.39</v>
+        <v>239.82</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>299.25</v>
+        <v>298.77</v>
       </c>
       <c r="E9" s="13">
-        <v>240.5</v>
+        <v>239.93</v>
       </c>
       <c r="F9" s="13">
-        <v>250.5</v>
+        <v>249.93</v>
       </c>
       <c r="G9" s="13">
-        <v>240.39</v>
+        <v>239.82</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>300.89999999999998</v>
+        <v>299.56</v>
       </c>
       <c r="E10" s="10">
-        <v>242.87</v>
+        <v>242.5</v>
       </c>
       <c r="F10" s="10">
-        <v>252.87</v>
+        <v>252.5</v>
       </c>
       <c r="G10" s="10">
-        <v>243.11</v>
+        <v>242.74</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>293.08999999999997</v>
+        <v>299.25</v>
       </c>
       <c r="E11" s="13">
-        <v>236.87</v>
+        <v>240.5</v>
       </c>
       <c r="F11" s="13">
-        <v>246.87</v>
+        <v>250.5</v>
       </c>
       <c r="G11" s="13">
-        <v>236.75</v>
+        <v>240.39</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>293.08999999999997</v>
+        <v>299.25</v>
       </c>
       <c r="E12" s="10">
-        <v>236.87</v>
+        <v>240.5</v>
       </c>
       <c r="F12" s="10">
-        <v>246.87</v>
+        <v>250.5</v>
       </c>
       <c r="G12" s="10">
-        <v>236.75</v>
+        <v>240.39</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>293.52</v>
+        <v>300.89999999999998</v>
       </c>
       <c r="E13" s="13">
-        <v>241.32</v>
+        <v>242.87</v>
       </c>
       <c r="F13" s="13">
-        <v>251.32</v>
+        <v>252.87</v>
       </c>
       <c r="G13" s="13">
-        <v>241.56</v>
+        <v>243.11</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>301.27999999999997</v>
+        <v>300.92</v>
       </c>
       <c r="E17" s="10">
-        <v>243.7</v>
+        <v>243.22</v>
       </c>
       <c r="F17" s="10">
-        <v>253.7</v>
+        <v>253.22</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>292.8</v>
+        <v>301.27999999999997</v>
       </c>
       <c r="E18" s="13">
-        <v>240.04</v>
+        <v>243.7</v>
       </c>
       <c r="F18" s="13">
-        <v>250.04</v>
+        <v>253.7</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>300</v>
+        <v>298.75</v>
       </c>
       <c r="E22" s="10">
-        <v>243.69</v>
+        <v>240.92</v>
       </c>
       <c r="F22" s="10">
-        <v>253.29</v>
+        <v>250.52</v>
       </c>
       <c r="G22" s="10">
-        <v>245.44</v>
+        <v>242.67</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>302.60000000000002</v>
+        <v>300.18</v>
       </c>
       <c r="E23" s="13">
-        <v>249.62</v>
+        <v>249.24</v>
       </c>
       <c r="F23" s="13">
-        <v>259.62</v>
+        <v>259.24</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>302.70999999999998</v>
+        <v>300.27</v>
       </c>
       <c r="E24" s="10">
-        <v>250.19</v>
+        <v>249.86</v>
       </c>
       <c r="F24" s="10">
-        <v>260.19</v>
+        <v>259.86</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>302.68</v>
+        <v>300.24</v>
       </c>
       <c r="E25" s="13">
-        <v>249.91</v>
+        <v>249.59</v>
       </c>
       <c r="F25" s="13">
-        <v>259.91000000000003</v>
+        <v>259.58999999999997</v>
       </c>
       <c r="G25" s="13">
-        <v>250.76</v>
+        <v>250.44</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>302.26</v>
+        <v>299.8</v>
       </c>
       <c r="E26" s="10">
-        <v>250.49</v>
+        <v>250.17</v>
       </c>
       <c r="F26" s="10">
-        <v>260.49</v>
+        <v>260.17</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>292.75</v>
+        <v>300</v>
       </c>
       <c r="E27" s="13">
-        <v>240.06</v>
+        <v>243.69</v>
       </c>
       <c r="F27" s="13">
-        <v>249.66</v>
+        <v>253.29</v>
       </c>
       <c r="G27" s="13">
-        <v>241.81</v>
+        <v>245.44</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>295.20999999999998</v>
+        <v>302.60000000000002</v>
       </c>
       <c r="E28" s="22">
-        <v>245.88</v>
+        <v>249.62</v>
       </c>
       <c r="F28" s="22">
-        <v>255.88</v>
+        <v>259.62</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>295.33</v>
+        <v>302.70999999999998</v>
       </c>
       <c r="E29" s="13">
-        <v>246.4</v>
+        <v>250.19</v>
       </c>
       <c r="F29" s="13">
-        <v>256.39999999999998</v>
+        <v>260.19</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>295.3</v>
+        <v>302.68</v>
       </c>
       <c r="E30" s="22">
-        <v>246.11</v>
+        <v>249.91</v>
       </c>
       <c r="F30" s="22">
-        <v>256.11</v>
+        <v>259.91000000000003</v>
       </c>
       <c r="G30" s="22">
-        <v>246.96</v>
+        <v>250.76</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>294.91000000000003</v>
+        <v>302.26</v>
       </c>
       <c r="E31" s="13">
-        <v>248.31</v>
+        <v>250.49</v>
       </c>
       <c r="F31" s="13">
-        <v>258.31</v>
+        <v>260.49</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>296.49</v>
+        <v>296.25</v>
       </c>
       <c r="E35" s="10">
-        <v>243.4</v>
+        <v>243.03</v>
       </c>
       <c r="F35" s="10">
-        <v>252.4</v>
+        <v>252.03</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>289.12</v>
+        <v>296.49</v>
       </c>
       <c r="E36" s="13">
-        <v>239.66</v>
+        <v>243.4</v>
       </c>
       <c r="F36" s="13">
-        <v>248.66</v>
+        <v>252.4</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>302.48</v>
+        <v>302.33</v>
       </c>
       <c r="E40" s="10">
-        <v>240.06</v>
+        <v>241.49</v>
       </c>
       <c r="F40" s="10">
-        <v>250.06</v>
+        <v>251.49</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>302.06</v>
+        <v>301.89999999999998</v>
       </c>
       <c r="E41" s="13">
-        <v>240.48</v>
+        <v>241.9</v>
       </c>
       <c r="F41" s="13">
-        <v>250.48</v>
+        <v>251.9</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>295.01</v>
+        <v>302.48</v>
       </c>
       <c r="E42" s="10">
-        <v>236.23</v>
+        <v>240.06</v>
       </c>
       <c r="F42" s="10">
-        <v>246.23</v>
+        <v>250.06</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>294.60000000000002</v>
+        <v>302.06</v>
       </c>
       <c r="E43" s="13">
-        <v>236.65</v>
+        <v>240.48</v>
       </c>
       <c r="F43" s="13">
-        <v>246.65</v>
+        <v>250.48</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>297.24</v>
+        <v>297.32</v>
       </c>
       <c r="E47" s="10">
-        <v>244.8</v>
+        <v>241.53</v>
       </c>
       <c r="F47" s="10">
-        <v>254.8</v>
+        <v>251.53</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>296.99</v>
+        <v>297.06</v>
       </c>
       <c r="E48" s="13">
-        <v>244.85</v>
+        <v>241.57</v>
       </c>
       <c r="F48" s="13">
-        <v>254.85</v>
+        <v>251.57</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>292.94</v>
+        <v>297.24</v>
       </c>
       <c r="E49" s="10">
-        <v>240.34</v>
+        <v>244.8</v>
       </c>
       <c r="F49" s="10">
-        <v>250.34</v>
+        <v>254.8</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>292.7</v>
+        <v>296.99</v>
       </c>
       <c r="E50" s="13">
-        <v>240.39</v>
+        <v>244.85</v>
       </c>
       <c r="F50" s="13">
-        <v>250.39</v>
+        <v>254.85</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>311.49</v>
+        <v>311.24</v>
       </c>
       <c r="E54" s="10">
-        <v>255.03</v>
+        <v>255.11</v>
       </c>
       <c r="F54" s="10">
-        <v>265.02999999999997</v>
+        <v>265.11</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>304.08999999999997</v>
+        <v>303.86</v>
       </c>
       <c r="E55" s="13">
-        <v>254.05</v>
+        <v>253.57</v>
       </c>
       <c r="F55" s="13">
-        <v>264.05</v>
+        <v>263.57</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>303.98</v>
+        <v>303.76</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>303.87</v>
+        <v>303.48</v>
       </c>
       <c r="E57" s="13">
-        <v>248.42</v>
+        <v>247.94</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>299.72000000000003</v>
+        <v>299.33</v>
       </c>
       <c r="E58" s="10">
-        <v>244.37</v>
+        <v>243.89</v>
       </c>
       <c r="F58" s="10">
-        <v>254.37</v>
+        <v>253.89</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>303.54000000000002</v>
+        <v>303.16000000000003</v>
       </c>
       <c r="E59" s="13">
-        <v>252.8</v>
+        <v>252.69</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>302.91000000000003</v>
+        <v>311.49</v>
       </c>
       <c r="E60" s="10">
-        <v>250.83</v>
+        <v>255.03</v>
       </c>
       <c r="F60" s="10">
-        <v>260.83</v>
+        <v>265.02999999999997</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>295.49</v>
+        <v>304.08999999999997</v>
       </c>
       <c r="E61" s="13">
-        <v>250.43</v>
+        <v>254.05</v>
       </c>
       <c r="F61" s="13">
-        <v>260.43</v>
+        <v>264.05</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>295.38</v>
+        <v>303.98</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>295.44</v>
+        <v>303.87</v>
       </c>
       <c r="E63" s="13">
-        <v>244.8</v>
+        <v>248.42</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>291.29000000000002</v>
+        <v>299.72000000000003</v>
       </c>
       <c r="E64" s="10">
-        <v>240.75</v>
+        <v>244.37</v>
       </c>
       <c r="F64" s="10">
-        <v>250.75</v>
+        <v>254.37</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46105</v>
+        <v>46106</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>295.08999999999997</v>
+        <v>303.54000000000002</v>
       </c>
       <c r="E65" s="13">
-        <v>248.8</v>
+        <v>252.8</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,26 +1850,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2129,33 +2109,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2175,6 +2149,32 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Thu Mar 26 04:06:30 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{F21BA19B-ACC8-4ABD-978C-F8695E10E534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{00E50267-B6CF-4CFA-8AF1-DDD27036EB07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>298.77</v>
+        <v>298.98</v>
       </c>
       <c r="E8" s="10">
-        <v>239.93</v>
+        <v>237.28</v>
       </c>
       <c r="F8" s="10">
-        <v>249.93</v>
+        <v>247.28</v>
       </c>
       <c r="G8" s="10">
-        <v>239.82</v>
+        <v>237.16</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>298.77</v>
+        <v>298.98</v>
       </c>
       <c r="E9" s="13">
-        <v>239.93</v>
+        <v>237.28</v>
       </c>
       <c r="F9" s="13">
-        <v>249.93</v>
+        <v>247.28</v>
       </c>
       <c r="G9" s="13">
-        <v>239.82</v>
+        <v>237.16</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>299.56</v>
+        <v>299.83999999999997</v>
       </c>
       <c r="E10" s="10">
-        <v>242.5</v>
+        <v>239.91</v>
       </c>
       <c r="F10" s="10">
-        <v>252.5</v>
+        <v>249.91</v>
       </c>
       <c r="G10" s="10">
-        <v>242.74</v>
+        <v>240.15</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>299.25</v>
+        <v>298.77</v>
       </c>
       <c r="E11" s="13">
-        <v>240.5</v>
+        <v>239.93</v>
       </c>
       <c r="F11" s="13">
-        <v>250.5</v>
+        <v>249.93</v>
       </c>
       <c r="G11" s="13">
-        <v>240.39</v>
+        <v>239.82</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>299.25</v>
+        <v>298.77</v>
       </c>
       <c r="E12" s="10">
-        <v>240.5</v>
+        <v>239.93</v>
       </c>
       <c r="F12" s="10">
-        <v>250.5</v>
+        <v>249.93</v>
       </c>
       <c r="G12" s="10">
-        <v>240.39</v>
+        <v>239.82</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>300.89999999999998</v>
+        <v>299.56</v>
       </c>
       <c r="E13" s="13">
-        <v>242.87</v>
+        <v>242.5</v>
       </c>
       <c r="F13" s="13">
-        <v>252.87</v>
+        <v>252.5</v>
       </c>
       <c r="G13" s="13">
-        <v>243.11</v>
+        <v>242.74</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>300.92</v>
+        <v>301.11</v>
       </c>
       <c r="E17" s="10">
-        <v>243.22</v>
+        <v>240.54</v>
       </c>
       <c r="F17" s="10">
-        <v>253.22</v>
+        <v>250.54</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>301.27999999999997</v>
+        <v>300.92</v>
       </c>
       <c r="E18" s="13">
-        <v>243.7</v>
+        <v>243.22</v>
       </c>
       <c r="F18" s="13">
-        <v>253.7</v>
+        <v>253.22</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>298.75</v>
+        <v>298.95</v>
       </c>
       <c r="E22" s="10">
-        <v>240.92</v>
+        <v>238.27</v>
       </c>
       <c r="F22" s="10">
-        <v>250.52</v>
+        <v>247.87</v>
       </c>
       <c r="G22" s="10">
-        <v>242.67</v>
+        <v>240.02</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>300.18</v>
+        <v>300.47000000000003</v>
       </c>
       <c r="E23" s="13">
-        <v>249.24</v>
+        <v>246.64</v>
       </c>
       <c r="F23" s="13">
-        <v>259.24</v>
+        <v>256.64</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>300.27</v>
+        <v>300.55</v>
       </c>
       <c r="E24" s="10">
-        <v>249.86</v>
+        <v>247.3</v>
       </c>
       <c r="F24" s="10">
-        <v>259.86</v>
+        <v>257.3</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>300.24</v>
+        <v>300.51</v>
       </c>
       <c r="E25" s="13">
-        <v>249.59</v>
+        <v>247.04</v>
       </c>
       <c r="F25" s="13">
-        <v>259.58999999999997</v>
+        <v>257.04000000000002</v>
       </c>
       <c r="G25" s="13">
-        <v>250.44</v>
+        <v>247.89</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>299.8</v>
+        <v>300.06</v>
       </c>
       <c r="E26" s="10">
-        <v>250.17</v>
+        <v>247.6</v>
       </c>
       <c r="F26" s="10">
-        <v>260.17</v>
+        <v>257.60000000000002</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>300</v>
+        <v>298.75</v>
       </c>
       <c r="E27" s="13">
-        <v>243.69</v>
+        <v>240.92</v>
       </c>
       <c r="F27" s="13">
-        <v>253.29</v>
+        <v>250.52</v>
       </c>
       <c r="G27" s="13">
-        <v>245.44</v>
+        <v>242.67</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>302.60000000000002</v>
+        <v>300.18</v>
       </c>
       <c r="E28" s="22">
-        <v>249.62</v>
+        <v>249.24</v>
       </c>
       <c r="F28" s="22">
-        <v>259.62</v>
+        <v>259.24</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>302.70999999999998</v>
+        <v>300.27</v>
       </c>
       <c r="E29" s="13">
-        <v>250.19</v>
+        <v>249.86</v>
       </c>
       <c r="F29" s="13">
-        <v>260.19</v>
+        <v>259.86</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>302.68</v>
+        <v>300.24</v>
       </c>
       <c r="E30" s="22">
-        <v>249.91</v>
+        <v>249.59</v>
       </c>
       <c r="F30" s="22">
-        <v>259.91000000000003</v>
+        <v>259.58999999999997</v>
       </c>
       <c r="G30" s="22">
-        <v>250.76</v>
+        <v>250.44</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>302.26</v>
+        <v>299.8</v>
       </c>
       <c r="E31" s="13">
-        <v>250.49</v>
+        <v>250.17</v>
       </c>
       <c r="F31" s="13">
-        <v>260.49</v>
+        <v>260.17</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>296.25</v>
+        <v>296.52</v>
       </c>
       <c r="E35" s="10">
-        <v>243.03</v>
+        <v>240.44</v>
       </c>
       <c r="F35" s="10">
-        <v>252.03</v>
+        <v>249.44</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>296.49</v>
+        <v>296.25</v>
       </c>
       <c r="E36" s="13">
-        <v>243.4</v>
+        <v>243.03</v>
       </c>
       <c r="F36" s="13">
-        <v>252.4</v>
+        <v>252.03</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>302.33</v>
+        <v>302.68</v>
       </c>
       <c r="E40" s="10">
-        <v>241.49</v>
+        <v>240.68</v>
       </c>
       <c r="F40" s="10">
-        <v>251.49</v>
+        <v>250.68</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>301.89999999999998</v>
+        <v>302.26</v>
       </c>
       <c r="E41" s="13">
-        <v>241.9</v>
+        <v>241.09</v>
       </c>
       <c r="F41" s="13">
-        <v>251.9</v>
+        <v>251.09</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>302.48</v>
+        <v>302.33</v>
       </c>
       <c r="E42" s="10">
-        <v>240.06</v>
+        <v>241.49</v>
       </c>
       <c r="F42" s="10">
-        <v>250.06</v>
+        <v>251.49</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>302.06</v>
+        <v>301.89999999999998</v>
       </c>
       <c r="E43" s="13">
-        <v>240.48</v>
+        <v>241.9</v>
       </c>
       <c r="F43" s="13">
-        <v>250.48</v>
+        <v>251.9</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>297.32</v>
+        <v>297.52</v>
       </c>
       <c r="E47" s="10">
-        <v>241.53</v>
+        <v>239.28</v>
       </c>
       <c r="F47" s="10">
-        <v>251.53</v>
+        <v>249.28</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>297.06</v>
+        <v>297.23</v>
       </c>
       <c r="E48" s="13">
-        <v>241.57</v>
+        <v>239.3</v>
       </c>
       <c r="F48" s="13">
-        <v>251.57</v>
+        <v>249.3</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>297.24</v>
+        <v>297.32</v>
       </c>
       <c r="E49" s="10">
-        <v>244.8</v>
+        <v>241.53</v>
       </c>
       <c r="F49" s="10">
-        <v>254.8</v>
+        <v>251.53</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>296.99</v>
+        <v>297.06</v>
       </c>
       <c r="E50" s="13">
-        <v>244.85</v>
+        <v>241.57</v>
       </c>
       <c r="F50" s="13">
-        <v>254.85</v>
+        <v>251.57</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>311.24</v>
+        <v>311.52</v>
       </c>
       <c r="E54" s="10">
-        <v>255.11</v>
+        <v>252.9</v>
       </c>
       <c r="F54" s="10">
-        <v>265.11</v>
+        <v>262.89999999999998</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>303.86</v>
+        <v>304.16000000000003</v>
       </c>
       <c r="E55" s="13">
-        <v>253.57</v>
+        <v>250.89</v>
       </c>
       <c r="F55" s="13">
-        <v>263.57</v>
+        <v>260.89</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>303.76</v>
+        <v>304.06</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>303.48</v>
+        <v>303.64</v>
       </c>
       <c r="E57" s="13">
-        <v>247.94</v>
+        <v>245.26</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>299.33</v>
+        <v>299.49</v>
       </c>
       <c r="E58" s="10">
-        <v>243.89</v>
+        <v>241.21</v>
       </c>
       <c r="F58" s="10">
-        <v>253.89</v>
+        <v>251.21</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>303.16000000000003</v>
+        <v>303.32</v>
       </c>
       <c r="E59" s="13">
-        <v>252.69</v>
+        <v>250.31</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>311.49</v>
+        <v>311.24</v>
       </c>
       <c r="E60" s="10">
-        <v>255.03</v>
+        <v>255.11</v>
       </c>
       <c r="F60" s="10">
-        <v>265.02999999999997</v>
+        <v>265.11</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>304.08999999999997</v>
+        <v>303.86</v>
       </c>
       <c r="E61" s="13">
-        <v>254.05</v>
+        <v>253.57</v>
       </c>
       <c r="F61" s="13">
-        <v>264.05</v>
+        <v>263.57</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>303.98</v>
+        <v>303.76</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>303.87</v>
+        <v>303.48</v>
       </c>
       <c r="E63" s="13">
-        <v>248.42</v>
+        <v>247.94</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>299.72000000000003</v>
+        <v>299.33</v>
       </c>
       <c r="E64" s="10">
-        <v>244.37</v>
+        <v>243.89</v>
       </c>
       <c r="F64" s="10">
-        <v>254.37</v>
+        <v>253.89</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>303.54000000000002</v>
+        <v>303.16000000000003</v>
       </c>
       <c r="E65" s="13">
-        <v>252.8</v>
+        <v>252.69</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1850,6 +1850,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2109,15 +2118,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2130,6 +2130,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2145,14 +2153,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Fri Mar 27 04:06:59 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{00E50267-B6CF-4CFA-8AF1-DDD27036EB07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{69D4A93B-6721-4548-8B72-8918F64557FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -802,128 +802,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>298.98</v>
+        <v>299.23</v>
       </c>
       <c r="E8" s="10">
-        <v>237.28</v>
+        <v>233.43</v>
       </c>
       <c r="F8" s="10">
-        <v>247.28</v>
+        <v>243.43</v>
       </c>
       <c r="G8" s="10">
-        <v>237.16</v>
+        <v>233.32</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>298.98</v>
+        <v>299.23</v>
       </c>
       <c r="E9" s="13">
-        <v>237.28</v>
+        <v>233.43</v>
       </c>
       <c r="F9" s="13">
-        <v>247.28</v>
+        <v>243.43</v>
       </c>
       <c r="G9" s="13">
-        <v>237.16</v>
+        <v>233.32</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>299.83999999999997</v>
+        <v>300.10000000000002</v>
       </c>
       <c r="E10" s="10">
-        <v>239.91</v>
+        <v>236.06</v>
       </c>
       <c r="F10" s="10">
-        <v>249.91</v>
+        <v>246.06</v>
       </c>
       <c r="G10" s="10">
-        <v>240.15</v>
+        <v>236.3</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>298.77</v>
+        <v>298.98</v>
       </c>
       <c r="E11" s="13">
-        <v>239.93</v>
+        <v>237.28</v>
       </c>
       <c r="F11" s="13">
-        <v>249.93</v>
+        <v>247.28</v>
       </c>
       <c r="G11" s="13">
-        <v>239.82</v>
+        <v>237.16</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>298.77</v>
+        <v>298.98</v>
       </c>
       <c r="E12" s="10">
-        <v>239.93</v>
+        <v>237.28</v>
       </c>
       <c r="F12" s="10">
-        <v>249.93</v>
+        <v>247.28</v>
       </c>
       <c r="G12" s="10">
-        <v>239.82</v>
+        <v>237.16</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>299.56</v>
+        <v>299.83999999999997</v>
       </c>
       <c r="E13" s="13">
-        <v>242.5</v>
+        <v>239.91</v>
       </c>
       <c r="F13" s="13">
-        <v>252.5</v>
+        <v>249.91</v>
       </c>
       <c r="G13" s="13">
-        <v>242.74</v>
+        <v>240.15</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -967,39 +967,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>301.11</v>
+        <v>302.39</v>
       </c>
       <c r="E17" s="10">
-        <v>240.54</v>
+        <v>236.6</v>
       </c>
       <c r="F17" s="10">
-        <v>250.54</v>
+        <v>246.6</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>300.92</v>
+        <v>301.11</v>
       </c>
       <c r="E18" s="13">
-        <v>243.22</v>
+        <v>240.54</v>
       </c>
       <c r="F18" s="13">
-        <v>253.22</v>
+        <v>250.54</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1046,41 +1046,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>298.95</v>
+        <v>298.98</v>
       </c>
       <c r="E22" s="10">
-        <v>238.27</v>
+        <v>234.42</v>
       </c>
       <c r="F22" s="10">
-        <v>247.87</v>
+        <v>244.02</v>
       </c>
       <c r="G22" s="10">
-        <v>240.02</v>
+        <v>236.17</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>300.47000000000003</v>
+        <v>301.83999999999997</v>
       </c>
       <c r="E23" s="13">
-        <v>246.64</v>
+        <v>241.67</v>
       </c>
       <c r="F23" s="13">
-        <v>256.64</v>
+        <v>251.67</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1088,20 +1088,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>300.55</v>
+        <v>301.91000000000003</v>
       </c>
       <c r="E24" s="10">
-        <v>247.3</v>
+        <v>242.38</v>
       </c>
       <c r="F24" s="10">
-        <v>257.3</v>
+        <v>252.38</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1109,41 +1109,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>300.51</v>
+        <v>301.87</v>
       </c>
       <c r="E25" s="13">
-        <v>247.04</v>
+        <v>242.12</v>
       </c>
       <c r="F25" s="13">
-        <v>257.04000000000002</v>
+        <v>252.12</v>
       </c>
       <c r="G25" s="13">
-        <v>247.89</v>
+        <v>242.96</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>300.06</v>
+        <v>301.39999999999998</v>
       </c>
       <c r="E26" s="10">
-        <v>247.6</v>
+        <v>242.63</v>
       </c>
       <c r="F26" s="10">
-        <v>257.60000000000002</v>
+        <v>252.63</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1151,41 +1151,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>298.75</v>
+        <v>298.95</v>
       </c>
       <c r="E27" s="13">
-        <v>240.92</v>
+        <v>238.27</v>
       </c>
       <c r="F27" s="13">
-        <v>250.52</v>
+        <v>247.87</v>
       </c>
       <c r="G27" s="13">
-        <v>242.67</v>
+        <v>240.02</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>300.18</v>
+        <v>300.47000000000003</v>
       </c>
       <c r="E28" s="22">
-        <v>249.24</v>
+        <v>246.64</v>
       </c>
       <c r="F28" s="22">
-        <v>259.24</v>
+        <v>256.64</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1193,20 +1193,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>300.27</v>
+        <v>300.55</v>
       </c>
       <c r="E29" s="13">
-        <v>249.86</v>
+        <v>247.3</v>
       </c>
       <c r="F29" s="13">
-        <v>259.86</v>
+        <v>257.3</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1214,41 +1214,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>300.24</v>
+        <v>300.51</v>
       </c>
       <c r="E30" s="22">
-        <v>249.59</v>
+        <v>247.04</v>
       </c>
       <c r="F30" s="22">
-        <v>259.58999999999997</v>
+        <v>257.04000000000002</v>
       </c>
       <c r="G30" s="22">
-        <v>250.44</v>
+        <v>247.89</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>299.8</v>
+        <v>300.06</v>
       </c>
       <c r="E31" s="13">
-        <v>250.17</v>
+        <v>247.6</v>
       </c>
       <c r="F31" s="13">
-        <v>260.17</v>
+        <v>257.60000000000002</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1295,39 +1295,39 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>296.52</v>
+        <v>297.89</v>
       </c>
       <c r="E35" s="10">
-        <v>240.44</v>
+        <v>236.6</v>
       </c>
       <c r="F35" s="10">
-        <v>249.44</v>
+        <v>245.6</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>296.25</v>
+        <v>296.52</v>
       </c>
       <c r="E36" s="13">
-        <v>243.03</v>
+        <v>240.44</v>
       </c>
       <c r="F36" s="13">
-        <v>252.03</v>
+        <v>249.44</v>
       </c>
       <c r="G36" s="17"/>
     </row>
@@ -1372,77 +1372,77 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B40" s="8"/>
       <c r="C40" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D40" s="10">
-        <v>302.68</v>
+        <v>305.20999999999998</v>
       </c>
       <c r="E40" s="10">
-        <v>240.68</v>
+        <v>241.93</v>
       </c>
       <c r="F40" s="10">
-        <v>250.68</v>
+        <v>251.93</v>
       </c>
       <c r="G40" s="17"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="13">
-        <v>302.26</v>
+        <v>304.77999999999997</v>
       </c>
       <c r="E41" s="13">
-        <v>241.09</v>
+        <v>242.34</v>
       </c>
       <c r="F41" s="13">
-        <v>251.09</v>
+        <v>252.34</v>
       </c>
       <c r="G41" s="17"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>25</v>
       </c>
       <c r="D42" s="10">
-        <v>302.33</v>
+        <v>302.68</v>
       </c>
       <c r="E42" s="10">
-        <v>241.49</v>
+        <v>240.68</v>
       </c>
       <c r="F42" s="10">
-        <v>251.49</v>
+        <v>250.68</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>26</v>
       </c>
       <c r="D43" s="13">
-        <v>301.89999999999998</v>
+        <v>302.26</v>
       </c>
       <c r="E43" s="13">
-        <v>241.9</v>
+        <v>241.09</v>
       </c>
       <c r="F43" s="13">
-        <v>251.9</v>
+        <v>251.09</v>
       </c>
       <c r="G43" s="17"/>
     </row>
@@ -1487,77 +1487,77 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B47" s="8"/>
       <c r="C47" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D47" s="10">
-        <v>297.52</v>
+        <v>300.82</v>
       </c>
       <c r="E47" s="10">
-        <v>239.28</v>
+        <v>239.2</v>
       </c>
       <c r="F47" s="10">
-        <v>249.28</v>
+        <v>249.2</v>
       </c>
       <c r="G47" s="17"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B48" s="12"/>
       <c r="C48" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D48" s="13">
-        <v>297.23</v>
+        <v>300.51</v>
       </c>
       <c r="E48" s="13">
-        <v>239.3</v>
+        <v>239.2</v>
       </c>
       <c r="F48" s="13">
-        <v>249.3</v>
+        <v>249.2</v>
       </c>
       <c r="G48" s="17"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>28</v>
       </c>
       <c r="D49" s="10">
-        <v>297.32</v>
+        <v>297.52</v>
       </c>
       <c r="E49" s="10">
-        <v>241.53</v>
+        <v>239.28</v>
       </c>
       <c r="F49" s="10">
-        <v>251.53</v>
+        <v>249.28</v>
       </c>
       <c r="G49" s="17"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="13">
-        <v>297.06</v>
+        <v>297.23</v>
       </c>
       <c r="E50" s="13">
-        <v>241.57</v>
+        <v>239.3</v>
       </c>
       <c r="F50" s="13">
-        <v>251.57</v>
+        <v>249.3</v>
       </c>
       <c r="G50" s="17"/>
     </row>
@@ -1602,52 +1602,52 @@
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B54" s="8"/>
       <c r="C54" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D54" s="10">
-        <v>311.52</v>
+        <v>312.86</v>
       </c>
       <c r="E54" s="10">
-        <v>252.9</v>
+        <v>249.38</v>
       </c>
       <c r="F54" s="10">
-        <v>262.89999999999998</v>
+        <v>259.38</v>
       </c>
       <c r="G54" s="17"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D55" s="13">
-        <v>304.16000000000003</v>
+        <v>305.52999999999997</v>
       </c>
       <c r="E55" s="13">
-        <v>250.89</v>
+        <v>246.98</v>
       </c>
       <c r="F55" s="13">
-        <v>260.89</v>
+        <v>256.98</v>
       </c>
       <c r="G55" s="17"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D56" s="10">
-        <v>304.06</v>
+        <v>305.44</v>
       </c>
       <c r="E56" s="10" t="s">
         <v>18</v>
@@ -1659,17 +1659,17 @@
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D57" s="13">
-        <v>303.64</v>
+        <v>304.89999999999998</v>
       </c>
       <c r="E57" s="13">
-        <v>245.26</v>
+        <v>241.36</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>18</v>
@@ -1678,36 +1678,36 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D58" s="10">
-        <v>299.49</v>
+        <v>300.76</v>
       </c>
       <c r="E58" s="10">
-        <v>241.21</v>
+        <v>237.3</v>
       </c>
       <c r="F58" s="10">
-        <v>251.21</v>
+        <v>247.3</v>
       </c>
       <c r="G58" s="17"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D59" s="13">
-        <v>303.32</v>
+        <v>304.58999999999997</v>
       </c>
       <c r="E59" s="13">
-        <v>250.31</v>
+        <v>246.64</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1716,52 +1716,52 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>31</v>
       </c>
       <c r="D60" s="10">
-        <v>311.24</v>
+        <v>311.52</v>
       </c>
       <c r="E60" s="10">
-        <v>255.11</v>
+        <v>252.9</v>
       </c>
       <c r="F60" s="10">
-        <v>265.11</v>
+        <v>262.89999999999998</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>32</v>
       </c>
       <c r="D61" s="13">
-        <v>303.86</v>
+        <v>304.16000000000003</v>
       </c>
       <c r="E61" s="13">
-        <v>253.57</v>
+        <v>250.89</v>
       </c>
       <c r="F61" s="13">
-        <v>263.57</v>
+        <v>260.89</v>
       </c>
       <c r="G61" s="17"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>33</v>
       </c>
       <c r="D62" s="10">
-        <v>303.76</v>
+        <v>304.06</v>
       </c>
       <c r="E62" s="10" t="s">
         <v>18</v>
@@ -1773,17 +1773,17 @@
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>34</v>
       </c>
       <c r="D63" s="13">
-        <v>303.48</v>
+        <v>303.64</v>
       </c>
       <c r="E63" s="13">
-        <v>247.94</v>
+        <v>245.26</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>18</v>
@@ -1792,36 +1792,36 @@
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>35</v>
       </c>
       <c r="D64" s="10">
-        <v>299.33</v>
+        <v>299.49</v>
       </c>
       <c r="E64" s="10">
-        <v>243.89</v>
+        <v>241.21</v>
       </c>
       <c r="F64" s="10">
-        <v>253.89</v>
+        <v>251.21</v>
       </c>
       <c r="G64" s="17"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46107</v>
+        <v>46108</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>36</v>
       </c>
       <c r="D65" s="13">
-        <v>303.16000000000003</v>
+        <v>303.32</v>
       </c>
       <c r="E65" s="13">
-        <v>252.69</v>
+        <v>250.31</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1859,6 +1859,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2118,17 +2129,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
@@ -2138,6 +2138,24 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2157,24 +2175,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Fri Mar 27 14:30:00 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{69D4A93B-6721-4548-8B72-8918F64557FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="14_{69D4A93B-6721-4548-8B72-8918F64557FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50CD192A-B954-4575-A57C-5B48438564AD}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="38">
   <si>
     <t>BP terminal gate pricing by state</t>
   </si>
@@ -147,6 +150,9 @@
   </si>
   <si>
     <t>Port Hedland</t>
+  </si>
+  <si>
+    <t>Port Bonython</t>
   </si>
 </sst>
 </file>
@@ -301,7 +307,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -383,6 +389,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -405,6 +414,69 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Front Page"/>
+      <sheetName val="PCNs"/>
+      <sheetName val="BM List"/>
+      <sheetName val="BM Check"/>
+      <sheetName val="ORP List"/>
+      <sheetName val="ZP01"/>
+      <sheetName val="Leader Price Movement"/>
+      <sheetName val="Leader Follower Check"/>
+      <sheetName val="New Database"/>
+      <sheetName val="Bottoms"/>
+      <sheetName val="PROS Dump Check"/>
+      <sheetName val="Web TGP"/>
+      <sheetName val="FuelWatch Check"/>
+      <sheetName val="FuelWatch Upload"/>
+      <sheetName val="FuelWatch"/>
+      <sheetName val="Web TGP Check"/>
+      <sheetName val="Rack Price - Card"/>
+      <sheetName val="Rack Notification"/>
+      <sheetName val="TGP Notification"/>
+      <sheetName val="Lookup"/>
+      <sheetName val="Comp TGP"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11">
+        <row r="2">
+          <cell r="J2">
+            <v>46109</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -707,7 +779,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
@@ -769,10 +841,10 @@
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="27"/>
+      <c r="B6" s="29"/>
       <c r="C6" s="1"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -936,10 +1008,10 @@
       <c r="G14" s="16"/>
     </row>
     <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="27"/>
+      <c r="B15" s="29"/>
       <c r="C15" s="1"/>
       <c r="D15" s="17"/>
       <c r="E15" s="17"/>
@@ -1013,10 +1085,10 @@
       <c r="G19" s="17"/>
     </row>
     <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="27"/>
+      <c r="B20" s="29"/>
       <c r="C20" s="1"/>
       <c r="D20" s="17"/>
       <c r="E20" s="17"/>
@@ -1264,10 +1336,10 @@
       <c r="G32" s="17"/>
     </row>
     <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A33" s="27" t="s">
+      <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="B33" s="27"/>
+      <c r="B33" s="29"/>
       <c r="C33" s="1"/>
       <c r="D33" s="17"/>
       <c r="E33" s="17"/>
@@ -1332,513 +1404,529 @@
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="14"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="15"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
+      <c r="A37" s="7">
+        <f>'[1]Web TGP'!$J$2</f>
+        <v>46109</v>
+      </c>
+      <c r="B37" s="8"/>
+      <c r="C37" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="D37" s="10">
+        <v>313.51</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F37" s="10" t="s">
+        <v>18</v>
+      </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A38" s="27" t="s">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="14"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="17"/>
+      <c r="G38" s="17"/>
+    </row>
+    <row r="39" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A39" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="B38" s="27"/>
-      <c r="C38" s="1"/>
-      <c r="D38" s="17"/>
-      <c r="E38" s="17"/>
-      <c r="F38" s="17"/>
-      <c r="G38" s="17"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="23" t="s">
+      <c r="B39" s="29"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="17"/>
+      <c r="G39" s="17"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B39" s="5"/>
-      <c r="C39" s="18" t="s">
+      <c r="B40" s="5"/>
+      <c r="C40" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D39" s="19" t="s">
+      <c r="D40" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E39" s="19" t="s">
+      <c r="E40" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="F39" s="19" t="s">
+      <c r="F40" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="G39" s="17"/>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="7">
+      <c r="G40" s="17"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="7">
         <v>46109</v>
       </c>
-      <c r="B40" s="8"/>
-      <c r="C40" s="20" t="s">
+      <c r="B41" s="8"/>
+      <c r="C41" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D40" s="10">
+      <c r="D41" s="10">
         <v>305.20999999999998</v>
       </c>
-      <c r="E40" s="10">
+      <c r="E41" s="10">
         <v>241.93</v>
       </c>
-      <c r="F40" s="10">
+      <c r="F41" s="10">
         <v>251.93</v>
       </c>
-      <c r="G40" s="17"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="11">
+      <c r="G41" s="17"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="11">
         <v>46109</v>
       </c>
-      <c r="B41" s="12"/>
-      <c r="C41" s="21" t="s">
+      <c r="B42" s="12"/>
+      <c r="C42" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D41" s="13">
+      <c r="D42" s="13">
         <v>304.77999999999997</v>
       </c>
-      <c r="E41" s="13">
+      <c r="E42" s="13">
         <v>242.34</v>
       </c>
-      <c r="F41" s="13">
+      <c r="F42" s="13">
         <v>252.34</v>
       </c>
-      <c r="G41" s="17"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="7">
+      <c r="G42" s="17"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="7">
         <v>46108</v>
       </c>
-      <c r="B42" s="8"/>
-      <c r="C42" s="20" t="s">
+      <c r="B43" s="8"/>
+      <c r="C43" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D42" s="10">
+      <c r="D43" s="10">
         <v>302.68</v>
       </c>
-      <c r="E42" s="10">
+      <c r="E43" s="10">
         <v>240.68</v>
       </c>
-      <c r="F42" s="10">
+      <c r="F43" s="10">
         <v>250.68</v>
       </c>
-      <c r="G42" s="17"/>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="11">
+      <c r="G43" s="17"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="11">
         <v>46108</v>
       </c>
-      <c r="B43" s="12"/>
-      <c r="C43" s="21" t="s">
+      <c r="B44" s="12"/>
+      <c r="C44" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D43" s="13">
+      <c r="D44" s="13">
         <v>302.26</v>
       </c>
-      <c r="E43" s="13">
+      <c r="E44" s="13">
         <v>241.09</v>
       </c>
-      <c r="F43" s="13">
+      <c r="F44" s="13">
         <v>251.09</v>
       </c>
-      <c r="G43" s="17"/>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="14"/>
-      <c r="B44" s="24"/>
-      <c r="C44" s="15"/>
-      <c r="D44" s="16"/>
-      <c r="E44" s="16"/>
-      <c r="F44" s="16"/>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="25" t="s">
+      <c r="A45" s="14"/>
+      <c r="B45" s="24"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="16"/>
+      <c r="E45" s="16"/>
+      <c r="F45" s="16"/>
+      <c r="G45" s="17"/>
+    </row>
+    <row r="46" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A46" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B45" s="26"/>
-      <c r="C45" s="1"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="23" t="s">
+      <c r="B46" s="26"/>
+      <c r="C46" s="1"/>
+      <c r="D46" s="17"/>
+      <c r="E46" s="17"/>
+      <c r="F46" s="17"/>
+      <c r="G46" s="17"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B46" s="5"/>
-      <c r="C46" s="18" t="s">
+      <c r="B47" s="5"/>
+      <c r="C47" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D46" s="19" t="s">
+      <c r="D47" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E46" s="19" t="s">
+      <c r="E47" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="F46" s="19" t="s">
+      <c r="F47" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="G46" s="17"/>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="7">
+      <c r="G47" s="17"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="7">
         <v>46109</v>
       </c>
-      <c r="B47" s="8"/>
-      <c r="C47" s="20" t="s">
+      <c r="B48" s="8"/>
+      <c r="C48" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D47" s="10">
+      <c r="D48" s="10">
         <v>300.82</v>
       </c>
-      <c r="E47" s="10">
+      <c r="E48" s="10">
         <v>239.2</v>
       </c>
-      <c r="F47" s="10">
+      <c r="F48" s="10">
         <v>249.2</v>
       </c>
-      <c r="G47" s="17"/>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="11">
+      <c r="G48" s="17"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="11">
         <v>46109</v>
       </c>
-      <c r="B48" s="12"/>
-      <c r="C48" s="21" t="s">
+      <c r="B49" s="12"/>
+      <c r="C49" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="D48" s="13">
+      <c r="D49" s="13">
         <v>300.51</v>
       </c>
-      <c r="E48" s="13">
+      <c r="E49" s="13">
         <v>239.2</v>
       </c>
-      <c r="F48" s="13">
+      <c r="F49" s="13">
         <v>249.2</v>
       </c>
-      <c r="G48" s="17"/>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="7">
+      <c r="G49" s="17"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="7">
         <v>46108</v>
       </c>
-      <c r="B49" s="8"/>
-      <c r="C49" s="20" t="s">
+      <c r="B50" s="8"/>
+      <c r="C50" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D49" s="10">
+      <c r="D50" s="10">
         <v>297.52</v>
       </c>
-      <c r="E49" s="10">
+      <c r="E50" s="10">
         <v>239.28</v>
       </c>
-      <c r="F49" s="10">
+      <c r="F50" s="10">
         <v>249.28</v>
       </c>
-      <c r="G49" s="17"/>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="11">
+      <c r="G50" s="17"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="11">
         <v>46108</v>
       </c>
-      <c r="B50" s="12"/>
-      <c r="C50" s="21" t="s">
+      <c r="B51" s="12"/>
+      <c r="C51" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="D50" s="13">
+      <c r="D51" s="13">
         <v>297.23</v>
       </c>
-      <c r="E50" s="13">
+      <c r="E51" s="13">
         <v>239.3</v>
       </c>
-      <c r="F50" s="13">
+      <c r="F51" s="13">
         <v>249.3</v>
       </c>
-      <c r="G50" s="17"/>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="14"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="15"/>
-      <c r="D51" s="16"/>
-      <c r="E51" s="16"/>
-      <c r="F51" s="16"/>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A52" s="27" t="s">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" s="14"/>
+      <c r="B52" s="14"/>
+      <c r="C52" s="15"/>
+      <c r="D52" s="16"/>
+      <c r="E52" s="16"/>
+      <c r="F52" s="16"/>
+      <c r="G52" s="17"/>
+    </row>
+    <row r="53" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A53" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="B52" s="27"/>
-      <c r="C52" s="1"/>
-      <c r="D52" s="17"/>
-      <c r="E52" s="17"/>
-      <c r="F52" s="17"/>
-      <c r="G52" s="17"/>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="23" t="s">
+      <c r="B53" s="27"/>
+      <c r="C53" s="1"/>
+      <c r="D53" s="17"/>
+      <c r="E53" s="17"/>
+      <c r="F53" s="17"/>
+      <c r="G53" s="17"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B53" s="5"/>
-      <c r="C53" s="18" t="s">
+      <c r="B54" s="5"/>
+      <c r="C54" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D53" s="19" t="s">
+      <c r="D54" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E53" s="19" t="s">
+      <c r="E54" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="F53" s="19" t="s">
+      <c r="F54" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="G53" s="17"/>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="7">
+      <c r="G54" s="17"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" s="7">
         <v>46109</v>
       </c>
-      <c r="B54" s="8"/>
-      <c r="C54" s="20" t="s">
+      <c r="B55" s="8"/>
+      <c r="C55" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="D54" s="10">
+      <c r="D55" s="10">
         <v>312.86</v>
       </c>
-      <c r="E54" s="10">
+      <c r="E55" s="10">
         <v>249.38</v>
       </c>
-      <c r="F54" s="10">
+      <c r="F55" s="10">
         <v>259.38</v>
       </c>
-      <c r="G54" s="17"/>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="11">
+      <c r="G55" s="17"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="11">
         <v>46109</v>
       </c>
-      <c r="B55" s="12"/>
-      <c r="C55" s="21" t="s">
+      <c r="B56" s="12"/>
+      <c r="C56" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="D55" s="13">
+      <c r="D56" s="13">
         <v>305.52999999999997</v>
       </c>
-      <c r="E55" s="13">
+      <c r="E56" s="13">
         <v>246.98</v>
       </c>
-      <c r="F55" s="13">
+      <c r="F56" s="13">
         <v>256.98</v>
       </c>
-      <c r="G55" s="17"/>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="7">
+      <c r="G56" s="17"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="7">
         <v>46109</v>
       </c>
-      <c r="B56" s="8"/>
-      <c r="C56" s="20" t="s">
+      <c r="B57" s="8"/>
+      <c r="C57" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="D56" s="10">
+      <c r="D57" s="10">
         <v>305.44</v>
       </c>
-      <c r="E56" s="10" t="s">
+      <c r="E57" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="F56" s="10" t="s">
+      <c r="F57" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="G56" s="17"/>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="11">
+      <c r="G57" s="17"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" s="11">
         <v>46109</v>
       </c>
-      <c r="B57" s="12"/>
-      <c r="C57" s="21" t="s">
+      <c r="B58" s="12"/>
+      <c r="C58" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="D57" s="13">
+      <c r="D58" s="13">
         <v>304.89999999999998</v>
       </c>
-      <c r="E57" s="13">
+      <c r="E58" s="13">
         <v>241.36</v>
       </c>
-      <c r="F57" s="13" t="s">
+      <c r="F58" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="G57" s="17"/>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="7">
+      <c r="G58" s="17"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" s="7">
         <v>46109</v>
       </c>
-      <c r="B58" s="8"/>
-      <c r="C58" s="20" t="s">
+      <c r="B59" s="8"/>
+      <c r="C59" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="D58" s="10">
+      <c r="D59" s="10">
         <v>300.76</v>
       </c>
-      <c r="E58" s="10">
+      <c r="E59" s="10">
         <v>237.3</v>
       </c>
-      <c r="F58" s="10">
+      <c r="F59" s="10">
         <v>247.3</v>
       </c>
-      <c r="G58" s="17"/>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" s="11">
+      <c r="G59" s="17"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="11">
         <v>46109</v>
       </c>
-      <c r="B59" s="12"/>
-      <c r="C59" s="21" t="s">
+      <c r="B60" s="12"/>
+      <c r="C60" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="D59" s="13">
+      <c r="D60" s="13">
         <v>304.58999999999997</v>
       </c>
-      <c r="E59" s="13">
+      <c r="E60" s="13">
         <v>246.64</v>
       </c>
-      <c r="F59" s="13" t="s">
+      <c r="F60" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="G59" s="17"/>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="7">
+      <c r="G60" s="17"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" s="7">
         <v>46108</v>
       </c>
-      <c r="B60" s="8"/>
-      <c r="C60" s="20" t="s">
+      <c r="B61" s="8"/>
+      <c r="C61" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="D60" s="10">
+      <c r="D61" s="10">
         <v>311.52</v>
       </c>
-      <c r="E60" s="10">
+      <c r="E61" s="10">
         <v>252.9</v>
       </c>
-      <c r="F60" s="10">
+      <c r="F61" s="10">
         <v>262.89999999999998</v>
       </c>
-      <c r="G60" s="17"/>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="11">
+      <c r="G61" s="17"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" s="11">
         <v>46108</v>
       </c>
-      <c r="B61" s="12"/>
-      <c r="C61" s="21" t="s">
+      <c r="B62" s="12"/>
+      <c r="C62" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="D61" s="13">
+      <c r="D62" s="13">
         <v>304.16000000000003</v>
       </c>
-      <c r="E61" s="13">
+      <c r="E62" s="13">
         <v>250.89</v>
       </c>
-      <c r="F61" s="13">
+      <c r="F62" s="13">
         <v>260.89</v>
       </c>
-      <c r="G61" s="17"/>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="7">
+      <c r="G62" s="17"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" s="7">
         <v>46108</v>
       </c>
-      <c r="B62" s="8"/>
-      <c r="C62" s="20" t="s">
+      <c r="B63" s="8"/>
+      <c r="C63" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="D62" s="10">
+      <c r="D63" s="10">
         <v>304.06</v>
       </c>
-      <c r="E62" s="10" t="s">
+      <c r="E63" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="F62" s="10" t="s">
+      <c r="F63" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="G62" s="17"/>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="11">
+      <c r="G63" s="17"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" s="11">
         <v>46108</v>
       </c>
-      <c r="B63" s="12"/>
-      <c r="C63" s="21" t="s">
+      <c r="B64" s="12"/>
+      <c r="C64" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="D63" s="13">
+      <c r="D64" s="13">
         <v>303.64</v>
       </c>
-      <c r="E63" s="13">
+      <c r="E64" s="13">
         <v>245.26</v>
       </c>
-      <c r="F63" s="13" t="s">
+      <c r="F64" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="G63" s="17"/>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" s="7">
+      <c r="G64" s="17"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="7">
         <v>46108</v>
       </c>
-      <c r="B64" s="8"/>
-      <c r="C64" s="20" t="s">
+      <c r="B65" s="8"/>
+      <c r="C65" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="D64" s="10">
+      <c r="D65" s="10">
         <v>299.49</v>
       </c>
-      <c r="E64" s="10">
+      <c r="E65" s="10">
         <v>241.21</v>
       </c>
-      <c r="F64" s="10">
+      <c r="F65" s="10">
         <v>251.21</v>
       </c>
-      <c r="G64" s="17"/>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="11">
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="11">
         <v>46108</v>
       </c>
-      <c r="B65" s="12"/>
-      <c r="C65" s="21" t="s">
+      <c r="B66" s="12"/>
+      <c r="C66" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="D65" s="13">
+      <c r="D66" s="13">
         <v>303.32</v>
       </c>
-      <c r="E65" s="13">
+      <c r="E66" s="13">
         <v>250.31</v>
       </c>
-      <c r="F65" s="13" t="s">
+      <c r="F66" s="13" t="s">
         <v>18</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A52:B52"/>
+  <mergeCells count="6">
+    <mergeCell ref="A39:B39"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A38:B38"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="67" orientation="portrait" r:id="rId1"/>
+  <pageSetup scale="66" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C
 # Confidential</oddHeader>
@@ -1850,26 +1938,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2129,33 +2197,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2175,6 +2237,32 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Mon Mar 30 04:19:24 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="14_{69D4A93B-6721-4548-8B72-8918F64557FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50CD192A-B954-4575-A57C-5B48438564AD}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="14_{4B60EC9E-6E37-4055-B12E-050B026604DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B96C2A63-C8ED-4D02-AC1D-9DF772E09555}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="38">
   <si>
     <t>BP terminal gate pricing by state</t>
   </si>
@@ -388,10 +385,10 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -414,69 +411,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Front Page"/>
-      <sheetName val="PCNs"/>
-      <sheetName val="BM List"/>
-      <sheetName val="BM Check"/>
-      <sheetName val="ORP List"/>
-      <sheetName val="ZP01"/>
-      <sheetName val="Leader Price Movement"/>
-      <sheetName val="Leader Follower Check"/>
-      <sheetName val="New Database"/>
-      <sheetName val="Bottoms"/>
-      <sheetName val="PROS Dump Check"/>
-      <sheetName val="Web TGP"/>
-      <sheetName val="FuelWatch Check"/>
-      <sheetName val="FuelWatch Upload"/>
-      <sheetName val="FuelWatch"/>
-      <sheetName val="Web TGP Check"/>
-      <sheetName val="Rack Price - Card"/>
-      <sheetName val="Rack Notification"/>
-      <sheetName val="TGP Notification"/>
-      <sheetName val="Lookup"/>
-      <sheetName val="Comp TGP"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11">
-        <row r="2">
-          <cell r="J2">
-            <v>46109</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -779,7 +713,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
@@ -790,10 +724,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
+      <c r="B1" s="29"/>
       <c r="C1" s="1"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -841,10 +775,10 @@
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="29"/>
+      <c r="B6" s="28"/>
       <c r="C6" s="1"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -874,128 +808,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>299.23</v>
+        <v>307.79000000000002</v>
       </c>
       <c r="E8" s="10">
-        <v>233.43</v>
+        <v>231.83</v>
       </c>
       <c r="F8" s="10">
-        <v>243.43</v>
+        <v>241.83</v>
       </c>
       <c r="G8" s="10">
-        <v>233.32</v>
+        <v>231.72</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>299.23</v>
+        <v>307.79000000000002</v>
       </c>
       <c r="E9" s="13">
-        <v>233.43</v>
+        <v>231.83</v>
       </c>
       <c r="F9" s="13">
-        <v>243.43</v>
+        <v>241.83</v>
       </c>
       <c r="G9" s="13">
-        <v>233.32</v>
+        <v>231.72</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>300.10000000000002</v>
+        <v>308.61</v>
       </c>
       <c r="E10" s="10">
-        <v>236.06</v>
+        <v>234.4</v>
       </c>
       <c r="F10" s="10">
-        <v>246.06</v>
+        <v>244.4</v>
       </c>
       <c r="G10" s="10">
-        <v>236.3</v>
+        <v>234.64</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>298.98</v>
+        <v>299.23</v>
       </c>
       <c r="E11" s="13">
-        <v>237.28</v>
+        <v>233.43</v>
       </c>
       <c r="F11" s="13">
-        <v>247.28</v>
+        <v>243.43</v>
       </c>
       <c r="G11" s="13">
-        <v>237.16</v>
+        <v>233.32</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>298.98</v>
+        <v>299.23</v>
       </c>
       <c r="E12" s="10">
-        <v>237.28</v>
+        <v>233.43</v>
       </c>
       <c r="F12" s="10">
-        <v>247.28</v>
+        <v>243.43</v>
       </c>
       <c r="G12" s="10">
-        <v>237.16</v>
+        <v>233.32</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>299.83999999999997</v>
+        <v>300.10000000000002</v>
       </c>
       <c r="E13" s="13">
-        <v>239.91</v>
+        <v>236.06</v>
       </c>
       <c r="F13" s="13">
-        <v>249.91</v>
+        <v>246.06</v>
       </c>
       <c r="G13" s="13">
-        <v>240.15</v>
+        <v>236.3</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1008,10 +942,10 @@
       <c r="G14" s="16"/>
     </row>
     <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A15" s="29" t="s">
+      <c r="A15" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="29"/>
+      <c r="B15" s="28"/>
       <c r="C15" s="1"/>
       <c r="D15" s="17"/>
       <c r="E15" s="17"/>
@@ -1039,39 +973,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>302.39</v>
+        <v>310.89</v>
       </c>
       <c r="E17" s="10">
-        <v>236.6</v>
+        <v>234.9</v>
       </c>
       <c r="F17" s="10">
-        <v>246.6</v>
+        <v>244.9</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>301.11</v>
+        <v>302.39</v>
       </c>
       <c r="E18" s="13">
-        <v>240.54</v>
+        <v>236.6</v>
       </c>
       <c r="F18" s="13">
-        <v>250.54</v>
+        <v>246.6</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1085,10 +1019,10 @@
       <c r="G19" s="17"/>
     </row>
     <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A20" s="29" t="s">
+      <c r="A20" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="29"/>
+      <c r="B20" s="28"/>
       <c r="C20" s="1"/>
       <c r="D20" s="17"/>
       <c r="E20" s="17"/>
@@ -1118,41 +1052,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>298.98</v>
+        <v>307.55</v>
       </c>
       <c r="E22" s="10">
-        <v>234.42</v>
+        <v>232.83</v>
       </c>
       <c r="F22" s="10">
-        <v>244.02</v>
+        <v>242.43</v>
       </c>
       <c r="G22" s="10">
-        <v>236.17</v>
+        <v>234.58</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>301.83999999999997</v>
+        <v>310.35000000000002</v>
       </c>
       <c r="E23" s="13">
-        <v>241.67</v>
+        <v>239.99</v>
       </c>
       <c r="F23" s="13">
-        <v>251.67</v>
+        <v>249.99</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1160,20 +1094,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>301.91000000000003</v>
+        <v>310.42</v>
       </c>
       <c r="E24" s="10">
-        <v>242.38</v>
+        <v>240.72</v>
       </c>
       <c r="F24" s="10">
-        <v>252.38</v>
+        <v>250.72</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1181,41 +1115,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>301.87</v>
+        <v>310.38</v>
       </c>
       <c r="E25" s="13">
-        <v>242.12</v>
+        <v>240.45</v>
       </c>
       <c r="F25" s="13">
-        <v>252.12</v>
+        <v>250.45</v>
       </c>
       <c r="G25" s="13">
-        <v>242.96</v>
+        <v>241.3</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>301.39999999999998</v>
+        <v>309.91000000000003</v>
       </c>
       <c r="E26" s="10">
-        <v>242.63</v>
+        <v>240.93</v>
       </c>
       <c r="F26" s="10">
-        <v>252.63</v>
+        <v>250.93</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1223,41 +1157,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>298.95</v>
+        <v>298.98</v>
       </c>
       <c r="E27" s="13">
-        <v>238.27</v>
+        <v>234.42</v>
       </c>
       <c r="F27" s="13">
-        <v>247.87</v>
+        <v>244.02</v>
       </c>
       <c r="G27" s="13">
-        <v>240.02</v>
+        <v>236.17</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>300.47000000000003</v>
+        <v>301.83999999999997</v>
       </c>
       <c r="E28" s="22">
-        <v>246.64</v>
+        <v>241.67</v>
       </c>
       <c r="F28" s="22">
-        <v>256.64</v>
+        <v>251.67</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1265,20 +1199,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>300.55</v>
+        <v>301.91000000000003</v>
       </c>
       <c r="E29" s="13">
-        <v>247.3</v>
+        <v>242.38</v>
       </c>
       <c r="F29" s="13">
-        <v>257.3</v>
+        <v>252.38</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1286,41 +1220,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>300.51</v>
+        <v>301.87</v>
       </c>
       <c r="E30" s="22">
-        <v>247.04</v>
+        <v>242.12</v>
       </c>
       <c r="F30" s="22">
-        <v>257.04000000000002</v>
+        <v>252.12</v>
       </c>
       <c r="G30" s="22">
-        <v>247.89</v>
+        <v>242.96</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>300.06</v>
+        <v>301.39999999999998</v>
       </c>
       <c r="E31" s="13">
-        <v>247.6</v>
+        <v>242.63</v>
       </c>
       <c r="F31" s="13">
-        <v>257.60000000000002</v>
+        <v>252.63</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1336,10 +1270,10 @@
       <c r="G32" s="17"/>
     </row>
     <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A33" s="29" t="s">
+      <c r="A33" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="B33" s="29"/>
+      <c r="B33" s="28"/>
       <c r="C33" s="1"/>
       <c r="D33" s="17"/>
       <c r="E33" s="17"/>
@@ -1367,53 +1301,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>297.89</v>
+        <v>306.39</v>
       </c>
       <c r="E35" s="10">
-        <v>236.6</v>
+        <v>234.95</v>
       </c>
       <c r="F35" s="10">
-        <v>245.6</v>
+        <v>243.95</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>296.52</v>
+        <v>297.89</v>
       </c>
       <c r="E36" s="13">
-        <v>240.44</v>
+        <v>236.6</v>
       </c>
       <c r="F36" s="13">
-        <v>249.44</v>
+        <v>245.6</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <f>'[1]Web TGP'!$J$2</f>
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>37</v>
       </c>
       <c r="D37" s="10">
-        <v>313.51</v>
+        <v>322.01</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1424,501 +1357,521 @@
       <c r="G37" s="17"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="14"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="15"/>
-      <c r="D38" s="17"/>
+      <c r="A38" s="11">
+        <v>46109</v>
+      </c>
+      <c r="B38" s="12"/>
+      <c r="C38" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D38" s="13">
+        <v>313.51</v>
+      </c>
+      <c r="E38" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="F38" s="13" t="s">
+        <v>18</v>
+      </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A39" s="29" t="s">
-        <v>24</v>
-      </c>
-      <c r="B39" s="29"/>
-      <c r="C39" s="1"/>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="24"/>
+      <c r="B39" s="24"/>
+      <c r="C39" s="15"/>
       <c r="D39" s="17"/>
       <c r="E39" s="17"/>
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="23" t="s">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A40" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="B40" s="28"/>
+      <c r="C40" s="1"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="17"/>
+      <c r="F40" s="17"/>
+      <c r="G40" s="17"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B40" s="5"/>
-      <c r="C40" s="18" t="s">
+      <c r="B41" s="5"/>
+      <c r="C41" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D40" s="19" t="s">
+      <c r="D41" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E40" s="19" t="s">
+      <c r="E41" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="F40" s="19" t="s">
+      <c r="F41" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="G40" s="17"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="7">
+      <c r="G41" s="17"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="7">
+        <v>46112</v>
+      </c>
+      <c r="B42" s="8"/>
+      <c r="C42" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="D42" s="10">
+        <v>313.73</v>
+      </c>
+      <c r="E42" s="10">
+        <v>242</v>
+      </c>
+      <c r="F42" s="10">
+        <v>252</v>
+      </c>
+      <c r="G42" s="17"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="11">
+        <v>46112</v>
+      </c>
+      <c r="B43" s="12"/>
+      <c r="C43" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="D43" s="13">
+        <v>313.29000000000002</v>
+      </c>
+      <c r="E43" s="13">
+        <v>242.41</v>
+      </c>
+      <c r="F43" s="13">
+        <v>252.41</v>
+      </c>
+      <c r="G43" s="17"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="7">
         <v>46109</v>
       </c>
-      <c r="B41" s="8"/>
-      <c r="C41" s="20" t="s">
+      <c r="B44" s="8"/>
+      <c r="C44" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="D41" s="10">
+      <c r="D44" s="10">
         <v>305.20999999999998</v>
       </c>
-      <c r="E41" s="10">
+      <c r="E44" s="10">
         <v>241.93</v>
       </c>
-      <c r="F41" s="10">
+      <c r="F44" s="10">
         <v>251.93</v>
       </c>
-      <c r="G41" s="17"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="11">
+      <c r="G44" s="17"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="11">
         <v>46109</v>
       </c>
-      <c r="B42" s="12"/>
-      <c r="C42" s="21" t="s">
+      <c r="B45" s="12"/>
+      <c r="C45" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D42" s="13">
+      <c r="D45" s="13">
         <v>304.77999999999997</v>
       </c>
-      <c r="E42" s="13">
+      <c r="E45" s="13">
         <v>242.34</v>
       </c>
-      <c r="F42" s="13">
+      <c r="F45" s="13">
         <v>252.34</v>
       </c>
-      <c r="G42" s="17"/>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="7">
-        <v>46108</v>
-      </c>
-      <c r="B43" s="8"/>
-      <c r="C43" s="20" t="s">
-        <v>25</v>
-      </c>
-      <c r="D43" s="10">
-        <v>302.68</v>
-      </c>
-      <c r="E43" s="10">
-        <v>240.68</v>
-      </c>
-      <c r="F43" s="10">
-        <v>250.68</v>
-      </c>
-      <c r="G43" s="17"/>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="11">
-        <v>46108</v>
-      </c>
-      <c r="B44" s="12"/>
-      <c r="C44" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="D44" s="13">
-        <v>302.26</v>
-      </c>
-      <c r="E44" s="13">
-        <v>241.09</v>
-      </c>
-      <c r="F44" s="13">
-        <v>251.09</v>
-      </c>
-      <c r="G44" s="17"/>
-    </row>
-    <row r="45" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="14"/>
-      <c r="B45" s="24"/>
-      <c r="C45" s="15"/>
-      <c r="D45" s="16"/>
-      <c r="E45" s="16"/>
-      <c r="F45" s="16"/>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A46" s="25" t="s">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="14"/>
+      <c r="B46" s="24"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="16"/>
+      <c r="E46" s="16"/>
+      <c r="F46" s="16"/>
+      <c r="G46" s="17"/>
+    </row>
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A47" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="B46" s="26"/>
-      <c r="C46" s="1"/>
-      <c r="D46" s="17"/>
-      <c r="E46" s="17"/>
-      <c r="F46" s="17"/>
-      <c r="G46" s="17"/>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="23" t="s">
+      <c r="B47" s="26"/>
+      <c r="C47" s="1"/>
+      <c r="D47" s="17"/>
+      <c r="E47" s="17"/>
+      <c r="F47" s="17"/>
+      <c r="G47" s="17"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B47" s="5"/>
-      <c r="C47" s="18" t="s">
+      <c r="B48" s="5"/>
+      <c r="C48" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D47" s="19" t="s">
+      <c r="D48" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E47" s="19" t="s">
+      <c r="E48" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="F47" s="19" t="s">
+      <c r="F48" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="G47" s="17"/>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="7">
+      <c r="G48" s="17"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="7">
+        <v>46112</v>
+      </c>
+      <c r="B49" s="8"/>
+      <c r="C49" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="D49" s="10">
+        <v>311.83</v>
+      </c>
+      <c r="E49" s="10">
+        <v>239.67</v>
+      </c>
+      <c r="F49" s="10">
+        <v>249.67</v>
+      </c>
+      <c r="G49" s="17"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="11">
+        <v>46112</v>
+      </c>
+      <c r="B50" s="12"/>
+      <c r="C50" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="D50" s="13">
+        <v>311.52</v>
+      </c>
+      <c r="E50" s="13">
+        <v>239.66</v>
+      </c>
+      <c r="F50" s="13">
+        <v>249.66</v>
+      </c>
+      <c r="G50" s="17"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="7">
         <v>46109</v>
       </c>
-      <c r="B48" s="8"/>
-      <c r="C48" s="20" t="s">
+      <c r="B51" s="8"/>
+      <c r="C51" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="D48" s="10">
+      <c r="D51" s="10">
         <v>300.82</v>
       </c>
-      <c r="E48" s="10">
+      <c r="E51" s="10">
         <v>239.2</v>
       </c>
-      <c r="F48" s="10">
+      <c r="F51" s="10">
         <v>249.2</v>
       </c>
-      <c r="G48" s="17"/>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="11">
+      <c r="G51" s="17"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" s="11">
         <v>46109</v>
       </c>
-      <c r="B49" s="12"/>
-      <c r="C49" s="21" t="s">
+      <c r="B52" s="12"/>
+      <c r="C52" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="D49" s="13">
+      <c r="D52" s="13">
         <v>300.51</v>
       </c>
-      <c r="E49" s="13">
+      <c r="E52" s="13">
         <v>239.2</v>
       </c>
-      <c r="F49" s="13">
+      <c r="F52" s="13">
         <v>249.2</v>
       </c>
-      <c r="G49" s="17"/>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="7">
-        <v>46108</v>
-      </c>
-      <c r="B50" s="8"/>
-      <c r="C50" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="D50" s="10">
-        <v>297.52</v>
-      </c>
-      <c r="E50" s="10">
-        <v>239.28</v>
-      </c>
-      <c r="F50" s="10">
-        <v>249.28</v>
-      </c>
-      <c r="G50" s="17"/>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="11">
-        <v>46108</v>
-      </c>
-      <c r="B51" s="12"/>
-      <c r="C51" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="D51" s="13">
-        <v>297.23</v>
-      </c>
-      <c r="E51" s="13">
-        <v>239.3</v>
-      </c>
-      <c r="F51" s="13">
-        <v>249.3</v>
-      </c>
-      <c r="G51" s="17"/>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="14"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="15"/>
-      <c r="D52" s="16"/>
-      <c r="E52" s="16"/>
-      <c r="F52" s="16"/>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A53" s="27" t="s">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" s="14"/>
+      <c r="B53" s="14"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="16"/>
+      <c r="E53" s="16"/>
+      <c r="F53" s="16"/>
+      <c r="G53" s="17"/>
+    </row>
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A54" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="B53" s="27"/>
-      <c r="C53" s="1"/>
-      <c r="D53" s="17"/>
-      <c r="E53" s="17"/>
-      <c r="F53" s="17"/>
-      <c r="G53" s="17"/>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="23" t="s">
+      <c r="B54" s="27"/>
+      <c r="C54" s="1"/>
+      <c r="D54" s="17"/>
+      <c r="E54" s="17"/>
+      <c r="F54" s="17"/>
+      <c r="G54" s="17"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B54" s="5"/>
-      <c r="C54" s="18" t="s">
+      <c r="B55" s="5"/>
+      <c r="C55" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D54" s="19" t="s">
+      <c r="D55" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E54" s="19" t="s">
+      <c r="E55" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="F54" s="19" t="s">
+      <c r="F55" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="G54" s="17"/>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="7">
+      <c r="G55" s="17"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="7">
+        <v>46112</v>
+      </c>
+      <c r="B56" s="8"/>
+      <c r="C56" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="D56" s="10">
+        <v>321.39999999999998</v>
+      </c>
+      <c r="E56" s="10">
+        <v>247.21</v>
+      </c>
+      <c r="F56" s="10">
+        <v>257.20999999999998</v>
+      </c>
+      <c r="G56" s="17"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="11">
+        <v>46112</v>
+      </c>
+      <c r="B57" s="12"/>
+      <c r="C57" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="D57" s="13">
+        <v>314.05</v>
+      </c>
+      <c r="E57" s="13">
+        <v>245.33</v>
+      </c>
+      <c r="F57" s="13">
+        <v>255.33</v>
+      </c>
+      <c r="G57" s="17"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" s="7">
+        <v>46112</v>
+      </c>
+      <c r="B58" s="8"/>
+      <c r="C58" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D58" s="10">
+        <v>313.95</v>
+      </c>
+      <c r="E58" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F58" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="G58" s="17"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" s="11">
+        <v>46112</v>
+      </c>
+      <c r="B59" s="12"/>
+      <c r="C59" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="D59" s="13">
+        <v>313.39</v>
+      </c>
+      <c r="E59" s="13">
+        <v>239.71</v>
+      </c>
+      <c r="F59" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="G59" s="17"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="7">
+        <v>46112</v>
+      </c>
+      <c r="B60" s="8"/>
+      <c r="C60" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="D60" s="10">
+        <v>309.24</v>
+      </c>
+      <c r="E60" s="10">
+        <v>235.65</v>
+      </c>
+      <c r="F60" s="10">
+        <v>245.65</v>
+      </c>
+      <c r="G60" s="17"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" s="11">
+        <v>46112</v>
+      </c>
+      <c r="B61" s="12"/>
+      <c r="C61" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="D61" s="13">
+        <v>313.07</v>
+      </c>
+      <c r="E61" s="13">
+        <v>245</v>
+      </c>
+      <c r="F61" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="G61" s="17"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" s="7">
         <v>46109</v>
       </c>
-      <c r="B55" s="8"/>
-      <c r="C55" s="20" t="s">
+      <c r="B62" s="8"/>
+      <c r="C62" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="D55" s="10">
+      <c r="D62" s="10">
         <v>312.86</v>
       </c>
-      <c r="E55" s="10">
+      <c r="E62" s="10">
         <v>249.38</v>
       </c>
-      <c r="F55" s="10">
+      <c r="F62" s="10">
         <v>259.38</v>
       </c>
-      <c r="G55" s="17"/>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="11">
+      <c r="G62" s="17"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" s="11">
         <v>46109</v>
       </c>
-      <c r="B56" s="12"/>
-      <c r="C56" s="21" t="s">
+      <c r="B63" s="12"/>
+      <c r="C63" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="D56" s="13">
+      <c r="D63" s="13">
         <v>305.52999999999997</v>
       </c>
-      <c r="E56" s="13">
+      <c r="E63" s="13">
         <v>246.98</v>
       </c>
-      <c r="F56" s="13">
+      <c r="F63" s="13">
         <v>256.98</v>
       </c>
-      <c r="G56" s="17"/>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="7">
+      <c r="G63" s="17"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" s="7">
         <v>46109</v>
       </c>
-      <c r="B57" s="8"/>
-      <c r="C57" s="20" t="s">
+      <c r="B64" s="8"/>
+      <c r="C64" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="D57" s="10">
+      <c r="D64" s="10">
         <v>305.44</v>
       </c>
-      <c r="E57" s="10" t="s">
+      <c r="E64" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="F57" s="10" t="s">
+      <c r="F64" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="G57" s="17"/>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="11">
+      <c r="G64" s="17"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="11">
         <v>46109</v>
       </c>
-      <c r="B58" s="12"/>
-      <c r="C58" s="21" t="s">
+      <c r="B65" s="12"/>
+      <c r="C65" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="D58" s="13">
+      <c r="D65" s="13">
         <v>304.89999999999998</v>
       </c>
-      <c r="E58" s="13">
+      <c r="E65" s="13">
         <v>241.36</v>
       </c>
-      <c r="F58" s="13" t="s">
+      <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="G58" s="17"/>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" s="7">
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="7">
         <v>46109</v>
       </c>
-      <c r="B59" s="8"/>
-      <c r="C59" s="20" t="s">
+      <c r="B66" s="8"/>
+      <c r="C66" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="D59" s="10">
+      <c r="D66" s="10">
         <v>300.76</v>
       </c>
-      <c r="E59" s="10">
+      <c r="E66" s="10">
         <v>237.3</v>
       </c>
-      <c r="F59" s="10">
+      <c r="F66" s="10">
         <v>247.3</v>
       </c>
-      <c r="G59" s="17"/>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="11">
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="11">
         <v>46109</v>
       </c>
-      <c r="B60" s="12"/>
-      <c r="C60" s="21" t="s">
+      <c r="B67" s="12"/>
+      <c r="C67" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="D60" s="13">
+      <c r="D67" s="13">
         <v>304.58999999999997</v>
       </c>
-      <c r="E60" s="13">
+      <c r="E67" s="13">
         <v>246.64</v>
       </c>
-      <c r="F60" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="G60" s="17"/>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="7">
-        <v>46108</v>
-      </c>
-      <c r="B61" s="8"/>
-      <c r="C61" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="D61" s="10">
-        <v>311.52</v>
-      </c>
-      <c r="E61" s="10">
-        <v>252.9</v>
-      </c>
-      <c r="F61" s="10">
-        <v>262.89999999999998</v>
-      </c>
-      <c r="G61" s="17"/>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="11">
-        <v>46108</v>
-      </c>
-      <c r="B62" s="12"/>
-      <c r="C62" s="21" t="s">
-        <v>32</v>
-      </c>
-      <c r="D62" s="13">
-        <v>304.16000000000003</v>
-      </c>
-      <c r="E62" s="13">
-        <v>250.89</v>
-      </c>
-      <c r="F62" s="13">
-        <v>260.89</v>
-      </c>
-      <c r="G62" s="17"/>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="7">
-        <v>46108</v>
-      </c>
-      <c r="B63" s="8"/>
-      <c r="C63" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="D63" s="10">
-        <v>304.06</v>
-      </c>
-      <c r="E63" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="F63" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="G63" s="17"/>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" s="11">
-        <v>46108</v>
-      </c>
-      <c r="B64" s="12"/>
-      <c r="C64" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="D64" s="13">
-        <v>303.64</v>
-      </c>
-      <c r="E64" s="13">
-        <v>245.26</v>
-      </c>
-      <c r="F64" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="G64" s="17"/>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="7">
-        <v>46108</v>
-      </c>
-      <c r="B65" s="8"/>
-      <c r="C65" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="D65" s="10">
-        <v>299.49</v>
-      </c>
-      <c r="E65" s="10">
-        <v>241.21</v>
-      </c>
-      <c r="F65" s="10">
-        <v>251.21</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" s="11">
-        <v>46108</v>
-      </c>
-      <c r="B66" s="12"/>
-      <c r="C66" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="D66" s="13">
-        <v>303.32</v>
-      </c>
-      <c r="E66" s="13">
-        <v>250.31</v>
-      </c>
-      <c r="F66" s="13" t="s">
+      <c r="F67" s="13" t="s">
         <v>18</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A15:B15"/>

</xml_diff>

<commit_message>
Tue Mar 31 14:44:35 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="14_{4B60EC9E-6E37-4055-B12E-050B026604DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B96C2A63-C8ED-4D02-AC1D-9DF772E09555}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="14_{45EEE00A-3DB3-4BE4-8402-66AB4272954C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63382CFB-184C-461F-8F43-CCE4FF1D7937}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -110,6 +110,9 @@
     <t>Adelaide</t>
   </si>
   <si>
+    <t>Port Bonython</t>
+  </si>
+  <si>
     <t>Tasmania</t>
   </si>
   <si>
@@ -147,9 +150,6 @@
   </si>
   <si>
     <t>Port Hedland</t>
-  </si>
-  <si>
-    <t>Port Bonython</t>
   </si>
 </sst>
 </file>
@@ -304,7 +304,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -385,6 +385,8 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -713,7 +715,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
@@ -724,10 +726,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
+      <c r="B1" s="31"/>
       <c r="C1" s="1"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -775,10 +777,10 @@
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="28"/>
+      <c r="B6" s="30"/>
       <c r="C6" s="1"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -808,128 +810,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>307.79000000000002</v>
+        <v>287.11</v>
       </c>
       <c r="E8" s="10">
-        <v>231.83</v>
+        <v>203.23</v>
       </c>
       <c r="F8" s="10">
-        <v>241.83</v>
+        <v>213.23</v>
       </c>
       <c r="G8" s="10">
-        <v>231.72</v>
+        <v>203.5</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>307.79000000000002</v>
+        <v>287.11</v>
       </c>
       <c r="E9" s="13">
-        <v>231.83</v>
+        <v>203.23</v>
       </c>
       <c r="F9" s="13">
-        <v>241.83</v>
+        <v>213.23</v>
       </c>
       <c r="G9" s="13">
-        <v>231.72</v>
+        <v>203.5</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>308.61</v>
+        <v>287.79000000000002</v>
       </c>
       <c r="E10" s="10">
-        <v>234.4</v>
+        <v>203.47</v>
       </c>
       <c r="F10" s="10">
-        <v>244.4</v>
+        <v>213.47</v>
       </c>
       <c r="G10" s="10">
-        <v>234.64</v>
+        <v>204.46</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>299.23</v>
+        <v>307.79000000000002</v>
       </c>
       <c r="E11" s="13">
-        <v>233.43</v>
+        <v>231.83</v>
       </c>
       <c r="F11" s="13">
-        <v>243.43</v>
+        <v>241.83</v>
       </c>
       <c r="G11" s="13">
-        <v>233.32</v>
+        <v>231.72</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>299.23</v>
+        <v>307.79000000000002</v>
       </c>
       <c r="E12" s="10">
-        <v>233.43</v>
+        <v>231.83</v>
       </c>
       <c r="F12" s="10">
-        <v>243.43</v>
+        <v>241.83</v>
       </c>
       <c r="G12" s="10">
-        <v>233.32</v>
+        <v>231.72</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>300.10000000000002</v>
+        <v>308.61</v>
       </c>
       <c r="E13" s="13">
-        <v>236.06</v>
+        <v>234.4</v>
       </c>
       <c r="F13" s="13">
-        <v>246.06</v>
+        <v>244.4</v>
       </c>
       <c r="G13" s="13">
-        <v>236.3</v>
+        <v>234.64</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -942,10 +944,10 @@
       <c r="G14" s="16"/>
     </row>
     <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="28"/>
+      <c r="B15" s="30"/>
       <c r="C15" s="1"/>
       <c r="D15" s="17"/>
       <c r="E15" s="17"/>
@@ -971,45 +973,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>310.89</v>
+        <v>290.07</v>
       </c>
       <c r="E17" s="10">
-        <v>234.9</v>
+        <v>203.97</v>
       </c>
       <c r="F17" s="10">
-        <v>244.9</v>
+        <v>213.97</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>302.39</v>
+        <v>310.89</v>
       </c>
       <c r="E18" s="13">
-        <v>236.6</v>
+        <v>234.9</v>
       </c>
       <c r="F18" s="13">
-        <v>246.6</v>
+        <v>244.9</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1018,18 +1020,18 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A20" s="28" t="s">
+    <row r="20" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A20" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="28"/>
+      <c r="B20" s="30"/>
       <c r="C20" s="1"/>
       <c r="D20" s="17"/>
       <c r="E20" s="17"/>
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1050,217 +1052,232 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>307.55</v>
+        <v>286.86</v>
       </c>
       <c r="E22" s="10">
-        <v>232.83</v>
+        <v>202.03</v>
       </c>
       <c r="F22" s="10">
-        <v>242.43</v>
+        <v>211.63</v>
       </c>
       <c r="G22" s="10">
-        <v>234.58</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>201.49</v>
+      </c>
+      <c r="I22" s="29"/>
+      <c r="J22" s="29"/>
+      <c r="K22" s="29"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>310.35000000000002</v>
+        <v>286.24</v>
       </c>
       <c r="E23" s="13">
-        <v>239.99</v>
+        <v>209.05</v>
       </c>
       <c r="F23" s="13">
-        <v>249.99</v>
+        <v>219.05</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I23" s="29"/>
+      <c r="J23" s="29"/>
+      <c r="K23" s="29"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>310.42</v>
+        <v>286.3</v>
       </c>
       <c r="E24" s="10">
-        <v>240.72</v>
+        <v>209.79</v>
       </c>
       <c r="F24" s="10">
-        <v>250.72</v>
+        <v>219.79</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I24" s="29"/>
+      <c r="J24" s="29"/>
+      <c r="K24" s="29"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>310.38</v>
+        <v>286.26</v>
       </c>
       <c r="E25" s="13">
-        <v>240.45</v>
+        <v>209.5</v>
       </c>
       <c r="F25" s="13">
-        <v>250.45</v>
+        <v>219.51</v>
       </c>
       <c r="G25" s="13">
-        <v>241.3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>208.04</v>
+      </c>
+      <c r="I25" s="29"/>
+      <c r="J25" s="29"/>
+      <c r="K25" s="29"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>309.91000000000003</v>
+        <v>285.8</v>
       </c>
       <c r="E26" s="10">
-        <v>240.93</v>
+        <v>209.96</v>
       </c>
       <c r="F26" s="10">
-        <v>250.93</v>
+        <v>219.96</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I26" s="29"/>
+      <c r="J26" s="29"/>
+      <c r="K26" s="29"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>298.98</v>
+        <v>307.55</v>
       </c>
       <c r="E27" s="13">
-        <v>234.42</v>
+        <v>232.83</v>
       </c>
       <c r="F27" s="13">
-        <v>244.02</v>
+        <v>242.43</v>
       </c>
       <c r="G27" s="13">
-        <v>236.17</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>234.58</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>301.83999999999997</v>
+        <v>310.35000000000002</v>
       </c>
       <c r="E28" s="22">
-        <v>241.67</v>
+        <v>239.99</v>
       </c>
       <c r="F28" s="22">
-        <v>251.67</v>
+        <v>249.99</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>301.91000000000003</v>
+        <v>310.42</v>
       </c>
       <c r="E29" s="13">
-        <v>242.38</v>
+        <v>240.72</v>
       </c>
       <c r="F29" s="13">
-        <v>252.38</v>
+        <v>250.72</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>301.87</v>
+        <v>310.38</v>
       </c>
       <c r="E30" s="22">
-        <v>242.12</v>
+        <v>240.45</v>
       </c>
       <c r="F30" s="22">
-        <v>252.12</v>
+        <v>250.45</v>
       </c>
       <c r="G30" s="22">
-        <v>242.96</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>241.3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>301.39999999999998</v>
+        <v>309.91000000000003</v>
       </c>
       <c r="E31" s="13">
-        <v>242.63</v>
+        <v>240.93</v>
       </c>
       <c r="F31" s="13">
-        <v>252.63</v>
+        <v>250.93</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1269,18 +1286,18 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A33" s="28" t="s">
+    <row r="33" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A33" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="B33" s="28"/>
+      <c r="B33" s="30"/>
       <c r="C33" s="1"/>
       <c r="D33" s="17"/>
       <c r="E33" s="17"/>
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1299,54 +1316,57 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>306.39</v>
+        <v>285.56</v>
       </c>
       <c r="E35" s="10">
-        <v>234.95</v>
+        <v>204.02</v>
       </c>
       <c r="F35" s="10">
-        <v>243.95</v>
+        <v>213.02</v>
       </c>
       <c r="G35" s="17"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I35" s="29"/>
+      <c r="J35" s="29"/>
+      <c r="K35" s="29"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>297.89</v>
+        <v>306.39</v>
       </c>
       <c r="E36" s="13">
-        <v>236.6</v>
+        <v>234.95</v>
       </c>
       <c r="F36" s="13">
-        <v>245.6</v>
+        <v>243.95</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>322.01</v>
+        <v>301.18</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1355,17 +1375,18 @@
         <v>18</v>
       </c>
       <c r="G37" s="17"/>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I37" s="29"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>313.51</v>
+        <v>322.01</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1375,7 +1396,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1384,18 +1405,18 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A40" s="28" t="s">
-        <v>24</v>
-      </c>
-      <c r="B40" s="28"/>
+    <row r="40" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A40" s="30" t="s">
+        <v>25</v>
+      </c>
+      <c r="B40" s="30"/>
       <c r="C40" s="1"/>
       <c r="D40" s="17"/>
       <c r="E40" s="17"/>
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1414,83 +1435,89 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>313.73</v>
+        <v>292.89999999999998</v>
       </c>
       <c r="E42" s="10">
-        <v>242</v>
+        <v>212.25</v>
       </c>
       <c r="F42" s="10">
-        <v>252</v>
+        <v>222.25</v>
       </c>
       <c r="G42" s="17"/>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I42" s="29"/>
+      <c r="J42" s="29"/>
+      <c r="K42" s="29"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>313.29000000000002</v>
+        <v>292.47000000000003</v>
       </c>
       <c r="E43" s="13">
-        <v>242.41</v>
+        <v>212.66</v>
       </c>
       <c r="F43" s="13">
-        <v>252.41</v>
+        <v>222.66</v>
       </c>
       <c r="G43" s="17"/>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I43" s="29"/>
+      <c r="J43" s="29"/>
+      <c r="K43" s="29"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>305.20999999999998</v>
+        <v>313.73</v>
       </c>
       <c r="E44" s="10">
-        <v>241.93</v>
+        <v>242</v>
       </c>
       <c r="F44" s="10">
-        <v>251.93</v>
+        <v>252</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>304.77999999999997</v>
+        <v>313.29000000000002</v>
       </c>
       <c r="E45" s="13">
-        <v>242.34</v>
+        <v>242.41</v>
       </c>
       <c r="F45" s="13">
-        <v>252.34</v>
+        <v>252.41</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1499,9 +1526,9 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B47" s="26"/>
       <c r="C47" s="1"/>
@@ -1510,7 +1537,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1529,83 +1556,89 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>311.83</v>
+        <v>291.13</v>
       </c>
       <c r="E49" s="10">
-        <v>239.67</v>
+        <v>211.09</v>
       </c>
       <c r="F49" s="10">
-        <v>249.67</v>
-      </c>
-      <c r="G49" s="17"/>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+        <v>221.09</v>
+      </c>
+      <c r="G49" s="28"/>
+      <c r="I49" s="29"/>
+      <c r="J49" s="29"/>
+      <c r="K49" s="29"/>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>311.52</v>
+        <v>290.8</v>
       </c>
       <c r="E50" s="13">
-        <v>239.66</v>
+        <v>211.06</v>
       </c>
       <c r="F50" s="13">
-        <v>249.66</v>
-      </c>
-      <c r="G50" s="17"/>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+        <v>221.06</v>
+      </c>
+      <c r="G50" s="28"/>
+      <c r="I50" s="29"/>
+      <c r="J50" s="29"/>
+      <c r="K50" s="29"/>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>300.82</v>
+        <v>311.83</v>
       </c>
       <c r="E51" s="10">
-        <v>239.2</v>
+        <v>239.67</v>
       </c>
       <c r="F51" s="10">
-        <v>249.2</v>
+        <v>249.67</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>300.51</v>
+        <v>311.52</v>
       </c>
       <c r="E52" s="13">
-        <v>239.2</v>
+        <v>239.66</v>
       </c>
       <c r="F52" s="13">
-        <v>249.2</v>
+        <v>249.66</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1614,9 +1647,9 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B54" s="27"/>
       <c r="C54" s="1"/>
@@ -1625,7 +1658,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1644,54 +1677,60 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>321.39999999999998</v>
+        <v>300.61</v>
       </c>
       <c r="E56" s="10">
-        <v>247.21</v>
+        <v>216.22</v>
       </c>
       <c r="F56" s="10">
-        <v>257.20999999999998</v>
+        <v>226.22</v>
       </c>
       <c r="G56" s="17"/>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I56" s="29"/>
+      <c r="J56" s="29"/>
+      <c r="K56" s="29"/>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>314.05</v>
+        <v>293.23</v>
       </c>
       <c r="E57" s="13">
-        <v>245.33</v>
+        <v>214.42</v>
       </c>
       <c r="F57" s="13">
-        <v>255.33</v>
+        <v>224.42</v>
       </c>
       <c r="G57" s="17"/>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I57" s="29"/>
+      <c r="J57" s="29"/>
+      <c r="K57" s="29"/>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>313.95</v>
+        <v>293.12</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1700,112 +1739,124 @@
         <v>18</v>
       </c>
       <c r="G58" s="17"/>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I58" s="29"/>
+      <c r="J58" s="29"/>
+      <c r="K58" s="29"/>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>313.39</v>
+        <v>292.57</v>
       </c>
       <c r="E59" s="13">
-        <v>239.71</v>
+        <v>208.81</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I59" s="29"/>
+      <c r="J59" s="29"/>
+      <c r="K59" s="29"/>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>309.24</v>
+        <v>288.43</v>
       </c>
       <c r="E60" s="10">
-        <v>235.65</v>
+        <v>204.74</v>
       </c>
       <c r="F60" s="10">
-        <v>245.65</v>
+        <v>214.74</v>
       </c>
       <c r="G60" s="17"/>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I60" s="29"/>
+      <c r="J60" s="29"/>
+      <c r="K60" s="29"/>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>313.07</v>
+        <v>292.26</v>
       </c>
       <c r="E61" s="13">
-        <v>245</v>
+        <v>214.04</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I61" s="29"/>
+      <c r="J61" s="29"/>
+      <c r="K61" s="29"/>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>312.86</v>
+        <v>321.39999999999998</v>
       </c>
       <c r="E62" s="10">
-        <v>249.38</v>
+        <v>247.21</v>
       </c>
       <c r="F62" s="10">
-        <v>259.38</v>
+        <v>257.20999999999998</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>305.52999999999997</v>
+        <v>314.05</v>
       </c>
       <c r="E63" s="13">
-        <v>246.98</v>
+        <v>245.33</v>
       </c>
       <c r="F63" s="13">
-        <v>256.98</v>
+        <v>255.33</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>305.44</v>
+        <v>313.95</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1817,17 +1868,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>304.89999999999998</v>
+        <v>313.39</v>
       </c>
       <c r="E65" s="13">
-        <v>241.36</v>
+        <v>239.71</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1835,35 +1886,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>300.76</v>
+        <v>309.24</v>
       </c>
       <c r="E66" s="10">
-        <v>237.3</v>
+        <v>235.65</v>
       </c>
       <c r="F66" s="10">
-        <v>247.3</v>
+        <v>245.65</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46109</v>
+        <v>46112</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>304.58999999999997</v>
+        <v>313.07</v>
       </c>
       <c r="E67" s="13">
-        <v>246.64</v>
+        <v>245</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -2151,15 +2202,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -2168,6 +2210,15 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2191,27 +2242,20 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Wed Apr  1 04:23:19 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="14_{45EEE00A-3DB3-4BE4-8402-66AB4272954C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63382CFB-184C-461F-8F43-CCE4FF1D7937}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{2AF9C2A8-0802-42A5-9565-D9B7F5003719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -304,7 +304,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -386,7 +386,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -715,7 +714,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K67"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
@@ -726,10 +725,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
+      <c r="B1" s="30"/>
       <c r="C1" s="1"/>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -777,10 +776,10 @@
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="30"/>
+      <c r="B6" s="29"/>
       <c r="C6" s="1"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
@@ -810,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>287.11</v>
+        <v>294.08</v>
       </c>
       <c r="E8" s="10">
-        <v>203.23</v>
+        <v>203.78</v>
       </c>
       <c r="F8" s="10">
-        <v>213.23</v>
+        <v>213.78</v>
       </c>
       <c r="G8" s="10">
-        <v>203.5</v>
+        <v>204.05</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>287.11</v>
+        <v>294.08</v>
       </c>
       <c r="E9" s="13">
-        <v>203.23</v>
+        <v>203.78</v>
       </c>
       <c r="F9" s="13">
-        <v>213.23</v>
+        <v>213.78</v>
       </c>
       <c r="G9" s="13">
-        <v>203.5</v>
+        <v>204.05</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>287.79000000000002</v>
+        <v>293.51</v>
       </c>
       <c r="E10" s="10">
-        <v>203.47</v>
+        <v>203.88</v>
       </c>
       <c r="F10" s="10">
-        <v>213.47</v>
+        <v>213.88</v>
       </c>
       <c r="G10" s="10">
-        <v>204.46</v>
+        <v>204.87</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>307.79000000000002</v>
+        <v>287.11</v>
       </c>
       <c r="E11" s="13">
-        <v>231.83</v>
+        <v>203.23</v>
       </c>
       <c r="F11" s="13">
-        <v>241.83</v>
+        <v>213.23</v>
       </c>
       <c r="G11" s="13">
-        <v>231.72</v>
+        <v>203.5</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>307.79000000000002</v>
+        <v>287.11</v>
       </c>
       <c r="E12" s="10">
-        <v>231.83</v>
+        <v>203.23</v>
       </c>
       <c r="F12" s="10">
-        <v>241.83</v>
+        <v>213.23</v>
       </c>
       <c r="G12" s="10">
-        <v>231.72</v>
+        <v>203.5</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>308.61</v>
+        <v>287.79000000000002</v>
       </c>
       <c r="E13" s="13">
-        <v>234.4</v>
+        <v>203.47</v>
       </c>
       <c r="F13" s="13">
-        <v>244.4</v>
+        <v>213.47</v>
       </c>
       <c r="G13" s="13">
-        <v>234.64</v>
+        <v>204.46</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -944,10 +943,10 @@
       <c r="G14" s="16"/>
     </row>
     <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A15" s="30" t="s">
+      <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="30"/>
+      <c r="B15" s="29"/>
       <c r="C15" s="1"/>
       <c r="D15" s="17"/>
       <c r="E15" s="17"/>
@@ -973,45 +972,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>290.07</v>
+        <v>294.69</v>
       </c>
       <c r="E17" s="10">
-        <v>203.97</v>
+        <v>204.37</v>
       </c>
       <c r="F17" s="10">
-        <v>213.97</v>
+        <v>214.37</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>310.89</v>
+        <v>290.07</v>
       </c>
       <c r="E18" s="13">
-        <v>234.9</v>
+        <v>203.97</v>
       </c>
       <c r="F18" s="13">
-        <v>244.9</v>
+        <v>213.97</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1020,18 +1019,18 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A20" s="30" t="s">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="30"/>
+      <c r="B20" s="29"/>
       <c r="C20" s="1"/>
       <c r="D20" s="17"/>
       <c r="E20" s="17"/>
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1052,232 +1051,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>286.86</v>
+        <v>292.73</v>
       </c>
       <c r="E22" s="10">
-        <v>202.03</v>
+        <v>202.58</v>
       </c>
       <c r="F22" s="10">
-        <v>211.63</v>
+        <v>212.18</v>
       </c>
       <c r="G22" s="10">
-        <v>201.49</v>
-      </c>
-      <c r="I22" s="29"/>
-      <c r="J22" s="29"/>
-      <c r="K22" s="29"/>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+        <v>202.04</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>286.24</v>
+        <v>294.16000000000003</v>
       </c>
       <c r="E23" s="13">
-        <v>209.05</v>
+        <v>209.46</v>
       </c>
       <c r="F23" s="13">
-        <v>219.05</v>
+        <v>219.46</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="I23" s="29"/>
-      <c r="J23" s="29"/>
-      <c r="K23" s="29"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>286.3</v>
+        <v>294.22000000000003</v>
       </c>
       <c r="E24" s="10">
-        <v>209.79</v>
+        <v>210.2</v>
       </c>
       <c r="F24" s="10">
-        <v>219.79</v>
+        <v>220.2</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I24" s="29"/>
-      <c r="J24" s="29"/>
-      <c r="K24" s="29"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>286.26</v>
+        <v>294.18</v>
       </c>
       <c r="E25" s="13">
-        <v>209.5</v>
+        <v>209.92</v>
       </c>
       <c r="F25" s="13">
-        <v>219.51</v>
+        <v>219.92</v>
       </c>
       <c r="G25" s="13">
-        <v>208.04</v>
-      </c>
-      <c r="I25" s="29"/>
-      <c r="J25" s="29"/>
-      <c r="K25" s="29"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+        <v>208.45</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>285.8</v>
+        <v>293.72000000000003</v>
       </c>
       <c r="E26" s="10">
-        <v>209.96</v>
+        <v>210.37</v>
       </c>
       <c r="F26" s="10">
-        <v>219.96</v>
+        <v>220.37</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="I26" s="29"/>
-      <c r="J26" s="29"/>
-      <c r="K26" s="29"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>307.55</v>
+        <v>286.86</v>
       </c>
       <c r="E27" s="13">
-        <v>232.83</v>
+        <v>202.03</v>
       </c>
       <c r="F27" s="13">
-        <v>242.43</v>
+        <v>211.63</v>
       </c>
       <c r="G27" s="13">
-        <v>234.58</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+        <v>201.49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>310.35000000000002</v>
+        <v>286.24</v>
       </c>
       <c r="E28" s="22">
-        <v>239.99</v>
+        <v>209.05</v>
       </c>
       <c r="F28" s="22">
-        <v>249.99</v>
+        <v>219.05</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>310.42</v>
+        <v>286.3</v>
       </c>
       <c r="E29" s="13">
-        <v>240.72</v>
+        <v>209.79</v>
       </c>
       <c r="F29" s="13">
-        <v>250.72</v>
+        <v>219.79</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>310.38</v>
+        <v>286.26</v>
       </c>
       <c r="E30" s="22">
-        <v>240.45</v>
+        <v>209.5</v>
       </c>
       <c r="F30" s="22">
-        <v>250.45</v>
+        <v>219.51</v>
       </c>
       <c r="G30" s="22">
-        <v>241.3</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+        <v>208.04</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>309.91000000000003</v>
+        <v>285.8</v>
       </c>
       <c r="E31" s="13">
-        <v>240.93</v>
+        <v>209.96</v>
       </c>
       <c r="F31" s="13">
-        <v>250.93</v>
+        <v>219.96</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1286,18 +1270,18 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A33" s="30" t="s">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="B33" s="30"/>
+      <c r="B33" s="29"/>
       <c r="C33" s="1"/>
       <c r="D33" s="17"/>
       <c r="E33" s="17"/>
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1316,57 +1300,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>285.56</v>
+        <v>292.37</v>
       </c>
       <c r="E35" s="10">
-        <v>204.02</v>
+        <v>204.43</v>
       </c>
       <c r="F35" s="10">
-        <v>213.02</v>
+        <v>213.43</v>
       </c>
       <c r="G35" s="17"/>
-      <c r="I35" s="29"/>
-      <c r="J35" s="29"/>
-      <c r="K35" s="29"/>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>306.39</v>
+        <v>285.56</v>
       </c>
       <c r="E36" s="13">
-        <v>234.95</v>
+        <v>204.02</v>
       </c>
       <c r="F36" s="13">
-        <v>243.95</v>
+        <v>213.02</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>301.18</v>
+        <v>307.99</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1375,18 +1356,17 @@
         <v>18</v>
       </c>
       <c r="G37" s="17"/>
-      <c r="I37" s="29"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>322.01</v>
+        <v>301.18</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1396,7 +1376,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1405,18 +1385,18 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A40" s="30" t="s">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="B40" s="30"/>
+      <c r="B40" s="29"/>
       <c r="C40" s="1"/>
       <c r="D40" s="17"/>
       <c r="E40" s="17"/>
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1435,89 +1415,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>292.89999999999998</v>
+        <v>297.52999999999997</v>
       </c>
       <c r="E42" s="10">
-        <v>212.25</v>
+        <v>212.09</v>
       </c>
       <c r="F42" s="10">
-        <v>222.25</v>
+        <v>222.09</v>
       </c>
       <c r="G42" s="17"/>
-      <c r="I42" s="29"/>
-      <c r="J42" s="29"/>
-      <c r="K42" s="29"/>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>292.47000000000003</v>
+        <v>297.08999999999997</v>
       </c>
       <c r="E43" s="13">
-        <v>212.66</v>
+        <v>212.5</v>
       </c>
       <c r="F43" s="13">
-        <v>222.66</v>
+        <v>222.5</v>
       </c>
       <c r="G43" s="17"/>
-      <c r="I43" s="29"/>
-      <c r="J43" s="29"/>
-      <c r="K43" s="29"/>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>313.73</v>
+        <v>292.89999999999998</v>
       </c>
       <c r="E44" s="10">
-        <v>242</v>
+        <v>212.25</v>
       </c>
       <c r="F44" s="10">
-        <v>252</v>
+        <v>222.25</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>313.29000000000002</v>
+        <v>292.47000000000003</v>
       </c>
       <c r="E45" s="13">
-        <v>242.41</v>
+        <v>212.66</v>
       </c>
       <c r="F45" s="13">
-        <v>252.41</v>
+        <v>222.66</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1526,7 +1500,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1537,7 +1511,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1556,89 +1530,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>291.13</v>
+        <v>294.60000000000002</v>
       </c>
       <c r="E49" s="10">
-        <v>211.09</v>
+        <v>209.32</v>
       </c>
       <c r="F49" s="10">
-        <v>221.09</v>
+        <v>219.32</v>
       </c>
       <c r="G49" s="28"/>
-      <c r="I49" s="29"/>
-      <c r="J49" s="29"/>
-      <c r="K49" s="29"/>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>290.8</v>
+        <v>294.27</v>
       </c>
       <c r="E50" s="13">
-        <v>211.06</v>
+        <v>209.28</v>
       </c>
       <c r="F50" s="13">
-        <v>221.06</v>
+        <v>219.28</v>
       </c>
       <c r="G50" s="28"/>
-      <c r="I50" s="29"/>
-      <c r="J50" s="29"/>
-      <c r="K50" s="29"/>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>311.83</v>
+        <v>291.13</v>
       </c>
       <c r="E51" s="10">
-        <v>239.67</v>
+        <v>211.09</v>
       </c>
       <c r="F51" s="10">
-        <v>249.67</v>
+        <v>221.09</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>311.52</v>
+        <v>290.8</v>
       </c>
       <c r="E52" s="13">
-        <v>239.66</v>
+        <v>211.06</v>
       </c>
       <c r="F52" s="13">
-        <v>249.66</v>
+        <v>221.06</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1647,7 +1615,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1658,7 +1626,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1677,60 +1645,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>300.61</v>
+        <v>305.26</v>
       </c>
       <c r="E56" s="10">
-        <v>216.22</v>
+        <v>216.64</v>
       </c>
       <c r="F56" s="10">
-        <v>226.22</v>
+        <v>226.64</v>
       </c>
       <c r="G56" s="17"/>
-      <c r="I56" s="29"/>
-      <c r="J56" s="29"/>
-      <c r="K56" s="29"/>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>293.23</v>
+        <v>297.87</v>
       </c>
       <c r="E57" s="13">
-        <v>214.42</v>
+        <v>214.83</v>
       </c>
       <c r="F57" s="13">
-        <v>224.42</v>
+        <v>224.83</v>
       </c>
       <c r="G57" s="17"/>
-      <c r="I57" s="29"/>
-      <c r="J57" s="29"/>
-      <c r="K57" s="29"/>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>293.12</v>
+        <v>297.74</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1739,124 +1701,112 @@
         <v>18</v>
       </c>
       <c r="G58" s="17"/>
-      <c r="I58" s="29"/>
-      <c r="J58" s="29"/>
-      <c r="K58" s="29"/>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>292.57</v>
+        <v>297.17</v>
       </c>
       <c r="E59" s="13">
-        <v>208.81</v>
+        <v>209.21</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
-      <c r="I59" s="29"/>
-      <c r="J59" s="29"/>
-      <c r="K59" s="29"/>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>288.43</v>
+        <v>293.04000000000002</v>
       </c>
       <c r="E60" s="10">
-        <v>204.74</v>
+        <v>205.15</v>
       </c>
       <c r="F60" s="10">
-        <v>214.74</v>
+        <v>215.15</v>
       </c>
       <c r="G60" s="17"/>
-      <c r="I60" s="29"/>
-      <c r="J60" s="29"/>
-      <c r="K60" s="29"/>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>292.26</v>
+        <v>296.87</v>
       </c>
       <c r="E61" s="13">
-        <v>214.04</v>
+        <v>214.45</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
-      <c r="I61" s="29"/>
-      <c r="J61" s="29"/>
-      <c r="K61" s="29"/>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>321.39999999999998</v>
+        <v>300.61</v>
       </c>
       <c r="E62" s="10">
-        <v>247.21</v>
+        <v>216.22</v>
       </c>
       <c r="F62" s="10">
-        <v>257.20999999999998</v>
+        <v>226.22</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>314.05</v>
+        <v>293.23</v>
       </c>
       <c r="E63" s="13">
-        <v>245.33</v>
+        <v>214.42</v>
       </c>
       <c r="F63" s="13">
-        <v>255.33</v>
+        <v>224.42</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>313.95</v>
+        <v>293.12</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1868,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>313.39</v>
+        <v>292.57</v>
       </c>
       <c r="E65" s="13">
-        <v>239.71</v>
+        <v>208.81</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1886,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>309.24</v>
+        <v>288.43</v>
       </c>
       <c r="E66" s="10">
-        <v>235.65</v>
+        <v>204.74</v>
       </c>
       <c r="F66" s="10">
-        <v>245.65</v>
+        <v>214.74</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>313.07</v>
+        <v>292.26</v>
       </c>
       <c r="E67" s="13">
-        <v>245</v>
+        <v>214.04</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1942,6 +1892,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2201,17 +2162,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2222,6 +2172,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2241,17 +2202,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Thu Apr  2 04:01:52 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{2AF9C2A8-0802-42A5-9565-D9B7F5003719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{182D821F-18DF-45ED-A3A4-169C74CA9CBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>294.08</v>
+        <v>300.79000000000002</v>
       </c>
       <c r="E8" s="10">
-        <v>203.78</v>
+        <v>205.91</v>
       </c>
       <c r="F8" s="10">
-        <v>213.78</v>
+        <v>215.91</v>
       </c>
       <c r="G8" s="10">
-        <v>204.05</v>
+        <v>206.18</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>294.08</v>
+        <v>300.79000000000002</v>
       </c>
       <c r="E9" s="13">
-        <v>203.78</v>
+        <v>205.91</v>
       </c>
       <c r="F9" s="13">
-        <v>213.78</v>
+        <v>215.91</v>
       </c>
       <c r="G9" s="13">
-        <v>204.05</v>
+        <v>206.18</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>293.51</v>
+        <v>299.99</v>
       </c>
       <c r="E10" s="10">
-        <v>203.88</v>
+        <v>205.8</v>
       </c>
       <c r="F10" s="10">
-        <v>213.88</v>
+        <v>215.8</v>
       </c>
       <c r="G10" s="10">
-        <v>204.87</v>
+        <v>206.79</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>287.11</v>
+        <v>294.08</v>
       </c>
       <c r="E11" s="13">
-        <v>203.23</v>
+        <v>203.78</v>
       </c>
       <c r="F11" s="13">
-        <v>213.23</v>
+        <v>213.78</v>
       </c>
       <c r="G11" s="13">
-        <v>203.5</v>
+        <v>204.05</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>287.11</v>
+        <v>294.08</v>
       </c>
       <c r="E12" s="10">
-        <v>203.23</v>
+        <v>203.78</v>
       </c>
       <c r="F12" s="10">
-        <v>213.23</v>
+        <v>213.78</v>
       </c>
       <c r="G12" s="10">
-        <v>203.5</v>
+        <v>204.05</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>287.79000000000002</v>
+        <v>293.51</v>
       </c>
       <c r="E13" s="13">
-        <v>203.47</v>
+        <v>203.88</v>
       </c>
       <c r="F13" s="13">
-        <v>213.47</v>
+        <v>213.88</v>
       </c>
       <c r="G13" s="13">
-        <v>204.46</v>
+        <v>204.87</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>294.69</v>
+        <v>303.33999999999997</v>
       </c>
       <c r="E17" s="10">
-        <v>204.37</v>
+        <v>206.27</v>
       </c>
       <c r="F17" s="10">
-        <v>214.37</v>
+        <v>216.27</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>290.07</v>
+        <v>294.69</v>
       </c>
       <c r="E18" s="13">
-        <v>203.97</v>
+        <v>204.37</v>
       </c>
       <c r="F18" s="13">
-        <v>213.97</v>
+        <v>214.37</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>292.73</v>
+        <v>299.44</v>
       </c>
       <c r="E22" s="10">
-        <v>202.58</v>
+        <v>204.7</v>
       </c>
       <c r="F22" s="10">
-        <v>212.18</v>
+        <v>214.3</v>
       </c>
       <c r="G22" s="10">
-        <v>202.04</v>
+        <v>204.17</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>294.16000000000003</v>
+        <v>300.64</v>
       </c>
       <c r="E23" s="13">
-        <v>209.46</v>
+        <v>211.38</v>
       </c>
       <c r="F23" s="13">
-        <v>219.46</v>
+        <v>221.38</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>294.22000000000003</v>
+        <v>300.7</v>
       </c>
       <c r="E24" s="10">
-        <v>210.2</v>
+        <v>212.13</v>
       </c>
       <c r="F24" s="10">
-        <v>220.2</v>
+        <v>222.13</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>294.18</v>
+        <v>300.64999999999998</v>
       </c>
       <c r="E25" s="13">
-        <v>209.92</v>
+        <v>211.85</v>
       </c>
       <c r="F25" s="13">
-        <v>219.92</v>
+        <v>221.85</v>
       </c>
       <c r="G25" s="13">
-        <v>208.45</v>
+        <v>210.38</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>293.72000000000003</v>
+        <v>301.3</v>
       </c>
       <c r="E26" s="10">
-        <v>210.37</v>
+        <v>212.32</v>
       </c>
       <c r="F26" s="10">
-        <v>220.37</v>
+        <v>222.32</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>286.86</v>
+        <v>292.73</v>
       </c>
       <c r="E27" s="13">
-        <v>202.03</v>
+        <v>202.58</v>
       </c>
       <c r="F27" s="13">
-        <v>211.63</v>
+        <v>212.18</v>
       </c>
       <c r="G27" s="13">
-        <v>201.49</v>
+        <v>202.04</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>286.24</v>
+        <v>294.16000000000003</v>
       </c>
       <c r="E28" s="22">
-        <v>209.05</v>
+        <v>209.46</v>
       </c>
       <c r="F28" s="22">
-        <v>219.05</v>
+        <v>219.46</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>286.3</v>
+        <v>294.22000000000003</v>
       </c>
       <c r="E29" s="13">
-        <v>209.79</v>
+        <v>210.2</v>
       </c>
       <c r="F29" s="13">
-        <v>219.79</v>
+        <v>220.2</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>286.26</v>
+        <v>294.18</v>
       </c>
       <c r="E30" s="22">
-        <v>209.5</v>
+        <v>209.92</v>
       </c>
       <c r="F30" s="22">
-        <v>219.51</v>
+        <v>219.92</v>
       </c>
       <c r="G30" s="22">
-        <v>208.04</v>
+        <v>208.45</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>285.8</v>
+        <v>293.72000000000003</v>
       </c>
       <c r="E31" s="13">
-        <v>209.96</v>
+        <v>210.37</v>
       </c>
       <c r="F31" s="13">
-        <v>219.96</v>
+        <v>220.37</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>292.37</v>
+        <v>298.85000000000002</v>
       </c>
       <c r="E35" s="10">
-        <v>204.43</v>
+        <v>206.34</v>
       </c>
       <c r="F35" s="10">
-        <v>213.43</v>
+        <v>215.34</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>285.56</v>
+        <v>292.37</v>
       </c>
       <c r="E36" s="13">
-        <v>204.02</v>
+        <v>204.43</v>
       </c>
       <c r="F36" s="13">
-        <v>213.02</v>
+        <v>213.43</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>307.99</v>
+        <v>314.47000000000003</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>301.18</v>
+        <v>307.99</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>297.52999999999997</v>
+        <v>304.04000000000002</v>
       </c>
       <c r="E42" s="10">
-        <v>212.09</v>
+        <v>213.47</v>
       </c>
       <c r="F42" s="10">
-        <v>222.09</v>
+        <v>223.47</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>297.08999999999997</v>
+        <v>303.58999999999997</v>
       </c>
       <c r="E43" s="13">
-        <v>212.5</v>
+        <v>213.89</v>
       </c>
       <c r="F43" s="13">
-        <v>222.5</v>
+        <v>223.89</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>292.89999999999998</v>
+        <v>297.52999999999997</v>
       </c>
       <c r="E44" s="10">
-        <v>212.25</v>
+        <v>212.09</v>
       </c>
       <c r="F44" s="10">
-        <v>222.25</v>
+        <v>222.09</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>292.47000000000003</v>
+        <v>297.08999999999997</v>
       </c>
       <c r="E45" s="13">
-        <v>212.66</v>
+        <v>212.5</v>
       </c>
       <c r="F45" s="13">
-        <v>222.66</v>
+        <v>222.5</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>294.60000000000002</v>
+        <v>295.43</v>
       </c>
       <c r="E49" s="10">
-        <v>209.32</v>
+        <v>205.68</v>
       </c>
       <c r="F49" s="10">
-        <v>219.32</v>
+        <v>215.68</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>294.27</v>
+        <v>295.10000000000002</v>
       </c>
       <c r="E50" s="13">
-        <v>209.28</v>
+        <v>205.63</v>
       </c>
       <c r="F50" s="13">
-        <v>219.28</v>
+        <v>215.63</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>291.13</v>
+        <v>294.60000000000002</v>
       </c>
       <c r="E51" s="10">
-        <v>211.09</v>
+        <v>209.32</v>
       </c>
       <c r="F51" s="10">
-        <v>221.09</v>
+        <v>219.32</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>290.8</v>
+        <v>294.27</v>
       </c>
       <c r="E52" s="13">
-        <v>211.06</v>
+        <v>209.28</v>
       </c>
       <c r="F52" s="13">
-        <v>221.06</v>
+        <v>219.28</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>305.26</v>
+        <v>313.95999999999998</v>
       </c>
       <c r="E56" s="10">
-        <v>216.64</v>
+        <v>218.66</v>
       </c>
       <c r="F56" s="10">
-        <v>226.64</v>
+        <v>228.66</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>297.87</v>
+        <v>306.55</v>
       </c>
       <c r="E57" s="13">
-        <v>214.83</v>
+        <v>216.71</v>
       </c>
       <c r="F57" s="13">
-        <v>224.83</v>
+        <v>226.71</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>297.74</v>
+        <v>306.42</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>297.17</v>
+        <v>305.8</v>
       </c>
       <c r="E59" s="13">
-        <v>209.21</v>
+        <v>211.09</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>293.04000000000002</v>
+        <v>301.66000000000003</v>
       </c>
       <c r="E60" s="10">
-        <v>205.15</v>
+        <v>207.03</v>
       </c>
       <c r="F60" s="10">
-        <v>215.15</v>
+        <v>217.03</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>296.87</v>
+        <v>305.51</v>
       </c>
       <c r="E61" s="13">
-        <v>214.45</v>
+        <v>216.44</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>300.61</v>
+        <v>305.26</v>
       </c>
       <c r="E62" s="10">
-        <v>216.22</v>
+        <v>216.64</v>
       </c>
       <c r="F62" s="10">
-        <v>226.22</v>
+        <v>226.64</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>293.23</v>
+        <v>297.87</v>
       </c>
       <c r="E63" s="13">
-        <v>214.42</v>
+        <v>214.83</v>
       </c>
       <c r="F63" s="13">
-        <v>224.42</v>
+        <v>224.83</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>293.12</v>
+        <v>297.74</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>292.57</v>
+        <v>297.17</v>
       </c>
       <c r="E65" s="13">
-        <v>208.81</v>
+        <v>209.21</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>288.43</v>
+        <v>293.04000000000002</v>
       </c>
       <c r="E66" s="10">
-        <v>204.74</v>
+        <v>205.15</v>
       </c>
       <c r="F66" s="10">
-        <v>214.74</v>
+        <v>215.15</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>292.26</v>
+        <v>296.87</v>
       </c>
       <c r="E67" s="13">
-        <v>214.04</v>
+        <v>214.45</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,17 +1892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2162,6 +2151,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2172,17 +2172,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2202,6 +2191,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Fri Apr  3 04:03:15 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{182D821F-18DF-45ED-A3A4-169C74CA9CBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{D162356C-1C79-46E3-B1F9-1F506698CC49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="9435" yWindow="-16320" windowWidth="38640" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,16 +715,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125"/>
-    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.3984375"/>
+    <col min="3" max="3" width="18.265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.86328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="6.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -735,7 +735,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -744,7 +744,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -755,7 +755,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -766,7 +766,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -775,7 +775,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -786,7 +786,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -807,7 +807,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
         <v>46115</v>
       </c>
@@ -816,19 +816,19 @@
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>300.79000000000002</v>
+        <v>294.52</v>
       </c>
       <c r="E8" s="10">
-        <v>205.91</v>
+        <v>199.64</v>
       </c>
       <c r="F8" s="10">
-        <v>215.91</v>
+        <v>209.64</v>
       </c>
       <c r="G8" s="10">
-        <v>206.18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>200.31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="11">
         <v>46115</v>
       </c>
@@ -837,19 +837,19 @@
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>300.79000000000002</v>
+        <v>294.52</v>
       </c>
       <c r="E9" s="13">
-        <v>205.91</v>
+        <v>199.64</v>
       </c>
       <c r="F9" s="13">
-        <v>215.91</v>
+        <v>209.64</v>
       </c>
       <c r="G9" s="13">
-        <v>206.18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>200.31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
         <v>46115</v>
       </c>
@@ -858,19 +858,19 @@
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>299.99</v>
+        <v>293.72000000000003</v>
       </c>
       <c r="E10" s="10">
-        <v>205.8</v>
+        <v>199.53</v>
       </c>
       <c r="F10" s="10">
-        <v>215.8</v>
+        <v>209.53</v>
       </c>
       <c r="G10" s="10">
-        <v>206.79</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>200.92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" s="11">
         <v>46114</v>
       </c>
@@ -891,7 +891,7 @@
         <v>204.05</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
         <v>46114</v>
       </c>
@@ -912,7 +912,7 @@
         <v>204.05</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" s="11">
         <v>46114</v>
       </c>
@@ -933,7 +933,7 @@
         <v>204.87</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -942,7 +942,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -953,7 +953,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -972,7 +972,7 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
         <v>46115</v>
       </c>
@@ -981,17 +981,17 @@
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>303.33999999999997</v>
+        <v>297.07</v>
       </c>
       <c r="E17" s="10">
-        <v>206.27</v>
+        <v>200</v>
       </c>
       <c r="F17" s="10">
-        <v>216.27</v>
+        <v>210</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="11">
         <v>46114</v>
       </c>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1019,7 +1019,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1030,7 +1030,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1051,7 +1051,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="7">
         <v>46115</v>
       </c>
@@ -1060,19 +1060,19 @@
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>299.44</v>
+        <v>293.17</v>
       </c>
       <c r="E22" s="10">
-        <v>204.7</v>
+        <v>198.43</v>
       </c>
       <c r="F22" s="10">
-        <v>214.3</v>
+        <v>208.03</v>
       </c>
       <c r="G22" s="10">
-        <v>204.17</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>197.9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="11">
         <v>46115</v>
       </c>
@@ -1081,19 +1081,19 @@
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>300.64</v>
+        <v>294.37</v>
       </c>
       <c r="E23" s="13">
-        <v>211.38</v>
+        <v>205.11</v>
       </c>
       <c r="F23" s="13">
-        <v>221.38</v>
+        <v>215.11</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="7">
         <v>46115</v>
       </c>
@@ -1102,19 +1102,19 @@
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>300.7</v>
+        <v>294.43</v>
       </c>
       <c r="E24" s="10">
-        <v>212.13</v>
+        <v>205.86</v>
       </c>
       <c r="F24" s="10">
-        <v>222.13</v>
+        <v>215.86</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="11">
         <v>46115</v>
       </c>
@@ -1123,19 +1123,19 @@
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>300.64999999999998</v>
+        <v>294.38</v>
       </c>
       <c r="E25" s="13">
-        <v>211.85</v>
+        <v>205.58</v>
       </c>
       <c r="F25" s="13">
-        <v>221.85</v>
+        <v>215.58</v>
       </c>
       <c r="G25" s="13">
-        <v>210.38</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>204.11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="7">
         <v>46115</v>
       </c>
@@ -1144,19 +1144,19 @@
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>301.3</v>
+        <v>295.02999999999997</v>
       </c>
       <c r="E26" s="10">
-        <v>212.32</v>
+        <v>206.05</v>
       </c>
       <c r="F26" s="10">
-        <v>222.32</v>
+        <v>216.05</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="11">
         <v>46114</v>
       </c>
@@ -1177,7 +1177,7 @@
         <v>202.04</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="7">
         <v>46114</v>
       </c>
@@ -1198,7 +1198,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="11">
         <v>46114</v>
       </c>
@@ -1219,7 +1219,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" s="7">
         <v>46114</v>
       </c>
@@ -1240,7 +1240,7 @@
         <v>208.45</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="11">
         <v>46114</v>
       </c>
@@ -1261,7 +1261,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1270,7 +1270,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1281,7 +1281,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="7">
         <v>46115</v>
       </c>
@@ -1309,17 +1309,17 @@
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>298.85000000000002</v>
+        <v>292.58</v>
       </c>
       <c r="E35" s="10">
-        <v>206.34</v>
+        <v>200.07</v>
       </c>
       <c r="F35" s="10">
-        <v>215.34</v>
+        <v>209.07</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="11">
         <v>46114</v>
       </c>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="7">
         <v>46115</v>
       </c>
@@ -1347,7 +1347,7 @@
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>314.47000000000003</v>
+        <v>308.2</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="11">
         <v>46114</v>
       </c>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1385,7 +1385,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1396,7 +1396,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="7">
         <v>46115</v>
       </c>
@@ -1424,17 +1424,17 @@
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>304.04000000000002</v>
+        <v>297.77</v>
       </c>
       <c r="E42" s="10">
-        <v>213.47</v>
+        <v>207.2</v>
       </c>
       <c r="F42" s="10">
-        <v>223.47</v>
+        <v>217.2</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" s="11">
         <v>46115</v>
       </c>
@@ -1443,17 +1443,17 @@
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>303.58999999999997</v>
+        <v>297.32</v>
       </c>
       <c r="E43" s="13">
-        <v>213.89</v>
+        <v>207.62</v>
       </c>
       <c r="F43" s="13">
-        <v>223.89</v>
+        <v>217.62</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" s="7">
         <v>46114</v>
       </c>
@@ -1472,7 +1472,7 @@
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" s="11">
         <v>46114</v>
       </c>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1500,7 +1500,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1511,7 +1511,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="7">
         <v>46115</v>
       </c>
@@ -1539,17 +1539,17 @@
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>295.43</v>
+        <v>289.16000000000003</v>
       </c>
       <c r="E49" s="10">
-        <v>205.68</v>
+        <v>199.41</v>
       </c>
       <c r="F49" s="10">
-        <v>215.68</v>
+        <v>209.41</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" s="11">
         <v>46115</v>
       </c>
@@ -1558,17 +1558,17 @@
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>295.10000000000002</v>
+        <v>288.83</v>
       </c>
       <c r="E50" s="13">
-        <v>205.63</v>
+        <v>199.36</v>
       </c>
       <c r="F50" s="13">
-        <v>215.63</v>
+        <v>209.36</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" s="7">
         <v>46114</v>
       </c>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" s="11">
         <v>46114</v>
       </c>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1615,7 +1615,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1626,7 +1626,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="7">
         <v>46115</v>
       </c>
@@ -1654,17 +1654,17 @@
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>313.95999999999998</v>
+        <v>307.69</v>
       </c>
       <c r="E56" s="10">
-        <v>218.66</v>
+        <v>212.39</v>
       </c>
       <c r="F56" s="10">
-        <v>228.66</v>
+        <v>222.39</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="11">
         <v>46115</v>
       </c>
@@ -1673,17 +1673,17 @@
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>306.55</v>
+        <v>300.27999999999997</v>
       </c>
       <c r="E57" s="13">
-        <v>216.71</v>
+        <v>210.44</v>
       </c>
       <c r="F57" s="13">
-        <v>226.71</v>
+        <v>220.44</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="7">
         <v>46115</v>
       </c>
@@ -1692,7 +1692,7 @@
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>306.42</v>
+        <v>300.14999999999998</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="11">
         <v>46115</v>
       </c>
@@ -1711,17 +1711,17 @@
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>305.8</v>
+        <v>299.52999999999997</v>
       </c>
       <c r="E59" s="13">
-        <v>211.09</v>
+        <v>204.82</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="7">
         <v>46115</v>
       </c>
@@ -1730,17 +1730,17 @@
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>301.66000000000003</v>
+        <v>295.39</v>
       </c>
       <c r="E60" s="10">
-        <v>207.03</v>
+        <v>200.76</v>
       </c>
       <c r="F60" s="10">
-        <v>217.03</v>
+        <v>210.76</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="11">
         <v>46115</v>
       </c>
@@ -1749,17 +1749,17 @@
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>305.51</v>
+        <v>299.24</v>
       </c>
       <c r="E61" s="13">
-        <v>216.44</v>
+        <v>210.17</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" s="7">
         <v>46114</v>
       </c>
@@ -1778,7 +1778,7 @@
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="11">
         <v>46114</v>
       </c>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" s="7">
         <v>46114</v>
       </c>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A65" s="11">
         <v>46114</v>
       </c>
@@ -1834,7 +1834,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A66" s="7">
         <v>46114</v>
       </c>
@@ -1852,7 +1852,7 @@
         <v>215.15</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A67" s="11">
         <v>46114</v>
       </c>
@@ -1892,6 +1892,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2151,7 +2160,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -2162,16 +2171,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2191,7 +2199,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2202,14 +2210,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Tue Apr  7 04:06:55 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{D162356C-1C79-46E3-B1F9-1F506698CC49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{E29374BD-8DDF-4823-B69F-3FB345B3D87C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9435" yWindow="-16320" windowWidth="38640" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" concurrentManualCount="12"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -715,16 +715,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.3984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.3984375"/>
-    <col min="3" max="3" width="18.265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.86328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="6.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125"/>
+    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="6.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.15" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -735,7 +735,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -744,7 +744,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -755,7 +755,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -766,7 +766,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -775,7 +775,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -786,7 +786,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -807,133 +807,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>294.52</v>
+        <v>320.72000000000003</v>
       </c>
       <c r="E8" s="10">
-        <v>199.64</v>
+        <v>208.3</v>
       </c>
       <c r="F8" s="10">
-        <v>209.64</v>
+        <v>218.3</v>
       </c>
       <c r="G8" s="10">
-        <v>200.31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+        <v>210.42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>294.52</v>
+        <v>320.72000000000003</v>
       </c>
       <c r="E9" s="13">
-        <v>199.64</v>
+        <v>208.3</v>
       </c>
       <c r="F9" s="13">
-        <v>209.64</v>
+        <v>218.3</v>
       </c>
       <c r="G9" s="13">
-        <v>200.31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+        <v>210.42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>293.72000000000003</v>
+        <v>319.20999999999998</v>
       </c>
       <c r="E10" s="10">
-        <v>199.53</v>
+        <v>207.56</v>
       </c>
       <c r="F10" s="10">
-        <v>209.53</v>
+        <v>217.56</v>
       </c>
       <c r="G10" s="10">
-        <v>200.92</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+        <v>210.4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>294.08</v>
+        <v>294.52</v>
       </c>
       <c r="E11" s="13">
-        <v>203.78</v>
+        <v>199.64</v>
       </c>
       <c r="F11" s="13">
-        <v>213.78</v>
+        <v>209.64</v>
       </c>
       <c r="G11" s="13">
-        <v>204.05</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+        <v>200.31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>294.08</v>
+        <v>294.52</v>
       </c>
       <c r="E12" s="10">
-        <v>203.78</v>
+        <v>199.64</v>
       </c>
       <c r="F12" s="10">
-        <v>213.78</v>
+        <v>209.64</v>
       </c>
       <c r="G12" s="10">
-        <v>204.05</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+        <v>200.31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>293.51</v>
+        <v>293.72000000000003</v>
       </c>
       <c r="E13" s="13">
-        <v>203.88</v>
+        <v>199.53</v>
       </c>
       <c r="F13" s="13">
-        <v>213.88</v>
+        <v>209.53</v>
       </c>
       <c r="G13" s="13">
-        <v>204.87</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+        <v>200.92</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -942,7 +942,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -953,7 +953,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -972,45 +972,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>297.07</v>
+        <v>322.48</v>
       </c>
       <c r="E17" s="10">
-        <v>200</v>
+        <v>207.98</v>
       </c>
       <c r="F17" s="10">
-        <v>210</v>
+        <v>217.98</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>294.69</v>
+        <v>297.07</v>
       </c>
       <c r="E18" s="13">
-        <v>204.37</v>
+        <v>200</v>
       </c>
       <c r="F18" s="13">
-        <v>214.37</v>
+        <v>210</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1019,7 +1019,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1030,7 +1030,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1051,217 +1051,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>293.17</v>
+        <v>319.35000000000002</v>
       </c>
       <c r="E22" s="10">
-        <v>198.43</v>
+        <v>207.09</v>
       </c>
       <c r="F22" s="10">
-        <v>208.03</v>
+        <v>216.69</v>
       </c>
       <c r="G22" s="10">
-        <v>197.9</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>294.37</v>
+        <v>319.89</v>
       </c>
       <c r="E23" s="13">
-        <v>205.11</v>
+        <v>213.16</v>
       </c>
       <c r="F23" s="13">
-        <v>215.11</v>
+        <v>223.16</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>294.43</v>
+        <v>319.94</v>
       </c>
       <c r="E24" s="10">
-        <v>205.86</v>
+        <v>213.92</v>
       </c>
       <c r="F24" s="10">
-        <v>215.86</v>
+        <v>223.92</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>294.38</v>
+        <v>319.88</v>
       </c>
       <c r="E25" s="13">
-        <v>205.58</v>
+        <v>213.67</v>
       </c>
       <c r="F25" s="13">
-        <v>215.58</v>
+        <v>223.67</v>
       </c>
       <c r="G25" s="13">
-        <v>204.11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+        <v>213.64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>295.02999999999997</v>
+        <v>320.52</v>
       </c>
       <c r="E26" s="10">
-        <v>206.05</v>
+        <v>214.2</v>
       </c>
       <c r="F26" s="10">
-        <v>216.05</v>
+        <v>224.2</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>292.73</v>
+        <v>293.17</v>
       </c>
       <c r="E27" s="13">
-        <v>202.58</v>
+        <v>198.43</v>
       </c>
       <c r="F27" s="13">
-        <v>212.18</v>
+        <v>208.03</v>
       </c>
       <c r="G27" s="13">
-        <v>202.04</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+        <v>197.9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>294.16000000000003</v>
+        <v>294.37</v>
       </c>
       <c r="E28" s="22">
-        <v>209.46</v>
+        <v>205.11</v>
       </c>
       <c r="F28" s="22">
-        <v>219.46</v>
+        <v>215.11</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>294.22000000000003</v>
+        <v>294.43</v>
       </c>
       <c r="E29" s="13">
-        <v>210.2</v>
+        <v>205.86</v>
       </c>
       <c r="F29" s="13">
-        <v>220.2</v>
+        <v>215.86</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>294.18</v>
+        <v>294.38</v>
       </c>
       <c r="E30" s="22">
-        <v>209.92</v>
+        <v>205.58</v>
       </c>
       <c r="F30" s="22">
-        <v>219.92</v>
+        <v>215.58</v>
       </c>
       <c r="G30" s="22">
-        <v>208.45</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+        <v>204.11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>293.72000000000003</v>
+        <v>295.02999999999997</v>
       </c>
       <c r="E31" s="13">
-        <v>210.37</v>
+        <v>206.05</v>
       </c>
       <c r="F31" s="13">
-        <v>220.37</v>
+        <v>216.05</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1270,7 +1270,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1281,7 +1281,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1300,54 +1300,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>292.58</v>
+        <v>318.05</v>
       </c>
       <c r="E35" s="10">
-        <v>200.07</v>
+        <v>208.09</v>
       </c>
       <c r="F35" s="10">
-        <v>209.07</v>
+        <v>217.09</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>292.37</v>
+        <v>292.58</v>
       </c>
       <c r="E36" s="13">
-        <v>204.43</v>
+        <v>200.07</v>
       </c>
       <c r="F36" s="13">
-        <v>213.43</v>
+        <v>209.07</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>308.2</v>
+        <v>333.67</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1357,16 +1357,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>307.99</v>
+        <v>308.2</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1385,7 +1385,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1396,7 +1396,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1415,83 +1415,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>297.77</v>
+        <v>323.33999999999997</v>
       </c>
       <c r="E42" s="10">
-        <v>207.2</v>
+        <v>213.76</v>
       </c>
       <c r="F42" s="10">
-        <v>217.2</v>
+        <v>223.76</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>297.32</v>
+        <v>322.86</v>
       </c>
       <c r="E43" s="13">
-        <v>207.62</v>
+        <v>214.18</v>
       </c>
       <c r="F43" s="13">
-        <v>217.62</v>
+        <v>224.18</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>297.52999999999997</v>
+        <v>297.77</v>
       </c>
       <c r="E44" s="10">
-        <v>212.09</v>
+        <v>207.2</v>
       </c>
       <c r="F44" s="10">
-        <v>222.09</v>
+        <v>217.2</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>297.08999999999997</v>
+        <v>297.32</v>
       </c>
       <c r="E45" s="13">
-        <v>212.5</v>
+        <v>207.62</v>
       </c>
       <c r="F45" s="13">
-        <v>222.5</v>
+        <v>217.62</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1500,7 +1500,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1511,7 +1511,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1530,83 +1530,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>289.16000000000003</v>
+        <v>316.39999999999998</v>
       </c>
       <c r="E49" s="10">
-        <v>199.41</v>
+        <v>205.24</v>
       </c>
       <c r="F49" s="10">
-        <v>209.41</v>
+        <v>215.24</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>288.83</v>
+        <v>316.10000000000002</v>
       </c>
       <c r="E50" s="13">
-        <v>199.36</v>
+        <v>205.19</v>
       </c>
       <c r="F50" s="13">
-        <v>209.36</v>
+        <v>215.19</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>294.60000000000002</v>
+        <v>289.16000000000003</v>
       </c>
       <c r="E51" s="10">
-        <v>209.32</v>
+        <v>199.41</v>
       </c>
       <c r="F51" s="10">
-        <v>219.32</v>
+        <v>209.41</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>294.27</v>
+        <v>288.83</v>
       </c>
       <c r="E52" s="13">
-        <v>209.28</v>
+        <v>199.36</v>
       </c>
       <c r="F52" s="13">
-        <v>219.28</v>
+        <v>209.36</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1615,7 +1615,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1626,7 +1626,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1645,54 +1645,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>307.69</v>
+        <v>333.24</v>
       </c>
       <c r="E56" s="10">
-        <v>212.39</v>
+        <v>220.75</v>
       </c>
       <c r="F56" s="10">
-        <v>222.39</v>
+        <v>230.75</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>300.27999999999997</v>
+        <v>325.81</v>
       </c>
       <c r="E57" s="13">
-        <v>210.44</v>
+        <v>218.36</v>
       </c>
       <c r="F57" s="13">
-        <v>220.44</v>
+        <v>228.36</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>300.14999999999998</v>
+        <v>325.64999999999998</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1702,111 +1702,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>299.52999999999997</v>
+        <v>324.85000000000002</v>
       </c>
       <c r="E59" s="13">
-        <v>204.82</v>
+        <v>212.73</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>295.39</v>
+        <v>320.74</v>
       </c>
       <c r="E60" s="10">
-        <v>200.76</v>
+        <v>208.68</v>
       </c>
       <c r="F60" s="10">
-        <v>210.76</v>
+        <v>218.68</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>299.24</v>
+        <v>324.62</v>
       </c>
       <c r="E61" s="13">
-        <v>210.17</v>
+        <v>218.4</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>305.26</v>
+        <v>307.69</v>
       </c>
       <c r="E62" s="10">
-        <v>216.64</v>
+        <v>212.39</v>
       </c>
       <c r="F62" s="10">
-        <v>226.64</v>
+        <v>222.39</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>297.87</v>
+        <v>300.27999999999997</v>
       </c>
       <c r="E63" s="13">
-        <v>214.83</v>
+        <v>210.44</v>
       </c>
       <c r="F63" s="13">
-        <v>224.83</v>
+        <v>220.44</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>297.74</v>
+        <v>300.14999999999998</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1816,55 +1816,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>297.17</v>
+        <v>299.52999999999997</v>
       </c>
       <c r="E65" s="13">
-        <v>209.21</v>
+        <v>204.82</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>293.04000000000002</v>
+        <v>295.39</v>
       </c>
       <c r="E66" s="10">
-        <v>205.15</v>
+        <v>200.76</v>
       </c>
       <c r="F66" s="10">
-        <v>215.15</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.45">
+        <v>210.76</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>296.87</v>
+        <v>299.24</v>
       </c>
       <c r="E67" s="13">
-        <v>214.45</v>
+        <v>210.17</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Wed Apr  8 04:10:11 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{E29374BD-8DDF-4823-B69F-3FB345B3D87C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{418CD5E4-FE70-48D0-9190-28E26F989E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -809,14 +809,14 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>320.72000000000003</v>
+        <v>318.64999999999998</v>
       </c>
       <c r="E8" s="10">
         <v>208.3</v>
@@ -825,19 +825,19 @@
         <v>218.3</v>
       </c>
       <c r="G8" s="10">
-        <v>210.42</v>
+        <v>208.98</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>320.72000000000003</v>
+        <v>318.64999999999998</v>
       </c>
       <c r="E9" s="13">
         <v>208.3</v>
@@ -846,91 +846,91 @@
         <v>218.3</v>
       </c>
       <c r="G9" s="13">
-        <v>210.42</v>
+        <v>208.98</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>319.20999999999998</v>
+        <v>316.95999999999998</v>
       </c>
       <c r="E10" s="10">
-        <v>207.56</v>
+        <v>207.4</v>
       </c>
       <c r="F10" s="10">
-        <v>217.56</v>
+        <v>217.4</v>
       </c>
       <c r="G10" s="10">
-        <v>210.4</v>
+        <v>208.8</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>294.52</v>
+        <v>320.72000000000003</v>
       </c>
       <c r="E11" s="13">
-        <v>199.64</v>
+        <v>208.3</v>
       </c>
       <c r="F11" s="13">
-        <v>209.64</v>
+        <v>218.3</v>
       </c>
       <c r="G11" s="13">
-        <v>200.31</v>
+        <v>210.42</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>294.52</v>
+        <v>320.72000000000003</v>
       </c>
       <c r="E12" s="10">
-        <v>199.64</v>
+        <v>208.3</v>
       </c>
       <c r="F12" s="10">
-        <v>209.64</v>
+        <v>218.3</v>
       </c>
       <c r="G12" s="10">
-        <v>200.31</v>
+        <v>210.42</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>293.72000000000003</v>
+        <v>319.20999999999998</v>
       </c>
       <c r="E13" s="13">
-        <v>199.53</v>
+        <v>207.56</v>
       </c>
       <c r="F13" s="13">
-        <v>209.53</v>
+        <v>217.56</v>
       </c>
       <c r="G13" s="13">
-        <v>200.92</v>
+        <v>210.4</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>322.48</v>
+        <v>320.24</v>
       </c>
       <c r="E17" s="10">
-        <v>207.98</v>
+        <v>207.82</v>
       </c>
       <c r="F17" s="10">
-        <v>217.98</v>
+        <v>217.82</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>297.07</v>
+        <v>322.48</v>
       </c>
       <c r="E18" s="13">
-        <v>200</v>
+        <v>207.98</v>
       </c>
       <c r="F18" s="13">
-        <v>210</v>
+        <v>217.98</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>319.35000000000002</v>
+        <v>317.27999999999997</v>
       </c>
       <c r="E22" s="10">
-        <v>207.09</v>
+        <v>207.1</v>
       </c>
       <c r="F22" s="10">
-        <v>216.69</v>
+        <v>216.7</v>
       </c>
       <c r="G22" s="10">
-        <v>208</v>
+        <v>206.56</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>319.89</v>
+        <v>317.64</v>
       </c>
       <c r="E23" s="13">
-        <v>213.16</v>
+        <v>213</v>
       </c>
       <c r="F23" s="13">
-        <v>223.16</v>
+        <v>223</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>319.94</v>
+        <v>317.69</v>
       </c>
       <c r="E24" s="10">
-        <v>213.92</v>
+        <v>213.77</v>
       </c>
       <c r="F24" s="10">
-        <v>223.92</v>
+        <v>223.77</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>319.88</v>
+        <v>317.63</v>
       </c>
       <c r="E25" s="13">
-        <v>213.67</v>
+        <v>213.51</v>
       </c>
       <c r="F25" s="13">
-        <v>223.67</v>
+        <v>223.51</v>
       </c>
       <c r="G25" s="13">
-        <v>213.64</v>
+        <v>212.04</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>320.52</v>
+        <v>318.27</v>
       </c>
       <c r="E26" s="10">
-        <v>214.2</v>
+        <v>214.04</v>
       </c>
       <c r="F26" s="10">
-        <v>224.2</v>
+        <v>224.04</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>293.17</v>
+        <v>319.35000000000002</v>
       </c>
       <c r="E27" s="13">
-        <v>198.43</v>
+        <v>207.09</v>
       </c>
       <c r="F27" s="13">
-        <v>208.03</v>
+        <v>216.69</v>
       </c>
       <c r="G27" s="13">
-        <v>197.9</v>
+        <v>208</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>294.37</v>
+        <v>319.89</v>
       </c>
       <c r="E28" s="22">
-        <v>205.11</v>
+        <v>213.16</v>
       </c>
       <c r="F28" s="22">
-        <v>215.11</v>
+        <v>223.16</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>294.43</v>
+        <v>319.94</v>
       </c>
       <c r="E29" s="13">
-        <v>205.86</v>
+        <v>213.92</v>
       </c>
       <c r="F29" s="13">
-        <v>215.86</v>
+        <v>223.92</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>294.38</v>
+        <v>319.88</v>
       </c>
       <c r="E30" s="22">
-        <v>205.58</v>
+        <v>213.67</v>
       </c>
       <c r="F30" s="22">
-        <v>215.58</v>
+        <v>223.67</v>
       </c>
       <c r="G30" s="22">
-        <v>204.11</v>
+        <v>213.64</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>295.02999999999997</v>
+        <v>320.52</v>
       </c>
       <c r="E31" s="13">
-        <v>206.05</v>
+        <v>214.2</v>
       </c>
       <c r="F31" s="13">
-        <v>216.05</v>
+        <v>224.2</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>318.05</v>
+        <v>318</v>
       </c>
       <c r="E35" s="10">
-        <v>208.09</v>
+        <v>207.93</v>
       </c>
       <c r="F35" s="10">
-        <v>217.09</v>
+        <v>216.93</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>292.58</v>
+        <v>318.05</v>
       </c>
       <c r="E36" s="13">
-        <v>200.07</v>
+        <v>208.09</v>
       </c>
       <c r="F36" s="13">
-        <v>209.07</v>
+        <v>217.09</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>333.67</v>
+        <v>333.62</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>308.2</v>
+        <v>333.67</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>323.33999999999997</v>
+        <v>321.10000000000002</v>
       </c>
       <c r="E42" s="10">
-        <v>213.76</v>
+        <v>213.21</v>
       </c>
       <c r="F42" s="10">
-        <v>223.76</v>
+        <v>223.21</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>322.86</v>
+        <v>320.62</v>
       </c>
       <c r="E43" s="13">
-        <v>214.18</v>
+        <v>213.63</v>
       </c>
       <c r="F43" s="13">
-        <v>224.18</v>
+        <v>223.63</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>297.77</v>
+        <v>323.33999999999997</v>
       </c>
       <c r="E44" s="10">
-        <v>207.2</v>
+        <v>213.76</v>
       </c>
       <c r="F44" s="10">
-        <v>217.2</v>
+        <v>223.76</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>297.32</v>
+        <v>322.86</v>
       </c>
       <c r="E45" s="13">
-        <v>207.62</v>
+        <v>214.18</v>
       </c>
       <c r="F45" s="13">
-        <v>217.62</v>
+        <v>224.18</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>316.39999999999998</v>
+        <v>319.37</v>
       </c>
       <c r="E49" s="10">
-        <v>205.24</v>
+        <v>207.31</v>
       </c>
       <c r="F49" s="10">
-        <v>215.24</v>
+        <v>217.31</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>316.10000000000002</v>
+        <v>319.07</v>
       </c>
       <c r="E50" s="13">
-        <v>205.19</v>
+        <v>207.27</v>
       </c>
       <c r="F50" s="13">
-        <v>215.19</v>
+        <v>217.27</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>289.16000000000003</v>
+        <v>316.39999999999998</v>
       </c>
       <c r="E51" s="10">
-        <v>199.41</v>
+        <v>205.24</v>
       </c>
       <c r="F51" s="10">
-        <v>209.41</v>
+        <v>215.24</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>288.83</v>
+        <v>316.10000000000002</v>
       </c>
       <c r="E52" s="13">
-        <v>199.36</v>
+        <v>205.19</v>
       </c>
       <c r="F52" s="13">
-        <v>209.36</v>
+        <v>215.19</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>333.24</v>
+        <v>330.99</v>
       </c>
       <c r="E56" s="10">
-        <v>220.75</v>
+        <v>220.62</v>
       </c>
       <c r="F56" s="10">
-        <v>230.75</v>
+        <v>230.62</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>325.81</v>
+        <v>323.56</v>
       </c>
       <c r="E57" s="13">
-        <v>218.36</v>
+        <v>218.2</v>
       </c>
       <c r="F57" s="13">
-        <v>228.36</v>
+        <v>228.2</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>325.64999999999998</v>
+        <v>323.39999999999998</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>324.85000000000002</v>
+        <v>322.60000000000002</v>
       </c>
       <c r="E59" s="13">
-        <v>212.73</v>
+        <v>212.57</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>320.74</v>
+        <v>318.48</v>
       </c>
       <c r="E60" s="10">
-        <v>208.68</v>
+        <v>208.52</v>
       </c>
       <c r="F60" s="10">
-        <v>218.68</v>
+        <v>218.52</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>324.62</v>
+        <v>322.38</v>
       </c>
       <c r="E61" s="13">
-        <v>218.4</v>
+        <v>218.25</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>307.69</v>
+        <v>333.24</v>
       </c>
       <c r="E62" s="10">
-        <v>212.39</v>
+        <v>220.75</v>
       </c>
       <c r="F62" s="10">
-        <v>222.39</v>
+        <v>230.75</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>300.27999999999997</v>
+        <v>325.81</v>
       </c>
       <c r="E63" s="13">
-        <v>210.44</v>
+        <v>218.36</v>
       </c>
       <c r="F63" s="13">
-        <v>220.44</v>
+        <v>228.36</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>300.14999999999998</v>
+        <v>325.64999999999998</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>299.52999999999997</v>
+        <v>324.85000000000002</v>
       </c>
       <c r="E65" s="13">
-        <v>204.82</v>
+        <v>212.73</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>295.39</v>
+        <v>320.74</v>
       </c>
       <c r="E66" s="10">
-        <v>200.76</v>
+        <v>208.68</v>
       </c>
       <c r="F66" s="10">
-        <v>210.76</v>
+        <v>218.68</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46115</v>
+        <v>46120</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>299.24</v>
+        <v>324.62</v>
       </c>
       <c r="E67" s="13">
-        <v>210.17</v>
+        <v>218.4</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,15 +1892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2160,6 +2151,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2172,14 +2172,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2195,6 +2187,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Thu Apr  9 04:04:50 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{418CD5E4-FE70-48D0-9190-28E26F989E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{AD306307-EA89-49C8-86E9-A05FAF1C6358}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" concurrentManualCount="12"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -809,77 +809,77 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>318.64999999999998</v>
+        <v>313.35000000000002</v>
       </c>
       <c r="E8" s="10">
-        <v>208.3</v>
+        <v>202.65</v>
       </c>
       <c r="F8" s="10">
-        <v>218.3</v>
+        <v>212.65</v>
       </c>
       <c r="G8" s="10">
-        <v>208.98</v>
+        <v>203.33</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>318.64999999999998</v>
+        <v>313.35000000000002</v>
       </c>
       <c r="E9" s="13">
-        <v>208.3</v>
+        <v>202.65</v>
       </c>
       <c r="F9" s="13">
-        <v>218.3</v>
+        <v>212.65</v>
       </c>
       <c r="G9" s="13">
-        <v>208.98</v>
+        <v>203.33</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>316.95999999999998</v>
+        <v>314.94</v>
       </c>
       <c r="E10" s="10">
-        <v>207.4</v>
+        <v>201.73</v>
       </c>
       <c r="F10" s="10">
-        <v>217.4</v>
+        <v>211.73</v>
       </c>
       <c r="G10" s="10">
-        <v>208.8</v>
+        <v>203.13</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>320.72000000000003</v>
+        <v>318.64999999999998</v>
       </c>
       <c r="E11" s="13">
         <v>208.3</v>
@@ -888,19 +888,19 @@
         <v>218.3</v>
       </c>
       <c r="G11" s="13">
-        <v>210.42</v>
+        <v>208.98</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>320.72000000000003</v>
+        <v>318.64999999999998</v>
       </c>
       <c r="E12" s="10">
         <v>208.3</v>
@@ -909,28 +909,28 @@
         <v>218.3</v>
       </c>
       <c r="G12" s="10">
-        <v>210.42</v>
+        <v>208.98</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>319.20999999999998</v>
+        <v>316.95999999999998</v>
       </c>
       <c r="E13" s="13">
-        <v>207.56</v>
+        <v>207.4</v>
       </c>
       <c r="F13" s="13">
-        <v>217.56</v>
+        <v>217.4</v>
       </c>
       <c r="G13" s="13">
-        <v>210.4</v>
+        <v>208.8</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>320.24</v>
+        <v>317.14</v>
       </c>
       <c r="E17" s="10">
-        <v>207.82</v>
+        <v>202.16</v>
       </c>
       <c r="F17" s="10">
-        <v>217.82</v>
+        <v>212.16</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>322.48</v>
+        <v>320.24</v>
       </c>
       <c r="E18" s="13">
-        <v>207.98</v>
+        <v>207.82</v>
       </c>
       <c r="F18" s="13">
-        <v>217.98</v>
+        <v>217.82</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>317.27999999999997</v>
+        <v>311.98</v>
       </c>
       <c r="E22" s="10">
-        <v>207.1</v>
+        <v>201.45</v>
       </c>
       <c r="F22" s="10">
-        <v>216.7</v>
+        <v>211.05</v>
       </c>
       <c r="G22" s="10">
-        <v>206.56</v>
+        <v>200.91</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>317.64</v>
+        <v>315.62</v>
       </c>
       <c r="E23" s="13">
-        <v>213</v>
+        <v>207.32</v>
       </c>
       <c r="F23" s="13">
-        <v>223</v>
+        <v>217.32</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>317.69</v>
+        <v>315.67</v>
       </c>
       <c r="E24" s="10">
-        <v>213.77</v>
+        <v>208.09</v>
       </c>
       <c r="F24" s="10">
-        <v>223.77</v>
+        <v>218.09</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>317.63</v>
+        <v>315.62</v>
       </c>
       <c r="E25" s="13">
-        <v>213.51</v>
+        <v>207.83</v>
       </c>
       <c r="F25" s="13">
-        <v>223.51</v>
+        <v>217.83</v>
       </c>
       <c r="G25" s="13">
-        <v>212.04</v>
+        <v>206.36</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>318.27</v>
+        <v>316.24</v>
       </c>
       <c r="E26" s="10">
-        <v>214.04</v>
+        <v>208.31</v>
       </c>
       <c r="F26" s="10">
-        <v>224.04</v>
+        <v>218.31</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>319.35000000000002</v>
+        <v>317.27999999999997</v>
       </c>
       <c r="E27" s="13">
-        <v>207.09</v>
+        <v>207.1</v>
       </c>
       <c r="F27" s="13">
-        <v>216.69</v>
+        <v>216.7</v>
       </c>
       <c r="G27" s="13">
-        <v>208</v>
+        <v>206.56</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>319.89</v>
+        <v>317.64</v>
       </c>
       <c r="E28" s="22">
-        <v>213.16</v>
+        <v>213</v>
       </c>
       <c r="F28" s="22">
-        <v>223.16</v>
+        <v>223</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>319.94</v>
+        <v>317.69</v>
       </c>
       <c r="E29" s="13">
-        <v>213.92</v>
+        <v>213.77</v>
       </c>
       <c r="F29" s="13">
-        <v>223.92</v>
+        <v>223.77</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>319.88</v>
+        <v>317.63</v>
       </c>
       <c r="E30" s="22">
-        <v>213.67</v>
+        <v>213.51</v>
       </c>
       <c r="F30" s="22">
-        <v>223.67</v>
+        <v>223.51</v>
       </c>
       <c r="G30" s="22">
-        <v>213.64</v>
+        <v>212.04</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>320.52</v>
+        <v>318.27</v>
       </c>
       <c r="E31" s="13">
-        <v>214.2</v>
+        <v>214.04</v>
       </c>
       <c r="F31" s="13">
-        <v>224.2</v>
+        <v>224.04</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>318</v>
+        <v>314.89999999999998</v>
       </c>
       <c r="E35" s="10">
-        <v>207.93</v>
+        <v>202.28</v>
       </c>
       <c r="F35" s="10">
-        <v>216.93</v>
+        <v>211.28</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>318.05</v>
+        <v>318</v>
       </c>
       <c r="E36" s="13">
-        <v>208.09</v>
+        <v>207.93</v>
       </c>
       <c r="F36" s="13">
-        <v>217.09</v>
+        <v>216.93</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>333.62</v>
+        <v>330.52</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>333.67</v>
+        <v>333.62</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>321.10000000000002</v>
+        <v>316.86</v>
       </c>
       <c r="E42" s="10">
-        <v>213.21</v>
+        <v>207.81</v>
       </c>
       <c r="F42" s="10">
-        <v>223.21</v>
+        <v>217.81</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>320.62</v>
+        <v>316.39999999999998</v>
       </c>
       <c r="E43" s="13">
-        <v>213.63</v>
+        <v>208.23</v>
       </c>
       <c r="F43" s="13">
-        <v>223.63</v>
+        <v>218.23</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>323.33999999999997</v>
+        <v>321.10000000000002</v>
       </c>
       <c r="E44" s="10">
-        <v>213.76</v>
+        <v>213.21</v>
       </c>
       <c r="F44" s="10">
-        <v>223.76</v>
+        <v>223.21</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>322.86</v>
+        <v>320.62</v>
       </c>
       <c r="E45" s="13">
-        <v>214.18</v>
+        <v>213.63</v>
       </c>
       <c r="F45" s="13">
-        <v>224.18</v>
+        <v>223.63</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>319.37</v>
+        <v>318.77</v>
       </c>
       <c r="E49" s="10">
-        <v>207.31</v>
+        <v>202.88</v>
       </c>
       <c r="F49" s="10">
-        <v>217.31</v>
+        <v>212.88</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>319.07</v>
+        <v>318.45</v>
       </c>
       <c r="E50" s="13">
-        <v>207.27</v>
+        <v>202.83</v>
       </c>
       <c r="F50" s="13">
-        <v>217.27</v>
+        <v>212.83</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>316.39999999999998</v>
+        <v>319.37</v>
       </c>
       <c r="E51" s="10">
-        <v>205.24</v>
+        <v>207.31</v>
       </c>
       <c r="F51" s="10">
-        <v>215.24</v>
+        <v>217.31</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>316.10000000000002</v>
+        <v>319.07</v>
       </c>
       <c r="E52" s="13">
-        <v>205.19</v>
+        <v>207.27</v>
       </c>
       <c r="F52" s="13">
-        <v>215.19</v>
+        <v>217.27</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>330.99</v>
+        <v>326.7</v>
       </c>
       <c r="E56" s="10">
-        <v>220.62</v>
+        <v>214.93</v>
       </c>
       <c r="F56" s="10">
-        <v>230.62</v>
+        <v>224.93</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>323.56</v>
+        <v>319.32</v>
       </c>
       <c r="E57" s="13">
-        <v>218.2</v>
+        <v>212.57</v>
       </c>
       <c r="F57" s="13">
-        <v>228.2</v>
+        <v>222.57</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>323.39999999999998</v>
+        <v>319.19</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>322.60000000000002</v>
+        <v>318.44</v>
       </c>
       <c r="E59" s="13">
-        <v>212.57</v>
+        <v>206.94</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>318.48</v>
+        <v>314.31</v>
       </c>
       <c r="E60" s="10">
-        <v>208.52</v>
+        <v>202.89</v>
       </c>
       <c r="F60" s="10">
-        <v>218.52</v>
+        <v>212.89</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>322.38</v>
+        <v>318.19</v>
       </c>
       <c r="E61" s="13">
-        <v>218.25</v>
+        <v>212.55</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>333.24</v>
+        <v>330.99</v>
       </c>
       <c r="E62" s="10">
-        <v>220.75</v>
+        <v>220.62</v>
       </c>
       <c r="F62" s="10">
-        <v>230.75</v>
+        <v>230.62</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>325.81</v>
+        <v>323.56</v>
       </c>
       <c r="E63" s="13">
-        <v>218.36</v>
+        <v>218.2</v>
       </c>
       <c r="F63" s="13">
-        <v>228.36</v>
+        <v>228.2</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>325.64999999999998</v>
+        <v>323.39999999999998</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>324.85000000000002</v>
+        <v>322.60000000000002</v>
       </c>
       <c r="E65" s="13">
-        <v>212.73</v>
+        <v>212.57</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>320.74</v>
+        <v>318.48</v>
       </c>
       <c r="E66" s="10">
-        <v>208.68</v>
+        <v>208.52</v>
       </c>
       <c r="F66" s="10">
-        <v>218.68</v>
+        <v>218.52</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>324.62</v>
+        <v>322.38</v>
       </c>
       <c r="E67" s="13">
-        <v>218.4</v>
+        <v>218.25</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,6 +1892,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2151,27 +2171,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2191,25 +2210,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Fri Apr 10 04:20:37 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{AD306307-EA89-49C8-86E9-A05FAF1C6358}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{711CBAC6-05D7-473C-8FFB-E8DA70566707}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>313.35000000000002</v>
+        <v>291.06</v>
       </c>
       <c r="E8" s="10">
-        <v>202.65</v>
+        <v>197.28</v>
       </c>
       <c r="F8" s="10">
-        <v>212.65</v>
+        <v>207.28</v>
       </c>
       <c r="G8" s="10">
-        <v>203.33</v>
+        <v>197.95</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>313.35000000000002</v>
+        <v>291.06</v>
       </c>
       <c r="E9" s="13">
-        <v>202.65</v>
+        <v>197.28</v>
       </c>
       <c r="F9" s="13">
-        <v>212.65</v>
+        <v>207.28</v>
       </c>
       <c r="G9" s="13">
-        <v>203.33</v>
+        <v>197.95</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>314.94</v>
+        <v>292.82</v>
       </c>
       <c r="E10" s="10">
-        <v>201.73</v>
+        <v>196.5</v>
       </c>
       <c r="F10" s="10">
-        <v>211.73</v>
+        <v>206.5</v>
       </c>
       <c r="G10" s="10">
-        <v>203.13</v>
+        <v>197.9</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>318.64999999999998</v>
+        <v>313.35000000000002</v>
       </c>
       <c r="E11" s="13">
-        <v>208.3</v>
+        <v>202.65</v>
       </c>
       <c r="F11" s="13">
-        <v>218.3</v>
+        <v>212.65</v>
       </c>
       <c r="G11" s="13">
-        <v>208.98</v>
+        <v>203.33</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>318.64999999999998</v>
+        <v>313.35000000000002</v>
       </c>
       <c r="E12" s="10">
-        <v>208.3</v>
+        <v>202.65</v>
       </c>
       <c r="F12" s="10">
-        <v>218.3</v>
+        <v>212.65</v>
       </c>
       <c r="G12" s="10">
-        <v>208.98</v>
+        <v>203.33</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>316.95999999999998</v>
+        <v>314.94</v>
       </c>
       <c r="E13" s="13">
-        <v>207.4</v>
+        <v>201.73</v>
       </c>
       <c r="F13" s="13">
-        <v>217.4</v>
+        <v>211.73</v>
       </c>
       <c r="G13" s="13">
-        <v>208.8</v>
+        <v>203.13</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>317.14</v>
+        <v>295</v>
       </c>
       <c r="E17" s="10">
-        <v>202.16</v>
+        <v>196.9</v>
       </c>
       <c r="F17" s="10">
-        <v>212.16</v>
+        <v>206.9</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>320.24</v>
+        <v>317.14</v>
       </c>
       <c r="E18" s="13">
-        <v>207.82</v>
+        <v>202.16</v>
       </c>
       <c r="F18" s="13">
-        <v>217.82</v>
+        <v>212.16</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>311.98</v>
+        <v>289.70999999999998</v>
       </c>
       <c r="E22" s="10">
-        <v>201.45</v>
+        <v>196.08</v>
       </c>
       <c r="F22" s="10">
-        <v>211.05</v>
+        <v>205.68</v>
       </c>
       <c r="G22" s="10">
-        <v>200.91</v>
+        <v>195.54</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>315.62</v>
+        <v>293.48</v>
       </c>
       <c r="E23" s="13">
-        <v>207.32</v>
+        <v>202.08</v>
       </c>
       <c r="F23" s="13">
-        <v>217.32</v>
+        <v>212.08</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>315.67</v>
+        <v>293.54000000000002</v>
       </c>
       <c r="E24" s="10">
-        <v>208.09</v>
+        <v>202.86</v>
       </c>
       <c r="F24" s="10">
-        <v>218.09</v>
+        <v>212.86</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>315.62</v>
+        <v>293.5</v>
       </c>
       <c r="E25" s="13">
-        <v>207.83</v>
+        <v>202.59</v>
       </c>
       <c r="F25" s="13">
-        <v>217.83</v>
+        <v>212.59</v>
       </c>
       <c r="G25" s="13">
-        <v>206.36</v>
+        <v>201.12</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>316.24</v>
+        <v>294.10000000000002</v>
       </c>
       <c r="E26" s="10">
-        <v>208.31</v>
+        <v>203.03</v>
       </c>
       <c r="F26" s="10">
-        <v>218.31</v>
+        <v>213.03</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>317.27999999999997</v>
+        <v>311.98</v>
       </c>
       <c r="E27" s="13">
-        <v>207.1</v>
+        <v>201.45</v>
       </c>
       <c r="F27" s="13">
-        <v>216.7</v>
+        <v>211.05</v>
       </c>
       <c r="G27" s="13">
-        <v>206.56</v>
+        <v>200.91</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>317.64</v>
+        <v>315.62</v>
       </c>
       <c r="E28" s="22">
-        <v>213</v>
+        <v>207.32</v>
       </c>
       <c r="F28" s="22">
-        <v>223</v>
+        <v>217.32</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>317.69</v>
+        <v>315.67</v>
       </c>
       <c r="E29" s="13">
-        <v>213.77</v>
+        <v>208.09</v>
       </c>
       <c r="F29" s="13">
-        <v>223.77</v>
+        <v>218.09</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>317.63</v>
+        <v>315.62</v>
       </c>
       <c r="E30" s="22">
-        <v>213.51</v>
+        <v>207.83</v>
       </c>
       <c r="F30" s="22">
-        <v>223.51</v>
+        <v>217.83</v>
       </c>
       <c r="G30" s="22">
-        <v>212.04</v>
+        <v>206.36</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>318.27</v>
+        <v>316.24</v>
       </c>
       <c r="E31" s="13">
-        <v>214.04</v>
+        <v>208.31</v>
       </c>
       <c r="F31" s="13">
-        <v>224.04</v>
+        <v>218.31</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>314.89999999999998</v>
+        <v>292.8</v>
       </c>
       <c r="E35" s="10">
-        <v>202.28</v>
+        <v>197.07</v>
       </c>
       <c r="F35" s="10">
-        <v>211.28</v>
+        <v>206.07</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>318</v>
+        <v>314.89999999999998</v>
       </c>
       <c r="E36" s="13">
-        <v>207.93</v>
+        <v>202.28</v>
       </c>
       <c r="F36" s="13">
-        <v>216.93</v>
+        <v>211.28</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>330.52</v>
+        <v>308.42</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>333.62</v>
+        <v>330.52</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>316.86</v>
+        <v>294.73</v>
       </c>
       <c r="E42" s="10">
-        <v>207.81</v>
+        <v>203.44</v>
       </c>
       <c r="F42" s="10">
-        <v>217.81</v>
+        <v>213.44</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>316.39999999999998</v>
+        <v>294.29000000000002</v>
       </c>
       <c r="E43" s="13">
-        <v>208.23</v>
+        <v>203.85</v>
       </c>
       <c r="F43" s="13">
-        <v>218.23</v>
+        <v>213.85</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>321.10000000000002</v>
+        <v>316.86</v>
       </c>
       <c r="E44" s="10">
-        <v>213.21</v>
+        <v>207.81</v>
       </c>
       <c r="F44" s="10">
-        <v>223.21</v>
+        <v>217.81</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>320.62</v>
+        <v>316.39999999999998</v>
       </c>
       <c r="E45" s="13">
-        <v>213.63</v>
+        <v>208.23</v>
       </c>
       <c r="F45" s="13">
-        <v>223.63</v>
+        <v>218.23</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>318.77</v>
+        <v>312.83</v>
       </c>
       <c r="E49" s="10">
-        <v>202.88</v>
+        <v>200.32</v>
       </c>
       <c r="F49" s="10">
-        <v>212.88</v>
+        <v>210.32</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>318.45</v>
+        <v>312.49</v>
       </c>
       <c r="E50" s="13">
-        <v>202.83</v>
+        <v>200.26</v>
       </c>
       <c r="F50" s="13">
-        <v>212.83</v>
+        <v>210.26</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>319.37</v>
+        <v>318.77</v>
       </c>
       <c r="E51" s="10">
-        <v>207.31</v>
+        <v>202.88</v>
       </c>
       <c r="F51" s="10">
-        <v>217.31</v>
+        <v>212.88</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>319.07</v>
+        <v>318.45</v>
       </c>
       <c r="E52" s="13">
-        <v>207.27</v>
+        <v>202.83</v>
       </c>
       <c r="F52" s="13">
-        <v>217.27</v>
+        <v>212.83</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>326.7</v>
+        <v>304.47000000000003</v>
       </c>
       <c r="E56" s="10">
-        <v>214.93</v>
+        <v>209.8</v>
       </c>
       <c r="F56" s="10">
-        <v>224.93</v>
+        <v>219.8</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>319.32</v>
+        <v>297.16000000000003</v>
       </c>
       <c r="E57" s="13">
-        <v>212.57</v>
+        <v>207.33</v>
       </c>
       <c r="F57" s="13">
-        <v>222.57</v>
+        <v>217.33</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>319.19</v>
+        <v>297.08</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>318.44</v>
+        <v>296.35000000000002</v>
       </c>
       <c r="E59" s="13">
-        <v>206.94</v>
+        <v>201.71</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>314.31</v>
+        <v>292.20999999999998</v>
       </c>
       <c r="E60" s="10">
-        <v>202.89</v>
+        <v>197.65</v>
       </c>
       <c r="F60" s="10">
-        <v>212.89</v>
+        <v>207.65</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>318.19</v>
+        <v>296.07</v>
       </c>
       <c r="E61" s="13">
-        <v>212.55</v>
+        <v>207.35</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>330.99</v>
+        <v>326.7</v>
       </c>
       <c r="E62" s="10">
-        <v>220.62</v>
+        <v>214.93</v>
       </c>
       <c r="F62" s="10">
-        <v>230.62</v>
+        <v>224.93</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>323.56</v>
+        <v>319.32</v>
       </c>
       <c r="E63" s="13">
-        <v>218.2</v>
+        <v>212.57</v>
       </c>
       <c r="F63" s="13">
-        <v>228.2</v>
+        <v>222.57</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>323.39999999999998</v>
+        <v>319.19</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>322.60000000000002</v>
+        <v>318.44</v>
       </c>
       <c r="E65" s="13">
-        <v>212.57</v>
+        <v>206.94</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>318.48</v>
+        <v>314.31</v>
       </c>
       <c r="E66" s="10">
-        <v>208.52</v>
+        <v>202.89</v>
       </c>
       <c r="F66" s="10">
-        <v>218.52</v>
+        <v>212.89</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>322.38</v>
+        <v>318.19</v>
       </c>
       <c r="E67" s="13">
-        <v>218.25</v>
+        <v>212.55</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1903,15 +1903,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2171,6 +2162,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
@@ -2183,14 +2183,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2210,6 +2202,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Mon Apr 13 04:32:21 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{711CBAC6-05D7-473C-8FFB-E8DA70566707}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{79FD157E-0D07-46CD-9D04-683A61148778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>291.06</v>
+        <v>289.12</v>
       </c>
       <c r="E8" s="10">
-        <v>197.28</v>
+        <v>196.95</v>
       </c>
       <c r="F8" s="10">
-        <v>207.28</v>
+        <v>206.95</v>
       </c>
       <c r="G8" s="10">
-        <v>197.95</v>
+        <v>197.62</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>291.06</v>
+        <v>289.12</v>
       </c>
       <c r="E9" s="13">
-        <v>197.28</v>
+        <v>196.95</v>
       </c>
       <c r="F9" s="13">
-        <v>207.28</v>
+        <v>206.95</v>
       </c>
       <c r="G9" s="13">
-        <v>197.95</v>
+        <v>197.62</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>292.82</v>
+        <v>290.86</v>
       </c>
       <c r="E10" s="10">
-        <v>196.5</v>
+        <v>196.16</v>
       </c>
       <c r="F10" s="10">
-        <v>206.5</v>
+        <v>206.16</v>
       </c>
       <c r="G10" s="10">
-        <v>197.9</v>
+        <v>197.56</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>313.35000000000002</v>
+        <v>291.06</v>
       </c>
       <c r="E11" s="13">
-        <v>202.65</v>
+        <v>197.28</v>
       </c>
       <c r="F11" s="13">
-        <v>212.65</v>
+        <v>207.28</v>
       </c>
       <c r="G11" s="13">
-        <v>203.33</v>
+        <v>197.95</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>313.35000000000002</v>
+        <v>291.06</v>
       </c>
       <c r="E12" s="10">
-        <v>202.65</v>
+        <v>197.28</v>
       </c>
       <c r="F12" s="10">
-        <v>212.65</v>
+        <v>207.28</v>
       </c>
       <c r="G12" s="10">
-        <v>203.33</v>
+        <v>197.95</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>314.94</v>
+        <v>292.82</v>
       </c>
       <c r="E13" s="13">
-        <v>201.73</v>
+        <v>196.5</v>
       </c>
       <c r="F13" s="13">
-        <v>211.73</v>
+        <v>206.5</v>
       </c>
       <c r="G13" s="13">
-        <v>203.13</v>
+        <v>197.9</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>295</v>
+        <v>293.02</v>
       </c>
       <c r="E17" s="10">
-        <v>196.9</v>
+        <v>196.54</v>
       </c>
       <c r="F17" s="10">
-        <v>206.9</v>
+        <v>206.54</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>317.14</v>
+        <v>295</v>
       </c>
       <c r="E18" s="13">
-        <v>202.16</v>
+        <v>196.9</v>
       </c>
       <c r="F18" s="13">
-        <v>212.16</v>
+        <v>206.9</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>289.70999999999998</v>
+        <v>287.77</v>
       </c>
       <c r="E22" s="10">
-        <v>196.08</v>
+        <v>195.75</v>
       </c>
       <c r="F22" s="10">
-        <v>205.68</v>
+        <v>205.35</v>
       </c>
       <c r="G22" s="10">
-        <v>195.54</v>
+        <v>195.21</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>293.48</v>
+        <v>291.52999999999997</v>
       </c>
       <c r="E23" s="13">
-        <v>202.08</v>
+        <v>201.73</v>
       </c>
       <c r="F23" s="13">
-        <v>212.08</v>
+        <v>211.73</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>293.54000000000002</v>
+        <v>291.58</v>
       </c>
       <c r="E24" s="10">
-        <v>202.86</v>
+        <v>202.53</v>
       </c>
       <c r="F24" s="10">
-        <v>212.86</v>
+        <v>212.53</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>293.5</v>
+        <v>291.54000000000002</v>
       </c>
       <c r="E25" s="13">
-        <v>202.59</v>
+        <v>202.26</v>
       </c>
       <c r="F25" s="13">
-        <v>212.59</v>
+        <v>212.26</v>
       </c>
       <c r="G25" s="13">
-        <v>201.12</v>
+        <v>200.79</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>294.10000000000002</v>
+        <v>292.13</v>
       </c>
       <c r="E26" s="10">
-        <v>203.03</v>
+        <v>202.69</v>
       </c>
       <c r="F26" s="10">
-        <v>213.03</v>
+        <v>212.69</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>311.98</v>
+        <v>289.70999999999998</v>
       </c>
       <c r="E27" s="13">
-        <v>201.45</v>
+        <v>196.08</v>
       </c>
       <c r="F27" s="13">
-        <v>211.05</v>
+        <v>205.68</v>
       </c>
       <c r="G27" s="13">
-        <v>200.91</v>
+        <v>195.54</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>315.62</v>
+        <v>293.48</v>
       </c>
       <c r="E28" s="22">
-        <v>207.32</v>
+        <v>202.08</v>
       </c>
       <c r="F28" s="22">
-        <v>217.32</v>
+        <v>212.08</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>315.67</v>
+        <v>293.54000000000002</v>
       </c>
       <c r="E29" s="13">
-        <v>208.09</v>
+        <v>202.86</v>
       </c>
       <c r="F29" s="13">
-        <v>218.09</v>
+        <v>212.86</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>315.62</v>
+        <v>293.5</v>
       </c>
       <c r="E30" s="22">
-        <v>207.83</v>
+        <v>202.59</v>
       </c>
       <c r="F30" s="22">
-        <v>217.83</v>
+        <v>212.59</v>
       </c>
       <c r="G30" s="22">
-        <v>206.36</v>
+        <v>201.12</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>316.24</v>
+        <v>294.10000000000002</v>
       </c>
       <c r="E31" s="13">
-        <v>208.31</v>
+        <v>203.03</v>
       </c>
       <c r="F31" s="13">
-        <v>218.31</v>
+        <v>213.03</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>292.8</v>
+        <v>290.85000000000002</v>
       </c>
       <c r="E35" s="10">
-        <v>197.07</v>
+        <v>196.73</v>
       </c>
       <c r="F35" s="10">
-        <v>206.07</v>
+        <v>205.73</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>314.89999999999998</v>
+        <v>292.8</v>
       </c>
       <c r="E36" s="13">
-        <v>202.28</v>
+        <v>197.07</v>
       </c>
       <c r="F36" s="13">
-        <v>211.28</v>
+        <v>206.07</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>308.42</v>
+        <v>306.47000000000003</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>330.52</v>
+        <v>308.42</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>294.73</v>
+        <v>292.79000000000002</v>
       </c>
       <c r="E42" s="10">
-        <v>203.44</v>
+        <v>203.41</v>
       </c>
       <c r="F42" s="10">
-        <v>213.44</v>
+        <v>213.41</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>294.29000000000002</v>
+        <v>292.35000000000002</v>
       </c>
       <c r="E43" s="13">
-        <v>203.85</v>
+        <v>203.82</v>
       </c>
       <c r="F43" s="13">
-        <v>213.85</v>
+        <v>213.82</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>316.86</v>
+        <v>294.73</v>
       </c>
       <c r="E44" s="10">
-        <v>207.81</v>
+        <v>203.44</v>
       </c>
       <c r="F44" s="10">
-        <v>217.81</v>
+        <v>213.44</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>316.39999999999998</v>
+        <v>294.29000000000002</v>
       </c>
       <c r="E45" s="13">
-        <v>208.23</v>
+        <v>203.85</v>
       </c>
       <c r="F45" s="13">
-        <v>218.23</v>
+        <v>213.85</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>312.83</v>
+        <v>305.79000000000002</v>
       </c>
       <c r="E49" s="10">
-        <v>200.32</v>
+        <v>200.3</v>
       </c>
       <c r="F49" s="10">
-        <v>210.32</v>
+        <v>210.3</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>312.49</v>
+        <v>305.43</v>
       </c>
       <c r="E50" s="13">
-        <v>200.26</v>
+        <v>200.24</v>
       </c>
       <c r="F50" s="13">
-        <v>210.26</v>
+        <v>210.24</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>318.77</v>
+        <v>312.83</v>
       </c>
       <c r="E51" s="10">
-        <v>202.88</v>
+        <v>200.32</v>
       </c>
       <c r="F51" s="10">
-        <v>212.88</v>
+        <v>210.32</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>318.45</v>
+        <v>312.49</v>
       </c>
       <c r="E52" s="13">
-        <v>202.83</v>
+        <v>200.26</v>
       </c>
       <c r="F52" s="13">
-        <v>212.83</v>
+        <v>210.26</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>304.47000000000003</v>
+        <v>302.48</v>
       </c>
       <c r="E56" s="10">
-        <v>209.8</v>
+        <v>209.55</v>
       </c>
       <c r="F56" s="10">
-        <v>219.8</v>
+        <v>219.55</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>297.16000000000003</v>
+        <v>295.2</v>
       </c>
       <c r="E57" s="13">
-        <v>207.33</v>
+        <v>206.97</v>
       </c>
       <c r="F57" s="13">
-        <v>217.33</v>
+        <v>216.97</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>297.08</v>
+        <v>295.14</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>296.35000000000002</v>
+        <v>294.38</v>
       </c>
       <c r="E59" s="13">
-        <v>201.71</v>
+        <v>201.36</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>292.20999999999998</v>
+        <v>290.24</v>
       </c>
       <c r="E60" s="10">
-        <v>197.65</v>
+        <v>197.29</v>
       </c>
       <c r="F60" s="10">
-        <v>207.65</v>
+        <v>207.29</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>296.07</v>
+        <v>294.08999999999997</v>
       </c>
       <c r="E61" s="13">
-        <v>207.35</v>
+        <v>207.06</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>326.7</v>
+        <v>304.47000000000003</v>
       </c>
       <c r="E62" s="10">
-        <v>214.93</v>
+        <v>209.8</v>
       </c>
       <c r="F62" s="10">
-        <v>224.93</v>
+        <v>219.8</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>319.32</v>
+        <v>297.16000000000003</v>
       </c>
       <c r="E63" s="13">
-        <v>212.57</v>
+        <v>207.33</v>
       </c>
       <c r="F63" s="13">
-        <v>222.57</v>
+        <v>217.33</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>319.19</v>
+        <v>297.08</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>318.44</v>
+        <v>296.35000000000002</v>
       </c>
       <c r="E65" s="13">
-        <v>206.94</v>
+        <v>201.71</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>314.31</v>
+        <v>292.20999999999998</v>
       </c>
       <c r="E66" s="10">
-        <v>202.89</v>
+        <v>197.65</v>
       </c>
       <c r="F66" s="10">
-        <v>212.89</v>
+        <v>207.65</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46122</v>
+        <v>46123</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>318.19</v>
+        <v>296.07</v>
       </c>
       <c r="E67" s="13">
-        <v>212.55</v>
+        <v>207.35</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,17 +1892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2162,6 +2151,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2172,17 +2172,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2202,6 +2191,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Tue Apr 14 04:20:27 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{79FD157E-0D07-46CD-9D04-683A61148778}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{4B5D9D85-3C29-45B3-9EAF-7DB685B4F12A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>289.12</v>
+        <v>278.13</v>
       </c>
       <c r="E8" s="10">
-        <v>196.95</v>
+        <v>193.99</v>
       </c>
       <c r="F8" s="10">
-        <v>206.95</v>
+        <v>203.99</v>
       </c>
       <c r="G8" s="10">
-        <v>197.62</v>
+        <v>194.66</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>289.12</v>
+        <v>278.13</v>
       </c>
       <c r="E9" s="13">
-        <v>196.95</v>
+        <v>193.99</v>
       </c>
       <c r="F9" s="13">
-        <v>206.95</v>
+        <v>203.99</v>
       </c>
       <c r="G9" s="13">
-        <v>197.62</v>
+        <v>194.66</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>290.86</v>
+        <v>279.89999999999998</v>
       </c>
       <c r="E10" s="10">
-        <v>196.16</v>
+        <v>193.22</v>
       </c>
       <c r="F10" s="10">
-        <v>206.16</v>
+        <v>203.22</v>
       </c>
       <c r="G10" s="10">
-        <v>197.56</v>
+        <v>194.62</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>291.06</v>
+        <v>289.12</v>
       </c>
       <c r="E11" s="13">
-        <v>197.28</v>
+        <v>196.95</v>
       </c>
       <c r="F11" s="13">
-        <v>207.28</v>
+        <v>206.95</v>
       </c>
       <c r="G11" s="13">
-        <v>197.95</v>
+        <v>197.62</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>291.06</v>
+        <v>289.12</v>
       </c>
       <c r="E12" s="10">
-        <v>197.28</v>
+        <v>196.95</v>
       </c>
       <c r="F12" s="10">
-        <v>207.28</v>
+        <v>206.95</v>
       </c>
       <c r="G12" s="10">
-        <v>197.95</v>
+        <v>197.62</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>292.82</v>
+        <v>290.86</v>
       </c>
       <c r="E13" s="13">
-        <v>196.5</v>
+        <v>196.16</v>
       </c>
       <c r="F13" s="13">
-        <v>206.5</v>
+        <v>206.16</v>
       </c>
       <c r="G13" s="13">
-        <v>197.9</v>
+        <v>197.56</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>293.02</v>
+        <v>282.01</v>
       </c>
       <c r="E17" s="10">
-        <v>196.54</v>
+        <v>193.55</v>
       </c>
       <c r="F17" s="10">
-        <v>206.54</v>
+        <v>203.56</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>295</v>
+        <v>293.02</v>
       </c>
       <c r="E18" s="13">
-        <v>196.9</v>
+        <v>196.54</v>
       </c>
       <c r="F18" s="13">
-        <v>206.9</v>
+        <v>206.54</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>287.77</v>
+        <v>276.79000000000002</v>
       </c>
       <c r="E22" s="10">
-        <v>195.75</v>
+        <v>192.79</v>
       </c>
       <c r="F22" s="10">
-        <v>205.35</v>
+        <v>202.39</v>
       </c>
       <c r="G22" s="10">
-        <v>195.21</v>
+        <v>192.25</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>291.52999999999997</v>
+        <v>280.56</v>
       </c>
       <c r="E23" s="13">
-        <v>201.73</v>
+        <v>198.78</v>
       </c>
       <c r="F23" s="13">
-        <v>211.73</v>
+        <v>208.78</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>291.58</v>
+        <v>280.61</v>
       </c>
       <c r="E24" s="10">
-        <v>202.53</v>
+        <v>199.6</v>
       </c>
       <c r="F24" s="10">
-        <v>212.53</v>
+        <v>209.6</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>291.54000000000002</v>
+        <v>280.57</v>
       </c>
       <c r="E25" s="13">
-        <v>202.26</v>
+        <v>199.33</v>
       </c>
       <c r="F25" s="13">
-        <v>212.26</v>
+        <v>209.33</v>
       </c>
       <c r="G25" s="13">
-        <v>200.79</v>
+        <v>197.86</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>292.13</v>
+        <v>281.14</v>
       </c>
       <c r="E26" s="10">
-        <v>202.69</v>
+        <v>199.74</v>
       </c>
       <c r="F26" s="10">
-        <v>212.69</v>
+        <v>209.74</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>289.70999999999998</v>
+        <v>287.77</v>
       </c>
       <c r="E27" s="13">
-        <v>196.08</v>
+        <v>195.75</v>
       </c>
       <c r="F27" s="13">
-        <v>205.68</v>
+        <v>205.35</v>
       </c>
       <c r="G27" s="13">
-        <v>195.54</v>
+        <v>195.21</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>293.48</v>
+        <v>291.52999999999997</v>
       </c>
       <c r="E28" s="22">
-        <v>202.08</v>
+        <v>201.73</v>
       </c>
       <c r="F28" s="22">
-        <v>212.08</v>
+        <v>211.73</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>293.54000000000002</v>
+        <v>291.58</v>
       </c>
       <c r="E29" s="13">
-        <v>202.86</v>
+        <v>202.53</v>
       </c>
       <c r="F29" s="13">
-        <v>212.86</v>
+        <v>212.53</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>293.5</v>
+        <v>291.54000000000002</v>
       </c>
       <c r="E30" s="22">
-        <v>202.59</v>
+        <v>202.26</v>
       </c>
       <c r="F30" s="22">
-        <v>212.59</v>
+        <v>212.26</v>
       </c>
       <c r="G30" s="22">
-        <v>201.12</v>
+        <v>200.79</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>294.10000000000002</v>
+        <v>292.13</v>
       </c>
       <c r="E31" s="13">
-        <v>203.03</v>
+        <v>202.69</v>
       </c>
       <c r="F31" s="13">
-        <v>213.03</v>
+        <v>212.69</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>290.85000000000002</v>
+        <v>279.89999999999998</v>
       </c>
       <c r="E35" s="10">
-        <v>196.73</v>
+        <v>193.8</v>
       </c>
       <c r="F35" s="10">
-        <v>205.73</v>
+        <v>202.8</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>292.8</v>
+        <v>290.85000000000002</v>
       </c>
       <c r="E36" s="13">
-        <v>197.07</v>
+        <v>196.73</v>
       </c>
       <c r="F36" s="13">
-        <v>206.07</v>
+        <v>205.73</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>306.47000000000003</v>
+        <v>295.52</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>308.42</v>
+        <v>306.47000000000003</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>292.79000000000002</v>
+        <v>281.83999999999997</v>
       </c>
       <c r="E42" s="10">
-        <v>203.41</v>
+        <v>200.82</v>
       </c>
       <c r="F42" s="10">
-        <v>213.41</v>
+        <v>210.82</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>292.35000000000002</v>
+        <v>281.42</v>
       </c>
       <c r="E43" s="13">
-        <v>203.82</v>
+        <v>201.23</v>
       </c>
       <c r="F43" s="13">
-        <v>213.82</v>
+        <v>211.23</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>294.73</v>
+        <v>292.79000000000002</v>
       </c>
       <c r="E44" s="10">
-        <v>203.44</v>
+        <v>203.41</v>
       </c>
       <c r="F44" s="10">
-        <v>213.44</v>
+        <v>213.41</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>294.29000000000002</v>
+        <v>292.35000000000002</v>
       </c>
       <c r="E45" s="13">
-        <v>203.85</v>
+        <v>203.82</v>
       </c>
       <c r="F45" s="13">
-        <v>213.85</v>
+        <v>213.82</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>305.79000000000002</v>
+        <v>285.63</v>
       </c>
       <c r="E49" s="10">
-        <v>200.3</v>
+        <v>197.07</v>
       </c>
       <c r="F49" s="10">
-        <v>210.3</v>
+        <v>207.07</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>305.43</v>
+        <v>285.24</v>
       </c>
       <c r="E50" s="13">
-        <v>200.24</v>
+        <v>197</v>
       </c>
       <c r="F50" s="13">
-        <v>210.24</v>
+        <v>207</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>312.83</v>
+        <v>305.79000000000002</v>
       </c>
       <c r="E51" s="10">
-        <v>200.32</v>
+        <v>200.3</v>
       </c>
       <c r="F51" s="10">
-        <v>210.32</v>
+        <v>210.3</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>312.49</v>
+        <v>305.43</v>
       </c>
       <c r="E52" s="13">
-        <v>200.26</v>
+        <v>200.24</v>
       </c>
       <c r="F52" s="13">
-        <v>210.26</v>
+        <v>210.24</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>302.48</v>
+        <v>291.45</v>
       </c>
       <c r="E56" s="10">
-        <v>209.55</v>
+        <v>206.77</v>
       </c>
       <c r="F56" s="10">
-        <v>219.55</v>
+        <v>216.77</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>295.2</v>
+        <v>284.22000000000003</v>
       </c>
       <c r="E57" s="13">
-        <v>206.97</v>
+        <v>204</v>
       </c>
       <c r="F57" s="13">
-        <v>216.97</v>
+        <v>214.01</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>295.14</v>
+        <v>284.18</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>294.38</v>
+        <v>283.39999999999998</v>
       </c>
       <c r="E59" s="13">
-        <v>201.36</v>
+        <v>198.39</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>290.24</v>
+        <v>279.25</v>
       </c>
       <c r="E60" s="10">
-        <v>197.29</v>
+        <v>194.32</v>
       </c>
       <c r="F60" s="10">
-        <v>207.29</v>
+        <v>204.33</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>294.08999999999997</v>
+        <v>283.08</v>
       </c>
       <c r="E61" s="13">
-        <v>207.06</v>
+        <v>204.2</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>304.47000000000003</v>
+        <v>302.48</v>
       </c>
       <c r="E62" s="10">
-        <v>209.8</v>
+        <v>209.55</v>
       </c>
       <c r="F62" s="10">
-        <v>219.8</v>
+        <v>219.55</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>297.16000000000003</v>
+        <v>295.2</v>
       </c>
       <c r="E63" s="13">
-        <v>207.33</v>
+        <v>206.97</v>
       </c>
       <c r="F63" s="13">
-        <v>217.33</v>
+        <v>216.97</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>297.08</v>
+        <v>295.14</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>296.35000000000002</v>
+        <v>294.38</v>
       </c>
       <c r="E65" s="13">
-        <v>201.71</v>
+        <v>201.36</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>292.20999999999998</v>
+        <v>290.24</v>
       </c>
       <c r="E66" s="10">
-        <v>197.65</v>
+        <v>197.29</v>
       </c>
       <c r="F66" s="10">
-        <v>207.65</v>
+        <v>207.29</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46123</v>
+        <v>46126</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>296.07</v>
+        <v>294.08999999999997</v>
       </c>
       <c r="E67" s="13">
-        <v>207.35</v>
+        <v>207.06</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,6 +1892,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2151,27 +2171,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2191,25 +2210,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Wed Apr 15 04:19:33 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{4B5D9D85-3C29-45B3-9EAF-7DB685B4F12A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{4946FB35-8835-4312-880C-1B132E052124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>278.13</v>
+        <v>267.47000000000003</v>
       </c>
       <c r="E8" s="10">
-        <v>193.99</v>
+        <v>187.64</v>
       </c>
       <c r="F8" s="10">
-        <v>203.99</v>
+        <v>197.64</v>
       </c>
       <c r="G8" s="10">
-        <v>194.66</v>
+        <v>188.31</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>278.13</v>
+        <v>267.47000000000003</v>
       </c>
       <c r="E9" s="13">
-        <v>193.99</v>
+        <v>187.64</v>
       </c>
       <c r="F9" s="13">
-        <v>203.99</v>
+        <v>197.64</v>
       </c>
       <c r="G9" s="13">
-        <v>194.66</v>
+        <v>188.31</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>279.89999999999998</v>
+        <v>269.27999999999997</v>
       </c>
       <c r="E10" s="10">
-        <v>193.22</v>
+        <v>186.9</v>
       </c>
       <c r="F10" s="10">
-        <v>203.22</v>
+        <v>196.9</v>
       </c>
       <c r="G10" s="10">
-        <v>194.62</v>
+        <v>188.29</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>289.12</v>
+        <v>278.13</v>
       </c>
       <c r="E11" s="13">
-        <v>196.95</v>
+        <v>193.99</v>
       </c>
       <c r="F11" s="13">
-        <v>206.95</v>
+        <v>203.99</v>
       </c>
       <c r="G11" s="13">
-        <v>197.62</v>
+        <v>194.66</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>289.12</v>
+        <v>278.13</v>
       </c>
       <c r="E12" s="10">
-        <v>196.95</v>
+        <v>193.99</v>
       </c>
       <c r="F12" s="10">
-        <v>206.95</v>
+        <v>203.99</v>
       </c>
       <c r="G12" s="10">
-        <v>197.62</v>
+        <v>194.66</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>290.86</v>
+        <v>279.89999999999998</v>
       </c>
       <c r="E13" s="13">
-        <v>196.16</v>
+        <v>193.22</v>
       </c>
       <c r="F13" s="13">
-        <v>206.16</v>
+        <v>203.22</v>
       </c>
       <c r="G13" s="13">
-        <v>197.56</v>
+        <v>194.62</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>282.01</v>
+        <v>271.33</v>
       </c>
       <c r="E17" s="10">
-        <v>193.55</v>
+        <v>187.17</v>
       </c>
       <c r="F17" s="10">
-        <v>203.56</v>
+        <v>197.17</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>293.02</v>
+        <v>282.01</v>
       </c>
       <c r="E18" s="13">
-        <v>196.54</v>
+        <v>193.55</v>
       </c>
       <c r="F18" s="13">
-        <v>206.54</v>
+        <v>203.56</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>276.79000000000002</v>
+        <v>266.14</v>
       </c>
       <c r="E22" s="10">
-        <v>192.79</v>
+        <v>186.44</v>
       </c>
       <c r="F22" s="10">
-        <v>202.39</v>
+        <v>196.04</v>
       </c>
       <c r="G22" s="10">
-        <v>192.25</v>
+        <v>185.9</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>280.56</v>
+        <v>269.93</v>
       </c>
       <c r="E23" s="13">
-        <v>198.78</v>
+        <v>192.45</v>
       </c>
       <c r="F23" s="13">
-        <v>208.78</v>
+        <v>202.45</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>280.61</v>
+        <v>269.98</v>
       </c>
       <c r="E24" s="10">
-        <v>199.6</v>
+        <v>193.3</v>
       </c>
       <c r="F24" s="10">
-        <v>209.6</v>
+        <v>203.3</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>280.57</v>
+        <v>269.95</v>
       </c>
       <c r="E25" s="13">
-        <v>199.33</v>
+        <v>193.02</v>
       </c>
       <c r="F25" s="13">
-        <v>209.33</v>
+        <v>203.02</v>
       </c>
       <c r="G25" s="13">
-        <v>197.86</v>
+        <v>191.55</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>281.14</v>
+        <v>270.49</v>
       </c>
       <c r="E26" s="10">
-        <v>199.74</v>
+        <v>193.4</v>
       </c>
       <c r="F26" s="10">
-        <v>209.74</v>
+        <v>203.4</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>287.77</v>
+        <v>276.79000000000002</v>
       </c>
       <c r="E27" s="13">
-        <v>195.75</v>
+        <v>192.79</v>
       </c>
       <c r="F27" s="13">
-        <v>205.35</v>
+        <v>202.39</v>
       </c>
       <c r="G27" s="13">
-        <v>195.21</v>
+        <v>192.25</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>291.52999999999997</v>
+        <v>280.56</v>
       </c>
       <c r="E28" s="22">
-        <v>201.73</v>
+        <v>198.78</v>
       </c>
       <c r="F28" s="22">
-        <v>211.73</v>
+        <v>208.78</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>291.58</v>
+        <v>280.61</v>
       </c>
       <c r="E29" s="13">
-        <v>202.53</v>
+        <v>199.6</v>
       </c>
       <c r="F29" s="13">
-        <v>212.53</v>
+        <v>209.6</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>291.54000000000002</v>
+        <v>280.57</v>
       </c>
       <c r="E30" s="22">
-        <v>202.26</v>
+        <v>199.33</v>
       </c>
       <c r="F30" s="22">
-        <v>212.26</v>
+        <v>209.33</v>
       </c>
       <c r="G30" s="22">
-        <v>200.79</v>
+        <v>197.86</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>292.13</v>
+        <v>281.14</v>
       </c>
       <c r="E31" s="13">
-        <v>202.69</v>
+        <v>199.74</v>
       </c>
       <c r="F31" s="13">
-        <v>212.69</v>
+        <v>209.74</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>279.89999999999998</v>
+        <v>269.29000000000002</v>
       </c>
       <c r="E35" s="10">
-        <v>193.8</v>
+        <v>187.49</v>
       </c>
       <c r="F35" s="10">
-        <v>202.8</v>
+        <v>196.49</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>290.85000000000002</v>
+        <v>279.89999999999998</v>
       </c>
       <c r="E36" s="13">
-        <v>196.73</v>
+        <v>193.8</v>
       </c>
       <c r="F36" s="13">
-        <v>205.73</v>
+        <v>202.8</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>295.52</v>
+        <v>284.91000000000003</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>306.47000000000003</v>
+        <v>295.52</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>281.83999999999997</v>
+        <v>271.25</v>
       </c>
       <c r="E42" s="10">
-        <v>200.82</v>
+        <v>195.34</v>
       </c>
       <c r="F42" s="10">
-        <v>210.82</v>
+        <v>205.34</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>281.42</v>
+        <v>270.85000000000002</v>
       </c>
       <c r="E43" s="13">
-        <v>201.23</v>
+        <v>195.76</v>
       </c>
       <c r="F43" s="13">
-        <v>211.23</v>
+        <v>205.76</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>292.79000000000002</v>
+        <v>281.83999999999997</v>
       </c>
       <c r="E44" s="10">
-        <v>203.41</v>
+        <v>200.82</v>
       </c>
       <c r="F44" s="10">
-        <v>213.41</v>
+        <v>210.82</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>292.35000000000002</v>
+        <v>281.42</v>
       </c>
       <c r="E45" s="13">
-        <v>203.82</v>
+        <v>201.23</v>
       </c>
       <c r="F45" s="13">
-        <v>213.82</v>
+        <v>211.23</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>285.63</v>
+        <v>277.44</v>
       </c>
       <c r="E49" s="10">
-        <v>197.07</v>
+        <v>193.48</v>
       </c>
       <c r="F49" s="10">
-        <v>207.07</v>
+        <v>203.48</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>285.24</v>
+        <v>277.02</v>
       </c>
       <c r="E50" s="13">
-        <v>197</v>
+        <v>193.4</v>
       </c>
       <c r="F50" s="13">
-        <v>207</v>
+        <v>203.4</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>305.79000000000002</v>
+        <v>285.63</v>
       </c>
       <c r="E51" s="10">
-        <v>200.3</v>
+        <v>197.07</v>
       </c>
       <c r="F51" s="10">
-        <v>210.3</v>
+        <v>207.07</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>305.43</v>
+        <v>285.24</v>
       </c>
       <c r="E52" s="13">
-        <v>200.24</v>
+        <v>197</v>
       </c>
       <c r="F52" s="13">
-        <v>210.24</v>
+        <v>207</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>291.45</v>
+        <v>280.74</v>
       </c>
       <c r="E56" s="10">
-        <v>206.77</v>
+        <v>200.71</v>
       </c>
       <c r="F56" s="10">
-        <v>216.77</v>
+        <v>210.71</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>284.22000000000003</v>
+        <v>273.58</v>
       </c>
       <c r="E57" s="13">
-        <v>204</v>
+        <v>197.64</v>
       </c>
       <c r="F57" s="13">
-        <v>214.01</v>
+        <v>207.64</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>284.18</v>
+        <v>273.58</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>283.39999999999998</v>
+        <v>272.74</v>
       </c>
       <c r="E59" s="13">
-        <v>198.39</v>
+        <v>192.02</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>279.25</v>
+        <v>268.58</v>
       </c>
       <c r="E60" s="10">
-        <v>194.32</v>
+        <v>187.96</v>
       </c>
       <c r="F60" s="10">
-        <v>204.33</v>
+        <v>197.96</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>283.08</v>
+        <v>272.39999999999998</v>
       </c>
       <c r="E61" s="13">
-        <v>204.2</v>
+        <v>198.01</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>302.48</v>
+        <v>291.45</v>
       </c>
       <c r="E62" s="10">
-        <v>209.55</v>
+        <v>206.77</v>
       </c>
       <c r="F62" s="10">
-        <v>219.55</v>
+        <v>216.77</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>295.2</v>
+        <v>284.22000000000003</v>
       </c>
       <c r="E63" s="13">
-        <v>206.97</v>
+        <v>204</v>
       </c>
       <c r="F63" s="13">
-        <v>216.97</v>
+        <v>214.01</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>295.14</v>
+        <v>284.18</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>294.38</v>
+        <v>283.39999999999998</v>
       </c>
       <c r="E65" s="13">
-        <v>201.36</v>
+        <v>198.39</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>290.24</v>
+        <v>279.25</v>
       </c>
       <c r="E66" s="10">
-        <v>197.29</v>
+        <v>194.32</v>
       </c>
       <c r="F66" s="10">
-        <v>207.29</v>
+        <v>204.33</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>294.08999999999997</v>
+        <v>283.08</v>
       </c>
       <c r="E67" s="13">
-        <v>207.06</v>
+        <v>204.2</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,26 +1892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2171,26 +2151,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2210,6 +2191,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Thu Apr 16 04:26:20 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{4946FB35-8835-4312-880C-1B132E052124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{95162A2F-2869-428B-8AF4-E6F3E8E730FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>267.47000000000003</v>
+        <v>259.98</v>
       </c>
       <c r="E8" s="10">
-        <v>187.64</v>
+        <v>187.25</v>
       </c>
       <c r="F8" s="10">
-        <v>197.64</v>
+        <v>197.25</v>
       </c>
       <c r="G8" s="10">
-        <v>188.31</v>
+        <v>187.93</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>267.47000000000003</v>
+        <v>259.98</v>
       </c>
       <c r="E9" s="13">
-        <v>187.64</v>
+        <v>187.25</v>
       </c>
       <c r="F9" s="13">
-        <v>197.64</v>
+        <v>197.25</v>
       </c>
       <c r="G9" s="13">
-        <v>188.31</v>
+        <v>187.93</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>269.27999999999997</v>
+        <v>260.91000000000003</v>
       </c>
       <c r="E10" s="10">
-        <v>186.9</v>
+        <v>186.72</v>
       </c>
       <c r="F10" s="10">
-        <v>196.9</v>
+        <v>196.72</v>
       </c>
       <c r="G10" s="10">
-        <v>188.29</v>
+        <v>188.12</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>278.13</v>
+        <v>267.47000000000003</v>
       </c>
       <c r="E11" s="13">
-        <v>193.99</v>
+        <v>187.64</v>
       </c>
       <c r="F11" s="13">
-        <v>203.99</v>
+        <v>197.64</v>
       </c>
       <c r="G11" s="13">
-        <v>194.66</v>
+        <v>188.31</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>278.13</v>
+        <v>267.47000000000003</v>
       </c>
       <c r="E12" s="10">
-        <v>193.99</v>
+        <v>187.64</v>
       </c>
       <c r="F12" s="10">
-        <v>203.99</v>
+        <v>197.64</v>
       </c>
       <c r="G12" s="10">
-        <v>194.66</v>
+        <v>188.31</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>279.89999999999998</v>
+        <v>269.27999999999997</v>
       </c>
       <c r="E13" s="13">
-        <v>193.22</v>
+        <v>186.9</v>
       </c>
       <c r="F13" s="13">
-        <v>203.22</v>
+        <v>196.9</v>
       </c>
       <c r="G13" s="13">
-        <v>194.62</v>
+        <v>188.29</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>271.33</v>
+        <v>262.88</v>
       </c>
       <c r="E17" s="10">
-        <v>187.17</v>
+        <v>186.92</v>
       </c>
       <c r="F17" s="10">
-        <v>197.17</v>
+        <v>196.92</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>282.01</v>
+        <v>271.33</v>
       </c>
       <c r="E18" s="13">
-        <v>193.55</v>
+        <v>187.17</v>
       </c>
       <c r="F18" s="13">
-        <v>203.56</v>
+        <v>197.17</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>266.14</v>
+        <v>257.55</v>
       </c>
       <c r="E22" s="10">
-        <v>186.44</v>
+        <v>186.06</v>
       </c>
       <c r="F22" s="10">
-        <v>196.04</v>
+        <v>195.66</v>
       </c>
       <c r="G22" s="10">
-        <v>185.9</v>
+        <v>185.52</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>269.93</v>
+        <v>261.57</v>
       </c>
       <c r="E23" s="13">
-        <v>192.45</v>
+        <v>192.26</v>
       </c>
       <c r="F23" s="13">
-        <v>202.45</v>
+        <v>202.26</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>269.98</v>
+        <v>261.61</v>
       </c>
       <c r="E24" s="10">
-        <v>193.3</v>
+        <v>193.15</v>
       </c>
       <c r="F24" s="10">
-        <v>203.3</v>
+        <v>203.15</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>269.95</v>
+        <v>261.58</v>
       </c>
       <c r="E25" s="13">
-        <v>193.02</v>
+        <v>192.88</v>
       </c>
       <c r="F25" s="13">
-        <v>203.02</v>
+        <v>202.88</v>
       </c>
       <c r="G25" s="13">
-        <v>191.55</v>
+        <v>191.41</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>270.49</v>
+        <v>262.10000000000002</v>
       </c>
       <c r="E26" s="10">
-        <v>193.4</v>
+        <v>193.25</v>
       </c>
       <c r="F26" s="10">
-        <v>203.4</v>
+        <v>203.25</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>276.79000000000002</v>
+        <v>266.14</v>
       </c>
       <c r="E27" s="13">
-        <v>192.79</v>
+        <v>186.44</v>
       </c>
       <c r="F27" s="13">
-        <v>202.39</v>
+        <v>196.04</v>
       </c>
       <c r="G27" s="13">
-        <v>192.25</v>
+        <v>185.9</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>280.56</v>
+        <v>269.93</v>
       </c>
       <c r="E28" s="22">
-        <v>198.78</v>
+        <v>192.45</v>
       </c>
       <c r="F28" s="22">
-        <v>208.78</v>
+        <v>202.45</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>280.61</v>
+        <v>269.98</v>
       </c>
       <c r="E29" s="13">
-        <v>199.6</v>
+        <v>193.3</v>
       </c>
       <c r="F29" s="13">
-        <v>209.6</v>
+        <v>203.3</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>280.57</v>
+        <v>269.95</v>
       </c>
       <c r="E30" s="22">
-        <v>199.33</v>
+        <v>193.02</v>
       </c>
       <c r="F30" s="22">
-        <v>209.33</v>
+        <v>203.02</v>
       </c>
       <c r="G30" s="22">
-        <v>197.86</v>
+        <v>191.55</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>281.14</v>
+        <v>270.49</v>
       </c>
       <c r="E31" s="13">
-        <v>199.74</v>
+        <v>193.4</v>
       </c>
       <c r="F31" s="13">
-        <v>209.74</v>
+        <v>203.4</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>269.29000000000002</v>
+        <v>260.93</v>
       </c>
       <c r="E35" s="10">
-        <v>187.49</v>
+        <v>187.32</v>
       </c>
       <c r="F35" s="10">
-        <v>196.49</v>
+        <v>196.32</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>279.89999999999998</v>
+        <v>269.29000000000002</v>
       </c>
       <c r="E36" s="13">
-        <v>193.8</v>
+        <v>187.49</v>
       </c>
       <c r="F36" s="13">
-        <v>202.8</v>
+        <v>196.49</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>284.91000000000003</v>
+        <v>276.55</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>295.52</v>
+        <v>284.91000000000003</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>271.25</v>
+        <v>262.94</v>
       </c>
       <c r="E42" s="10">
-        <v>195.34</v>
+        <v>195.27</v>
       </c>
       <c r="F42" s="10">
-        <v>205.34</v>
+        <v>205.27</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>270.85000000000002</v>
+        <v>262.54000000000002</v>
       </c>
       <c r="E43" s="13">
-        <v>195.76</v>
+        <v>195.69</v>
       </c>
       <c r="F43" s="13">
-        <v>205.76</v>
+        <v>205.69</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>281.83999999999997</v>
+        <v>271.25</v>
       </c>
       <c r="E44" s="10">
-        <v>200.82</v>
+        <v>195.34</v>
       </c>
       <c r="F44" s="10">
-        <v>210.82</v>
+        <v>205.34</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>281.42</v>
+        <v>270.85000000000002</v>
       </c>
       <c r="E45" s="13">
-        <v>201.23</v>
+        <v>195.76</v>
       </c>
       <c r="F45" s="13">
-        <v>211.23</v>
+        <v>205.76</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>277.44</v>
+        <v>261.01</v>
       </c>
       <c r="E49" s="10">
-        <v>193.48</v>
+        <v>189.72</v>
       </c>
       <c r="F49" s="10">
-        <v>203.48</v>
+        <v>199.72</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>277.02</v>
+        <v>260.55</v>
       </c>
       <c r="E50" s="13">
-        <v>193.4</v>
+        <v>189.62</v>
       </c>
       <c r="F50" s="13">
-        <v>203.4</v>
+        <v>199.62</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>285.63</v>
+        <v>277.44</v>
       </c>
       <c r="E51" s="10">
-        <v>197.07</v>
+        <v>193.48</v>
       </c>
       <c r="F51" s="10">
-        <v>207.07</v>
+        <v>203.48</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>285.24</v>
+        <v>277.02</v>
       </c>
       <c r="E52" s="13">
-        <v>197</v>
+        <v>193.4</v>
       </c>
       <c r="F52" s="13">
-        <v>207</v>
+        <v>203.4</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>280.74</v>
+        <v>272.32</v>
       </c>
       <c r="E56" s="10">
-        <v>200.71</v>
+        <v>200.87</v>
       </c>
       <c r="F56" s="10">
-        <v>210.71</v>
+        <v>210.87</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>273.58</v>
+        <v>265.20999999999998</v>
       </c>
       <c r="E57" s="13">
-        <v>197.64</v>
+        <v>197.37</v>
       </c>
       <c r="F57" s="13">
-        <v>207.64</v>
+        <v>207.37</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>273.58</v>
+        <v>265.24</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>272.74</v>
+        <v>264.29000000000002</v>
       </c>
       <c r="E59" s="13">
-        <v>192.02</v>
+        <v>191.76</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>268.58</v>
+        <v>260.13</v>
       </c>
       <c r="E60" s="10">
-        <v>187.96</v>
+        <v>187.69</v>
       </c>
       <c r="F60" s="10">
-        <v>197.96</v>
+        <v>197.69</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>272.39999999999998</v>
+        <v>263.94</v>
       </c>
       <c r="E61" s="13">
-        <v>198.01</v>
+        <v>198.02</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>291.45</v>
+        <v>280.74</v>
       </c>
       <c r="E62" s="10">
-        <v>206.77</v>
+        <v>200.71</v>
       </c>
       <c r="F62" s="10">
-        <v>216.77</v>
+        <v>210.71</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>284.22000000000003</v>
+        <v>273.58</v>
       </c>
       <c r="E63" s="13">
-        <v>204</v>
+        <v>197.64</v>
       </c>
       <c r="F63" s="13">
-        <v>214.01</v>
+        <v>207.64</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>284.18</v>
+        <v>273.58</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>283.39999999999998</v>
+        <v>272.74</v>
       </c>
       <c r="E65" s="13">
-        <v>198.39</v>
+        <v>192.02</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>279.25</v>
+        <v>268.58</v>
       </c>
       <c r="E66" s="10">
-        <v>194.32</v>
+        <v>187.96</v>
       </c>
       <c r="F66" s="10">
-        <v>204.33</v>
+        <v>197.96</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>283.08</v>
+        <v>272.39999999999998</v>
       </c>
       <c r="E67" s="13">
-        <v>204.2</v>
+        <v>198.01</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,6 +1892,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2151,17 +2162,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2172,6 +2172,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2191,17 +2202,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Fri Apr 17 04:24:07 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{95162A2F-2869-428B-8AF4-E6F3E8E730FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{C0430A54-8956-4365-826C-6B297643ADE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>259.98</v>
+        <v>253.09</v>
       </c>
       <c r="E8" s="10">
-        <v>187.25</v>
+        <v>184.08</v>
       </c>
       <c r="F8" s="10">
-        <v>197.25</v>
+        <v>194.08</v>
       </c>
       <c r="G8" s="10">
-        <v>187.93</v>
+        <v>184.76</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>259.98</v>
+        <v>253.09</v>
       </c>
       <c r="E9" s="13">
-        <v>187.25</v>
+        <v>184.08</v>
       </c>
       <c r="F9" s="13">
-        <v>197.25</v>
+        <v>194.08</v>
       </c>
       <c r="G9" s="13">
-        <v>187.93</v>
+        <v>184.76</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>260.91000000000003</v>
+        <v>254.32</v>
       </c>
       <c r="E10" s="10">
-        <v>186.72</v>
+        <v>183.81</v>
       </c>
       <c r="F10" s="10">
-        <v>196.72</v>
+        <v>193.81</v>
       </c>
       <c r="G10" s="10">
-        <v>188.12</v>
+        <v>185.21</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>267.47000000000003</v>
+        <v>259.98</v>
       </c>
       <c r="E11" s="13">
-        <v>187.64</v>
+        <v>187.25</v>
       </c>
       <c r="F11" s="13">
-        <v>197.64</v>
+        <v>197.25</v>
       </c>
       <c r="G11" s="13">
-        <v>188.31</v>
+        <v>187.93</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>267.47000000000003</v>
+        <v>259.98</v>
       </c>
       <c r="E12" s="10">
-        <v>187.64</v>
+        <v>187.25</v>
       </c>
       <c r="F12" s="10">
-        <v>197.64</v>
+        <v>197.25</v>
       </c>
       <c r="G12" s="10">
-        <v>188.31</v>
+        <v>187.93</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>269.27999999999997</v>
+        <v>260.91000000000003</v>
       </c>
       <c r="E13" s="13">
-        <v>186.9</v>
+        <v>186.72</v>
       </c>
       <c r="F13" s="13">
-        <v>196.9</v>
+        <v>196.72</v>
       </c>
       <c r="G13" s="13">
-        <v>188.29</v>
+        <v>188.12</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>262.88</v>
+        <v>256.22000000000003</v>
       </c>
       <c r="E17" s="10">
-        <v>186.92</v>
+        <v>183.94</v>
       </c>
       <c r="F17" s="10">
-        <v>196.92</v>
+        <v>193.94</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>271.33</v>
+        <v>262.88</v>
       </c>
       <c r="E18" s="13">
-        <v>187.17</v>
+        <v>186.92</v>
       </c>
       <c r="F18" s="13">
-        <v>197.17</v>
+        <v>196.92</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>257.55</v>
+        <v>250.67</v>
       </c>
       <c r="E22" s="10">
-        <v>186.06</v>
+        <v>182.88</v>
       </c>
       <c r="F22" s="10">
-        <v>195.66</v>
+        <v>192.48</v>
       </c>
       <c r="G22" s="10">
-        <v>185.52</v>
+        <v>182.35</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>261.57</v>
+        <v>254.99</v>
       </c>
       <c r="E23" s="13">
-        <v>192.26</v>
+        <v>189.34</v>
       </c>
       <c r="F23" s="13">
-        <v>202.26</v>
+        <v>199.34</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>261.61</v>
+        <v>255.02</v>
       </c>
       <c r="E24" s="10">
-        <v>193.15</v>
+        <v>190.26</v>
       </c>
       <c r="F24" s="10">
-        <v>203.15</v>
+        <v>200.26</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>261.58</v>
+        <v>254.99</v>
       </c>
       <c r="E25" s="13">
-        <v>192.88</v>
+        <v>190</v>
       </c>
       <c r="F25" s="13">
-        <v>202.88</v>
+        <v>200</v>
       </c>
       <c r="G25" s="13">
-        <v>191.41</v>
+        <v>188.53</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>262.10000000000002</v>
+        <v>255.48</v>
       </c>
       <c r="E26" s="10">
-        <v>193.25</v>
+        <v>190.35</v>
       </c>
       <c r="F26" s="10">
-        <v>203.25</v>
+        <v>200.35</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>266.14</v>
+        <v>257.55</v>
       </c>
       <c r="E27" s="13">
-        <v>186.44</v>
+        <v>186.06</v>
       </c>
       <c r="F27" s="13">
-        <v>196.04</v>
+        <v>195.66</v>
       </c>
       <c r="G27" s="13">
-        <v>185.9</v>
+        <v>185.52</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>269.93</v>
+        <v>261.57</v>
       </c>
       <c r="E28" s="22">
-        <v>192.45</v>
+        <v>192.26</v>
       </c>
       <c r="F28" s="22">
-        <v>202.45</v>
+        <v>202.26</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>269.98</v>
+        <v>261.61</v>
       </c>
       <c r="E29" s="13">
-        <v>193.3</v>
+        <v>193.15</v>
       </c>
       <c r="F29" s="13">
-        <v>203.3</v>
+        <v>203.15</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>269.95</v>
+        <v>261.58</v>
       </c>
       <c r="E30" s="22">
-        <v>193.02</v>
+        <v>192.88</v>
       </c>
       <c r="F30" s="22">
-        <v>203.02</v>
+        <v>202.88</v>
       </c>
       <c r="G30" s="22">
-        <v>191.55</v>
+        <v>191.41</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>270.49</v>
+        <v>262.10000000000002</v>
       </c>
       <c r="E31" s="13">
-        <v>193.4</v>
+        <v>193.25</v>
       </c>
       <c r="F31" s="13">
-        <v>203.4</v>
+        <v>203.25</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>260.93</v>
+        <v>254.35</v>
       </c>
       <c r="E35" s="10">
-        <v>187.32</v>
+        <v>184.42</v>
       </c>
       <c r="F35" s="10">
-        <v>196.32</v>
+        <v>193.42</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>269.29000000000002</v>
+        <v>260.93</v>
       </c>
       <c r="E36" s="13">
-        <v>187.49</v>
+        <v>187.32</v>
       </c>
       <c r="F36" s="13">
-        <v>196.49</v>
+        <v>196.32</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>276.55</v>
+        <v>269.97000000000003</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>284.91000000000003</v>
+        <v>276.55</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>262.94</v>
+        <v>256.41000000000003</v>
       </c>
       <c r="E42" s="10">
-        <v>195.27</v>
+        <v>192.97</v>
       </c>
       <c r="F42" s="10">
-        <v>205.27</v>
+        <v>202.97</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>262.54000000000002</v>
+        <v>256.01</v>
       </c>
       <c r="E43" s="13">
-        <v>195.69</v>
+        <v>193.38</v>
       </c>
       <c r="F43" s="13">
-        <v>205.69</v>
+        <v>203.38</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>271.25</v>
+        <v>262.94</v>
       </c>
       <c r="E44" s="10">
-        <v>195.34</v>
+        <v>195.27</v>
       </c>
       <c r="F44" s="10">
-        <v>205.34</v>
+        <v>205.27</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>270.85000000000002</v>
+        <v>262.54000000000002</v>
       </c>
       <c r="E45" s="13">
-        <v>195.76</v>
+        <v>195.69</v>
       </c>
       <c r="F45" s="13">
-        <v>205.76</v>
+        <v>205.69</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>261.01</v>
+        <v>251.77</v>
       </c>
       <c r="E49" s="10">
-        <v>189.72</v>
+        <v>185.65</v>
       </c>
       <c r="F49" s="10">
-        <v>199.72</v>
+        <v>195.65</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>260.55</v>
+        <v>251.27</v>
       </c>
       <c r="E50" s="13">
-        <v>189.62</v>
+        <v>185.54</v>
       </c>
       <c r="F50" s="13">
-        <v>199.62</v>
+        <v>195.54</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>277.44</v>
+        <v>261.01</v>
       </c>
       <c r="E51" s="10">
-        <v>193.48</v>
+        <v>189.72</v>
       </c>
       <c r="F51" s="10">
-        <v>203.48</v>
+        <v>199.72</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>277.02</v>
+        <v>260.55</v>
       </c>
       <c r="E52" s="13">
-        <v>193.4</v>
+        <v>189.62</v>
       </c>
       <c r="F52" s="13">
-        <v>203.4</v>
+        <v>199.62</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>272.32</v>
+        <v>265.66000000000003</v>
       </c>
       <c r="E56" s="10">
-        <v>200.87</v>
+        <v>198.29</v>
       </c>
       <c r="F56" s="10">
-        <v>210.87</v>
+        <v>208.29</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>265.20999999999998</v>
+        <v>258.61</v>
       </c>
       <c r="E57" s="13">
-        <v>197.37</v>
+        <v>194.4</v>
       </c>
       <c r="F57" s="13">
-        <v>207.37</v>
+        <v>204.4</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>265.24</v>
+        <v>258.67</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>264.29000000000002</v>
+        <v>257.63</v>
       </c>
       <c r="E59" s="13">
-        <v>191.76</v>
+        <v>188.79</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>260.13</v>
+        <v>253.47</v>
       </c>
       <c r="E60" s="10">
-        <v>187.69</v>
+        <v>184.72</v>
       </c>
       <c r="F60" s="10">
-        <v>197.69</v>
+        <v>194.72</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>263.94</v>
+        <v>257.27</v>
       </c>
       <c r="E61" s="13">
-        <v>198.02</v>
+        <v>195.28</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>280.74</v>
+        <v>272.32</v>
       </c>
       <c r="E62" s="10">
-        <v>200.71</v>
+        <v>200.87</v>
       </c>
       <c r="F62" s="10">
-        <v>210.71</v>
+        <v>210.87</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>273.58</v>
+        <v>265.20999999999998</v>
       </c>
       <c r="E63" s="13">
-        <v>197.64</v>
+        <v>197.37</v>
       </c>
       <c r="F63" s="13">
-        <v>207.64</v>
+        <v>207.37</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>273.58</v>
+        <v>265.24</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>272.74</v>
+        <v>264.29000000000002</v>
       </c>
       <c r="E65" s="13">
-        <v>192.02</v>
+        <v>191.76</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>268.58</v>
+        <v>260.13</v>
       </c>
       <c r="E66" s="10">
-        <v>187.96</v>
+        <v>187.69</v>
       </c>
       <c r="F66" s="10">
-        <v>197.96</v>
+        <v>197.69</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46128</v>
+        <v>46129</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>272.39999999999998</v>
+        <v>263.94</v>
       </c>
       <c r="E67" s="13">
-        <v>198.01</v>
+        <v>198.02</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,6 +1892,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -1902,7 +1911,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2162,16 +2171,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2182,7 +2190,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2202,14 +2210,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Mon Apr 20 04:32:43 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{C0430A54-8956-4365-826C-6B297643ADE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{ECEBC45E-0106-4CB2-9BBC-21364A845CF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>253.09</v>
+        <v>245.74</v>
       </c>
       <c r="E8" s="10">
-        <v>184.08</v>
+        <v>182.46</v>
       </c>
       <c r="F8" s="10">
-        <v>194.08</v>
+        <v>192.46</v>
       </c>
       <c r="G8" s="10">
-        <v>184.76</v>
+        <v>183.13</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>253.09</v>
+        <v>245.74</v>
       </c>
       <c r="E9" s="13">
-        <v>184.08</v>
+        <v>182.46</v>
       </c>
       <c r="F9" s="13">
-        <v>194.08</v>
+        <v>192.46</v>
       </c>
       <c r="G9" s="13">
-        <v>184.76</v>
+        <v>183.13</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>254.32</v>
+        <v>247.35</v>
       </c>
       <c r="E10" s="10">
-        <v>183.81</v>
+        <v>182.52</v>
       </c>
       <c r="F10" s="10">
-        <v>193.81</v>
+        <v>192.52</v>
       </c>
       <c r="G10" s="10">
-        <v>185.21</v>
+        <v>183.92</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>259.98</v>
+        <v>253.09</v>
       </c>
       <c r="E11" s="13">
-        <v>187.25</v>
+        <v>184.08</v>
       </c>
       <c r="F11" s="13">
-        <v>197.25</v>
+        <v>194.08</v>
       </c>
       <c r="G11" s="13">
-        <v>187.93</v>
+        <v>184.76</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>259.98</v>
+        <v>253.09</v>
       </c>
       <c r="E12" s="10">
-        <v>187.25</v>
+        <v>184.08</v>
       </c>
       <c r="F12" s="10">
-        <v>197.25</v>
+        <v>194.08</v>
       </c>
       <c r="G12" s="10">
-        <v>187.93</v>
+        <v>184.76</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>260.91000000000003</v>
+        <v>254.32</v>
       </c>
       <c r="E13" s="13">
-        <v>186.72</v>
+        <v>183.81</v>
       </c>
       <c r="F13" s="13">
-        <v>196.72</v>
+        <v>193.81</v>
       </c>
       <c r="G13" s="13">
-        <v>188.12</v>
+        <v>185.21</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>256.22000000000003</v>
+        <v>248.07</v>
       </c>
       <c r="E17" s="10">
-        <v>183.94</v>
+        <v>182.58</v>
       </c>
       <c r="F17" s="10">
-        <v>193.94</v>
+        <v>192.58</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>262.88</v>
+        <v>256.22000000000003</v>
       </c>
       <c r="E18" s="13">
-        <v>186.92</v>
+        <v>183.94</v>
       </c>
       <c r="F18" s="13">
-        <v>196.92</v>
+        <v>193.94</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>250.67</v>
+        <v>243.33</v>
       </c>
       <c r="E22" s="10">
-        <v>182.88</v>
+        <v>181.26</v>
       </c>
       <c r="F22" s="10">
-        <v>192.48</v>
+        <v>190.86</v>
       </c>
       <c r="G22" s="10">
-        <v>182.35</v>
+        <v>180.72</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>254.99</v>
+        <v>248.02</v>
       </c>
       <c r="E23" s="13">
-        <v>189.34</v>
+        <v>188.05</v>
       </c>
       <c r="F23" s="13">
-        <v>199.34</v>
+        <v>198.05</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>255.02</v>
+        <v>248.04</v>
       </c>
       <c r="E24" s="10">
-        <v>190.26</v>
+        <v>189.01</v>
       </c>
       <c r="F24" s="10">
-        <v>200.26</v>
+        <v>199.01</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>254.99</v>
+        <v>248.02</v>
       </c>
       <c r="E25" s="13">
-        <v>190</v>
+        <v>188.75</v>
       </c>
       <c r="F25" s="13">
-        <v>200</v>
+        <v>198.75</v>
       </c>
       <c r="G25" s="13">
-        <v>188.53</v>
+        <v>187.28</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>255.48</v>
+        <v>248.48</v>
       </c>
       <c r="E26" s="10">
-        <v>190.35</v>
+        <v>189.09</v>
       </c>
       <c r="F26" s="10">
-        <v>200.35</v>
+        <v>199.09</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>257.55</v>
+        <v>250.67</v>
       </c>
       <c r="E27" s="13">
-        <v>186.06</v>
+        <v>182.88</v>
       </c>
       <c r="F27" s="13">
-        <v>195.66</v>
+        <v>192.48</v>
       </c>
       <c r="G27" s="13">
-        <v>185.52</v>
+        <v>182.35</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>261.57</v>
+        <v>254.99</v>
       </c>
       <c r="E28" s="22">
-        <v>192.26</v>
+        <v>189.34</v>
       </c>
       <c r="F28" s="22">
-        <v>202.26</v>
+        <v>199.34</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>261.61</v>
+        <v>255.02</v>
       </c>
       <c r="E29" s="13">
-        <v>193.15</v>
+        <v>190.26</v>
       </c>
       <c r="F29" s="13">
-        <v>203.15</v>
+        <v>200.26</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>261.58</v>
+        <v>254.99</v>
       </c>
       <c r="E30" s="22">
-        <v>192.88</v>
+        <v>190</v>
       </c>
       <c r="F30" s="22">
-        <v>202.88</v>
+        <v>200</v>
       </c>
       <c r="G30" s="22">
-        <v>191.41</v>
+        <v>188.53</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>262.10000000000002</v>
+        <v>255.48</v>
       </c>
       <c r="E31" s="13">
-        <v>193.25</v>
+        <v>190.35</v>
       </c>
       <c r="F31" s="13">
-        <v>203.25</v>
+        <v>200.35</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>254.35</v>
+        <v>246.29</v>
       </c>
       <c r="E35" s="10">
-        <v>184.42</v>
+        <v>183.14</v>
       </c>
       <c r="F35" s="10">
-        <v>193.42</v>
+        <v>192.14</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>260.93</v>
+        <v>254.35</v>
       </c>
       <c r="E36" s="13">
-        <v>187.32</v>
+        <v>184.42</v>
       </c>
       <c r="F36" s="13">
-        <v>196.32</v>
+        <v>193.42</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>269.97000000000003</v>
+        <v>261.91000000000003</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>276.55</v>
+        <v>269.97000000000003</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>256.41000000000003</v>
+        <v>249.49</v>
       </c>
       <c r="E42" s="10">
-        <v>192.97</v>
+        <v>191.71</v>
       </c>
       <c r="F42" s="10">
-        <v>202.97</v>
+        <v>201.71</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>256.01</v>
+        <v>249.11</v>
       </c>
       <c r="E43" s="13">
-        <v>193.38</v>
+        <v>192.12</v>
       </c>
       <c r="F43" s="13">
-        <v>203.38</v>
+        <v>202.13</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>262.94</v>
+        <v>256.41000000000003</v>
       </c>
       <c r="E44" s="10">
-        <v>195.27</v>
+        <v>192.97</v>
       </c>
       <c r="F44" s="10">
-        <v>205.27</v>
+        <v>202.97</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>262.54000000000002</v>
+        <v>256.01</v>
       </c>
       <c r="E45" s="13">
-        <v>195.69</v>
+        <v>193.38</v>
       </c>
       <c r="F45" s="13">
-        <v>205.69</v>
+        <v>203.38</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>251.77</v>
+        <v>247.71</v>
       </c>
       <c r="E49" s="10">
-        <v>185.65</v>
+        <v>185.92</v>
       </c>
       <c r="F49" s="10">
-        <v>195.65</v>
+        <v>195.92</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>251.27</v>
+        <v>247.18</v>
       </c>
       <c r="E50" s="13">
-        <v>185.54</v>
+        <v>185.8</v>
       </c>
       <c r="F50" s="13">
-        <v>195.54</v>
+        <v>195.8</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>261.01</v>
+        <v>251.77</v>
       </c>
       <c r="E51" s="10">
-        <v>189.72</v>
+        <v>185.65</v>
       </c>
       <c r="F51" s="10">
-        <v>199.72</v>
+        <v>195.65</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>260.55</v>
+        <v>251.27</v>
       </c>
       <c r="E52" s="13">
-        <v>189.62</v>
+        <v>185.54</v>
       </c>
       <c r="F52" s="13">
-        <v>199.62</v>
+        <v>195.54</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>265.66000000000003</v>
+        <v>257.52999999999997</v>
       </c>
       <c r="E56" s="10">
-        <v>198.29</v>
+        <v>197.36</v>
       </c>
       <c r="F56" s="10">
-        <v>208.29</v>
+        <v>207.36</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>258.61</v>
+        <v>250.54</v>
       </c>
       <c r="E57" s="13">
-        <v>194.4</v>
+        <v>193.03</v>
       </c>
       <c r="F57" s="13">
-        <v>204.4</v>
+        <v>203.03</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>258.67</v>
+        <v>250.63</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>257.63</v>
+        <v>249.48</v>
       </c>
       <c r="E59" s="13">
-        <v>188.79</v>
+        <v>187.42</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>253.47</v>
+        <v>245.31</v>
       </c>
       <c r="E60" s="10">
-        <v>184.72</v>
+        <v>183.35</v>
       </c>
       <c r="F60" s="10">
-        <v>194.72</v>
+        <v>193.35</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>257.27</v>
+        <v>249.11</v>
       </c>
       <c r="E61" s="13">
-        <v>195.28</v>
+        <v>194.19</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>272.32</v>
+        <v>265.66000000000003</v>
       </c>
       <c r="E62" s="10">
-        <v>200.87</v>
+        <v>198.29</v>
       </c>
       <c r="F62" s="10">
-        <v>210.87</v>
+        <v>208.29</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>265.20999999999998</v>
+        <v>258.61</v>
       </c>
       <c r="E63" s="13">
-        <v>197.37</v>
+        <v>194.4</v>
       </c>
       <c r="F63" s="13">
-        <v>207.37</v>
+        <v>204.4</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>265.24</v>
+        <v>258.67</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>264.29000000000002</v>
+        <v>257.63</v>
       </c>
       <c r="E65" s="13">
-        <v>191.76</v>
+        <v>188.79</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>260.13</v>
+        <v>253.47</v>
       </c>
       <c r="E66" s="10">
-        <v>187.69</v>
+        <v>184.72</v>
       </c>
       <c r="F66" s="10">
-        <v>197.69</v>
+        <v>194.72</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46129</v>
+        <v>46130</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>263.94</v>
+        <v>257.27</v>
       </c>
       <c r="E67" s="13">
-        <v>198.02</v>
+        <v>195.28</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,26 +1892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2171,26 +2151,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2210,6 +2191,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Tue Apr 21 04:22:39 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{ECEBC45E-0106-4CB2-9BBC-21364A845CF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{6DD4CDA3-0EEB-4076-87F6-59E070199835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>245.74</v>
+        <v>233</v>
       </c>
       <c r="E8" s="10">
-        <v>182.46</v>
+        <v>178.64</v>
       </c>
       <c r="F8" s="10">
-        <v>192.46</v>
+        <v>188.64</v>
       </c>
       <c r="G8" s="10">
-        <v>183.13</v>
+        <v>179.32</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>245.74</v>
+        <v>233</v>
       </c>
       <c r="E9" s="13">
-        <v>182.46</v>
+        <v>178.64</v>
       </c>
       <c r="F9" s="13">
-        <v>192.46</v>
+        <v>188.64</v>
       </c>
       <c r="G9" s="13">
-        <v>183.13</v>
+        <v>179.32</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>247.35</v>
+        <v>234.91</v>
       </c>
       <c r="E10" s="10">
-        <v>182.52</v>
+        <v>178.97</v>
       </c>
       <c r="F10" s="10">
-        <v>192.52</v>
+        <v>188.97</v>
       </c>
       <c r="G10" s="10">
-        <v>183.92</v>
+        <v>180.37</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>253.09</v>
+        <v>245.74</v>
       </c>
       <c r="E11" s="13">
-        <v>184.08</v>
+        <v>182.46</v>
       </c>
       <c r="F11" s="13">
-        <v>194.08</v>
+        <v>192.46</v>
       </c>
       <c r="G11" s="13">
-        <v>184.76</v>
+        <v>183.13</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>253.09</v>
+        <v>245.74</v>
       </c>
       <c r="E12" s="10">
-        <v>184.08</v>
+        <v>182.46</v>
       </c>
       <c r="F12" s="10">
-        <v>194.08</v>
+        <v>192.46</v>
       </c>
       <c r="G12" s="10">
-        <v>184.76</v>
+        <v>183.13</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>254.32</v>
+        <v>247.35</v>
       </c>
       <c r="E13" s="13">
-        <v>183.81</v>
+        <v>182.52</v>
       </c>
       <c r="F13" s="13">
-        <v>193.81</v>
+        <v>192.52</v>
       </c>
       <c r="G13" s="13">
-        <v>185.21</v>
+        <v>183.92</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>248.07</v>
+        <v>237.2</v>
       </c>
       <c r="E17" s="10">
-        <v>182.58</v>
+        <v>178.95</v>
       </c>
       <c r="F17" s="10">
-        <v>192.58</v>
+        <v>188.95</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>256.22000000000003</v>
+        <v>248.07</v>
       </c>
       <c r="E18" s="13">
-        <v>183.94</v>
+        <v>182.58</v>
       </c>
       <c r="F18" s="13">
-        <v>193.94</v>
+        <v>192.58</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>243.33</v>
+        <v>233.34</v>
       </c>
       <c r="E22" s="10">
-        <v>181.26</v>
+        <v>177.45</v>
       </c>
       <c r="F22" s="10">
-        <v>190.86</v>
+        <v>187.05</v>
       </c>
       <c r="G22" s="10">
-        <v>180.72</v>
+        <v>176.91</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>248.02</v>
+        <v>236.14</v>
       </c>
       <c r="E23" s="13">
-        <v>188.05</v>
+        <v>184.48</v>
       </c>
       <c r="F23" s="13">
-        <v>198.05</v>
+        <v>194.48</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>248.04</v>
+        <v>236.15</v>
       </c>
       <c r="E24" s="10">
-        <v>189.01</v>
+        <v>185.48</v>
       </c>
       <c r="F24" s="10">
-        <v>199.01</v>
+        <v>195.48</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>248.02</v>
+        <v>236.13</v>
       </c>
       <c r="E25" s="13">
-        <v>188.75</v>
+        <v>185.23</v>
       </c>
       <c r="F25" s="13">
-        <v>198.75</v>
+        <v>195.23</v>
       </c>
       <c r="G25" s="13">
-        <v>187.28</v>
+        <v>183.76</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>248.48</v>
+        <v>236.56</v>
       </c>
       <c r="E26" s="10">
-        <v>189.09</v>
+        <v>185.55</v>
       </c>
       <c r="F26" s="10">
-        <v>199.09</v>
+        <v>195.55</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>250.67</v>
+        <v>243.33</v>
       </c>
       <c r="E27" s="13">
-        <v>182.88</v>
+        <v>181.26</v>
       </c>
       <c r="F27" s="13">
-        <v>192.48</v>
+        <v>190.86</v>
       </c>
       <c r="G27" s="13">
-        <v>182.35</v>
+        <v>180.72</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>254.99</v>
+        <v>248.02</v>
       </c>
       <c r="E28" s="22">
-        <v>189.34</v>
+        <v>188.05</v>
       </c>
       <c r="F28" s="22">
-        <v>199.34</v>
+        <v>198.05</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>255.02</v>
+        <v>248.04</v>
       </c>
       <c r="E29" s="13">
-        <v>190.26</v>
+        <v>189.01</v>
       </c>
       <c r="F29" s="13">
-        <v>200.26</v>
+        <v>199.01</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>254.99</v>
+        <v>248.02</v>
       </c>
       <c r="E30" s="22">
-        <v>190</v>
+        <v>188.75</v>
       </c>
       <c r="F30" s="22">
-        <v>200</v>
+        <v>198.75</v>
       </c>
       <c r="G30" s="22">
-        <v>188.53</v>
+        <v>187.28</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>255.48</v>
+        <v>248.48</v>
       </c>
       <c r="E31" s="13">
-        <v>190.35</v>
+        <v>189.09</v>
       </c>
       <c r="F31" s="13">
-        <v>200.35</v>
+        <v>199.09</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>246.29</v>
+        <v>232.77</v>
       </c>
       <c r="E35" s="10">
-        <v>183.14</v>
+        <v>179.6</v>
       </c>
       <c r="F35" s="10">
-        <v>192.14</v>
+        <v>188.6</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>254.35</v>
+        <v>246.29</v>
       </c>
       <c r="E36" s="13">
-        <v>184.42</v>
+        <v>183.14</v>
       </c>
       <c r="F36" s="13">
-        <v>193.42</v>
+        <v>192.14</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>261.91000000000003</v>
+        <v>248.39</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>269.97000000000003</v>
+        <v>261.91000000000003</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>249.49</v>
+        <v>238.76</v>
       </c>
       <c r="E42" s="10">
-        <v>191.71</v>
+        <v>188.57</v>
       </c>
       <c r="F42" s="10">
-        <v>201.71</v>
+        <v>198.57</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>249.11</v>
+        <v>238.38</v>
       </c>
       <c r="E43" s="13">
-        <v>192.12</v>
+        <v>188.99</v>
       </c>
       <c r="F43" s="13">
-        <v>202.13</v>
+        <v>198.99</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>256.41000000000003</v>
+        <v>249.49</v>
       </c>
       <c r="E44" s="10">
-        <v>192.97</v>
+        <v>191.71</v>
       </c>
       <c r="F44" s="10">
-        <v>202.97</v>
+        <v>201.71</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>256.01</v>
+        <v>249.11</v>
       </c>
       <c r="E45" s="13">
-        <v>193.38</v>
+        <v>192.12</v>
       </c>
       <c r="F45" s="13">
-        <v>203.38</v>
+        <v>202.13</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>247.71</v>
+        <v>237.48</v>
       </c>
       <c r="E49" s="10">
-        <v>185.92</v>
+        <v>183.19</v>
       </c>
       <c r="F49" s="10">
-        <v>195.92</v>
+        <v>193.19</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>247.18</v>
+        <v>236.91</v>
       </c>
       <c r="E50" s="13">
-        <v>185.8</v>
+        <v>183.05</v>
       </c>
       <c r="F50" s="13">
-        <v>195.8</v>
+        <v>193.05</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>251.77</v>
+        <v>247.71</v>
       </c>
       <c r="E51" s="10">
-        <v>185.65</v>
+        <v>185.92</v>
       </c>
       <c r="F51" s="10">
-        <v>195.65</v>
+        <v>195.92</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>251.27</v>
+        <v>247.18</v>
       </c>
       <c r="E52" s="13">
-        <v>185.54</v>
+        <v>185.8</v>
       </c>
       <c r="F52" s="13">
-        <v>195.54</v>
+        <v>195.8</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>257.52999999999997</v>
+        <v>246.67</v>
       </c>
       <c r="E56" s="10">
-        <v>197.36</v>
+        <v>194.16</v>
       </c>
       <c r="F56" s="10">
-        <v>207.36</v>
+        <v>204.16</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>250.54</v>
+        <v>236.99</v>
       </c>
       <c r="E57" s="13">
-        <v>193.03</v>
+        <v>189.41</v>
       </c>
       <c r="F57" s="13">
-        <v>203.03</v>
+        <v>199.41</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>250.63</v>
+        <v>237.11</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>249.48</v>
+        <v>235.87</v>
       </c>
       <c r="E59" s="13">
-        <v>187.42</v>
+        <v>183.8</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>245.31</v>
+        <v>231.7</v>
       </c>
       <c r="E60" s="10">
-        <v>183.35</v>
+        <v>179.73</v>
       </c>
       <c r="F60" s="10">
-        <v>193.35</v>
+        <v>189.73</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>249.11</v>
+        <v>235.48</v>
       </c>
       <c r="E61" s="13">
-        <v>194.19</v>
+        <v>190.82</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>265.66000000000003</v>
+        <v>257.52999999999997</v>
       </c>
       <c r="E62" s="10">
-        <v>198.29</v>
+        <v>197.36</v>
       </c>
       <c r="F62" s="10">
-        <v>208.29</v>
+        <v>207.36</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>258.61</v>
+        <v>250.54</v>
       </c>
       <c r="E63" s="13">
-        <v>194.4</v>
+        <v>193.03</v>
       </c>
       <c r="F63" s="13">
-        <v>204.4</v>
+        <v>203.03</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>258.67</v>
+        <v>250.63</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>257.63</v>
+        <v>249.48</v>
       </c>
       <c r="E65" s="13">
-        <v>188.79</v>
+        <v>187.42</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>253.47</v>
+        <v>245.31</v>
       </c>
       <c r="E66" s="10">
-        <v>184.72</v>
+        <v>183.35</v>
       </c>
       <c r="F66" s="10">
-        <v>194.72</v>
+        <v>193.35</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46130</v>
+        <v>46133</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>257.27</v>
+        <v>249.11</v>
       </c>
       <c r="E67" s="13">
-        <v>195.28</v>
+        <v>194.19</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -2152,15 +2152,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -2169,6 +2160,15 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2192,14 +2192,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2210,6 +2202,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Wed Apr 22 04:21:07 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{6DD4CDA3-0EEB-4076-87F6-59E070199835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{37E4677C-2C50-48D7-BEB1-0952CF49F897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>233</v>
+        <v>222.74</v>
       </c>
       <c r="E8" s="10">
-        <v>178.64</v>
+        <v>176.15</v>
       </c>
       <c r="F8" s="10">
-        <v>188.64</v>
+        <v>186.15</v>
       </c>
       <c r="G8" s="10">
-        <v>179.32</v>
+        <v>176.83</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>233</v>
+        <v>222.74</v>
       </c>
       <c r="E9" s="13">
-        <v>178.64</v>
+        <v>176.15</v>
       </c>
       <c r="F9" s="13">
-        <v>188.64</v>
+        <v>186.15</v>
       </c>
       <c r="G9" s="13">
-        <v>179.32</v>
+        <v>176.83</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>234.91</v>
+        <v>223.8</v>
       </c>
       <c r="E10" s="10">
-        <v>178.97</v>
+        <v>176.71</v>
       </c>
       <c r="F10" s="10">
-        <v>188.97</v>
+        <v>186.71</v>
       </c>
       <c r="G10" s="10">
-        <v>180.37</v>
+        <v>178.1</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>245.74</v>
+        <v>233</v>
       </c>
       <c r="E11" s="13">
-        <v>182.46</v>
+        <v>178.64</v>
       </c>
       <c r="F11" s="13">
-        <v>192.46</v>
+        <v>188.64</v>
       </c>
       <c r="G11" s="13">
-        <v>183.13</v>
+        <v>179.32</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>245.74</v>
+        <v>233</v>
       </c>
       <c r="E12" s="10">
-        <v>182.46</v>
+        <v>178.64</v>
       </c>
       <c r="F12" s="10">
-        <v>192.46</v>
+        <v>188.64</v>
       </c>
       <c r="G12" s="10">
-        <v>183.13</v>
+        <v>179.32</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>247.35</v>
+        <v>234.91</v>
       </c>
       <c r="E13" s="13">
-        <v>182.52</v>
+        <v>178.97</v>
       </c>
       <c r="F13" s="13">
-        <v>192.52</v>
+        <v>188.97</v>
       </c>
       <c r="G13" s="13">
-        <v>183.92</v>
+        <v>180.37</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>237.2</v>
+        <v>227.14</v>
       </c>
       <c r="E17" s="10">
-        <v>178.95</v>
+        <v>176.65</v>
       </c>
       <c r="F17" s="10">
-        <v>188.95</v>
+        <v>186.65</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>248.07</v>
+        <v>237.2</v>
       </c>
       <c r="E18" s="13">
-        <v>182.58</v>
+        <v>178.95</v>
       </c>
       <c r="F18" s="13">
-        <v>192.58</v>
+        <v>188.95</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>233.34</v>
+        <v>223.63</v>
       </c>
       <c r="E22" s="10">
-        <v>177.45</v>
+        <v>176.06</v>
       </c>
       <c r="F22" s="10">
-        <v>187.05</v>
+        <v>185.66</v>
       </c>
       <c r="G22" s="10">
-        <v>176.91</v>
+        <v>175.52</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>236.14</v>
+        <v>227.22</v>
       </c>
       <c r="E23" s="13">
-        <v>184.48</v>
+        <v>181.66</v>
       </c>
       <c r="F23" s="13">
-        <v>194.48</v>
+        <v>191.66</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>236.15</v>
+        <v>227.23</v>
       </c>
       <c r="E24" s="10">
-        <v>185.48</v>
+        <v>182.68</v>
       </c>
       <c r="F24" s="10">
-        <v>195.48</v>
+        <v>192.68</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>236.13</v>
+        <v>227.21</v>
       </c>
       <c r="E25" s="13">
-        <v>185.23</v>
+        <v>182.43</v>
       </c>
       <c r="F25" s="13">
-        <v>195.23</v>
+        <v>192.43</v>
       </c>
       <c r="G25" s="13">
-        <v>183.76</v>
+        <v>180.96</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>236.56</v>
+        <v>226.53</v>
       </c>
       <c r="E26" s="10">
-        <v>185.55</v>
+        <v>184.39</v>
       </c>
       <c r="F26" s="10">
-        <v>195.55</v>
+        <v>194.39</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>243.33</v>
+        <v>233.34</v>
       </c>
       <c r="E27" s="13">
-        <v>181.26</v>
+        <v>177.45</v>
       </c>
       <c r="F27" s="13">
-        <v>190.86</v>
+        <v>187.05</v>
       </c>
       <c r="G27" s="13">
-        <v>180.72</v>
+        <v>176.91</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>248.02</v>
+        <v>236.14</v>
       </c>
       <c r="E28" s="22">
-        <v>188.05</v>
+        <v>184.48</v>
       </c>
       <c r="F28" s="22">
-        <v>198.05</v>
+        <v>194.48</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>248.04</v>
+        <v>236.15</v>
       </c>
       <c r="E29" s="13">
-        <v>189.01</v>
+        <v>185.48</v>
       </c>
       <c r="F29" s="13">
-        <v>199.01</v>
+        <v>195.48</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>248.02</v>
+        <v>236.13</v>
       </c>
       <c r="E30" s="22">
-        <v>188.75</v>
+        <v>185.23</v>
       </c>
       <c r="F30" s="22">
-        <v>198.75</v>
+        <v>195.23</v>
       </c>
       <c r="G30" s="22">
-        <v>187.28</v>
+        <v>183.76</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>248.48</v>
+        <v>236.56</v>
       </c>
       <c r="E31" s="13">
-        <v>189.09</v>
+        <v>185.55</v>
       </c>
       <c r="F31" s="13">
-        <v>199.09</v>
+        <v>195.55</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>232.77</v>
+        <v>222.21</v>
       </c>
       <c r="E35" s="10">
-        <v>179.6</v>
+        <v>176.79</v>
       </c>
       <c r="F35" s="10">
-        <v>188.6</v>
+        <v>185.79</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>246.29</v>
+        <v>232.77</v>
       </c>
       <c r="E36" s="13">
-        <v>183.14</v>
+        <v>179.6</v>
       </c>
       <c r="F36" s="13">
-        <v>192.14</v>
+        <v>188.6</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>248.39</v>
+        <v>237.83</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>261.91000000000003</v>
+        <v>248.39</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>238.76</v>
+        <v>229.87</v>
       </c>
       <c r="E42" s="10">
-        <v>188.57</v>
+        <v>185.13</v>
       </c>
       <c r="F42" s="10">
-        <v>198.57</v>
+        <v>195.13</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>238.38</v>
+        <v>229.5</v>
       </c>
       <c r="E43" s="13">
-        <v>188.99</v>
+        <v>185.55</v>
       </c>
       <c r="F43" s="13">
-        <v>198.99</v>
+        <v>195.55</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>249.49</v>
+        <v>238.76</v>
       </c>
       <c r="E44" s="10">
-        <v>191.71</v>
+        <v>188.57</v>
       </c>
       <c r="F44" s="10">
-        <v>201.71</v>
+        <v>198.57</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>249.11</v>
+        <v>238.38</v>
       </c>
       <c r="E45" s="13">
-        <v>192.12</v>
+        <v>188.99</v>
       </c>
       <c r="F45" s="13">
-        <v>202.13</v>
+        <v>198.99</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>237.48</v>
+        <v>228.24</v>
       </c>
       <c r="E49" s="10">
-        <v>183.19</v>
+        <v>179.5</v>
       </c>
       <c r="F49" s="10">
-        <v>193.19</v>
+        <v>189.5</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>236.91</v>
+        <v>227.64</v>
       </c>
       <c r="E50" s="13">
-        <v>183.05</v>
+        <v>179.35</v>
       </c>
       <c r="F50" s="13">
-        <v>193.05</v>
+        <v>189.35</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>247.71</v>
+        <v>237.48</v>
       </c>
       <c r="E51" s="10">
-        <v>185.92</v>
+        <v>183.19</v>
       </c>
       <c r="F51" s="10">
-        <v>195.92</v>
+        <v>193.19</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>247.18</v>
+        <v>236.91</v>
       </c>
       <c r="E52" s="13">
-        <v>185.8</v>
+        <v>183.05</v>
       </c>
       <c r="F52" s="13">
-        <v>195.8</v>
+        <v>193.05</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>246.67</v>
+        <v>236.6</v>
       </c>
       <c r="E56" s="10">
-        <v>194.16</v>
+        <v>191.32</v>
       </c>
       <c r="F56" s="10">
-        <v>204.16</v>
+        <v>201.32</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>236.99</v>
+        <v>226.97</v>
       </c>
       <c r="E57" s="13">
-        <v>189.41</v>
+        <v>186.33</v>
       </c>
       <c r="F57" s="13">
-        <v>199.41</v>
+        <v>196.33</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>237.11</v>
+        <v>227.11</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>235.87</v>
+        <v>225.82</v>
       </c>
       <c r="E59" s="13">
-        <v>183.8</v>
+        <v>180.72</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>231.7</v>
+        <v>221.64</v>
       </c>
       <c r="E60" s="10">
-        <v>179.73</v>
+        <v>176.65</v>
       </c>
       <c r="F60" s="10">
-        <v>189.73</v>
+        <v>186.65</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>235.48</v>
+        <v>225.42</v>
       </c>
       <c r="E61" s="13">
-        <v>190.82</v>
+        <v>187.89</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>257.52999999999997</v>
+        <v>246.67</v>
       </c>
       <c r="E62" s="10">
-        <v>197.36</v>
+        <v>194.16</v>
       </c>
       <c r="F62" s="10">
-        <v>207.36</v>
+        <v>204.16</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>250.54</v>
+        <v>236.99</v>
       </c>
       <c r="E63" s="13">
-        <v>193.03</v>
+        <v>189.41</v>
       </c>
       <c r="F63" s="13">
-        <v>203.03</v>
+        <v>199.41</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>250.63</v>
+        <v>237.11</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>249.48</v>
+        <v>235.87</v>
       </c>
       <c r="E65" s="13">
-        <v>187.42</v>
+        <v>183.8</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>245.31</v>
+        <v>231.7</v>
       </c>
       <c r="E66" s="10">
-        <v>183.35</v>
+        <v>179.73</v>
       </c>
       <c r="F66" s="10">
-        <v>193.35</v>
+        <v>189.73</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46133</v>
+        <v>46134</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>249.11</v>
+        <v>235.48</v>
       </c>
       <c r="E67" s="13">
-        <v>194.19</v>
+        <v>190.82</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,6 +1892,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2151,7 +2160,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -2162,16 +2171,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2191,7 +2199,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2202,14 +2210,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Thu Apr 23 04:25:07 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{37E4677C-2C50-48D7-BEB1-0952CF49F897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{D4423F0A-01F8-471A-970D-AE925447E857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>222.74</v>
+        <v>221.4</v>
       </c>
       <c r="E8" s="10">
-        <v>176.15</v>
+        <v>176.74</v>
       </c>
       <c r="F8" s="10">
-        <v>186.15</v>
+        <v>186.74</v>
       </c>
       <c r="G8" s="10">
-        <v>176.83</v>
+        <v>177.42</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>222.74</v>
+        <v>221.4</v>
       </c>
       <c r="E9" s="13">
-        <v>176.15</v>
+        <v>176.74</v>
       </c>
       <c r="F9" s="13">
-        <v>186.15</v>
+        <v>186.74</v>
       </c>
       <c r="G9" s="13">
-        <v>176.83</v>
+        <v>177.42</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>223.8</v>
+        <v>222.53</v>
       </c>
       <c r="E10" s="10">
-        <v>176.71</v>
+        <v>177.36</v>
       </c>
       <c r="F10" s="10">
-        <v>186.71</v>
+        <v>187.36</v>
       </c>
       <c r="G10" s="10">
-        <v>178.1</v>
+        <v>178.76</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>233</v>
+        <v>222.74</v>
       </c>
       <c r="E11" s="13">
-        <v>178.64</v>
+        <v>176.15</v>
       </c>
       <c r="F11" s="13">
-        <v>188.64</v>
+        <v>186.15</v>
       </c>
       <c r="G11" s="13">
-        <v>179.32</v>
+        <v>176.83</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>233</v>
+        <v>222.74</v>
       </c>
       <c r="E12" s="10">
-        <v>178.64</v>
+        <v>176.15</v>
       </c>
       <c r="F12" s="10">
-        <v>188.64</v>
+        <v>186.15</v>
       </c>
       <c r="G12" s="10">
-        <v>179.32</v>
+        <v>176.83</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>234.91</v>
+        <v>223.8</v>
       </c>
       <c r="E13" s="13">
-        <v>178.97</v>
+        <v>176.71</v>
       </c>
       <c r="F13" s="13">
-        <v>188.97</v>
+        <v>186.71</v>
       </c>
       <c r="G13" s="13">
-        <v>180.37</v>
+        <v>178.1</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>227.14</v>
+        <v>225.85</v>
       </c>
       <c r="E17" s="10">
-        <v>176.65</v>
+        <v>177.28</v>
       </c>
       <c r="F17" s="10">
-        <v>186.65</v>
+        <v>187.28</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>237.2</v>
+        <v>227.14</v>
       </c>
       <c r="E18" s="13">
-        <v>178.95</v>
+        <v>176.65</v>
       </c>
       <c r="F18" s="13">
-        <v>188.95</v>
+        <v>186.65</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>223.63</v>
+        <v>222.3</v>
       </c>
       <c r="E22" s="10">
-        <v>176.06</v>
+        <v>174.45</v>
       </c>
       <c r="F22" s="10">
-        <v>185.66</v>
+        <v>184.05</v>
       </c>
       <c r="G22" s="10">
-        <v>175.52</v>
+        <v>173.91</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>227.22</v>
+        <v>225.95</v>
       </c>
       <c r="E23" s="13">
-        <v>181.66</v>
+        <v>179.02</v>
       </c>
       <c r="F23" s="13">
-        <v>191.66</v>
+        <v>189.02</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>227.23</v>
+        <v>225.96</v>
       </c>
       <c r="E24" s="10">
-        <v>182.68</v>
+        <v>180.05</v>
       </c>
       <c r="F24" s="10">
-        <v>192.68</v>
+        <v>190.05</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>227.21</v>
+        <v>225.95</v>
       </c>
       <c r="E25" s="13">
-        <v>182.43</v>
+        <v>179.8</v>
       </c>
       <c r="F25" s="13">
-        <v>192.43</v>
+        <v>189.8</v>
       </c>
       <c r="G25" s="13">
-        <v>180.96</v>
+        <v>178.33</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>226.53</v>
+        <v>225.25</v>
       </c>
       <c r="E26" s="10">
-        <v>184.39</v>
+        <v>181.77</v>
       </c>
       <c r="F26" s="10">
-        <v>194.39</v>
+        <v>191.77</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>233.34</v>
+        <v>223.63</v>
       </c>
       <c r="E27" s="13">
-        <v>177.45</v>
+        <v>176.06</v>
       </c>
       <c r="F27" s="13">
-        <v>187.05</v>
+        <v>185.66</v>
       </c>
       <c r="G27" s="13">
-        <v>176.91</v>
+        <v>175.52</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>236.14</v>
+        <v>227.22</v>
       </c>
       <c r="E28" s="22">
-        <v>184.48</v>
+        <v>181.66</v>
       </c>
       <c r="F28" s="22">
-        <v>194.48</v>
+        <v>191.66</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>236.15</v>
+        <v>227.23</v>
       </c>
       <c r="E29" s="13">
-        <v>185.48</v>
+        <v>182.68</v>
       </c>
       <c r="F29" s="13">
-        <v>195.48</v>
+        <v>192.68</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>236.13</v>
+        <v>227.21</v>
       </c>
       <c r="E30" s="22">
-        <v>185.23</v>
+        <v>182.43</v>
       </c>
       <c r="F30" s="22">
-        <v>195.23</v>
+        <v>192.43</v>
       </c>
       <c r="G30" s="22">
-        <v>183.76</v>
+        <v>180.96</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>236.56</v>
+        <v>226.53</v>
       </c>
       <c r="E31" s="13">
-        <v>185.55</v>
+        <v>184.39</v>
       </c>
       <c r="F31" s="13">
-        <v>195.55</v>
+        <v>194.39</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>222.21</v>
+        <v>220.94</v>
       </c>
       <c r="E35" s="10">
-        <v>176.79</v>
+        <v>174.14</v>
       </c>
       <c r="F35" s="10">
-        <v>185.79</v>
+        <v>183.14</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>232.77</v>
+        <v>222.21</v>
       </c>
       <c r="E36" s="13">
-        <v>179.6</v>
+        <v>176.79</v>
       </c>
       <c r="F36" s="13">
-        <v>188.6</v>
+        <v>185.79</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>237.83</v>
+        <v>236.56</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>248.39</v>
+        <v>237.83</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>229.87</v>
+        <v>228.61</v>
       </c>
       <c r="E42" s="10">
-        <v>185.13</v>
+        <v>182.81</v>
       </c>
       <c r="F42" s="10">
-        <v>195.13</v>
+        <v>192.81</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>229.5</v>
+        <v>228.25</v>
       </c>
       <c r="E43" s="13">
-        <v>185.55</v>
+        <v>183.23</v>
       </c>
       <c r="F43" s="13">
-        <v>195.55</v>
+        <v>193.23</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>238.76</v>
+        <v>229.87</v>
       </c>
       <c r="E44" s="10">
-        <v>188.57</v>
+        <v>185.13</v>
       </c>
       <c r="F44" s="10">
-        <v>198.57</v>
+        <v>195.13</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>238.38</v>
+        <v>229.5</v>
       </c>
       <c r="E45" s="13">
-        <v>188.99</v>
+        <v>185.55</v>
       </c>
       <c r="F45" s="13">
-        <v>198.99</v>
+        <v>195.55</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>228.24</v>
+        <v>222.94</v>
       </c>
       <c r="E49" s="10">
-        <v>179.5</v>
+        <v>175</v>
       </c>
       <c r="F49" s="10">
-        <v>189.5</v>
+        <v>185</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>227.64</v>
+        <v>222.31</v>
       </c>
       <c r="E50" s="13">
-        <v>179.35</v>
+        <v>174.84</v>
       </c>
       <c r="F50" s="13">
-        <v>189.35</v>
+        <v>184.84</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>237.48</v>
+        <v>228.24</v>
       </c>
       <c r="E51" s="10">
-        <v>183.19</v>
+        <v>179.5</v>
       </c>
       <c r="F51" s="10">
-        <v>193.19</v>
+        <v>189.5</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>236.91</v>
+        <v>227.64</v>
       </c>
       <c r="E52" s="13">
-        <v>183.05</v>
+        <v>179.35</v>
       </c>
       <c r="F52" s="13">
-        <v>193.05</v>
+        <v>189.35</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>236.6</v>
+        <v>235.31</v>
       </c>
       <c r="E56" s="10">
-        <v>191.32</v>
+        <v>188.77</v>
       </c>
       <c r="F56" s="10">
-        <v>201.32</v>
+        <v>198.77</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>226.97</v>
+        <v>225.7</v>
       </c>
       <c r="E57" s="13">
-        <v>186.33</v>
+        <v>183.66</v>
       </c>
       <c r="F57" s="13">
-        <v>196.33</v>
+        <v>193.66</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>227.11</v>
+        <v>225.85</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>225.82</v>
+        <v>224.53</v>
       </c>
       <c r="E59" s="13">
-        <v>180.72</v>
+        <v>178.05</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>221.64</v>
+        <v>220.34</v>
       </c>
       <c r="E60" s="10">
-        <v>176.65</v>
+        <v>173.98</v>
       </c>
       <c r="F60" s="10">
-        <v>186.65</v>
+        <v>183.98</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>225.42</v>
+        <v>224.13</v>
       </c>
       <c r="E61" s="13">
-        <v>187.89</v>
+        <v>185.3</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>246.67</v>
+        <v>236.6</v>
       </c>
       <c r="E62" s="10">
-        <v>194.16</v>
+        <v>191.32</v>
       </c>
       <c r="F62" s="10">
-        <v>204.16</v>
+        <v>201.32</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>236.99</v>
+        <v>226.97</v>
       </c>
       <c r="E63" s="13">
-        <v>189.41</v>
+        <v>186.33</v>
       </c>
       <c r="F63" s="13">
-        <v>199.41</v>
+        <v>196.33</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>237.11</v>
+        <v>227.11</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>235.87</v>
+        <v>225.82</v>
       </c>
       <c r="E65" s="13">
-        <v>183.8</v>
+        <v>180.72</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>231.7</v>
+        <v>221.64</v>
       </c>
       <c r="E66" s="10">
-        <v>179.73</v>
+        <v>176.65</v>
       </c>
       <c r="F66" s="10">
-        <v>189.73</v>
+        <v>186.65</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>235.48</v>
+        <v>225.42</v>
       </c>
       <c r="E67" s="13">
-        <v>190.82</v>
+        <v>187.89</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,15 +1892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2160,7 +2151,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -2171,15 +2162,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2199,7 +2191,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2210,6 +2202,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Fri Apr 24 04:28:52 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{D4423F0A-01F8-471A-970D-AE925447E857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{102C88C3-B25E-4B31-AB77-916CD5680C22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" concurrentManualCount="12"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>221.4</v>
+        <v>221.48</v>
       </c>
       <c r="E8" s="10">
-        <v>176.74</v>
+        <v>175.26</v>
       </c>
       <c r="F8" s="10">
-        <v>186.74</v>
+        <v>185.26</v>
       </c>
       <c r="G8" s="10">
-        <v>177.42</v>
+        <v>175.94</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>221.4</v>
+        <v>221.48</v>
       </c>
       <c r="E9" s="13">
-        <v>176.74</v>
+        <v>175.26</v>
       </c>
       <c r="F9" s="13">
-        <v>186.74</v>
+        <v>185.26</v>
       </c>
       <c r="G9" s="13">
-        <v>177.42</v>
+        <v>175.94</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>222.53</v>
+        <v>222.46</v>
       </c>
       <c r="E10" s="10">
-        <v>177.36</v>
+        <v>175.76</v>
       </c>
       <c r="F10" s="10">
-        <v>187.36</v>
+        <v>185.76</v>
       </c>
       <c r="G10" s="10">
-        <v>178.76</v>
+        <v>177.16</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>222.74</v>
+        <v>221.4</v>
       </c>
       <c r="E11" s="13">
-        <v>176.15</v>
+        <v>176.74</v>
       </c>
       <c r="F11" s="13">
-        <v>186.15</v>
+        <v>186.74</v>
       </c>
       <c r="G11" s="13">
-        <v>176.83</v>
+        <v>177.42</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>222.74</v>
+        <v>221.4</v>
       </c>
       <c r="E12" s="10">
-        <v>176.15</v>
+        <v>176.74</v>
       </c>
       <c r="F12" s="10">
-        <v>186.15</v>
+        <v>186.74</v>
       </c>
       <c r="G12" s="10">
-        <v>176.83</v>
+        <v>177.42</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>223.8</v>
+        <v>222.53</v>
       </c>
       <c r="E13" s="13">
-        <v>176.71</v>
+        <v>177.36</v>
       </c>
       <c r="F13" s="13">
-        <v>186.71</v>
+        <v>187.36</v>
       </c>
       <c r="G13" s="13">
-        <v>178.1</v>
+        <v>178.76</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>225.85</v>
+        <v>225.8</v>
       </c>
       <c r="E17" s="10">
-        <v>177.28</v>
+        <v>179</v>
       </c>
       <c r="F17" s="10">
-        <v>187.28</v>
+        <v>189</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>227.14</v>
+        <v>225.85</v>
       </c>
       <c r="E18" s="13">
-        <v>176.65</v>
+        <v>177.28</v>
       </c>
       <c r="F18" s="13">
-        <v>186.65</v>
+        <v>187.28</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>222.3</v>
+        <v>222.37</v>
       </c>
       <c r="E22" s="10">
-        <v>174.45</v>
+        <v>174.84</v>
       </c>
       <c r="F22" s="10">
-        <v>184.05</v>
+        <v>184.44</v>
       </c>
       <c r="G22" s="10">
-        <v>173.91</v>
+        <v>174.3</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>225.95</v>
+        <v>225.89</v>
       </c>
       <c r="E23" s="13">
-        <v>179.02</v>
+        <v>179.62</v>
       </c>
       <c r="F23" s="13">
-        <v>189.02</v>
+        <v>189.62</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>225.96</v>
+        <v>225.9</v>
       </c>
       <c r="E24" s="10">
-        <v>180.05</v>
+        <v>180.64</v>
       </c>
       <c r="F24" s="10">
-        <v>190.05</v>
+        <v>190.64</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>225.95</v>
+        <v>225.88</v>
       </c>
       <c r="E25" s="13">
-        <v>179.8</v>
+        <v>180.4</v>
       </c>
       <c r="F25" s="13">
-        <v>189.8</v>
+        <v>190.4</v>
       </c>
       <c r="G25" s="13">
-        <v>178.33</v>
+        <v>178.93</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>225.25</v>
+        <v>225.19</v>
       </c>
       <c r="E26" s="10">
-        <v>181.77</v>
+        <v>182.37</v>
       </c>
       <c r="F26" s="10">
-        <v>191.77</v>
+        <v>192.37</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>223.63</v>
+        <v>222.3</v>
       </c>
       <c r="E27" s="13">
-        <v>176.06</v>
+        <v>174.45</v>
       </c>
       <c r="F27" s="13">
-        <v>185.66</v>
+        <v>184.05</v>
       </c>
       <c r="G27" s="13">
-        <v>175.52</v>
+        <v>173.91</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>227.22</v>
+        <v>225.95</v>
       </c>
       <c r="E28" s="22">
-        <v>181.66</v>
+        <v>179.02</v>
       </c>
       <c r="F28" s="22">
-        <v>191.66</v>
+        <v>189.02</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>227.23</v>
+        <v>225.96</v>
       </c>
       <c r="E29" s="13">
-        <v>182.68</v>
+        <v>180.05</v>
       </c>
       <c r="F29" s="13">
-        <v>192.68</v>
+        <v>190.05</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>227.21</v>
+        <v>225.95</v>
       </c>
       <c r="E30" s="22">
-        <v>182.43</v>
+        <v>179.8</v>
       </c>
       <c r="F30" s="22">
-        <v>192.43</v>
+        <v>189.8</v>
       </c>
       <c r="G30" s="22">
-        <v>180.96</v>
+        <v>178.33</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>226.53</v>
+        <v>225.25</v>
       </c>
       <c r="E31" s="13">
-        <v>184.39</v>
+        <v>181.77</v>
       </c>
       <c r="F31" s="13">
-        <v>194.39</v>
+        <v>191.77</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>220.94</v>
+        <v>220.88</v>
       </c>
       <c r="E35" s="10">
-        <v>174.14</v>
+        <v>170.34</v>
       </c>
       <c r="F35" s="10">
-        <v>183.14</v>
+        <v>179.34</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>222.21</v>
+        <v>220.94</v>
       </c>
       <c r="E36" s="13">
-        <v>176.79</v>
+        <v>174.14</v>
       </c>
       <c r="F36" s="13">
-        <v>185.79</v>
+        <v>183.14</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>236.56</v>
+        <v>236.5</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>237.83</v>
+        <v>236.56</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>228.61</v>
+        <v>228.54</v>
       </c>
       <c r="E42" s="10">
-        <v>182.81</v>
+        <v>181.67</v>
       </c>
       <c r="F42" s="10">
-        <v>192.81</v>
+        <v>191.67</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>228.25</v>
+        <v>228.18</v>
       </c>
       <c r="E43" s="13">
-        <v>183.23</v>
+        <v>182.08</v>
       </c>
       <c r="F43" s="13">
-        <v>193.23</v>
+        <v>192.08</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>229.87</v>
+        <v>228.61</v>
       </c>
       <c r="E44" s="10">
-        <v>185.13</v>
+        <v>182.81</v>
       </c>
       <c r="F44" s="10">
-        <v>195.13</v>
+        <v>192.81</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>229.5</v>
+        <v>228.25</v>
       </c>
       <c r="E45" s="13">
-        <v>185.55</v>
+        <v>183.23</v>
       </c>
       <c r="F45" s="13">
-        <v>195.55</v>
+        <v>193.23</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>222.94</v>
+        <v>221.57</v>
       </c>
       <c r="E49" s="10">
-        <v>175</v>
+        <v>173.98</v>
       </c>
       <c r="F49" s="10">
-        <v>185</v>
+        <v>183.98</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>222.31</v>
+        <v>220.93</v>
       </c>
       <c r="E50" s="13">
-        <v>174.84</v>
+        <v>173.82</v>
       </c>
       <c r="F50" s="13">
-        <v>184.84</v>
+        <v>183.82</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>228.24</v>
+        <v>222.94</v>
       </c>
       <c r="E51" s="10">
-        <v>179.5</v>
+        <v>175</v>
       </c>
       <c r="F51" s="10">
-        <v>189.5</v>
+        <v>185</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>227.64</v>
+        <v>222.31</v>
       </c>
       <c r="E52" s="13">
-        <v>179.35</v>
+        <v>174.84</v>
       </c>
       <c r="F52" s="13">
-        <v>189.35</v>
+        <v>184.84</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>235.31</v>
+        <v>235.26</v>
       </c>
       <c r="E56" s="10">
-        <v>188.77</v>
+        <v>189.3</v>
       </c>
       <c r="F56" s="10">
-        <v>198.77</v>
+        <v>199.3</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>225.7</v>
+        <v>225.64</v>
       </c>
       <c r="E57" s="13">
-        <v>183.66</v>
+        <v>184.27</v>
       </c>
       <c r="F57" s="13">
-        <v>193.66</v>
+        <v>194.27</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>225.85</v>
+        <v>225.78</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>224.53</v>
+        <v>224.48</v>
       </c>
       <c r="E59" s="13">
-        <v>178.05</v>
+        <v>178.66</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>220.34</v>
+        <v>220.3</v>
       </c>
       <c r="E60" s="10">
-        <v>173.98</v>
+        <v>174.59</v>
       </c>
       <c r="F60" s="10">
-        <v>183.98</v>
+        <v>184.59</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>224.13</v>
+        <v>224.08</v>
       </c>
       <c r="E61" s="13">
-        <v>185.3</v>
+        <v>185.87</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>236.6</v>
+        <v>235.31</v>
       </c>
       <c r="E62" s="10">
-        <v>191.32</v>
+        <v>188.77</v>
       </c>
       <c r="F62" s="10">
-        <v>201.32</v>
+        <v>198.77</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>226.97</v>
+        <v>225.7</v>
       </c>
       <c r="E63" s="13">
-        <v>186.33</v>
+        <v>183.66</v>
       </c>
       <c r="F63" s="13">
-        <v>196.33</v>
+        <v>193.66</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>227.11</v>
+        <v>225.85</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>225.82</v>
+        <v>224.53</v>
       </c>
       <c r="E65" s="13">
-        <v>180.72</v>
+        <v>178.05</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>221.64</v>
+        <v>220.34</v>
       </c>
       <c r="E66" s="10">
-        <v>176.65</v>
+        <v>173.98</v>
       </c>
       <c r="F66" s="10">
-        <v>186.65</v>
+        <v>183.98</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>225.42</v>
+        <v>224.13</v>
       </c>
       <c r="E67" s="13">
-        <v>187.89</v>
+        <v>185.3</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,6 +1892,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2151,27 +2171,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2191,25 +2210,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Mon Apr 27 04:43:44 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{102C88C3-B25E-4B31-AB77-916CD5680C22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{C61E42DD-FAA2-4F68-B42E-A6AA953CF448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" concurrentManualCount="12"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>221.48</v>
+        <v>220.04</v>
       </c>
       <c r="E8" s="10">
-        <v>175.26</v>
+        <v>173.42</v>
       </c>
       <c r="F8" s="10">
-        <v>185.26</v>
+        <v>183.42</v>
       </c>
       <c r="G8" s="10">
-        <v>175.94</v>
+        <v>174.1</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>221.48</v>
+        <v>220.04</v>
       </c>
       <c r="E9" s="13">
-        <v>175.26</v>
+        <v>173.42</v>
       </c>
       <c r="F9" s="13">
-        <v>185.26</v>
+        <v>183.42</v>
       </c>
       <c r="G9" s="13">
-        <v>175.94</v>
+        <v>174.1</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>222.46</v>
+        <v>220.9</v>
       </c>
       <c r="E10" s="10">
-        <v>175.76</v>
+        <v>173.81</v>
       </c>
       <c r="F10" s="10">
-        <v>185.76</v>
+        <v>183.81</v>
       </c>
       <c r="G10" s="10">
-        <v>177.16</v>
+        <v>175.21</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>221.4</v>
+        <v>221.48</v>
       </c>
       <c r="E11" s="13">
-        <v>176.74</v>
+        <v>175.26</v>
       </c>
       <c r="F11" s="13">
-        <v>186.74</v>
+        <v>185.26</v>
       </c>
       <c r="G11" s="13">
-        <v>177.42</v>
+        <v>175.94</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>221.4</v>
+        <v>221.48</v>
       </c>
       <c r="E12" s="10">
-        <v>176.74</v>
+        <v>175.26</v>
       </c>
       <c r="F12" s="10">
-        <v>186.74</v>
+        <v>185.26</v>
       </c>
       <c r="G12" s="10">
-        <v>177.42</v>
+        <v>175.94</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>222.53</v>
+        <v>222.46</v>
       </c>
       <c r="E13" s="13">
-        <v>177.36</v>
+        <v>175.76</v>
       </c>
       <c r="F13" s="13">
-        <v>187.36</v>
+        <v>185.76</v>
       </c>
       <c r="G13" s="13">
-        <v>178.76</v>
+        <v>177.16</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>225.8</v>
+        <v>224.25</v>
       </c>
       <c r="E17" s="10">
-        <v>179</v>
+        <v>178.71</v>
       </c>
       <c r="F17" s="10">
-        <v>189</v>
+        <v>188.71</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>225.85</v>
+        <v>225.8</v>
       </c>
       <c r="E18" s="13">
-        <v>177.28</v>
+        <v>179</v>
       </c>
       <c r="F18" s="13">
-        <v>187.28</v>
+        <v>189</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>222.37</v>
+        <v>220.93</v>
       </c>
       <c r="E22" s="10">
-        <v>174.84</v>
+        <v>174.1</v>
       </c>
       <c r="F22" s="10">
-        <v>184.44</v>
+        <v>183.7</v>
       </c>
       <c r="G22" s="10">
-        <v>174.3</v>
+        <v>173.56</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>225.89</v>
+        <v>225.42</v>
       </c>
       <c r="E23" s="13">
-        <v>179.62</v>
+        <v>180.42</v>
       </c>
       <c r="F23" s="13">
-        <v>189.62</v>
+        <v>190.42</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>225.9</v>
+        <v>225.43</v>
       </c>
       <c r="E24" s="10">
-        <v>180.64</v>
+        <v>181.43</v>
       </c>
       <c r="F24" s="10">
-        <v>190.64</v>
+        <v>191.43</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>225.88</v>
+        <v>225.42</v>
       </c>
       <c r="E25" s="13">
-        <v>180.4</v>
+        <v>181.19</v>
       </c>
       <c r="F25" s="13">
-        <v>190.4</v>
+        <v>191.19</v>
       </c>
       <c r="G25" s="13">
-        <v>178.93</v>
+        <v>179.72</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>225.19</v>
+        <v>224.73</v>
       </c>
       <c r="E26" s="10">
-        <v>182.37</v>
+        <v>183.17</v>
       </c>
       <c r="F26" s="10">
-        <v>192.37</v>
+        <v>193.17</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>222.3</v>
+        <v>222.37</v>
       </c>
       <c r="E27" s="13">
-        <v>174.45</v>
+        <v>174.84</v>
       </c>
       <c r="F27" s="13">
-        <v>184.05</v>
+        <v>184.44</v>
       </c>
       <c r="G27" s="13">
-        <v>173.91</v>
+        <v>174.3</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>225.95</v>
+        <v>225.89</v>
       </c>
       <c r="E28" s="22">
-        <v>179.02</v>
+        <v>179.62</v>
       </c>
       <c r="F28" s="22">
-        <v>189.02</v>
+        <v>189.62</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>225.96</v>
+        <v>225.9</v>
       </c>
       <c r="E29" s="13">
-        <v>180.05</v>
+        <v>180.64</v>
       </c>
       <c r="F29" s="13">
-        <v>190.05</v>
+        <v>190.64</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>225.95</v>
+        <v>225.88</v>
       </c>
       <c r="E30" s="22">
-        <v>179.8</v>
+        <v>180.4</v>
       </c>
       <c r="F30" s="22">
-        <v>189.8</v>
+        <v>190.4</v>
       </c>
       <c r="G30" s="22">
-        <v>178.33</v>
+        <v>178.93</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>225.25</v>
+        <v>225.19</v>
       </c>
       <c r="E31" s="13">
-        <v>181.77</v>
+        <v>182.37</v>
       </c>
       <c r="F31" s="13">
-        <v>191.77</v>
+        <v>192.37</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>220.88</v>
+        <v>219.31</v>
       </c>
       <c r="E35" s="10">
-        <v>170.34</v>
+        <v>169.49</v>
       </c>
       <c r="F35" s="10">
-        <v>179.34</v>
+        <v>178.49</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>220.94</v>
+        <v>220.88</v>
       </c>
       <c r="E36" s="13">
-        <v>174.14</v>
+        <v>170.34</v>
       </c>
       <c r="F36" s="13">
-        <v>183.14</v>
+        <v>179.34</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>236.5</v>
+        <v>234.93</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>236.56</v>
+        <v>236.5</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>228.54</v>
+        <v>229.16</v>
       </c>
       <c r="E42" s="10">
-        <v>181.67</v>
+        <v>179.5</v>
       </c>
       <c r="F42" s="10">
-        <v>191.67</v>
+        <v>189.5</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>228.18</v>
+        <v>228.79</v>
       </c>
       <c r="E43" s="13">
-        <v>182.08</v>
+        <v>179.91</v>
       </c>
       <c r="F43" s="13">
-        <v>192.08</v>
+        <v>189.91</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>228.61</v>
+        <v>228.54</v>
       </c>
       <c r="E44" s="10">
-        <v>182.81</v>
+        <v>181.67</v>
       </c>
       <c r="F44" s="10">
-        <v>192.81</v>
+        <v>191.67</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>228.25</v>
+        <v>228.18</v>
       </c>
       <c r="E45" s="13">
-        <v>183.23</v>
+        <v>182.08</v>
       </c>
       <c r="F45" s="13">
-        <v>193.23</v>
+        <v>192.08</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>221.57</v>
+        <v>219.38</v>
       </c>
       <c r="E49" s="10">
-        <v>173.98</v>
+        <v>172.74</v>
       </c>
       <c r="F49" s="10">
-        <v>183.98</v>
+        <v>182.74</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>220.93</v>
+        <v>218.73</v>
       </c>
       <c r="E50" s="13">
-        <v>173.82</v>
+        <v>172.58</v>
       </c>
       <c r="F50" s="13">
-        <v>183.82</v>
+        <v>182.58</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>222.94</v>
+        <v>221.57</v>
       </c>
       <c r="E51" s="10">
-        <v>175</v>
+        <v>173.98</v>
       </c>
       <c r="F51" s="10">
-        <v>185</v>
+        <v>183.98</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>222.31</v>
+        <v>220.93</v>
       </c>
       <c r="E52" s="13">
-        <v>174.84</v>
+        <v>173.82</v>
       </c>
       <c r="F52" s="13">
-        <v>184.84</v>
+        <v>183.82</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>235.26</v>
+        <v>233.71</v>
       </c>
       <c r="E56" s="10">
-        <v>189.3</v>
+        <v>190.02</v>
       </c>
       <c r="F56" s="10">
-        <v>199.3</v>
+        <v>200.02</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>225.64</v>
+        <v>224.07</v>
       </c>
       <c r="E57" s="13">
-        <v>184.27</v>
+        <v>183.98</v>
       </c>
       <c r="F57" s="13">
-        <v>194.27</v>
+        <v>193.98</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>225.78</v>
+        <v>224.21</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>224.48</v>
+        <v>222.94</v>
       </c>
       <c r="E59" s="13">
-        <v>178.66</v>
+        <v>178.37</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>220.3</v>
+        <v>218.75</v>
       </c>
       <c r="E60" s="10">
-        <v>174.59</v>
+        <v>174.3</v>
       </c>
       <c r="F60" s="10">
-        <v>184.59</v>
+        <v>184.3</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>224.08</v>
+        <v>222.53</v>
       </c>
       <c r="E61" s="13">
-        <v>185.87</v>
+        <v>186.63</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>235.31</v>
+        <v>235.26</v>
       </c>
       <c r="E62" s="10">
-        <v>188.77</v>
+        <v>189.3</v>
       </c>
       <c r="F62" s="10">
-        <v>198.77</v>
+        <v>199.3</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>225.7</v>
+        <v>225.64</v>
       </c>
       <c r="E63" s="13">
-        <v>183.66</v>
+        <v>184.27</v>
       </c>
       <c r="F63" s="13">
-        <v>193.66</v>
+        <v>194.27</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>225.85</v>
+        <v>225.78</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>224.53</v>
+        <v>224.48</v>
       </c>
       <c r="E65" s="13">
-        <v>178.05</v>
+        <v>178.66</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>220.34</v>
+        <v>220.3</v>
       </c>
       <c r="E66" s="10">
-        <v>173.98</v>
+        <v>174.59</v>
       </c>
       <c r="F66" s="10">
-        <v>183.98</v>
+        <v>184.59</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>224.13</v>
+        <v>224.08</v>
       </c>
       <c r="E67" s="13">
-        <v>185.3</v>
+        <v>185.87</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,6 +1892,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -1900,15 +1909,6 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2172,20 +2172,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
     <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Tue Apr 28 04:47:22 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{C61E42DD-FAA2-4F68-B42E-A6AA953CF448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{9EDD2943-5C8D-497E-8F08-189238EE712D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" concurrentManualCount="12"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>220.04</v>
+        <v>221.49</v>
       </c>
       <c r="E8" s="10">
-        <v>173.42</v>
+        <v>172.87</v>
       </c>
       <c r="F8" s="10">
-        <v>183.42</v>
+        <v>182.87</v>
       </c>
       <c r="G8" s="10">
-        <v>174.1</v>
+        <v>173.55</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>220.04</v>
+        <v>221.49</v>
       </c>
       <c r="E9" s="13">
-        <v>173.42</v>
+        <v>172.87</v>
       </c>
       <c r="F9" s="13">
-        <v>183.42</v>
+        <v>182.87</v>
       </c>
       <c r="G9" s="13">
-        <v>174.1</v>
+        <v>173.55</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>220.9</v>
+        <v>222.28</v>
       </c>
       <c r="E10" s="10">
-        <v>173.81</v>
+        <v>173.2</v>
       </c>
       <c r="F10" s="10">
-        <v>183.81</v>
+        <v>183.2</v>
       </c>
       <c r="G10" s="10">
-        <v>175.21</v>
+        <v>174.6</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>221.48</v>
+        <v>220.04</v>
       </c>
       <c r="E11" s="13">
-        <v>175.26</v>
+        <v>173.42</v>
       </c>
       <c r="F11" s="13">
-        <v>185.26</v>
+        <v>183.42</v>
       </c>
       <c r="G11" s="13">
-        <v>175.94</v>
+        <v>174.1</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>221.48</v>
+        <v>220.04</v>
       </c>
       <c r="E12" s="10">
-        <v>175.26</v>
+        <v>173.42</v>
       </c>
       <c r="F12" s="10">
-        <v>185.26</v>
+        <v>183.42</v>
       </c>
       <c r="G12" s="10">
-        <v>175.94</v>
+        <v>174.1</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>222.46</v>
+        <v>220.9</v>
       </c>
       <c r="E13" s="13">
-        <v>175.76</v>
+        <v>173.81</v>
       </c>
       <c r="F13" s="13">
-        <v>185.76</v>
+        <v>183.81</v>
       </c>
       <c r="G13" s="13">
-        <v>177.16</v>
+        <v>175.21</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>224.25</v>
+        <v>225.66</v>
       </c>
       <c r="E17" s="10">
-        <v>178.71</v>
+        <v>178.14</v>
       </c>
       <c r="F17" s="10">
-        <v>188.71</v>
+        <v>188.14</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>225.8</v>
+        <v>224.25</v>
       </c>
       <c r="E18" s="13">
-        <v>179</v>
+        <v>178.71</v>
       </c>
       <c r="F18" s="13">
-        <v>189</v>
+        <v>188.71</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>220.93</v>
+        <v>222.38</v>
       </c>
       <c r="E22" s="10">
-        <v>174.1</v>
+        <v>172.45</v>
       </c>
       <c r="F22" s="10">
-        <v>183.7</v>
+        <v>182.05</v>
       </c>
       <c r="G22" s="10">
-        <v>173.56</v>
+        <v>171.91</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>225.42</v>
+        <v>226.8</v>
       </c>
       <c r="E23" s="13">
-        <v>180.42</v>
+        <v>179.82</v>
       </c>
       <c r="F23" s="13">
-        <v>190.42</v>
+        <v>189.82</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>225.43</v>
+        <v>226.81</v>
       </c>
       <c r="E24" s="10">
-        <v>181.43</v>
+        <v>180.82</v>
       </c>
       <c r="F24" s="10">
-        <v>191.43</v>
+        <v>190.82</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>225.42</v>
+        <v>226.8</v>
       </c>
       <c r="E25" s="13">
-        <v>181.19</v>
+        <v>180.57</v>
       </c>
       <c r="F25" s="13">
-        <v>191.19</v>
+        <v>190.57</v>
       </c>
       <c r="G25" s="13">
-        <v>179.72</v>
+        <v>179.1</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>224.73</v>
+        <v>226.12</v>
       </c>
       <c r="E26" s="10">
-        <v>183.17</v>
+        <v>182.57</v>
       </c>
       <c r="F26" s="10">
-        <v>193.17</v>
+        <v>192.57</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>222.37</v>
+        <v>220.93</v>
       </c>
       <c r="E27" s="13">
-        <v>174.84</v>
+        <v>174.1</v>
       </c>
       <c r="F27" s="13">
-        <v>184.44</v>
+        <v>183.7</v>
       </c>
       <c r="G27" s="13">
-        <v>174.3</v>
+        <v>173.56</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>225.89</v>
+        <v>225.42</v>
       </c>
       <c r="E28" s="22">
-        <v>179.62</v>
+        <v>180.42</v>
       </c>
       <c r="F28" s="22">
-        <v>189.62</v>
+        <v>190.42</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>225.9</v>
+        <v>225.43</v>
       </c>
       <c r="E29" s="13">
-        <v>180.64</v>
+        <v>181.43</v>
       </c>
       <c r="F29" s="13">
-        <v>190.64</v>
+        <v>191.43</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>225.88</v>
+        <v>225.42</v>
       </c>
       <c r="E30" s="22">
-        <v>180.4</v>
+        <v>181.19</v>
       </c>
       <c r="F30" s="22">
-        <v>190.4</v>
+        <v>191.19</v>
       </c>
       <c r="G30" s="22">
-        <v>178.93</v>
+        <v>179.72</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>225.19</v>
+        <v>224.73</v>
       </c>
       <c r="E31" s="13">
-        <v>182.37</v>
+        <v>183.17</v>
       </c>
       <c r="F31" s="13">
-        <v>192.37</v>
+        <v>193.17</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>219.31</v>
+        <v>220.69</v>
       </c>
       <c r="E35" s="10">
-        <v>169.49</v>
+        <v>168.88</v>
       </c>
       <c r="F35" s="10">
-        <v>178.49</v>
+        <v>177.88</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>220.88</v>
+        <v>219.31</v>
       </c>
       <c r="E36" s="13">
-        <v>170.34</v>
+        <v>169.49</v>
       </c>
       <c r="F36" s="13">
-        <v>179.34</v>
+        <v>178.49</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>234.93</v>
+        <v>236.31</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>236.5</v>
+        <v>234.93</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>229.16</v>
+        <v>230.52</v>
       </c>
       <c r="E42" s="10">
-        <v>179.5</v>
+        <v>180.11</v>
       </c>
       <c r="F42" s="10">
-        <v>189.5</v>
+        <v>190.11</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>228.79</v>
+        <v>230.15</v>
       </c>
       <c r="E43" s="13">
-        <v>179.91</v>
+        <v>180.52</v>
       </c>
       <c r="F43" s="13">
-        <v>189.91</v>
+        <v>190.52</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>228.54</v>
+        <v>229.16</v>
       </c>
       <c r="E44" s="10">
-        <v>181.67</v>
+        <v>179.5</v>
       </c>
       <c r="F44" s="10">
-        <v>191.67</v>
+        <v>189.5</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>228.18</v>
+        <v>228.79</v>
       </c>
       <c r="E45" s="13">
-        <v>182.08</v>
+        <v>179.91</v>
       </c>
       <c r="F45" s="13">
-        <v>192.08</v>
+        <v>189.91</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>219.38</v>
+        <v>219.15</v>
       </c>
       <c r="E49" s="10">
-        <v>172.74</v>
+        <v>172.53</v>
       </c>
       <c r="F49" s="10">
-        <v>182.74</v>
+        <v>182.53</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>218.73</v>
+        <v>218.51</v>
       </c>
       <c r="E50" s="13">
-        <v>172.58</v>
+        <v>172.37</v>
       </c>
       <c r="F50" s="13">
-        <v>182.58</v>
+        <v>182.37</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>221.57</v>
+        <v>219.38</v>
       </c>
       <c r="E51" s="10">
-        <v>173.98</v>
+        <v>172.74</v>
       </c>
       <c r="F51" s="10">
-        <v>183.98</v>
+        <v>182.74</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>220.93</v>
+        <v>218.73</v>
       </c>
       <c r="E52" s="13">
-        <v>173.82</v>
+        <v>172.58</v>
       </c>
       <c r="F52" s="13">
-        <v>183.82</v>
+        <v>182.58</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>233.71</v>
+        <v>235.11</v>
       </c>
       <c r="E56" s="10">
-        <v>190.02</v>
+        <v>189.3</v>
       </c>
       <c r="F56" s="10">
-        <v>200.02</v>
+        <v>199.3</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>224.07</v>
+        <v>225.45</v>
       </c>
       <c r="E57" s="13">
-        <v>183.98</v>
+        <v>183.39</v>
       </c>
       <c r="F57" s="13">
-        <v>193.98</v>
+        <v>193.39</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>224.21</v>
+        <v>225.58</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>222.94</v>
+        <v>224.34</v>
       </c>
       <c r="E59" s="13">
-        <v>178.37</v>
+        <v>177.78</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>218.75</v>
+        <v>220.16</v>
       </c>
       <c r="E60" s="10">
-        <v>174.3</v>
+        <v>173.71</v>
       </c>
       <c r="F60" s="10">
-        <v>184.3</v>
+        <v>183.71</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>222.53</v>
+        <v>223.95</v>
       </c>
       <c r="E61" s="13">
-        <v>186.63</v>
+        <v>185.96</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>235.26</v>
+        <v>233.71</v>
       </c>
       <c r="E62" s="10">
-        <v>189.3</v>
+        <v>190.02</v>
       </c>
       <c r="F62" s="10">
-        <v>199.3</v>
+        <v>200.02</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>225.64</v>
+        <v>224.07</v>
       </c>
       <c r="E63" s="13">
-        <v>184.27</v>
+        <v>183.98</v>
       </c>
       <c r="F63" s="13">
-        <v>194.27</v>
+        <v>193.98</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>225.78</v>
+        <v>224.21</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>224.48</v>
+        <v>222.94</v>
       </c>
       <c r="E65" s="13">
-        <v>178.66</v>
+        <v>178.37</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>220.3</v>
+        <v>218.75</v>
       </c>
       <c r="E66" s="10">
-        <v>174.59</v>
+        <v>174.3</v>
       </c>
       <c r="F66" s="10">
-        <v>184.59</v>
+        <v>184.3</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46137</v>
+        <v>46140</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>224.08</v>
+        <v>222.53</v>
       </c>
       <c r="E67" s="13">
-        <v>185.87</v>
+        <v>186.63</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,15 +1892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -1909,6 +1900,15 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2172,20 +2172,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
     <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Wed Apr 29 04:42:27 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{9EDD2943-5C8D-497E-8F08-189238EE712D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{4D47BCB1-D82C-410A-8CF6-A64DAD79CAE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" concurrentManualCount="12"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>221.49</v>
+        <v>220.73</v>
       </c>
       <c r="E8" s="10">
-        <v>172.87</v>
+        <v>172.64</v>
       </c>
       <c r="F8" s="10">
-        <v>182.87</v>
+        <v>182.64</v>
       </c>
       <c r="G8" s="10">
-        <v>173.55</v>
+        <v>173.32</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>221.49</v>
+        <v>220.73</v>
       </c>
       <c r="E9" s="13">
-        <v>172.87</v>
+        <v>172.64</v>
       </c>
       <c r="F9" s="13">
-        <v>182.87</v>
+        <v>182.64</v>
       </c>
       <c r="G9" s="13">
-        <v>173.55</v>
+        <v>173.32</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>222.28</v>
+        <v>221.16</v>
       </c>
       <c r="E10" s="10">
-        <v>173.2</v>
+        <v>173.5</v>
       </c>
       <c r="F10" s="10">
-        <v>183.2</v>
+        <v>183.5</v>
       </c>
       <c r="G10" s="10">
-        <v>174.6</v>
+        <v>174.89</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>220.04</v>
+        <v>221.49</v>
       </c>
       <c r="E11" s="13">
-        <v>173.42</v>
+        <v>172.87</v>
       </c>
       <c r="F11" s="13">
-        <v>183.42</v>
+        <v>182.87</v>
       </c>
       <c r="G11" s="13">
-        <v>174.1</v>
+        <v>173.55</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>220.04</v>
+        <v>221.49</v>
       </c>
       <c r="E12" s="10">
-        <v>173.42</v>
+        <v>172.87</v>
       </c>
       <c r="F12" s="10">
-        <v>183.42</v>
+        <v>182.87</v>
       </c>
       <c r="G12" s="10">
-        <v>174.1</v>
+        <v>173.55</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>220.9</v>
+        <v>222.28</v>
       </c>
       <c r="E13" s="13">
-        <v>173.81</v>
+        <v>173.2</v>
       </c>
       <c r="F13" s="13">
-        <v>183.81</v>
+        <v>183.2</v>
       </c>
       <c r="G13" s="13">
-        <v>175.21</v>
+        <v>174.6</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>225.66</v>
+        <v>225.56</v>
       </c>
       <c r="E17" s="10">
-        <v>178.14</v>
+        <v>179.55</v>
       </c>
       <c r="F17" s="10">
-        <v>188.14</v>
+        <v>189.55</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>224.25</v>
+        <v>225.66</v>
       </c>
       <c r="E18" s="13">
-        <v>178.71</v>
+        <v>178.14</v>
       </c>
       <c r="F18" s="13">
-        <v>188.71</v>
+        <v>188.14</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>222.38</v>
+        <v>221.84</v>
       </c>
       <c r="E22" s="10">
-        <v>172.45</v>
+        <v>172.77</v>
       </c>
       <c r="F22" s="10">
-        <v>182.05</v>
+        <v>182.37</v>
       </c>
       <c r="G22" s="10">
-        <v>171.91</v>
+        <v>172.23</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>226.8</v>
+        <v>227.33</v>
       </c>
       <c r="E23" s="13">
-        <v>179.82</v>
+        <v>180.12</v>
       </c>
       <c r="F23" s="13">
-        <v>189.82</v>
+        <v>190.12</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>226.81</v>
+        <v>227.35</v>
       </c>
       <c r="E24" s="10">
-        <v>180.82</v>
+        <v>181.1</v>
       </c>
       <c r="F24" s="10">
-        <v>190.82</v>
+        <v>191.1</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>226.8</v>
+        <v>227.33</v>
       </c>
       <c r="E25" s="13">
-        <v>180.57</v>
+        <v>180.86</v>
       </c>
       <c r="F25" s="13">
-        <v>190.57</v>
+        <v>190.86</v>
       </c>
       <c r="G25" s="13">
-        <v>179.1</v>
+        <v>179.39</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>226.12</v>
+        <v>226.66</v>
       </c>
       <c r="E26" s="10">
-        <v>182.57</v>
+        <v>182.86</v>
       </c>
       <c r="F26" s="10">
-        <v>192.57</v>
+        <v>192.86</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>220.93</v>
+        <v>222.38</v>
       </c>
       <c r="E27" s="13">
-        <v>174.1</v>
+        <v>172.45</v>
       </c>
       <c r="F27" s="13">
-        <v>183.7</v>
+        <v>182.05</v>
       </c>
       <c r="G27" s="13">
-        <v>173.56</v>
+        <v>171.91</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>225.42</v>
+        <v>226.8</v>
       </c>
       <c r="E28" s="22">
-        <v>180.42</v>
+        <v>179.82</v>
       </c>
       <c r="F28" s="22">
-        <v>190.42</v>
+        <v>189.82</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>225.43</v>
+        <v>226.81</v>
       </c>
       <c r="E29" s="13">
-        <v>181.43</v>
+        <v>180.82</v>
       </c>
       <c r="F29" s="13">
-        <v>191.43</v>
+        <v>190.82</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>225.42</v>
+        <v>226.8</v>
       </c>
       <c r="E30" s="22">
-        <v>181.19</v>
+        <v>180.57</v>
       </c>
       <c r="F30" s="22">
-        <v>191.19</v>
+        <v>190.57</v>
       </c>
       <c r="G30" s="22">
-        <v>179.72</v>
+        <v>179.1</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>224.73</v>
+        <v>226.12</v>
       </c>
       <c r="E31" s="13">
-        <v>183.17</v>
+        <v>182.57</v>
       </c>
       <c r="F31" s="13">
-        <v>193.17</v>
+        <v>192.57</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>220.69</v>
+        <v>219.35</v>
       </c>
       <c r="E35" s="10">
-        <v>168.88</v>
+        <v>169.72</v>
       </c>
       <c r="F35" s="10">
-        <v>177.88</v>
+        <v>178.72</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>219.31</v>
+        <v>220.69</v>
       </c>
       <c r="E36" s="13">
-        <v>169.49</v>
+        <v>168.88</v>
       </c>
       <c r="F36" s="13">
-        <v>178.49</v>
+        <v>177.88</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>236.31</v>
+        <v>234.97</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>234.93</v>
+        <v>236.31</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>230.52</v>
+        <v>231.04</v>
       </c>
       <c r="E42" s="10">
-        <v>180.11</v>
+        <v>178.88</v>
       </c>
       <c r="F42" s="10">
-        <v>190.11</v>
+        <v>188.88</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>230.15</v>
+        <v>230.67</v>
       </c>
       <c r="E43" s="13">
-        <v>180.52</v>
+        <v>179.29</v>
       </c>
       <c r="F43" s="13">
-        <v>190.52</v>
+        <v>189.29</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>229.16</v>
+        <v>230.52</v>
       </c>
       <c r="E44" s="10">
-        <v>179.5</v>
+        <v>180.11</v>
       </c>
       <c r="F44" s="10">
-        <v>189.5</v>
+        <v>190.11</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>228.79</v>
+        <v>230.15</v>
       </c>
       <c r="E45" s="13">
-        <v>179.91</v>
+        <v>180.52</v>
       </c>
       <c r="F45" s="13">
-        <v>189.91</v>
+        <v>190.52</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>219.15</v>
+        <v>218.69</v>
       </c>
       <c r="E49" s="10">
-        <v>172.53</v>
+        <v>171.4</v>
       </c>
       <c r="F49" s="10">
-        <v>182.53</v>
+        <v>181.4</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>218.51</v>
+        <v>218.06</v>
       </c>
       <c r="E50" s="13">
-        <v>172.37</v>
+        <v>171.25</v>
       </c>
       <c r="F50" s="13">
-        <v>182.37</v>
+        <v>181.25</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>219.38</v>
+        <v>219.15</v>
       </c>
       <c r="E51" s="10">
-        <v>172.74</v>
+        <v>172.53</v>
       </c>
       <c r="F51" s="10">
-        <v>182.74</v>
+        <v>182.53</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>218.73</v>
+        <v>218.51</v>
       </c>
       <c r="E52" s="13">
-        <v>172.58</v>
+        <v>172.37</v>
       </c>
       <c r="F52" s="13">
-        <v>182.58</v>
+        <v>182.37</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>235.11</v>
+        <v>234.56</v>
       </c>
       <c r="E56" s="10">
-        <v>189.3</v>
+        <v>190.6</v>
       </c>
       <c r="F56" s="10">
-        <v>199.3</v>
+        <v>200.6</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>225.45</v>
+        <v>224.89</v>
       </c>
       <c r="E57" s="13">
-        <v>183.39</v>
+        <v>182.61</v>
       </c>
       <c r="F57" s="13">
-        <v>193.39</v>
+        <v>192.61</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>225.58</v>
+        <v>225.01</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>224.34</v>
+        <v>223.8</v>
       </c>
       <c r="E59" s="13">
-        <v>177.78</v>
+        <v>176.99</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>220.16</v>
+        <v>219.62</v>
       </c>
       <c r="E60" s="10">
-        <v>173.71</v>
+        <v>172.93</v>
       </c>
       <c r="F60" s="10">
-        <v>183.71</v>
+        <v>182.93</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>223.95</v>
+        <v>223.41</v>
       </c>
       <c r="E61" s="13">
-        <v>185.96</v>
+        <v>187.3</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>233.71</v>
+        <v>235.11</v>
       </c>
       <c r="E62" s="10">
-        <v>190.02</v>
+        <v>189.3</v>
       </c>
       <c r="F62" s="10">
-        <v>200.02</v>
+        <v>199.3</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>224.07</v>
+        <v>225.45</v>
       </c>
       <c r="E63" s="13">
-        <v>183.98</v>
+        <v>183.39</v>
       </c>
       <c r="F63" s="13">
-        <v>193.98</v>
+        <v>193.39</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>224.21</v>
+        <v>225.58</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>222.94</v>
+        <v>224.34</v>
       </c>
       <c r="E65" s="13">
-        <v>178.37</v>
+        <v>177.78</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>218.75</v>
+        <v>220.16</v>
       </c>
       <c r="E66" s="10">
-        <v>174.3</v>
+        <v>173.71</v>
       </c>
       <c r="F66" s="10">
-        <v>184.3</v>
+        <v>183.71</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>222.53</v>
+        <v>223.95</v>
       </c>
       <c r="E67" s="13">
-        <v>186.63</v>
+        <v>185.96</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,26 +1892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2171,26 +2151,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2210,6 +2191,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Thu Apr 30 04:46:23 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{4D47BCB1-D82C-410A-8CF6-A64DAD79CAE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{107CBC12-09B3-4A00-AE15-5C8E77DFF538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>220.73</v>
+        <v>220.53</v>
       </c>
       <c r="E8" s="10">
-        <v>172.64</v>
+        <v>173.01</v>
       </c>
       <c r="F8" s="10">
-        <v>182.64</v>
+        <v>183.01</v>
       </c>
       <c r="G8" s="10">
-        <v>173.32</v>
+        <v>173.59</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>220.73</v>
+        <v>220.53</v>
       </c>
       <c r="E9" s="13">
-        <v>172.64</v>
+        <v>173.01</v>
       </c>
       <c r="F9" s="13">
-        <v>182.64</v>
+        <v>183.01</v>
       </c>
       <c r="G9" s="13">
-        <v>173.32</v>
+        <v>173.59</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>221.16</v>
+        <v>221.05</v>
       </c>
       <c r="E10" s="10">
-        <v>173.5</v>
+        <v>174.5</v>
       </c>
       <c r="F10" s="10">
-        <v>183.5</v>
+        <v>184.5</v>
       </c>
       <c r="G10" s="10">
-        <v>174.89</v>
+        <v>175.52</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>221.49</v>
+        <v>220.73</v>
       </c>
       <c r="E11" s="13">
-        <v>172.87</v>
+        <v>172.64</v>
       </c>
       <c r="F11" s="13">
-        <v>182.87</v>
+        <v>182.64</v>
       </c>
       <c r="G11" s="13">
-        <v>173.55</v>
+        <v>173.32</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>221.49</v>
+        <v>220.73</v>
       </c>
       <c r="E12" s="10">
-        <v>172.87</v>
+        <v>172.64</v>
       </c>
       <c r="F12" s="10">
-        <v>182.87</v>
+        <v>182.64</v>
       </c>
       <c r="G12" s="10">
-        <v>173.55</v>
+        <v>173.32</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>222.28</v>
+        <v>221.16</v>
       </c>
       <c r="E13" s="13">
-        <v>173.2</v>
+        <v>173.5</v>
       </c>
       <c r="F13" s="13">
-        <v>183.2</v>
+        <v>183.5</v>
       </c>
       <c r="G13" s="13">
-        <v>174.6</v>
+        <v>174.89</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>225.56</v>
+        <v>225.46</v>
       </c>
       <c r="E17" s="10">
-        <v>179.55</v>
+        <v>180.57</v>
       </c>
       <c r="F17" s="10">
-        <v>189.55</v>
+        <v>190.57</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>225.66</v>
+        <v>225.56</v>
       </c>
       <c r="E18" s="13">
-        <v>178.14</v>
+        <v>179.55</v>
       </c>
       <c r="F18" s="13">
-        <v>188.14</v>
+        <v>189.55</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>221.84</v>
+        <v>221.65</v>
       </c>
       <c r="E22" s="10">
-        <v>172.77</v>
+        <v>172.59</v>
       </c>
       <c r="F22" s="10">
-        <v>182.37</v>
+        <v>182.19</v>
       </c>
       <c r="G22" s="10">
-        <v>172.23</v>
+        <v>172.05</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>227.33</v>
+        <v>227.22</v>
       </c>
       <c r="E23" s="13">
-        <v>180.12</v>
+        <v>181.12</v>
       </c>
       <c r="F23" s="13">
-        <v>190.12</v>
+        <v>191.13</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>227.35</v>
+        <v>227.24</v>
       </c>
       <c r="E24" s="10">
-        <v>181.1</v>
+        <v>182.1</v>
       </c>
       <c r="F24" s="10">
-        <v>191.1</v>
+        <v>192.1</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>227.33</v>
+        <v>227.22</v>
       </c>
       <c r="E25" s="13">
-        <v>180.86</v>
+        <v>181.85</v>
       </c>
       <c r="F25" s="13">
-        <v>190.86</v>
+        <v>191.85</v>
       </c>
       <c r="G25" s="13">
-        <v>179.39</v>
+        <v>182.21</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>226.66</v>
+        <v>226.56</v>
       </c>
       <c r="E26" s="10">
-        <v>182.86</v>
+        <v>183.87</v>
       </c>
       <c r="F26" s="10">
-        <v>192.86</v>
+        <v>193.87</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>222.38</v>
+        <v>221.84</v>
       </c>
       <c r="E27" s="13">
-        <v>172.45</v>
+        <v>172.77</v>
       </c>
       <c r="F27" s="13">
-        <v>182.05</v>
+        <v>182.37</v>
       </c>
       <c r="G27" s="13">
-        <v>171.91</v>
+        <v>172.23</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>226.8</v>
+        <v>227.33</v>
       </c>
       <c r="E28" s="22">
-        <v>179.82</v>
+        <v>180.12</v>
       </c>
       <c r="F28" s="22">
-        <v>189.82</v>
+        <v>190.12</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>226.81</v>
+        <v>227.35</v>
       </c>
       <c r="E29" s="13">
-        <v>180.82</v>
+        <v>181.1</v>
       </c>
       <c r="F29" s="13">
-        <v>190.82</v>
+        <v>191.1</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>226.8</v>
+        <v>227.33</v>
       </c>
       <c r="E30" s="22">
-        <v>180.57</v>
+        <v>180.86</v>
       </c>
       <c r="F30" s="22">
-        <v>190.57</v>
+        <v>190.86</v>
       </c>
       <c r="G30" s="22">
-        <v>179.1</v>
+        <v>179.39</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>226.12</v>
+        <v>226.66</v>
       </c>
       <c r="E31" s="13">
-        <v>182.57</v>
+        <v>182.86</v>
       </c>
       <c r="F31" s="13">
-        <v>192.57</v>
+        <v>192.86</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>219.35</v>
+        <v>219.24</v>
       </c>
       <c r="E35" s="10">
-        <v>169.72</v>
+        <v>170.72</v>
       </c>
       <c r="F35" s="10">
-        <v>178.72</v>
+        <v>179.72</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>220.69</v>
+        <v>219.35</v>
       </c>
       <c r="E36" s="13">
-        <v>168.88</v>
+        <v>169.72</v>
       </c>
       <c r="F36" s="13">
-        <v>177.88</v>
+        <v>178.72</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>234.97</v>
+        <v>234.86</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>236.31</v>
+        <v>234.97</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>231.04</v>
+        <v>230.92</v>
       </c>
       <c r="E42" s="10">
-        <v>178.88</v>
+        <v>179.94</v>
       </c>
       <c r="F42" s="10">
-        <v>188.88</v>
+        <v>189.94</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>230.67</v>
+        <v>230.55</v>
       </c>
       <c r="E43" s="13">
-        <v>179.29</v>
+        <v>180.36</v>
       </c>
       <c r="F43" s="13">
-        <v>189.29</v>
+        <v>190.36</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>230.52</v>
+        <v>231.04</v>
       </c>
       <c r="E44" s="10">
-        <v>180.11</v>
+        <v>178.88</v>
       </c>
       <c r="F44" s="10">
-        <v>190.11</v>
+        <v>188.88</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>230.15</v>
+        <v>230.67</v>
       </c>
       <c r="E45" s="13">
-        <v>180.52</v>
+        <v>179.29</v>
       </c>
       <c r="F45" s="13">
-        <v>190.52</v>
+        <v>189.29</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>218.69</v>
+        <v>218.37</v>
       </c>
       <c r="E49" s="10">
-        <v>171.4</v>
+        <v>172.63</v>
       </c>
       <c r="F49" s="10">
-        <v>181.4</v>
+        <v>182.63</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>218.06</v>
+        <v>217.74</v>
       </c>
       <c r="E50" s="13">
-        <v>171.25</v>
+        <v>172.49</v>
       </c>
       <c r="F50" s="13">
-        <v>181.25</v>
+        <v>182.49</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>219.15</v>
+        <v>218.69</v>
       </c>
       <c r="E51" s="10">
-        <v>172.53</v>
+        <v>171.4</v>
       </c>
       <c r="F51" s="10">
-        <v>182.53</v>
+        <v>181.4</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>218.51</v>
+        <v>218.06</v>
       </c>
       <c r="E52" s="13">
-        <v>172.37</v>
+        <v>171.25</v>
       </c>
       <c r="F52" s="13">
-        <v>182.37</v>
+        <v>181.25</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>234.56</v>
+        <v>234.46</v>
       </c>
       <c r="E56" s="10">
-        <v>190.6</v>
+        <v>191.52</v>
       </c>
       <c r="F56" s="10">
-        <v>200.6</v>
+        <v>201.52</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>224.89</v>
+        <v>224.78</v>
       </c>
       <c r="E57" s="13">
-        <v>182.61</v>
+        <v>183.62</v>
       </c>
       <c r="F57" s="13">
-        <v>192.61</v>
+        <v>193.62</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>225.01</v>
+        <v>224.9</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>223.8</v>
+        <v>223.71</v>
       </c>
       <c r="E59" s="13">
-        <v>176.99</v>
+        <v>178.01</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>219.62</v>
+        <v>219.53</v>
       </c>
       <c r="E60" s="10">
-        <v>172.93</v>
+        <v>173.94</v>
       </c>
       <c r="F60" s="10">
-        <v>182.93</v>
+        <v>183.94</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>223.41</v>
+        <v>226.06</v>
       </c>
       <c r="E61" s="13">
-        <v>187.3</v>
+        <v>188.26</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>235.11</v>
+        <v>234.56</v>
       </c>
       <c r="E62" s="10">
-        <v>189.3</v>
+        <v>190.6</v>
       </c>
       <c r="F62" s="10">
-        <v>199.3</v>
+        <v>200.6</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>225.45</v>
+        <v>224.89</v>
       </c>
       <c r="E63" s="13">
-        <v>183.39</v>
+        <v>182.61</v>
       </c>
       <c r="F63" s="13">
-        <v>193.39</v>
+        <v>192.61</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>225.58</v>
+        <v>225.01</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>224.34</v>
+        <v>223.8</v>
       </c>
       <c r="E65" s="13">
-        <v>177.78</v>
+        <v>176.99</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>220.16</v>
+        <v>219.62</v>
       </c>
       <c r="E66" s="10">
-        <v>173.71</v>
+        <v>172.93</v>
       </c>
       <c r="F66" s="10">
-        <v>183.71</v>
+        <v>182.93</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>223.95</v>
+        <v>223.41</v>
       </c>
       <c r="E67" s="13">
-        <v>185.96</v>
+        <v>187.3</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,6 +1892,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2151,15 +2160,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2172,6 +2172,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2187,14 +2195,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Fri May  1 04:58:21 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{107CBC12-09B3-4A00-AE15-5C8E77DFF538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{F21B2DBE-60DC-401D-BB26-91A194644804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>220.53</v>
+        <v>222.06</v>
       </c>
       <c r="E8" s="10">
-        <v>173.01</v>
+        <v>174.45</v>
       </c>
       <c r="F8" s="10">
-        <v>183.01</v>
+        <v>184.45</v>
       </c>
       <c r="G8" s="10">
-        <v>173.59</v>
+        <v>175.02</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>220.53</v>
+        <v>222.06</v>
       </c>
       <c r="E9" s="13">
-        <v>173.01</v>
+        <v>174.45</v>
       </c>
       <c r="F9" s="13">
-        <v>183.01</v>
+        <v>184.45</v>
       </c>
       <c r="G9" s="13">
-        <v>173.59</v>
+        <v>175.02</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>221.05</v>
+        <v>222.71</v>
       </c>
       <c r="E10" s="10">
-        <v>174.5</v>
+        <v>176.05</v>
       </c>
       <c r="F10" s="10">
-        <v>184.5</v>
+        <v>186.05</v>
       </c>
       <c r="G10" s="10">
-        <v>175.52</v>
+        <v>177.07</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>220.73</v>
+        <v>220.53</v>
       </c>
       <c r="E11" s="13">
-        <v>172.64</v>
+        <v>173.01</v>
       </c>
       <c r="F11" s="13">
-        <v>182.64</v>
+        <v>183.01</v>
       </c>
       <c r="G11" s="13">
-        <v>173.32</v>
+        <v>173.59</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>220.73</v>
+        <v>220.53</v>
       </c>
       <c r="E12" s="10">
-        <v>172.64</v>
+        <v>173.01</v>
       </c>
       <c r="F12" s="10">
-        <v>182.64</v>
+        <v>183.01</v>
       </c>
       <c r="G12" s="10">
-        <v>173.32</v>
+        <v>173.59</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>221.16</v>
+        <v>221.05</v>
       </c>
       <c r="E13" s="13">
-        <v>173.5</v>
+        <v>174.5</v>
       </c>
       <c r="F13" s="13">
-        <v>183.5</v>
+        <v>184.5</v>
       </c>
       <c r="G13" s="13">
-        <v>174.89</v>
+        <v>175.52</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>225.46</v>
+        <v>227.13</v>
       </c>
       <c r="E17" s="10">
-        <v>180.57</v>
+        <v>182.13</v>
       </c>
       <c r="F17" s="10">
-        <v>190.57</v>
+        <v>192.13</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>225.56</v>
+        <v>225.46</v>
       </c>
       <c r="E18" s="13">
-        <v>179.55</v>
+        <v>180.57</v>
       </c>
       <c r="F18" s="13">
-        <v>189.55</v>
+        <v>190.57</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>221.65</v>
+        <v>223.17</v>
       </c>
       <c r="E22" s="10">
-        <v>172.59</v>
+        <v>174.02</v>
       </c>
       <c r="F22" s="10">
-        <v>182.19</v>
+        <v>183.62</v>
       </c>
       <c r="G22" s="10">
-        <v>172.05</v>
+        <v>173.48</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>227.22</v>
+        <v>228.88</v>
       </c>
       <c r="E23" s="13">
-        <v>181.12</v>
+        <v>182.68</v>
       </c>
       <c r="F23" s="13">
-        <v>191.13</v>
+        <v>192.68</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>227.24</v>
+        <v>228.9</v>
       </c>
       <c r="E24" s="10">
-        <v>182.1</v>
+        <v>183.64</v>
       </c>
       <c r="F24" s="10">
-        <v>192.1</v>
+        <v>193.64</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>227.22</v>
+        <v>228.88</v>
       </c>
       <c r="E25" s="13">
-        <v>181.85</v>
+        <v>183.4</v>
       </c>
       <c r="F25" s="13">
-        <v>191.85</v>
+        <v>193.4</v>
       </c>
       <c r="G25" s="13">
-        <v>182.21</v>
+        <v>183.76</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>226.56</v>
+        <v>228.22</v>
       </c>
       <c r="E26" s="10">
-        <v>183.87</v>
+        <v>185.43</v>
       </c>
       <c r="F26" s="10">
-        <v>193.87</v>
+        <v>195.43</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>221.84</v>
+        <v>221.65</v>
       </c>
       <c r="E27" s="13">
-        <v>172.77</v>
+        <v>172.59</v>
       </c>
       <c r="F27" s="13">
-        <v>182.37</v>
+        <v>182.19</v>
       </c>
       <c r="G27" s="13">
-        <v>172.23</v>
+        <v>172.05</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>227.33</v>
+        <v>227.22</v>
       </c>
       <c r="E28" s="22">
-        <v>180.12</v>
+        <v>181.12</v>
       </c>
       <c r="F28" s="22">
-        <v>190.12</v>
+        <v>191.13</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>227.35</v>
+        <v>227.24</v>
       </c>
       <c r="E29" s="13">
-        <v>181.1</v>
+        <v>182.1</v>
       </c>
       <c r="F29" s="13">
-        <v>191.1</v>
+        <v>192.1</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>227.33</v>
+        <v>227.22</v>
       </c>
       <c r="E30" s="22">
-        <v>180.86</v>
+        <v>181.85</v>
       </c>
       <c r="F30" s="22">
-        <v>190.86</v>
+        <v>191.85</v>
       </c>
       <c r="G30" s="22">
-        <v>179.39</v>
+        <v>182.21</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>226.66</v>
+        <v>226.56</v>
       </c>
       <c r="E31" s="13">
-        <v>182.86</v>
+        <v>183.87</v>
       </c>
       <c r="F31" s="13">
-        <v>192.86</v>
+        <v>193.87</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>219.24</v>
+        <v>220.9</v>
       </c>
       <c r="E35" s="10">
-        <v>170.72</v>
+        <v>172.26</v>
       </c>
       <c r="F35" s="10">
-        <v>179.72</v>
+        <v>181.26</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>219.35</v>
+        <v>219.24</v>
       </c>
       <c r="E36" s="13">
-        <v>169.72</v>
+        <v>170.72</v>
       </c>
       <c r="F36" s="13">
-        <v>178.72</v>
+        <v>179.72</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>234.86</v>
+        <v>236.52</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>234.97</v>
+        <v>234.86</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>230.92</v>
+        <v>232.57</v>
       </c>
       <c r="E42" s="10">
-        <v>179.94</v>
+        <v>181.73</v>
       </c>
       <c r="F42" s="10">
-        <v>189.94</v>
+        <v>191.73</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>230.55</v>
+        <v>232.2</v>
       </c>
       <c r="E43" s="13">
-        <v>180.36</v>
+        <v>182.15</v>
       </c>
       <c r="F43" s="13">
-        <v>190.36</v>
+        <v>192.15</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>231.04</v>
+        <v>230.92</v>
       </c>
       <c r="E44" s="10">
-        <v>178.88</v>
+        <v>179.94</v>
       </c>
       <c r="F44" s="10">
-        <v>188.88</v>
+        <v>189.94</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>230.67</v>
+        <v>230.55</v>
       </c>
       <c r="E45" s="13">
-        <v>179.29</v>
+        <v>180.36</v>
       </c>
       <c r="F45" s="13">
-        <v>189.29</v>
+        <v>190.36</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>218.37</v>
+        <v>222.09</v>
       </c>
       <c r="E49" s="10">
-        <v>172.63</v>
+        <v>174.64</v>
       </c>
       <c r="F49" s="10">
-        <v>182.63</v>
+        <v>184.64</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>217.74</v>
+        <v>221.48</v>
       </c>
       <c r="E50" s="13">
-        <v>172.49</v>
+        <v>174.5</v>
       </c>
       <c r="F50" s="13">
-        <v>182.49</v>
+        <v>184.5</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>218.69</v>
+        <v>218.37</v>
       </c>
       <c r="E51" s="10">
-        <v>171.4</v>
+        <v>172.63</v>
       </c>
       <c r="F51" s="10">
-        <v>181.4</v>
+        <v>182.63</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>218.06</v>
+        <v>217.74</v>
       </c>
       <c r="E52" s="13">
-        <v>171.25</v>
+        <v>172.49</v>
       </c>
       <c r="F52" s="13">
-        <v>181.25</v>
+        <v>182.49</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>234.46</v>
+        <v>236.13</v>
       </c>
       <c r="E56" s="10">
-        <v>191.52</v>
+        <v>193.03</v>
       </c>
       <c r="F56" s="10">
-        <v>201.52</v>
+        <v>203.03</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>224.78</v>
+        <v>226.44</v>
       </c>
       <c r="E57" s="13">
-        <v>183.62</v>
+        <v>185.18</v>
       </c>
       <c r="F57" s="13">
-        <v>193.62</v>
+        <v>195.18</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>224.9</v>
+        <v>226.55</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>223.71</v>
+        <v>225.37</v>
       </c>
       <c r="E59" s="13">
-        <v>178.01</v>
+        <v>179.56</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>219.53</v>
+        <v>221.19</v>
       </c>
       <c r="E60" s="10">
-        <v>173.94</v>
+        <v>175.5</v>
       </c>
       <c r="F60" s="10">
-        <v>183.94</v>
+        <v>185.5</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>226.06</v>
+        <v>227.73</v>
       </c>
       <c r="E61" s="13">
-        <v>188.26</v>
+        <v>189.79</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>234.56</v>
+        <v>234.46</v>
       </c>
       <c r="E62" s="10">
-        <v>190.6</v>
+        <v>191.52</v>
       </c>
       <c r="F62" s="10">
-        <v>200.6</v>
+        <v>201.52</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>224.89</v>
+        <v>224.78</v>
       </c>
       <c r="E63" s="13">
-        <v>182.61</v>
+        <v>183.62</v>
       </c>
       <c r="F63" s="13">
-        <v>192.61</v>
+        <v>193.62</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>225.01</v>
+        <v>224.9</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>223.8</v>
+        <v>223.71</v>
       </c>
       <c r="E65" s="13">
-        <v>176.99</v>
+        <v>178.01</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>219.62</v>
+        <v>219.53</v>
       </c>
       <c r="E66" s="10">
-        <v>172.93</v>
+        <v>173.94</v>
       </c>
       <c r="F66" s="10">
-        <v>182.93</v>
+        <v>183.94</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>223.41</v>
+        <v>226.06</v>
       </c>
       <c r="E67" s="13">
-        <v>187.3</v>
+        <v>188.26</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,15 +1892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2160,6 +2151,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2172,14 +2172,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2195,6 +2187,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Mon May  4 04:51:49 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{F21B2DBE-60DC-401D-BB26-91A194644804}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{D9B8151E-6EB9-401E-8E25-ACF2A2C38AC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>222.06</v>
+        <v>220.41</v>
       </c>
       <c r="E8" s="10">
-        <v>174.45</v>
+        <v>173.42</v>
       </c>
       <c r="F8" s="10">
-        <v>184.45</v>
+        <v>183.42</v>
       </c>
       <c r="G8" s="10">
-        <v>175.02</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>222.06</v>
+        <v>220.41</v>
       </c>
       <c r="E9" s="13">
-        <v>174.45</v>
+        <v>173.42</v>
       </c>
       <c r="F9" s="13">
-        <v>184.45</v>
+        <v>183.42</v>
       </c>
       <c r="G9" s="13">
-        <v>175.02</v>
+        <v>174</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>222.71</v>
+        <v>221.12</v>
       </c>
       <c r="E10" s="10">
-        <v>176.05</v>
+        <v>174.52</v>
       </c>
       <c r="F10" s="10">
-        <v>186.05</v>
+        <v>184.52</v>
       </c>
       <c r="G10" s="10">
-        <v>177.07</v>
+        <v>175.55</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>220.53</v>
+        <v>222.06</v>
       </c>
       <c r="E11" s="13">
-        <v>173.01</v>
+        <v>174.45</v>
       </c>
       <c r="F11" s="13">
-        <v>183.01</v>
+        <v>184.45</v>
       </c>
       <c r="G11" s="13">
-        <v>173.59</v>
+        <v>175.02</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>220.53</v>
+        <v>222.06</v>
       </c>
       <c r="E12" s="10">
-        <v>173.01</v>
+        <v>174.45</v>
       </c>
       <c r="F12" s="10">
-        <v>183.01</v>
+        <v>184.45</v>
       </c>
       <c r="G12" s="10">
-        <v>173.59</v>
+        <v>175.02</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>221.05</v>
+        <v>222.71</v>
       </c>
       <c r="E13" s="13">
-        <v>174.5</v>
+        <v>176.05</v>
       </c>
       <c r="F13" s="13">
-        <v>184.5</v>
+        <v>186.05</v>
       </c>
       <c r="G13" s="13">
-        <v>175.52</v>
+        <v>177.07</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>227.13</v>
+        <v>225.55</v>
       </c>
       <c r="E17" s="10">
-        <v>182.13</v>
+        <v>181.72</v>
       </c>
       <c r="F17" s="10">
-        <v>192.13</v>
+        <v>191.72</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>225.46</v>
+        <v>227.13</v>
       </c>
       <c r="E18" s="13">
-        <v>180.57</v>
+        <v>182.13</v>
       </c>
       <c r="F18" s="13">
-        <v>190.57</v>
+        <v>192.13</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>223.17</v>
+        <v>221.52</v>
       </c>
       <c r="E22" s="10">
-        <v>174.02</v>
+        <v>173.54</v>
       </c>
       <c r="F22" s="10">
-        <v>183.62</v>
+        <v>183.14</v>
       </c>
       <c r="G22" s="10">
-        <v>173.48</v>
+        <v>173</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>228.88</v>
+        <v>227.28</v>
       </c>
       <c r="E23" s="13">
-        <v>182.68</v>
+        <v>180.61</v>
       </c>
       <c r="F23" s="13">
-        <v>192.68</v>
+        <v>190.61</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>228.9</v>
+        <v>227.3</v>
       </c>
       <c r="E24" s="10">
-        <v>183.64</v>
+        <v>181.56</v>
       </c>
       <c r="F24" s="10">
-        <v>193.64</v>
+        <v>191.57</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>228.88</v>
+        <v>227.29</v>
       </c>
       <c r="E25" s="13">
-        <v>183.4</v>
+        <v>181.32</v>
       </c>
       <c r="F25" s="13">
-        <v>193.4</v>
+        <v>191.32</v>
       </c>
       <c r="G25" s="13">
-        <v>183.76</v>
+        <v>181.68</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>228.22</v>
+        <v>226.63</v>
       </c>
       <c r="E26" s="10">
-        <v>185.43</v>
+        <v>183.35</v>
       </c>
       <c r="F26" s="10">
-        <v>195.43</v>
+        <v>193.35</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>221.65</v>
+        <v>223.17</v>
       </c>
       <c r="E27" s="13">
-        <v>172.59</v>
+        <v>174.02</v>
       </c>
       <c r="F27" s="13">
-        <v>182.19</v>
+        <v>183.62</v>
       </c>
       <c r="G27" s="13">
-        <v>172.05</v>
+        <v>173.48</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>227.22</v>
+        <v>228.88</v>
       </c>
       <c r="E28" s="22">
-        <v>181.12</v>
+        <v>182.68</v>
       </c>
       <c r="F28" s="22">
-        <v>191.13</v>
+        <v>192.68</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>227.24</v>
+        <v>228.9</v>
       </c>
       <c r="E29" s="13">
-        <v>182.1</v>
+        <v>183.64</v>
       </c>
       <c r="F29" s="13">
-        <v>192.1</v>
+        <v>193.64</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>227.22</v>
+        <v>228.88</v>
       </c>
       <c r="E30" s="22">
-        <v>181.85</v>
+        <v>183.4</v>
       </c>
       <c r="F30" s="22">
-        <v>191.85</v>
+        <v>193.4</v>
       </c>
       <c r="G30" s="22">
-        <v>182.21</v>
+        <v>183.76</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>226.56</v>
+        <v>228.22</v>
       </c>
       <c r="E31" s="13">
-        <v>183.87</v>
+        <v>185.43</v>
       </c>
       <c r="F31" s="13">
-        <v>193.87</v>
+        <v>195.43</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>220.9</v>
+        <v>219.31</v>
       </c>
       <c r="E35" s="10">
-        <v>172.26</v>
+        <v>172.39</v>
       </c>
       <c r="F35" s="10">
-        <v>181.26</v>
+        <v>181.39</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>219.24</v>
+        <v>220.9</v>
       </c>
       <c r="E36" s="13">
-        <v>170.72</v>
+        <v>172.26</v>
       </c>
       <c r="F36" s="13">
-        <v>179.72</v>
+        <v>181.26</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>236.52</v>
+        <v>234.93</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>234.86</v>
+        <v>236.52</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>232.57</v>
+        <v>230.96</v>
       </c>
       <c r="E42" s="10">
-        <v>181.73</v>
+        <v>181.27</v>
       </c>
       <c r="F42" s="10">
-        <v>191.73</v>
+        <v>191.27</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>232.2</v>
+        <v>230.59</v>
       </c>
       <c r="E43" s="13">
-        <v>182.15</v>
+        <v>181.68</v>
       </c>
       <c r="F43" s="13">
-        <v>192.15</v>
+        <v>191.68</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>230.92</v>
+        <v>232.57</v>
       </c>
       <c r="E44" s="10">
-        <v>179.94</v>
+        <v>181.73</v>
       </c>
       <c r="F44" s="10">
-        <v>189.94</v>
+        <v>191.73</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>230.55</v>
+        <v>232.2</v>
       </c>
       <c r="E45" s="13">
-        <v>180.36</v>
+        <v>182.15</v>
       </c>
       <c r="F45" s="13">
-        <v>190.36</v>
+        <v>192.15</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>222.09</v>
+        <v>221.59</v>
       </c>
       <c r="E49" s="10">
-        <v>174.64</v>
+        <v>173.48</v>
       </c>
       <c r="F49" s="10">
-        <v>184.64</v>
+        <v>183.48</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>221.48</v>
+        <v>220.98</v>
       </c>
       <c r="E50" s="13">
-        <v>174.5</v>
+        <v>173.35</v>
       </c>
       <c r="F50" s="13">
-        <v>184.5</v>
+        <v>183.35</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>218.37</v>
+        <v>222.09</v>
       </c>
       <c r="E51" s="10">
-        <v>172.63</v>
+        <v>174.64</v>
       </c>
       <c r="F51" s="10">
-        <v>182.63</v>
+        <v>184.64</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>217.74</v>
+        <v>221.48</v>
       </c>
       <c r="E52" s="13">
-        <v>172.49</v>
+        <v>174.5</v>
       </c>
       <c r="F52" s="13">
-        <v>182.49</v>
+        <v>184.5</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>236.13</v>
+        <v>234.53</v>
       </c>
       <c r="E56" s="10">
-        <v>193.03</v>
+        <v>193.11</v>
       </c>
       <c r="F56" s="10">
-        <v>203.03</v>
+        <v>203.11</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>226.44</v>
+        <v>224.84</v>
       </c>
       <c r="E57" s="13">
-        <v>185.18</v>
+        <v>184.21</v>
       </c>
       <c r="F57" s="13">
-        <v>195.18</v>
+        <v>194.21</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>226.55</v>
+        <v>224.96</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>225.37</v>
+        <v>223.8</v>
       </c>
       <c r="E59" s="13">
-        <v>179.56</v>
+        <v>178.6</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>221.19</v>
+        <v>219.62</v>
       </c>
       <c r="E60" s="10">
-        <v>175.5</v>
+        <v>174.53</v>
       </c>
       <c r="F60" s="10">
-        <v>185.5</v>
+        <v>184.53</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>227.73</v>
+        <v>226.15</v>
       </c>
       <c r="E61" s="13">
-        <v>189.79</v>
+        <v>189.56</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>234.46</v>
+        <v>236.13</v>
       </c>
       <c r="E62" s="10">
-        <v>191.52</v>
+        <v>193.03</v>
       </c>
       <c r="F62" s="10">
-        <v>201.52</v>
+        <v>203.03</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>224.78</v>
+        <v>226.44</v>
       </c>
       <c r="E63" s="13">
-        <v>183.62</v>
+        <v>185.18</v>
       </c>
       <c r="F63" s="13">
-        <v>193.62</v>
+        <v>195.18</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>224.9</v>
+        <v>226.55</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>223.71</v>
+        <v>225.37</v>
       </c>
       <c r="E65" s="13">
-        <v>178.01</v>
+        <v>179.56</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>219.53</v>
+        <v>221.19</v>
       </c>
       <c r="E66" s="10">
-        <v>173.94</v>
+        <v>175.5</v>
       </c>
       <c r="F66" s="10">
-        <v>183.94</v>
+        <v>185.5</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46143</v>
+        <v>46144</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>226.06</v>
+        <v>227.73</v>
       </c>
       <c r="E67" s="13">
-        <v>188.26</v>
+        <v>189.79</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,6 +1892,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2151,7 +2162,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2160,18 +2171,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2191,21 +2202,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Tue May  5 04:30:00 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{D9B8151E-6EB9-401E-8E25-ACF2A2C38AC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{DC887F39-D310-410B-A106-41A9CA687F02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>220.41</v>
+        <v>215.13</v>
       </c>
       <c r="E8" s="10">
-        <v>173.42</v>
+        <v>173.13</v>
       </c>
       <c r="F8" s="10">
-        <v>183.42</v>
+        <v>183.13</v>
       </c>
       <c r="G8" s="10">
-        <v>174</v>
+        <v>173.71</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>220.41</v>
+        <v>215.13</v>
       </c>
       <c r="E9" s="13">
-        <v>173.42</v>
+        <v>173.13</v>
       </c>
       <c r="F9" s="13">
-        <v>183.42</v>
+        <v>183.13</v>
       </c>
       <c r="G9" s="13">
-        <v>174</v>
+        <v>173.71</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>221.12</v>
+        <v>215.97</v>
       </c>
       <c r="E10" s="10">
-        <v>174.52</v>
+        <v>174.36</v>
       </c>
       <c r="F10" s="10">
-        <v>184.52</v>
+        <v>184.36</v>
       </c>
       <c r="G10" s="10">
-        <v>175.55</v>
+        <v>175.38</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>222.06</v>
+        <v>220.41</v>
       </c>
       <c r="E11" s="13">
-        <v>174.45</v>
+        <v>173.42</v>
       </c>
       <c r="F11" s="13">
-        <v>184.45</v>
+        <v>183.42</v>
       </c>
       <c r="G11" s="13">
-        <v>175.02</v>
+        <v>174</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>222.06</v>
+        <v>220.41</v>
       </c>
       <c r="E12" s="10">
-        <v>174.45</v>
+        <v>173.42</v>
       </c>
       <c r="F12" s="10">
-        <v>184.45</v>
+        <v>183.42</v>
       </c>
       <c r="G12" s="10">
-        <v>175.02</v>
+        <v>174</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>222.71</v>
+        <v>221.12</v>
       </c>
       <c r="E13" s="13">
-        <v>176.05</v>
+        <v>174.52</v>
       </c>
       <c r="F13" s="13">
-        <v>186.05</v>
+        <v>184.52</v>
       </c>
       <c r="G13" s="13">
-        <v>177.07</v>
+        <v>175.55</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>225.55</v>
+        <v>220.42</v>
       </c>
       <c r="E17" s="10">
-        <v>181.72</v>
+        <v>180.47</v>
       </c>
       <c r="F17" s="10">
-        <v>191.72</v>
+        <v>190.47</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>227.13</v>
+        <v>225.55</v>
       </c>
       <c r="E18" s="13">
-        <v>182.13</v>
+        <v>181.72</v>
       </c>
       <c r="F18" s="13">
-        <v>192.13</v>
+        <v>191.72</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>221.52</v>
+        <v>216.25</v>
       </c>
       <c r="E22" s="10">
-        <v>173.54</v>
+        <v>173.25</v>
       </c>
       <c r="F22" s="10">
-        <v>183.14</v>
+        <v>182.85</v>
       </c>
       <c r="G22" s="10">
-        <v>173</v>
+        <v>172.51</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>227.28</v>
+        <v>222.13</v>
       </c>
       <c r="E23" s="13">
-        <v>180.61</v>
+        <v>180.44</v>
       </c>
       <c r="F23" s="13">
-        <v>190.61</v>
+        <v>190.44</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>227.3</v>
+        <v>222.16</v>
       </c>
       <c r="E24" s="10">
-        <v>181.56</v>
+        <v>181.39</v>
       </c>
       <c r="F24" s="10">
-        <v>191.57</v>
+        <v>191.39</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>227.29</v>
+        <v>222.14</v>
       </c>
       <c r="E25" s="13">
-        <v>181.32</v>
+        <v>181.15</v>
       </c>
       <c r="F25" s="13">
-        <v>191.32</v>
+        <v>191.15</v>
       </c>
       <c r="G25" s="13">
-        <v>181.68</v>
+        <v>179.64</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>226.63</v>
+        <v>221.49</v>
       </c>
       <c r="E26" s="10">
-        <v>183.35</v>
+        <v>183.17</v>
       </c>
       <c r="F26" s="10">
-        <v>193.35</v>
+        <v>193.17</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>223.17</v>
+        <v>221.52</v>
       </c>
       <c r="E27" s="13">
-        <v>174.02</v>
+        <v>173.54</v>
       </c>
       <c r="F27" s="13">
-        <v>183.62</v>
+        <v>183.14</v>
       </c>
       <c r="G27" s="13">
-        <v>173.48</v>
+        <v>173</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>228.88</v>
+        <v>227.28</v>
       </c>
       <c r="E28" s="22">
-        <v>182.68</v>
+        <v>180.61</v>
       </c>
       <c r="F28" s="22">
-        <v>192.68</v>
+        <v>190.61</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>228.9</v>
+        <v>227.3</v>
       </c>
       <c r="E29" s="13">
-        <v>183.64</v>
+        <v>181.56</v>
       </c>
       <c r="F29" s="13">
-        <v>193.64</v>
+        <v>191.57</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>228.88</v>
+        <v>227.29</v>
       </c>
       <c r="E30" s="22">
-        <v>183.4</v>
+        <v>181.32</v>
       </c>
       <c r="F30" s="22">
-        <v>193.4</v>
+        <v>191.32</v>
       </c>
       <c r="G30" s="22">
-        <v>183.76</v>
+        <v>181.68</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>228.22</v>
+        <v>226.63</v>
       </c>
       <c r="E31" s="13">
-        <v>185.43</v>
+        <v>183.35</v>
       </c>
       <c r="F31" s="13">
-        <v>195.43</v>
+        <v>193.35</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>219.31</v>
+        <v>214.16</v>
       </c>
       <c r="E35" s="10">
-        <v>172.39</v>
+        <v>172.22</v>
       </c>
       <c r="F35" s="10">
-        <v>181.39</v>
+        <v>181.22</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>220.9</v>
+        <v>219.31</v>
       </c>
       <c r="E36" s="13">
-        <v>172.26</v>
+        <v>172.39</v>
       </c>
       <c r="F36" s="13">
-        <v>181.26</v>
+        <v>181.39</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>234.93</v>
+        <v>229.78</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>236.52</v>
+        <v>234.93</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>230.96</v>
+        <v>225.8</v>
       </c>
       <c r="E42" s="10">
-        <v>181.27</v>
+        <v>180.63</v>
       </c>
       <c r="F42" s="10">
-        <v>191.27</v>
+        <v>190.63</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>230.59</v>
+        <v>225.43</v>
       </c>
       <c r="E43" s="13">
-        <v>181.68</v>
+        <v>181.04</v>
       </c>
       <c r="F43" s="13">
-        <v>191.68</v>
+        <v>191.04</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>232.57</v>
+        <v>230.96</v>
       </c>
       <c r="E44" s="10">
-        <v>181.73</v>
+        <v>181.27</v>
       </c>
       <c r="F44" s="10">
-        <v>191.73</v>
+        <v>191.27</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>232.2</v>
+        <v>230.59</v>
       </c>
       <c r="E45" s="13">
-        <v>182.15</v>
+        <v>181.68</v>
       </c>
       <c r="F45" s="13">
-        <v>192.15</v>
+        <v>191.68</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>221.59</v>
+        <v>217.99</v>
       </c>
       <c r="E49" s="10">
-        <v>173.48</v>
+        <v>173.72</v>
       </c>
       <c r="F49" s="10">
-        <v>183.48</v>
+        <v>183.72</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>220.98</v>
+        <v>217.38</v>
       </c>
       <c r="E50" s="13">
-        <v>173.35</v>
+        <v>173.59</v>
       </c>
       <c r="F50" s="13">
-        <v>183.35</v>
+        <v>183.59</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>222.09</v>
+        <v>221.59</v>
       </c>
       <c r="E51" s="10">
-        <v>174.64</v>
+        <v>173.48</v>
       </c>
       <c r="F51" s="10">
-        <v>184.64</v>
+        <v>183.48</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>221.48</v>
+        <v>220.98</v>
       </c>
       <c r="E52" s="13">
-        <v>174.5</v>
+        <v>173.35</v>
       </c>
       <c r="F52" s="13">
-        <v>184.5</v>
+        <v>183.35</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>234.53</v>
+        <v>229.37</v>
       </c>
       <c r="E56" s="10">
-        <v>193.11</v>
+        <v>192.87</v>
       </c>
       <c r="F56" s="10">
-        <v>203.11</v>
+        <v>202.87</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>224.84</v>
+        <v>219.69</v>
       </c>
       <c r="E57" s="13">
-        <v>184.21</v>
+        <v>184.07</v>
       </c>
       <c r="F57" s="13">
-        <v>194.21</v>
+        <v>194.07</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>224.96</v>
+        <v>219.81</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>223.8</v>
+        <v>218.68</v>
       </c>
       <c r="E59" s="13">
-        <v>178.6</v>
+        <v>178.45</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>219.62</v>
+        <v>214.5</v>
       </c>
       <c r="E60" s="10">
-        <v>174.53</v>
+        <v>174.39</v>
       </c>
       <c r="F60" s="10">
-        <v>184.53</v>
+        <v>184.39</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>226.15</v>
+        <v>221.03</v>
       </c>
       <c r="E61" s="13">
-        <v>189.56</v>
+        <v>189.35</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>236.13</v>
+        <v>234.53</v>
       </c>
       <c r="E62" s="10">
-        <v>193.03</v>
+        <v>193.11</v>
       </c>
       <c r="F62" s="10">
-        <v>203.03</v>
+        <v>203.11</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>226.44</v>
+        <v>224.84</v>
       </c>
       <c r="E63" s="13">
-        <v>185.18</v>
+        <v>184.21</v>
       </c>
       <c r="F63" s="13">
-        <v>195.18</v>
+        <v>194.21</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>226.55</v>
+        <v>224.96</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>225.37</v>
+        <v>223.8</v>
       </c>
       <c r="E65" s="13">
-        <v>179.56</v>
+        <v>178.6</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>221.19</v>
+        <v>219.62</v>
       </c>
       <c r="E66" s="10">
-        <v>175.5</v>
+        <v>174.53</v>
       </c>
       <c r="F66" s="10">
-        <v>185.5</v>
+        <v>184.53</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46144</v>
+        <v>46147</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>227.73</v>
+        <v>226.15</v>
       </c>
       <c r="E67" s="13">
-        <v>189.79</v>
+        <v>189.56</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,17 +1892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2162,6 +2151,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2172,17 +2172,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2202,6 +2191,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Wed May  6 04:46:55 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{DC887F39-D310-410B-A106-41A9CA687F02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{08954749-2497-4E93-87B2-29C0E1D96961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>215.13</v>
+        <v>213.55</v>
       </c>
       <c r="E8" s="10">
-        <v>173.13</v>
+        <v>174.59</v>
       </c>
       <c r="F8" s="10">
-        <v>183.13</v>
+        <v>184.59</v>
       </c>
       <c r="G8" s="10">
-        <v>173.71</v>
+        <v>175.16</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>215.13</v>
+        <v>213.55</v>
       </c>
       <c r="E9" s="13">
-        <v>173.13</v>
+        <v>174.59</v>
       </c>
       <c r="F9" s="13">
-        <v>183.13</v>
+        <v>184.59</v>
       </c>
       <c r="G9" s="13">
-        <v>173.71</v>
+        <v>175.16</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>215.97</v>
+        <v>214.46</v>
       </c>
       <c r="E10" s="10">
-        <v>174.36</v>
+        <v>175.88</v>
       </c>
       <c r="F10" s="10">
-        <v>184.36</v>
+        <v>185.88</v>
       </c>
       <c r="G10" s="10">
-        <v>175.38</v>
+        <v>176.9</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>220.41</v>
+        <v>215.13</v>
       </c>
       <c r="E11" s="13">
-        <v>173.42</v>
+        <v>173.13</v>
       </c>
       <c r="F11" s="13">
-        <v>183.42</v>
+        <v>183.13</v>
       </c>
       <c r="G11" s="13">
-        <v>174</v>
+        <v>173.71</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>220.41</v>
+        <v>215.13</v>
       </c>
       <c r="E12" s="10">
-        <v>173.42</v>
+        <v>173.13</v>
       </c>
       <c r="F12" s="10">
-        <v>183.42</v>
+        <v>183.13</v>
       </c>
       <c r="G12" s="10">
-        <v>174</v>
+        <v>173.71</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>221.12</v>
+        <v>215.97</v>
       </c>
       <c r="E13" s="13">
-        <v>174.52</v>
+        <v>174.36</v>
       </c>
       <c r="F13" s="13">
-        <v>184.52</v>
+        <v>184.36</v>
       </c>
       <c r="G13" s="13">
-        <v>175.55</v>
+        <v>175.38</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>220.42</v>
+        <v>218.95</v>
       </c>
       <c r="E17" s="10">
-        <v>180.47</v>
+        <v>182.03</v>
       </c>
       <c r="F17" s="10">
-        <v>190.47</v>
+        <v>192.03</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>225.55</v>
+        <v>220.42</v>
       </c>
       <c r="E18" s="13">
-        <v>181.72</v>
+        <v>180.47</v>
       </c>
       <c r="F18" s="13">
-        <v>191.72</v>
+        <v>190.47</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>216.25</v>
+        <v>214.67</v>
       </c>
       <c r="E22" s="10">
-        <v>173.25</v>
+        <v>174.71</v>
       </c>
       <c r="F22" s="10">
-        <v>182.85</v>
+        <v>184.31</v>
       </c>
       <c r="G22" s="10">
-        <v>172.51</v>
+        <v>173.96</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>222.13</v>
+        <v>220.62</v>
       </c>
       <c r="E23" s="13">
-        <v>180.44</v>
+        <v>180.88</v>
       </c>
       <c r="F23" s="13">
-        <v>190.44</v>
+        <v>190.88</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>222.16</v>
+        <v>220.65</v>
       </c>
       <c r="E24" s="10">
-        <v>181.39</v>
+        <v>181.81</v>
       </c>
       <c r="F24" s="10">
-        <v>191.39</v>
+        <v>191.81</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>222.14</v>
+        <v>220.63</v>
       </c>
       <c r="E25" s="13">
-        <v>181.15</v>
+        <v>181.56</v>
       </c>
       <c r="F25" s="13">
-        <v>191.15</v>
+        <v>191.56</v>
       </c>
       <c r="G25" s="13">
-        <v>179.64</v>
+        <v>180.05</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>221.49</v>
+        <v>219.98</v>
       </c>
       <c r="E26" s="10">
-        <v>183.17</v>
+        <v>183.6</v>
       </c>
       <c r="F26" s="10">
-        <v>193.17</v>
+        <v>193.6</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>221.52</v>
+        <v>216.25</v>
       </c>
       <c r="E27" s="13">
-        <v>173.54</v>
+        <v>173.25</v>
       </c>
       <c r="F27" s="13">
-        <v>183.14</v>
+        <v>182.85</v>
       </c>
       <c r="G27" s="13">
-        <v>173</v>
+        <v>172.51</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>227.28</v>
+        <v>222.13</v>
       </c>
       <c r="E28" s="22">
-        <v>180.61</v>
+        <v>180.44</v>
       </c>
       <c r="F28" s="22">
-        <v>190.61</v>
+        <v>190.44</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>227.3</v>
+        <v>222.16</v>
       </c>
       <c r="E29" s="13">
-        <v>181.56</v>
+        <v>181.39</v>
       </c>
       <c r="F29" s="13">
-        <v>191.57</v>
+        <v>191.39</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>227.29</v>
+        <v>222.14</v>
       </c>
       <c r="E30" s="22">
-        <v>181.32</v>
+        <v>181.15</v>
       </c>
       <c r="F30" s="22">
-        <v>191.32</v>
+        <v>191.15</v>
       </c>
       <c r="G30" s="22">
-        <v>181.68</v>
+        <v>179.64</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>226.63</v>
+        <v>221.49</v>
       </c>
       <c r="E31" s="13">
-        <v>183.35</v>
+        <v>183.17</v>
       </c>
       <c r="F31" s="13">
-        <v>193.35</v>
+        <v>193.17</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>214.16</v>
+        <v>212.65</v>
       </c>
       <c r="E35" s="10">
-        <v>172.22</v>
+        <v>173.74</v>
       </c>
       <c r="F35" s="10">
-        <v>181.22</v>
+        <v>182.74</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>219.31</v>
+        <v>214.16</v>
       </c>
       <c r="E36" s="13">
-        <v>172.39</v>
+        <v>172.22</v>
       </c>
       <c r="F36" s="13">
-        <v>181.39</v>
+        <v>181.22</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>229.78</v>
+        <v>228.27</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>234.93</v>
+        <v>229.78</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>225.8</v>
+        <v>224.27</v>
       </c>
       <c r="E42" s="10">
-        <v>180.63</v>
+        <v>181.99</v>
       </c>
       <c r="F42" s="10">
-        <v>190.63</v>
+        <v>191.99</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>225.43</v>
+        <v>223.9</v>
       </c>
       <c r="E43" s="13">
-        <v>181.04</v>
+        <v>182.4</v>
       </c>
       <c r="F43" s="13">
-        <v>191.04</v>
+        <v>192.4</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>230.96</v>
+        <v>225.8</v>
       </c>
       <c r="E44" s="10">
-        <v>181.27</v>
+        <v>180.63</v>
       </c>
       <c r="F44" s="10">
-        <v>191.27</v>
+        <v>190.63</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>230.59</v>
+        <v>225.43</v>
       </c>
       <c r="E45" s="13">
-        <v>181.68</v>
+        <v>181.04</v>
       </c>
       <c r="F45" s="13">
-        <v>191.68</v>
+        <v>191.04</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>217.99</v>
+        <v>215.94</v>
       </c>
       <c r="E49" s="10">
-        <v>173.72</v>
+        <v>174.57</v>
       </c>
       <c r="F49" s="10">
-        <v>183.72</v>
+        <v>184.57</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>217.38</v>
+        <v>215.34</v>
       </c>
       <c r="E50" s="13">
-        <v>173.59</v>
+        <v>174.44</v>
       </c>
       <c r="F50" s="13">
-        <v>183.59</v>
+        <v>184.44</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>221.59</v>
+        <v>217.99</v>
       </c>
       <c r="E51" s="10">
-        <v>173.48</v>
+        <v>173.72</v>
       </c>
       <c r="F51" s="10">
-        <v>183.48</v>
+        <v>183.72</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>220.98</v>
+        <v>217.38</v>
       </c>
       <c r="E52" s="13">
-        <v>173.35</v>
+        <v>173.59</v>
       </c>
       <c r="F52" s="13">
-        <v>183.35</v>
+        <v>183.59</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>229.37</v>
+        <v>227.87</v>
       </c>
       <c r="E56" s="10">
-        <v>192.87</v>
+        <v>194.25</v>
       </c>
       <c r="F56" s="10">
-        <v>202.87</v>
+        <v>204.25</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>219.69</v>
+        <v>218.18</v>
       </c>
       <c r="E57" s="13">
-        <v>184.07</v>
+        <v>185.62</v>
       </c>
       <c r="F57" s="13">
-        <v>194.07</v>
+        <v>195.62</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>219.81</v>
+        <v>218.29</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>218.68</v>
+        <v>217.22</v>
       </c>
       <c r="E59" s="13">
-        <v>178.45</v>
+        <v>180.01</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>214.5</v>
+        <v>213.03</v>
       </c>
       <c r="E60" s="10">
-        <v>174.39</v>
+        <v>175.94</v>
       </c>
       <c r="F60" s="10">
-        <v>184.39</v>
+        <v>185.94</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>221.03</v>
+        <v>219.56</v>
       </c>
       <c r="E61" s="13">
-        <v>189.35</v>
+        <v>190.8</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>234.53</v>
+        <v>229.37</v>
       </c>
       <c r="E62" s="10">
-        <v>193.11</v>
+        <v>192.87</v>
       </c>
       <c r="F62" s="10">
-        <v>203.11</v>
+        <v>202.87</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>224.84</v>
+        <v>219.69</v>
       </c>
       <c r="E63" s="13">
-        <v>184.21</v>
+        <v>184.07</v>
       </c>
       <c r="F63" s="13">
-        <v>194.21</v>
+        <v>194.07</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>224.96</v>
+        <v>219.81</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>223.8</v>
+        <v>218.68</v>
       </c>
       <c r="E65" s="13">
-        <v>178.6</v>
+        <v>178.45</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>219.62</v>
+        <v>214.5</v>
       </c>
       <c r="E66" s="10">
-        <v>174.53</v>
+        <v>174.39</v>
       </c>
       <c r="F66" s="10">
-        <v>184.53</v>
+        <v>184.39</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>226.15</v>
+        <v>221.03</v>
       </c>
       <c r="E67" s="13">
-        <v>189.56</v>
+        <v>189.35</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -2152,6 +2152,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -2160,15 +2169,6 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2192,6 +2192,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2202,14 +2210,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Thu May  7 04:46:45 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{08954749-2497-4E93-87B2-29C0E1D96961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{A23002CE-DF9C-423F-BDA5-4AAC83059A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>213.55</v>
+        <v>207.85</v>
       </c>
       <c r="E8" s="10">
-        <v>174.59</v>
+        <v>174.25</v>
       </c>
       <c r="F8" s="10">
-        <v>184.59</v>
+        <v>184.25</v>
       </c>
       <c r="G8" s="10">
-        <v>175.16</v>
+        <v>174.82</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>213.55</v>
+        <v>207.85</v>
       </c>
       <c r="E9" s="13">
-        <v>174.59</v>
+        <v>174.25</v>
       </c>
       <c r="F9" s="13">
-        <v>184.59</v>
+        <v>184.25</v>
       </c>
       <c r="G9" s="13">
-        <v>175.16</v>
+        <v>174.82</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>214.46</v>
+        <v>208.74</v>
       </c>
       <c r="E10" s="10">
-        <v>175.88</v>
+        <v>175.52</v>
       </c>
       <c r="F10" s="10">
-        <v>185.88</v>
+        <v>185.52</v>
       </c>
       <c r="G10" s="10">
-        <v>176.9</v>
+        <v>176.54</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>215.13</v>
+        <v>213.55</v>
       </c>
       <c r="E11" s="13">
-        <v>173.13</v>
+        <v>174.59</v>
       </c>
       <c r="F11" s="13">
-        <v>183.13</v>
+        <v>184.59</v>
       </c>
       <c r="G11" s="13">
-        <v>173.71</v>
+        <v>175.16</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>215.13</v>
+        <v>213.55</v>
       </c>
       <c r="E12" s="10">
-        <v>173.13</v>
+        <v>174.59</v>
       </c>
       <c r="F12" s="10">
-        <v>183.13</v>
+        <v>184.59</v>
       </c>
       <c r="G12" s="10">
-        <v>173.71</v>
+        <v>175.16</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>215.97</v>
+        <v>214.46</v>
       </c>
       <c r="E13" s="13">
-        <v>174.36</v>
+        <v>175.88</v>
       </c>
       <c r="F13" s="13">
-        <v>184.36</v>
+        <v>185.88</v>
       </c>
       <c r="G13" s="13">
-        <v>175.38</v>
+        <v>176.9</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>218.95</v>
+        <v>213.27</v>
       </c>
       <c r="E17" s="10">
-        <v>182.03</v>
+        <v>181.71</v>
       </c>
       <c r="F17" s="10">
-        <v>192.03</v>
+        <v>191.71</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>220.42</v>
+        <v>218.95</v>
       </c>
       <c r="E18" s="13">
-        <v>180.47</v>
+        <v>182.03</v>
       </c>
       <c r="F18" s="13">
-        <v>190.47</v>
+        <v>192.03</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>214.67</v>
+        <v>208.97</v>
       </c>
       <c r="E22" s="10">
-        <v>174.71</v>
+        <v>174.37</v>
       </c>
       <c r="F22" s="10">
-        <v>184.31</v>
+        <v>183.97</v>
       </c>
       <c r="G22" s="10">
-        <v>173.96</v>
+        <v>173.62</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>220.62</v>
+        <v>214.89</v>
       </c>
       <c r="E23" s="13">
-        <v>180.88</v>
+        <v>180.52</v>
       </c>
       <c r="F23" s="13">
-        <v>190.88</v>
+        <v>190.52</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>220.65</v>
+        <v>214.92</v>
       </c>
       <c r="E24" s="10">
-        <v>181.81</v>
+        <v>181.43</v>
       </c>
       <c r="F24" s="10">
-        <v>191.81</v>
+        <v>191.43</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>220.63</v>
+        <v>214.91</v>
       </c>
       <c r="E25" s="13">
-        <v>181.56</v>
+        <v>181.18</v>
       </c>
       <c r="F25" s="13">
-        <v>191.56</v>
+        <v>191.18</v>
       </c>
       <c r="G25" s="13">
-        <v>180.05</v>
+        <v>179.67</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>219.98</v>
+        <v>214.27</v>
       </c>
       <c r="E26" s="10">
-        <v>183.6</v>
+        <v>183.21</v>
       </c>
       <c r="F26" s="10">
-        <v>193.6</v>
+        <v>193.21</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>216.25</v>
+        <v>214.67</v>
       </c>
       <c r="E27" s="13">
-        <v>173.25</v>
+        <v>174.71</v>
       </c>
       <c r="F27" s="13">
-        <v>182.85</v>
+        <v>184.31</v>
       </c>
       <c r="G27" s="13">
-        <v>172.51</v>
+        <v>173.96</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>222.13</v>
+        <v>220.62</v>
       </c>
       <c r="E28" s="22">
-        <v>180.44</v>
+        <v>180.88</v>
       </c>
       <c r="F28" s="22">
-        <v>190.44</v>
+        <v>190.88</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>222.16</v>
+        <v>220.65</v>
       </c>
       <c r="E29" s="13">
-        <v>181.39</v>
+        <v>181.81</v>
       </c>
       <c r="F29" s="13">
-        <v>191.39</v>
+        <v>191.81</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>222.14</v>
+        <v>220.63</v>
       </c>
       <c r="E30" s="22">
-        <v>181.15</v>
+        <v>181.56</v>
       </c>
       <c r="F30" s="22">
-        <v>191.15</v>
+        <v>191.56</v>
       </c>
       <c r="G30" s="22">
-        <v>179.64</v>
+        <v>180.05</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>221.49</v>
+        <v>219.98</v>
       </c>
       <c r="E31" s="13">
-        <v>183.17</v>
+        <v>183.6</v>
       </c>
       <c r="F31" s="13">
-        <v>193.17</v>
+        <v>193.6</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>212.65</v>
+        <v>206.93</v>
       </c>
       <c r="E35" s="10">
-        <v>173.74</v>
+        <v>173.39</v>
       </c>
       <c r="F35" s="10">
-        <v>182.74</v>
+        <v>182.39</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>214.16</v>
+        <v>212.65</v>
       </c>
       <c r="E36" s="13">
-        <v>172.22</v>
+        <v>173.74</v>
       </c>
       <c r="F36" s="13">
-        <v>181.22</v>
+        <v>182.74</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>228.27</v>
+        <v>222.55</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>229.78</v>
+        <v>228.27</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>224.27</v>
+        <v>218.5</v>
       </c>
       <c r="E42" s="10">
-        <v>181.99</v>
+        <v>182.36</v>
       </c>
       <c r="F42" s="10">
-        <v>191.99</v>
+        <v>192.36</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>223.9</v>
+        <v>218.14</v>
       </c>
       <c r="E43" s="13">
-        <v>182.4</v>
+        <v>182.77</v>
       </c>
       <c r="F43" s="13">
-        <v>192.4</v>
+        <v>192.77</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>225.8</v>
+        <v>224.27</v>
       </c>
       <c r="E44" s="10">
-        <v>180.63</v>
+        <v>181.99</v>
       </c>
       <c r="F44" s="10">
-        <v>190.63</v>
+        <v>191.99</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>225.43</v>
+        <v>223.9</v>
       </c>
       <c r="E45" s="13">
-        <v>181.04</v>
+        <v>182.4</v>
       </c>
       <c r="F45" s="13">
-        <v>191.04</v>
+        <v>192.4</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>215.94</v>
+        <v>210.63</v>
       </c>
       <c r="E49" s="10">
-        <v>174.57</v>
+        <v>174.46</v>
       </c>
       <c r="F49" s="10">
-        <v>184.57</v>
+        <v>184.46</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>215.34</v>
+        <v>210.04</v>
       </c>
       <c r="E50" s="13">
-        <v>174.44</v>
+        <v>174.35</v>
       </c>
       <c r="F50" s="13">
-        <v>184.44</v>
+        <v>184.35</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>217.99</v>
+        <v>215.94</v>
       </c>
       <c r="E51" s="10">
-        <v>173.72</v>
+        <v>174.57</v>
       </c>
       <c r="F51" s="10">
-        <v>183.72</v>
+        <v>184.57</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>217.38</v>
+        <v>215.34</v>
       </c>
       <c r="E52" s="13">
-        <v>173.59</v>
+        <v>174.44</v>
       </c>
       <c r="F52" s="13">
-        <v>183.59</v>
+        <v>184.44</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>227.87</v>
+        <v>222.15</v>
       </c>
       <c r="E56" s="10">
-        <v>194.25</v>
+        <v>193.71</v>
       </c>
       <c r="F56" s="10">
-        <v>204.25</v>
+        <v>203.71</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>218.18</v>
+        <v>212.45</v>
       </c>
       <c r="E57" s="13">
-        <v>185.62</v>
+        <v>185.31</v>
       </c>
       <c r="F57" s="13">
-        <v>195.62</v>
+        <v>195.31</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>218.29</v>
+        <v>212.56</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>217.22</v>
+        <v>211.56</v>
       </c>
       <c r="E59" s="13">
-        <v>180.01</v>
+        <v>179.7</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>213.03</v>
+        <v>207.38</v>
       </c>
       <c r="E60" s="10">
-        <v>175.94</v>
+        <v>175.63</v>
       </c>
       <c r="F60" s="10">
-        <v>185.94</v>
+        <v>185.63</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>219.56</v>
+        <v>213.9</v>
       </c>
       <c r="E61" s="13">
-        <v>190.8</v>
+        <v>190.33</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>229.37</v>
+        <v>227.87</v>
       </c>
       <c r="E62" s="10">
-        <v>192.87</v>
+        <v>194.25</v>
       </c>
       <c r="F62" s="10">
-        <v>202.87</v>
+        <v>204.25</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>219.69</v>
+        <v>218.18</v>
       </c>
       <c r="E63" s="13">
-        <v>184.07</v>
+        <v>185.62</v>
       </c>
       <c r="F63" s="13">
-        <v>194.07</v>
+        <v>195.62</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>219.81</v>
+        <v>218.29</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>218.68</v>
+        <v>217.22</v>
       </c>
       <c r="E65" s="13">
-        <v>178.45</v>
+        <v>180.01</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>214.5</v>
+        <v>213.03</v>
       </c>
       <c r="E66" s="10">
-        <v>174.39</v>
+        <v>175.94</v>
       </c>
       <c r="F66" s="10">
-        <v>184.39</v>
+        <v>185.94</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>221.03</v>
+        <v>219.56</v>
       </c>
       <c r="E67" s="13">
-        <v>189.35</v>
+        <v>190.8</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -2152,15 +2152,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -2169,6 +2160,15 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2192,14 +2192,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2210,6 +2202,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Fri May  8 04:26:39 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{A23002CE-DF9C-423F-BDA5-4AAC83059A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{16927DAA-8284-4E19-A775-138891D37E82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>207.85</v>
+        <v>197.84</v>
       </c>
       <c r="E8" s="10">
-        <v>174.25</v>
+        <v>171.18</v>
       </c>
       <c r="F8" s="10">
-        <v>184.25</v>
+        <v>181.18</v>
       </c>
       <c r="G8" s="10">
-        <v>174.82</v>
+        <v>171.76</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>207.85</v>
+        <v>197.84</v>
       </c>
       <c r="E9" s="13">
-        <v>174.25</v>
+        <v>171.18</v>
       </c>
       <c r="F9" s="13">
-        <v>184.25</v>
+        <v>181.18</v>
       </c>
       <c r="G9" s="13">
-        <v>174.82</v>
+        <v>171.76</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>208.74</v>
+        <v>198.74</v>
       </c>
       <c r="E10" s="10">
-        <v>175.52</v>
+        <v>172.46</v>
       </c>
       <c r="F10" s="10">
-        <v>185.52</v>
+        <v>182.46</v>
       </c>
       <c r="G10" s="10">
-        <v>176.54</v>
+        <v>173.48</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>213.55</v>
+        <v>207.85</v>
       </c>
       <c r="E11" s="13">
-        <v>174.59</v>
+        <v>174.25</v>
       </c>
       <c r="F11" s="13">
-        <v>184.59</v>
+        <v>184.25</v>
       </c>
       <c r="G11" s="13">
-        <v>175.16</v>
+        <v>174.82</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>213.55</v>
+        <v>207.85</v>
       </c>
       <c r="E12" s="10">
-        <v>174.59</v>
+        <v>174.25</v>
       </c>
       <c r="F12" s="10">
-        <v>184.59</v>
+        <v>184.25</v>
       </c>
       <c r="G12" s="10">
-        <v>175.16</v>
+        <v>174.82</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>214.46</v>
+        <v>208.74</v>
       </c>
       <c r="E13" s="13">
-        <v>175.88</v>
+        <v>175.52</v>
       </c>
       <c r="F13" s="13">
-        <v>185.88</v>
+        <v>185.52</v>
       </c>
       <c r="G13" s="13">
-        <v>176.9</v>
+        <v>176.54</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>213.27</v>
+        <v>203.32</v>
       </c>
       <c r="E17" s="10">
-        <v>181.71</v>
+        <v>178.69</v>
       </c>
       <c r="F17" s="10">
-        <v>191.71</v>
+        <v>188.69</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>218.95</v>
+        <v>213.27</v>
       </c>
       <c r="E18" s="13">
-        <v>182.03</v>
+        <v>181.71</v>
       </c>
       <c r="F18" s="13">
-        <v>192.03</v>
+        <v>191.71</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>208.97</v>
+        <v>198.96</v>
       </c>
       <c r="E22" s="10">
-        <v>174.37</v>
+        <v>171.3</v>
       </c>
       <c r="F22" s="10">
-        <v>183.97</v>
+        <v>180.9</v>
       </c>
       <c r="G22" s="10">
-        <v>173.62</v>
+        <v>170.56</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>214.89</v>
+        <v>204.89</v>
       </c>
       <c r="E23" s="13">
-        <v>180.52</v>
+        <v>177.45</v>
       </c>
       <c r="F23" s="13">
-        <v>190.52</v>
+        <v>187.45</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>214.92</v>
+        <v>204.93</v>
       </c>
       <c r="E24" s="10">
-        <v>181.43</v>
+        <v>178.35</v>
       </c>
       <c r="F24" s="10">
-        <v>191.43</v>
+        <v>188.35</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>214.91</v>
+        <v>204.92</v>
       </c>
       <c r="E25" s="13">
-        <v>181.18</v>
+        <v>178.09</v>
       </c>
       <c r="F25" s="13">
-        <v>191.18</v>
+        <v>188.09</v>
       </c>
       <c r="G25" s="13">
-        <v>179.67</v>
+        <v>176.58</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>214.27</v>
+        <v>204.28</v>
       </c>
       <c r="E26" s="10">
-        <v>183.21</v>
+        <v>180.1</v>
       </c>
       <c r="F26" s="10">
-        <v>193.21</v>
+        <v>190.1</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>214.67</v>
+        <v>208.97</v>
       </c>
       <c r="E27" s="13">
-        <v>174.71</v>
+        <v>174.37</v>
       </c>
       <c r="F27" s="13">
-        <v>184.31</v>
+        <v>183.97</v>
       </c>
       <c r="G27" s="13">
-        <v>173.96</v>
+        <v>173.62</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>220.62</v>
+        <v>214.89</v>
       </c>
       <c r="E28" s="22">
-        <v>180.88</v>
+        <v>180.52</v>
       </c>
       <c r="F28" s="22">
-        <v>190.88</v>
+        <v>190.52</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>220.65</v>
+        <v>214.92</v>
       </c>
       <c r="E29" s="13">
-        <v>181.81</v>
+        <v>181.43</v>
       </c>
       <c r="F29" s="13">
-        <v>191.81</v>
+        <v>191.43</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>220.63</v>
+        <v>214.91</v>
       </c>
       <c r="E30" s="22">
-        <v>181.56</v>
+        <v>181.18</v>
       </c>
       <c r="F30" s="22">
-        <v>191.56</v>
+        <v>191.18</v>
       </c>
       <c r="G30" s="22">
-        <v>180.05</v>
+        <v>179.67</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>219.98</v>
+        <v>214.27</v>
       </c>
       <c r="E31" s="13">
-        <v>183.6</v>
+        <v>183.21</v>
       </c>
       <c r="F31" s="13">
-        <v>193.6</v>
+        <v>193.21</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>206.93</v>
+        <v>196.95</v>
       </c>
       <c r="E35" s="10">
-        <v>173.39</v>
+        <v>170.33</v>
       </c>
       <c r="F35" s="10">
-        <v>182.39</v>
+        <v>179.33</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>212.65</v>
+        <v>206.93</v>
       </c>
       <c r="E36" s="13">
-        <v>173.74</v>
+        <v>173.39</v>
       </c>
       <c r="F36" s="13">
-        <v>182.74</v>
+        <v>182.39</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>222.55</v>
+        <v>212.57</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>228.27</v>
+        <v>222.55</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>218.5</v>
+        <v>208.47</v>
       </c>
       <c r="E42" s="10">
-        <v>182.36</v>
+        <v>179.73</v>
       </c>
       <c r="F42" s="10">
-        <v>192.36</v>
+        <v>189.73</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>218.14</v>
+        <v>208.11</v>
       </c>
       <c r="E43" s="13">
-        <v>182.77</v>
+        <v>180.15</v>
       </c>
       <c r="F43" s="13">
-        <v>192.77</v>
+        <v>190.15</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>224.27</v>
+        <v>218.5</v>
       </c>
       <c r="E44" s="10">
-        <v>181.99</v>
+        <v>182.36</v>
       </c>
       <c r="F44" s="10">
-        <v>191.99</v>
+        <v>192.36</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>223.9</v>
+        <v>218.14</v>
       </c>
       <c r="E45" s="13">
-        <v>182.4</v>
+        <v>182.77</v>
       </c>
       <c r="F45" s="13">
-        <v>192.4</v>
+        <v>192.77</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>210.63</v>
+        <v>205.19</v>
       </c>
       <c r="E49" s="10">
-        <v>174.46</v>
+        <v>173.53</v>
       </c>
       <c r="F49" s="10">
-        <v>184.46</v>
+        <v>183.53</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>210.04</v>
+        <v>204.61</v>
       </c>
       <c r="E50" s="13">
-        <v>174.35</v>
+        <v>173.41</v>
       </c>
       <c r="F50" s="13">
-        <v>184.35</v>
+        <v>183.41</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>215.94</v>
+        <v>210.63</v>
       </c>
       <c r="E51" s="10">
-        <v>174.57</v>
+        <v>174.46</v>
       </c>
       <c r="F51" s="10">
-        <v>184.57</v>
+        <v>184.46</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>215.34</v>
+        <v>210.04</v>
       </c>
       <c r="E52" s="13">
-        <v>174.44</v>
+        <v>174.35</v>
       </c>
       <c r="F52" s="13">
-        <v>184.44</v>
+        <v>184.35</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>222.15</v>
+        <v>212.13</v>
       </c>
       <c r="E56" s="10">
-        <v>193.71</v>
+        <v>190.47</v>
       </c>
       <c r="F56" s="10">
-        <v>203.71</v>
+        <v>200.47</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>212.45</v>
+        <v>202.43</v>
       </c>
       <c r="E57" s="13">
-        <v>185.31</v>
+        <v>182.31</v>
       </c>
       <c r="F57" s="13">
-        <v>195.31</v>
+        <v>192.31</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>212.56</v>
+        <v>202.56</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>211.56</v>
+        <v>201.64</v>
       </c>
       <c r="E59" s="13">
-        <v>179.7</v>
+        <v>176.7</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>207.38</v>
+        <v>197.45</v>
       </c>
       <c r="E60" s="10">
-        <v>175.63</v>
+        <v>172.63</v>
       </c>
       <c r="F60" s="10">
-        <v>185.63</v>
+        <v>182.63</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>213.9</v>
+        <v>203.97</v>
       </c>
       <c r="E61" s="13">
-        <v>190.33</v>
+        <v>187.16</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>227.87</v>
+        <v>222.15</v>
       </c>
       <c r="E62" s="10">
-        <v>194.25</v>
+        <v>193.71</v>
       </c>
       <c r="F62" s="10">
-        <v>204.25</v>
+        <v>203.71</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>218.18</v>
+        <v>212.45</v>
       </c>
       <c r="E63" s="13">
-        <v>185.62</v>
+        <v>185.31</v>
       </c>
       <c r="F63" s="13">
-        <v>195.62</v>
+        <v>195.31</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>218.29</v>
+        <v>212.56</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>217.22</v>
+        <v>211.56</v>
       </c>
       <c r="E65" s="13">
-        <v>180.01</v>
+        <v>179.7</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>213.03</v>
+        <v>207.38</v>
       </c>
       <c r="E66" s="10">
-        <v>175.94</v>
+        <v>175.63</v>
       </c>
       <c r="F66" s="10">
-        <v>185.94</v>
+        <v>185.63</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46149</v>
+        <v>46150</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>219.56</v>
+        <v>213.9</v>
       </c>
       <c r="E67" s="13">
-        <v>190.8</v>
+        <v>190.33</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -2152,6 +2152,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -2160,15 +2169,6 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2192,6 +2192,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2202,14 +2210,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Mon May 11 05:08:05 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{16927DAA-8284-4E19-A775-138891D37E82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{126E8927-785E-475E-889B-DC8822BC2986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>197.84</v>
+        <v>196.96</v>
       </c>
       <c r="E8" s="10">
-        <v>171.18</v>
+        <v>169.39</v>
       </c>
       <c r="F8" s="10">
-        <v>181.18</v>
+        <v>179.39</v>
       </c>
       <c r="G8" s="10">
-        <v>171.76</v>
+        <v>169.97</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>197.84</v>
+        <v>196.96</v>
       </c>
       <c r="E9" s="13">
-        <v>171.18</v>
+        <v>169.39</v>
       </c>
       <c r="F9" s="13">
-        <v>181.18</v>
+        <v>179.39</v>
       </c>
       <c r="G9" s="13">
-        <v>171.76</v>
+        <v>169.97</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>198.74</v>
+        <v>197.88</v>
       </c>
       <c r="E10" s="10">
-        <v>172.46</v>
+        <v>170.14</v>
       </c>
       <c r="F10" s="10">
-        <v>182.46</v>
+        <v>180.14</v>
       </c>
       <c r="G10" s="10">
-        <v>173.48</v>
+        <v>171.16</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>207.85</v>
+        <v>197.84</v>
       </c>
       <c r="E11" s="13">
-        <v>174.25</v>
+        <v>171.18</v>
       </c>
       <c r="F11" s="13">
-        <v>184.25</v>
+        <v>181.18</v>
       </c>
       <c r="G11" s="13">
-        <v>174.82</v>
+        <v>171.76</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>207.85</v>
+        <v>197.84</v>
       </c>
       <c r="E12" s="10">
-        <v>174.25</v>
+        <v>171.18</v>
       </c>
       <c r="F12" s="10">
-        <v>184.25</v>
+        <v>181.18</v>
       </c>
       <c r="G12" s="10">
-        <v>174.82</v>
+        <v>171.76</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>208.74</v>
+        <v>198.74</v>
       </c>
       <c r="E13" s="13">
-        <v>175.52</v>
+        <v>172.46</v>
       </c>
       <c r="F13" s="13">
-        <v>185.52</v>
+        <v>182.46</v>
       </c>
       <c r="G13" s="13">
-        <v>176.54</v>
+        <v>173.48</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>203.32</v>
+        <v>202.47</v>
       </c>
       <c r="E17" s="10">
-        <v>178.69</v>
+        <v>175.83</v>
       </c>
       <c r="F17" s="10">
-        <v>188.69</v>
+        <v>185.83</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>213.27</v>
+        <v>203.32</v>
       </c>
       <c r="E18" s="13">
-        <v>181.71</v>
+        <v>178.69</v>
       </c>
       <c r="F18" s="13">
-        <v>191.71</v>
+        <v>188.69</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>198.96</v>
+        <v>198.08</v>
       </c>
       <c r="E22" s="10">
-        <v>171.3</v>
+        <v>169.52</v>
       </c>
       <c r="F22" s="10">
-        <v>180.9</v>
+        <v>179.12</v>
       </c>
       <c r="G22" s="10">
-        <v>170.56</v>
+        <v>168.77</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>204.89</v>
+        <v>204.02</v>
       </c>
       <c r="E23" s="13">
-        <v>177.45</v>
+        <v>175.68</v>
       </c>
       <c r="F23" s="13">
-        <v>187.45</v>
+        <v>185.68</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>204.93</v>
+        <v>204.06</v>
       </c>
       <c r="E24" s="10">
-        <v>178.35</v>
+        <v>176.57</v>
       </c>
       <c r="F24" s="10">
-        <v>188.35</v>
+        <v>186.57</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>204.92</v>
+        <v>204.05</v>
       </c>
       <c r="E25" s="13">
-        <v>178.09</v>
+        <v>176.3</v>
       </c>
       <c r="F25" s="13">
-        <v>188.09</v>
+        <v>186.3</v>
       </c>
       <c r="G25" s="13">
-        <v>176.58</v>
+        <v>174.8</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>204.28</v>
+        <v>203.42</v>
       </c>
       <c r="E26" s="10">
-        <v>180.1</v>
+        <v>178.3</v>
       </c>
       <c r="F26" s="10">
-        <v>190.1</v>
+        <v>188.3</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>208.97</v>
+        <v>198.96</v>
       </c>
       <c r="E27" s="13">
-        <v>174.37</v>
+        <v>171.3</v>
       </c>
       <c r="F27" s="13">
-        <v>183.97</v>
+        <v>180.9</v>
       </c>
       <c r="G27" s="13">
-        <v>173.62</v>
+        <v>170.56</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>214.89</v>
+        <v>204.89</v>
       </c>
       <c r="E28" s="22">
-        <v>180.52</v>
+        <v>177.45</v>
       </c>
       <c r="F28" s="22">
-        <v>190.52</v>
+        <v>187.45</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>214.92</v>
+        <v>204.93</v>
       </c>
       <c r="E29" s="13">
-        <v>181.43</v>
+        <v>178.35</v>
       </c>
       <c r="F29" s="13">
-        <v>191.43</v>
+        <v>188.35</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>214.91</v>
+        <v>204.92</v>
       </c>
       <c r="E30" s="22">
-        <v>181.18</v>
+        <v>178.09</v>
       </c>
       <c r="F30" s="22">
-        <v>191.18</v>
+        <v>188.09</v>
       </c>
       <c r="G30" s="22">
-        <v>179.67</v>
+        <v>176.58</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>214.27</v>
+        <v>204.28</v>
       </c>
       <c r="E31" s="13">
-        <v>183.21</v>
+        <v>180.1</v>
       </c>
       <c r="F31" s="13">
-        <v>193.21</v>
+        <v>190.1</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>196.95</v>
+        <v>196.08</v>
       </c>
       <c r="E35" s="10">
-        <v>170.33</v>
+        <v>168.56</v>
       </c>
       <c r="F35" s="10">
-        <v>179.33</v>
+        <v>177.56</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>206.93</v>
+        <v>196.95</v>
       </c>
       <c r="E36" s="13">
-        <v>173.39</v>
+        <v>170.33</v>
       </c>
       <c r="F36" s="13">
-        <v>182.39</v>
+        <v>179.33</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>212.57</v>
+        <v>211.7</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>222.55</v>
+        <v>212.57</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>208.47</v>
+        <v>207.59</v>
       </c>
       <c r="E42" s="10">
-        <v>179.73</v>
+        <v>177.86</v>
       </c>
       <c r="F42" s="10">
-        <v>189.73</v>
+        <v>187.86</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>208.11</v>
+        <v>207.23</v>
       </c>
       <c r="E43" s="13">
-        <v>180.15</v>
+        <v>178.28</v>
       </c>
       <c r="F43" s="13">
-        <v>190.15</v>
+        <v>188.28</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>218.5</v>
+        <v>208.47</v>
       </c>
       <c r="E44" s="10">
-        <v>182.36</v>
+        <v>179.73</v>
       </c>
       <c r="F44" s="10">
-        <v>192.36</v>
+        <v>189.73</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>218.14</v>
+        <v>208.11</v>
       </c>
       <c r="E45" s="13">
-        <v>182.77</v>
+        <v>180.15</v>
       </c>
       <c r="F45" s="13">
-        <v>192.77</v>
+        <v>190.15</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>205.19</v>
+        <v>202.33</v>
       </c>
       <c r="E49" s="10">
-        <v>173.53</v>
+        <v>171.25</v>
       </c>
       <c r="F49" s="10">
-        <v>183.53</v>
+        <v>181.25</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>204.61</v>
+        <v>201.76</v>
       </c>
       <c r="E50" s="13">
-        <v>173.41</v>
+        <v>171.14</v>
       </c>
       <c r="F50" s="13">
-        <v>183.41</v>
+        <v>181.14</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>210.63</v>
+        <v>205.19</v>
       </c>
       <c r="E51" s="10">
-        <v>174.46</v>
+        <v>173.53</v>
       </c>
       <c r="F51" s="10">
-        <v>184.46</v>
+        <v>183.53</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>210.04</v>
+        <v>204.61</v>
       </c>
       <c r="E52" s="13">
-        <v>174.35</v>
+        <v>173.41</v>
       </c>
       <c r="F52" s="13">
-        <v>184.35</v>
+        <v>183.41</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>212.13</v>
+        <v>211.26</v>
       </c>
       <c r="E56" s="10">
-        <v>190.47</v>
+        <v>188.63</v>
       </c>
       <c r="F56" s="10">
-        <v>200.47</v>
+        <v>198.63</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>202.43</v>
+        <v>201.56</v>
       </c>
       <c r="E57" s="13">
-        <v>182.31</v>
+        <v>180.56</v>
       </c>
       <c r="F57" s="13">
-        <v>192.31</v>
+        <v>190.56</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>202.56</v>
+        <v>201.69</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>201.64</v>
+        <v>200.8</v>
       </c>
       <c r="E59" s="13">
-        <v>176.7</v>
+        <v>174.95</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>197.45</v>
+        <v>196.61</v>
       </c>
       <c r="E60" s="10">
-        <v>172.63</v>
+        <v>170.88</v>
       </c>
       <c r="F60" s="10">
-        <v>182.63</v>
+        <v>180.88</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>203.97</v>
+        <v>203.12</v>
       </c>
       <c r="E61" s="13">
-        <v>187.16</v>
+        <v>185.34</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>222.15</v>
+        <v>212.13</v>
       </c>
       <c r="E62" s="10">
-        <v>193.71</v>
+        <v>190.47</v>
       </c>
       <c r="F62" s="10">
-        <v>203.71</v>
+        <v>200.47</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>212.45</v>
+        <v>202.43</v>
       </c>
       <c r="E63" s="13">
-        <v>185.31</v>
+        <v>182.31</v>
       </c>
       <c r="F63" s="13">
-        <v>195.31</v>
+        <v>192.31</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>212.56</v>
+        <v>202.56</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>211.56</v>
+        <v>201.64</v>
       </c>
       <c r="E65" s="13">
-        <v>179.7</v>
+        <v>176.7</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>207.38</v>
+        <v>197.45</v>
       </c>
       <c r="E66" s="10">
-        <v>175.63</v>
+        <v>172.63</v>
       </c>
       <c r="F66" s="10">
-        <v>185.63</v>
+        <v>182.63</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46150</v>
+        <v>46151</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>213.9</v>
+        <v>203.97</v>
       </c>
       <c r="E67" s="13">
-        <v>190.33</v>
+        <v>187.16</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,6 +1892,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2151,7 +2162,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2160,18 +2171,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2191,21 +2202,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Tue May 12 04:51:08 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{126E8927-785E-475E-889B-DC8822BC2986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{8A3B80C1-4912-4406-B8A6-D6A2AE711775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>196.96</v>
+        <v>195.69</v>
       </c>
       <c r="E8" s="10">
-        <v>169.39</v>
+        <v>168.56</v>
       </c>
       <c r="F8" s="10">
-        <v>179.39</v>
+        <v>178.56</v>
       </c>
       <c r="G8" s="10">
-        <v>169.97</v>
+        <v>169.14</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>196.96</v>
+        <v>195.69</v>
       </c>
       <c r="E9" s="13">
-        <v>169.39</v>
+        <v>168.56</v>
       </c>
       <c r="F9" s="13">
-        <v>179.39</v>
+        <v>178.56</v>
       </c>
       <c r="G9" s="13">
-        <v>169.97</v>
+        <v>169.14</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>197.88</v>
+        <v>196.64</v>
       </c>
       <c r="E10" s="10">
-        <v>170.14</v>
+        <v>169.33</v>
       </c>
       <c r="F10" s="10">
-        <v>180.14</v>
+        <v>179.33</v>
       </c>
       <c r="G10" s="10">
-        <v>171.16</v>
+        <v>170.35</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>197.84</v>
+        <v>196.96</v>
       </c>
       <c r="E11" s="13">
-        <v>171.18</v>
+        <v>169.39</v>
       </c>
       <c r="F11" s="13">
-        <v>181.18</v>
+        <v>179.39</v>
       </c>
       <c r="G11" s="13">
-        <v>171.76</v>
+        <v>169.97</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>197.84</v>
+        <v>196.96</v>
       </c>
       <c r="E12" s="10">
-        <v>171.18</v>
+        <v>169.39</v>
       </c>
       <c r="F12" s="10">
-        <v>181.18</v>
+        <v>179.39</v>
       </c>
       <c r="G12" s="10">
-        <v>171.76</v>
+        <v>169.97</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>198.74</v>
+        <v>197.88</v>
       </c>
       <c r="E13" s="13">
-        <v>172.46</v>
+        <v>170.14</v>
       </c>
       <c r="F13" s="13">
-        <v>182.46</v>
+        <v>180.14</v>
       </c>
       <c r="G13" s="13">
-        <v>173.48</v>
+        <v>171.16</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>202.47</v>
+        <v>201.27</v>
       </c>
       <c r="E17" s="10">
-        <v>175.83</v>
+        <v>175.05</v>
       </c>
       <c r="F17" s="10">
-        <v>185.83</v>
+        <v>185.05</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>203.32</v>
+        <v>202.47</v>
       </c>
       <c r="E18" s="13">
-        <v>178.69</v>
+        <v>175.83</v>
       </c>
       <c r="F18" s="13">
-        <v>188.69</v>
+        <v>185.83</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>198.08</v>
+        <v>196.81</v>
       </c>
       <c r="E22" s="10">
-        <v>169.52</v>
+        <v>168.69</v>
       </c>
       <c r="F22" s="10">
-        <v>179.12</v>
+        <v>178.29</v>
       </c>
       <c r="G22" s="10">
-        <v>168.77</v>
+        <v>167.94</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>204.02</v>
+        <v>202.77</v>
       </c>
       <c r="E23" s="13">
-        <v>175.68</v>
+        <v>174.87</v>
       </c>
       <c r="F23" s="13">
-        <v>185.68</v>
+        <v>184.87</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>204.06</v>
+        <v>202.82</v>
       </c>
       <c r="E24" s="10">
-        <v>176.57</v>
+        <v>175.75</v>
       </c>
       <c r="F24" s="10">
-        <v>186.57</v>
+        <v>185.75</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>204.05</v>
+        <v>202.81</v>
       </c>
       <c r="E25" s="13">
-        <v>176.3</v>
+        <v>175.48</v>
       </c>
       <c r="F25" s="13">
-        <v>186.3</v>
+        <v>185.48</v>
       </c>
       <c r="G25" s="13">
-        <v>174.8</v>
+        <v>173.97</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>203.42</v>
+        <v>202.18</v>
       </c>
       <c r="E26" s="10">
-        <v>178.3</v>
+        <v>177.46</v>
       </c>
       <c r="F26" s="10">
-        <v>188.3</v>
+        <v>187.46</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>198.96</v>
+        <v>198.08</v>
       </c>
       <c r="E27" s="13">
-        <v>171.3</v>
+        <v>169.52</v>
       </c>
       <c r="F27" s="13">
-        <v>180.9</v>
+        <v>179.12</v>
       </c>
       <c r="G27" s="13">
-        <v>170.56</v>
+        <v>168.77</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>204.89</v>
+        <v>204.02</v>
       </c>
       <c r="E28" s="22">
-        <v>177.45</v>
+        <v>175.68</v>
       </c>
       <c r="F28" s="22">
-        <v>187.45</v>
+        <v>185.68</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>204.93</v>
+        <v>204.06</v>
       </c>
       <c r="E29" s="13">
-        <v>178.35</v>
+        <v>176.57</v>
       </c>
       <c r="F29" s="13">
-        <v>188.35</v>
+        <v>186.57</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>204.92</v>
+        <v>204.05</v>
       </c>
       <c r="E30" s="22">
-        <v>178.09</v>
+        <v>176.3</v>
       </c>
       <c r="F30" s="22">
-        <v>188.09</v>
+        <v>186.3</v>
       </c>
       <c r="G30" s="22">
-        <v>176.58</v>
+        <v>174.8</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>204.28</v>
+        <v>203.42</v>
       </c>
       <c r="E31" s="13">
-        <v>180.1</v>
+        <v>178.3</v>
       </c>
       <c r="F31" s="13">
-        <v>190.1</v>
+        <v>188.3</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>196.08</v>
+        <v>194.84</v>
       </c>
       <c r="E35" s="10">
-        <v>168.56</v>
+        <v>167.75</v>
       </c>
       <c r="F35" s="10">
-        <v>177.56</v>
+        <v>176.75</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>196.95</v>
+        <v>196.08</v>
       </c>
       <c r="E36" s="13">
-        <v>170.33</v>
+        <v>168.56</v>
       </c>
       <c r="F36" s="13">
-        <v>179.33</v>
+        <v>177.56</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>211.7</v>
+        <v>210.46</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>212.57</v>
+        <v>211.7</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>207.59</v>
+        <v>206.31</v>
       </c>
       <c r="E42" s="10">
-        <v>177.86</v>
+        <v>176.97</v>
       </c>
       <c r="F42" s="10">
-        <v>187.86</v>
+        <v>186.97</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>207.23</v>
+        <v>205.96</v>
       </c>
       <c r="E43" s="13">
-        <v>178.28</v>
+        <v>177.38</v>
       </c>
       <c r="F43" s="13">
-        <v>188.28</v>
+        <v>187.39</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>208.47</v>
+        <v>207.59</v>
       </c>
       <c r="E44" s="10">
-        <v>179.73</v>
+        <v>177.86</v>
       </c>
       <c r="F44" s="10">
-        <v>189.73</v>
+        <v>187.86</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>208.11</v>
+        <v>207.23</v>
       </c>
       <c r="E45" s="13">
-        <v>180.15</v>
+        <v>178.28</v>
       </c>
       <c r="F45" s="13">
-        <v>190.15</v>
+        <v>188.28</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>202.33</v>
+        <v>198.13</v>
       </c>
       <c r="E49" s="10">
-        <v>171.25</v>
+        <v>169.63</v>
       </c>
       <c r="F49" s="10">
-        <v>181.25</v>
+        <v>179.63</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>201.76</v>
+        <v>197.56</v>
       </c>
       <c r="E50" s="13">
-        <v>171.14</v>
+        <v>169.53</v>
       </c>
       <c r="F50" s="13">
-        <v>181.14</v>
+        <v>179.53</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>205.19</v>
+        <v>202.33</v>
       </c>
       <c r="E51" s="10">
-        <v>173.53</v>
+        <v>171.25</v>
       </c>
       <c r="F51" s="10">
-        <v>183.53</v>
+        <v>181.25</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>204.61</v>
+        <v>201.76</v>
       </c>
       <c r="E52" s="13">
-        <v>173.41</v>
+        <v>171.14</v>
       </c>
       <c r="F52" s="13">
-        <v>183.41</v>
+        <v>181.14</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>211.26</v>
+        <v>210.02</v>
       </c>
       <c r="E56" s="10">
-        <v>188.63</v>
+        <v>187.66</v>
       </c>
       <c r="F56" s="10">
-        <v>198.63</v>
+        <v>197.66</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>201.56</v>
+        <v>200.32</v>
       </c>
       <c r="E57" s="13">
-        <v>180.56</v>
+        <v>179.79</v>
       </c>
       <c r="F57" s="13">
-        <v>190.56</v>
+        <v>189.79</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>201.69</v>
+        <v>200.44</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>200.8</v>
+        <v>199.6</v>
       </c>
       <c r="E59" s="13">
-        <v>174.95</v>
+        <v>174.18</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>196.61</v>
+        <v>195.42</v>
       </c>
       <c r="E60" s="10">
-        <v>170.88</v>
+        <v>170.11</v>
       </c>
       <c r="F60" s="10">
-        <v>180.88</v>
+        <v>180.11</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>203.12</v>
+        <v>201.93</v>
       </c>
       <c r="E61" s="13">
-        <v>185.34</v>
+        <v>184.44</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>212.13</v>
+        <v>211.26</v>
       </c>
       <c r="E62" s="10">
-        <v>190.47</v>
+        <v>188.63</v>
       </c>
       <c r="F62" s="10">
-        <v>200.47</v>
+        <v>198.63</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>202.43</v>
+        <v>201.56</v>
       </c>
       <c r="E63" s="13">
-        <v>182.31</v>
+        <v>180.56</v>
       </c>
       <c r="F63" s="13">
-        <v>192.31</v>
+        <v>190.56</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>202.56</v>
+        <v>201.69</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>201.64</v>
+        <v>200.8</v>
       </c>
       <c r="E65" s="13">
-        <v>176.7</v>
+        <v>174.95</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>197.45</v>
+        <v>196.61</v>
       </c>
       <c r="E66" s="10">
-        <v>172.63</v>
+        <v>170.88</v>
       </c>
       <c r="F66" s="10">
-        <v>182.63</v>
+        <v>180.88</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46151</v>
+        <v>46154</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>203.97</v>
+        <v>203.12</v>
       </c>
       <c r="E67" s="13">
-        <v>187.16</v>
+        <v>185.34</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,14 +1892,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2163,21 +2161,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2203,9 +2200,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Wed May 13 04:59:24 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{8A3B80C1-4912-4406-B8A6-D6A2AE711775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{FFA27C10-AAB1-4203-9521-211925F6AF01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>195.69</v>
+        <v>195.04</v>
       </c>
       <c r="E8" s="10">
-        <v>168.56</v>
+        <v>167.54</v>
       </c>
       <c r="F8" s="10">
-        <v>178.56</v>
+        <v>177.54</v>
       </c>
       <c r="G8" s="10">
-        <v>169.14</v>
+        <v>168.12</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>195.69</v>
+        <v>195.04</v>
       </c>
       <c r="E9" s="13">
-        <v>168.56</v>
+        <v>167.54</v>
       </c>
       <c r="F9" s="13">
-        <v>178.56</v>
+        <v>177.54</v>
       </c>
       <c r="G9" s="13">
-        <v>169.14</v>
+        <v>168.12</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>196.64</v>
+        <v>196.06</v>
       </c>
       <c r="E10" s="10">
-        <v>169.33</v>
+        <v>168.38</v>
       </c>
       <c r="F10" s="10">
-        <v>179.33</v>
+        <v>178.38</v>
       </c>
       <c r="G10" s="10">
-        <v>170.35</v>
+        <v>169.4</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>196.96</v>
+        <v>195.69</v>
       </c>
       <c r="E11" s="13">
-        <v>169.39</v>
+        <v>168.56</v>
       </c>
       <c r="F11" s="13">
-        <v>179.39</v>
+        <v>178.56</v>
       </c>
       <c r="G11" s="13">
-        <v>169.97</v>
+        <v>169.14</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>196.96</v>
+        <v>195.69</v>
       </c>
       <c r="E12" s="10">
-        <v>169.39</v>
+        <v>168.56</v>
       </c>
       <c r="F12" s="10">
-        <v>179.39</v>
+        <v>178.56</v>
       </c>
       <c r="G12" s="10">
-        <v>169.97</v>
+        <v>169.14</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>197.88</v>
+        <v>196.64</v>
       </c>
       <c r="E13" s="13">
-        <v>170.14</v>
+        <v>169.33</v>
       </c>
       <c r="F13" s="13">
-        <v>180.14</v>
+        <v>179.33</v>
       </c>
       <c r="G13" s="13">
-        <v>171.16</v>
+        <v>170.35</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>201.27</v>
+        <v>200.72</v>
       </c>
       <c r="E17" s="10">
-        <v>175.05</v>
+        <v>174.12</v>
       </c>
       <c r="F17" s="10">
-        <v>185.05</v>
+        <v>184.12</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>202.47</v>
+        <v>201.27</v>
       </c>
       <c r="E18" s="13">
-        <v>175.83</v>
+        <v>175.05</v>
       </c>
       <c r="F18" s="13">
-        <v>185.83</v>
+        <v>185.05</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>196.81</v>
+        <v>196.16</v>
       </c>
       <c r="E22" s="10">
-        <v>168.69</v>
+        <v>167.67</v>
       </c>
       <c r="F22" s="10">
-        <v>178.29</v>
+        <v>177.27</v>
       </c>
       <c r="G22" s="10">
-        <v>167.94</v>
+        <v>166.92</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>202.77</v>
+        <v>202.19</v>
       </c>
       <c r="E23" s="13">
-        <v>174.87</v>
+        <v>173.92</v>
       </c>
       <c r="F23" s="13">
-        <v>184.87</v>
+        <v>183.92</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>202.82</v>
+        <v>202.24</v>
       </c>
       <c r="E24" s="10">
-        <v>175.75</v>
+        <v>174.79</v>
       </c>
       <c r="F24" s="10">
-        <v>185.75</v>
+        <v>184.79</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>202.81</v>
+        <v>202.24</v>
       </c>
       <c r="E25" s="13">
-        <v>175.48</v>
+        <v>174.51</v>
       </c>
       <c r="F25" s="13">
-        <v>185.48</v>
+        <v>184.51</v>
       </c>
       <c r="G25" s="13">
-        <v>173.97</v>
+        <v>173</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>202.18</v>
+        <v>201.62</v>
       </c>
       <c r="E26" s="10">
-        <v>177.46</v>
+        <v>176.49</v>
       </c>
       <c r="F26" s="10">
-        <v>187.46</v>
+        <v>186.49</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>198.08</v>
+        <v>196.81</v>
       </c>
       <c r="E27" s="13">
-        <v>169.52</v>
+        <v>168.69</v>
       </c>
       <c r="F27" s="13">
-        <v>179.12</v>
+        <v>178.29</v>
       </c>
       <c r="G27" s="13">
-        <v>168.77</v>
+        <v>167.94</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>204.02</v>
+        <v>202.77</v>
       </c>
       <c r="E28" s="22">
-        <v>175.68</v>
+        <v>174.87</v>
       </c>
       <c r="F28" s="22">
-        <v>185.68</v>
+        <v>184.87</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>204.06</v>
+        <v>202.82</v>
       </c>
       <c r="E29" s="13">
-        <v>176.57</v>
+        <v>175.75</v>
       </c>
       <c r="F29" s="13">
-        <v>186.57</v>
+        <v>185.75</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>204.05</v>
+        <v>202.81</v>
       </c>
       <c r="E30" s="22">
-        <v>176.3</v>
+        <v>175.48</v>
       </c>
       <c r="F30" s="22">
-        <v>186.3</v>
+        <v>185.48</v>
       </c>
       <c r="G30" s="22">
-        <v>174.8</v>
+        <v>173.97</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>203.42</v>
+        <v>202.18</v>
       </c>
       <c r="E31" s="13">
-        <v>178.3</v>
+        <v>177.46</v>
       </c>
       <c r="F31" s="13">
-        <v>188.3</v>
+        <v>187.46</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>194.84</v>
+        <v>194.27</v>
       </c>
       <c r="E35" s="10">
-        <v>167.75</v>
+        <v>166.81</v>
       </c>
       <c r="F35" s="10">
-        <v>176.75</v>
+        <v>175.81</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>196.08</v>
+        <v>194.84</v>
       </c>
       <c r="E36" s="13">
-        <v>168.56</v>
+        <v>167.75</v>
       </c>
       <c r="F36" s="13">
-        <v>177.56</v>
+        <v>176.75</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>210.46</v>
+        <v>209.89</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>211.7</v>
+        <v>210.46</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>206.31</v>
+        <v>205.72</v>
       </c>
       <c r="E42" s="10">
-        <v>176.97</v>
+        <v>175.76</v>
       </c>
       <c r="F42" s="10">
-        <v>186.97</v>
+        <v>185.76</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>205.96</v>
+        <v>205.37</v>
       </c>
       <c r="E43" s="13">
-        <v>177.38</v>
+        <v>176.18</v>
       </c>
       <c r="F43" s="13">
-        <v>187.39</v>
+        <v>186.18</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>207.59</v>
+        <v>206.31</v>
       </c>
       <c r="E44" s="10">
-        <v>177.86</v>
+        <v>176.97</v>
       </c>
       <c r="F44" s="10">
-        <v>187.86</v>
+        <v>186.97</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>207.23</v>
+        <v>205.96</v>
       </c>
       <c r="E45" s="13">
-        <v>178.28</v>
+        <v>177.38</v>
       </c>
       <c r="F45" s="13">
-        <v>188.28</v>
+        <v>187.39</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>198.13</v>
+        <v>198.54</v>
       </c>
       <c r="E49" s="10">
-        <v>169.63</v>
+        <v>169.97</v>
       </c>
       <c r="F49" s="10">
-        <v>179.63</v>
+        <v>179.97</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>197.56</v>
+        <v>197.98</v>
       </c>
       <c r="E50" s="13">
-        <v>169.53</v>
+        <v>169.87</v>
       </c>
       <c r="F50" s="13">
-        <v>179.53</v>
+        <v>179.87</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>202.33</v>
+        <v>198.13</v>
       </c>
       <c r="E51" s="10">
-        <v>171.25</v>
+        <v>169.63</v>
       </c>
       <c r="F51" s="10">
-        <v>181.25</v>
+        <v>179.63</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>201.76</v>
+        <v>197.56</v>
       </c>
       <c r="E52" s="13">
-        <v>171.14</v>
+        <v>169.53</v>
       </c>
       <c r="F52" s="13">
-        <v>181.14</v>
+        <v>179.53</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>210.02</v>
+        <v>209.45</v>
       </c>
       <c r="E56" s="10">
-        <v>187.66</v>
+        <v>186.62</v>
       </c>
       <c r="F56" s="10">
-        <v>197.66</v>
+        <v>196.62</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>200.32</v>
+        <v>199.74</v>
       </c>
       <c r="E57" s="13">
-        <v>179.79</v>
+        <v>178.87</v>
       </c>
       <c r="F57" s="13">
-        <v>189.79</v>
+        <v>188.87</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>200.44</v>
+        <v>199.86</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>199.6</v>
+        <v>199.06</v>
       </c>
       <c r="E59" s="13">
-        <v>174.18</v>
+        <v>173.26</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>195.42</v>
+        <v>194.87</v>
       </c>
       <c r="E60" s="10">
-        <v>170.11</v>
+        <v>169.19</v>
       </c>
       <c r="F60" s="10">
-        <v>180.11</v>
+        <v>179.19</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>201.93</v>
+        <v>201.39</v>
       </c>
       <c r="E61" s="13">
-        <v>184.44</v>
+        <v>183.44</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>211.26</v>
+        <v>210.02</v>
       </c>
       <c r="E62" s="10">
-        <v>188.63</v>
+        <v>187.66</v>
       </c>
       <c r="F62" s="10">
-        <v>198.63</v>
+        <v>197.66</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>201.56</v>
+        <v>200.32</v>
       </c>
       <c r="E63" s="13">
-        <v>180.56</v>
+        <v>179.79</v>
       </c>
       <c r="F63" s="13">
-        <v>190.56</v>
+        <v>189.79</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>201.69</v>
+        <v>200.44</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>200.8</v>
+        <v>199.6</v>
       </c>
       <c r="E65" s="13">
-        <v>174.95</v>
+        <v>174.18</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>196.61</v>
+        <v>195.42</v>
       </c>
       <c r="E66" s="10">
-        <v>170.88</v>
+        <v>170.11</v>
       </c>
       <c r="F66" s="10">
-        <v>180.88</v>
+        <v>180.11</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46154</v>
+        <v>46155</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>203.12</v>
+        <v>201.93</v>
       </c>
       <c r="E67" s="13">
-        <v>185.34</v>
+        <v>184.44</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1880,7 +1880,7 @@
     <mergeCell ref="A33:B33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="66" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C
 # Confidential</oddHeader>
@@ -1892,15 +1892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2160,7 +2151,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -2171,15 +2162,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2199,7 +2191,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2210,6 +2202,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Thu May 14 04:58:50 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{FFA27C10-AAB1-4203-9521-211925F6AF01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{1ECC6180-8E92-4F27-89BF-D8171BBDD964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>195.04</v>
+        <v>196.57</v>
       </c>
       <c r="E8" s="10">
-        <v>167.54</v>
+        <v>167.98</v>
       </c>
       <c r="F8" s="10">
-        <v>177.54</v>
+        <v>177.98</v>
       </c>
       <c r="G8" s="10">
-        <v>168.12</v>
+        <v>168.56</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>195.04</v>
+        <v>196.57</v>
       </c>
       <c r="E9" s="13">
-        <v>167.54</v>
+        <v>167.98</v>
       </c>
       <c r="F9" s="13">
-        <v>177.54</v>
+        <v>177.98</v>
       </c>
       <c r="G9" s="13">
-        <v>168.12</v>
+        <v>168.56</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>196.06</v>
+        <v>197.64</v>
       </c>
       <c r="E10" s="10">
-        <v>168.38</v>
+        <v>168.85</v>
       </c>
       <c r="F10" s="10">
-        <v>178.38</v>
+        <v>178.85</v>
       </c>
       <c r="G10" s="10">
-        <v>169.4</v>
+        <v>169.87</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>195.69</v>
+        <v>195.04</v>
       </c>
       <c r="E11" s="13">
-        <v>168.56</v>
+        <v>167.54</v>
       </c>
       <c r="F11" s="13">
-        <v>178.56</v>
+        <v>177.54</v>
       </c>
       <c r="G11" s="13">
-        <v>169.14</v>
+        <v>168.12</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>195.69</v>
+        <v>195.04</v>
       </c>
       <c r="E12" s="10">
-        <v>168.56</v>
+        <v>167.54</v>
       </c>
       <c r="F12" s="10">
-        <v>178.56</v>
+        <v>177.54</v>
       </c>
       <c r="G12" s="10">
-        <v>169.14</v>
+        <v>168.12</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>196.64</v>
+        <v>196.06</v>
       </c>
       <c r="E13" s="13">
-        <v>169.33</v>
+        <v>168.38</v>
       </c>
       <c r="F13" s="13">
-        <v>179.33</v>
+        <v>178.38</v>
       </c>
       <c r="G13" s="13">
-        <v>170.35</v>
+        <v>169.4</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>200.72</v>
+        <v>202.32</v>
       </c>
       <c r="E17" s="10">
-        <v>174.12</v>
+        <v>174.62</v>
       </c>
       <c r="F17" s="10">
-        <v>184.12</v>
+        <v>184.62</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>201.27</v>
+        <v>200.72</v>
       </c>
       <c r="E18" s="13">
-        <v>175.05</v>
+        <v>174.12</v>
       </c>
       <c r="F18" s="13">
-        <v>185.05</v>
+        <v>184.12</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>196.16</v>
+        <v>197.7</v>
       </c>
       <c r="E22" s="10">
-        <v>167.67</v>
+        <v>168.11</v>
       </c>
       <c r="F22" s="10">
-        <v>177.27</v>
+        <v>177.71</v>
       </c>
       <c r="G22" s="10">
-        <v>166.92</v>
+        <v>167.36</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>202.19</v>
+        <v>203.77</v>
       </c>
       <c r="E23" s="13">
-        <v>173.92</v>
+        <v>174.39</v>
       </c>
       <c r="F23" s="13">
-        <v>183.92</v>
+        <v>184.39</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>202.24</v>
+        <v>203.82</v>
       </c>
       <c r="E24" s="10">
-        <v>174.79</v>
+        <v>175.25</v>
       </c>
       <c r="F24" s="10">
-        <v>184.79</v>
+        <v>185.25</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>202.24</v>
+        <v>203.81</v>
       </c>
       <c r="E25" s="13">
-        <v>174.51</v>
+        <v>174.97</v>
       </c>
       <c r="F25" s="13">
-        <v>184.51</v>
+        <v>184.97</v>
       </c>
       <c r="G25" s="13">
-        <v>173</v>
+        <v>173.47</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>201.62</v>
+        <v>203.2</v>
       </c>
       <c r="E26" s="10">
-        <v>176.49</v>
+        <v>176.96</v>
       </c>
       <c r="F26" s="10">
-        <v>186.49</v>
+        <v>186.96</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>196.81</v>
+        <v>196.16</v>
       </c>
       <c r="E27" s="13">
-        <v>168.69</v>
+        <v>167.67</v>
       </c>
       <c r="F27" s="13">
-        <v>178.29</v>
+        <v>177.27</v>
       </c>
       <c r="G27" s="13">
-        <v>167.94</v>
+        <v>166.92</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>202.77</v>
+        <v>202.19</v>
       </c>
       <c r="E28" s="22">
-        <v>174.87</v>
+        <v>173.92</v>
       </c>
       <c r="F28" s="22">
-        <v>184.87</v>
+        <v>183.92</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>202.82</v>
+        <v>202.24</v>
       </c>
       <c r="E29" s="13">
-        <v>175.75</v>
+        <v>174.79</v>
       </c>
       <c r="F29" s="13">
-        <v>185.75</v>
+        <v>184.79</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>202.81</v>
+        <v>202.24</v>
       </c>
       <c r="E30" s="22">
-        <v>175.48</v>
+        <v>174.51</v>
       </c>
       <c r="F30" s="22">
-        <v>185.48</v>
+        <v>184.51</v>
       </c>
       <c r="G30" s="22">
-        <v>173.97</v>
+        <v>173</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>202.18</v>
+        <v>201.62</v>
       </c>
       <c r="E31" s="13">
-        <v>177.46</v>
+        <v>176.49</v>
       </c>
       <c r="F31" s="13">
-        <v>187.46</v>
+        <v>186.49</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>194.27</v>
+        <v>195.84</v>
       </c>
       <c r="E35" s="10">
-        <v>166.81</v>
+        <v>167.28</v>
       </c>
       <c r="F35" s="10">
-        <v>175.81</v>
+        <v>176.28</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>194.84</v>
+        <v>194.27</v>
       </c>
       <c r="E36" s="13">
-        <v>167.75</v>
+        <v>166.81</v>
       </c>
       <c r="F36" s="13">
-        <v>176.75</v>
+        <v>175.81</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>209.89</v>
+        <v>211.46</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>210.46</v>
+        <v>209.89</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>205.72</v>
+        <v>207.28</v>
       </c>
       <c r="E42" s="10">
-        <v>175.76</v>
+        <v>175.97</v>
       </c>
       <c r="F42" s="10">
-        <v>185.76</v>
+        <v>185.97</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>205.37</v>
+        <v>206.92</v>
       </c>
       <c r="E43" s="13">
-        <v>176.18</v>
+        <v>176.39</v>
       </c>
       <c r="F43" s="13">
-        <v>186.18</v>
+        <v>186.39</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>206.31</v>
+        <v>205.72</v>
       </c>
       <c r="E44" s="10">
-        <v>176.97</v>
+        <v>175.76</v>
       </c>
       <c r="F44" s="10">
-        <v>186.97</v>
+        <v>185.76</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>205.96</v>
+        <v>205.37</v>
       </c>
       <c r="E45" s="13">
-        <v>177.38</v>
+        <v>176.18</v>
       </c>
       <c r="F45" s="13">
-        <v>187.39</v>
+        <v>186.18</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>198.54</v>
+        <v>198.98</v>
       </c>
       <c r="E49" s="10">
-        <v>169.97</v>
+        <v>170.3</v>
       </c>
       <c r="F49" s="10">
-        <v>179.97</v>
+        <v>180.3</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>197.98</v>
+        <v>198.43</v>
       </c>
       <c r="E50" s="13">
-        <v>169.87</v>
+        <v>170.2</v>
       </c>
       <c r="F50" s="13">
-        <v>179.87</v>
+        <v>180.2</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>198.13</v>
+        <v>198.54</v>
       </c>
       <c r="E51" s="10">
-        <v>169.63</v>
+        <v>169.97</v>
       </c>
       <c r="F51" s="10">
-        <v>179.63</v>
+        <v>179.97</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>197.56</v>
+        <v>197.98</v>
       </c>
       <c r="E52" s="13">
-        <v>169.53</v>
+        <v>169.87</v>
       </c>
       <c r="F52" s="13">
-        <v>179.53</v>
+        <v>179.87</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>209.45</v>
+        <v>211.04</v>
       </c>
       <c r="E56" s="10">
-        <v>186.62</v>
+        <v>186.99</v>
       </c>
       <c r="F56" s="10">
-        <v>196.62</v>
+        <v>196.99</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>199.74</v>
+        <v>201.31</v>
       </c>
       <c r="E57" s="13">
-        <v>178.87</v>
+        <v>178.81</v>
       </c>
       <c r="F57" s="13">
-        <v>188.87</v>
+        <v>188.82</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>199.86</v>
+        <v>201.43</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>199.06</v>
+        <v>200.66</v>
       </c>
       <c r="E59" s="13">
-        <v>173.26</v>
+        <v>173.2</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>194.87</v>
+        <v>196.47</v>
       </c>
       <c r="E60" s="10">
-        <v>169.19</v>
+        <v>169.13</v>
       </c>
       <c r="F60" s="10">
-        <v>179.19</v>
+        <v>179.14</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>201.39</v>
+        <v>202.99</v>
       </c>
       <c r="E61" s="13">
-        <v>183.44</v>
+        <v>183.85</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>210.02</v>
+        <v>209.45</v>
       </c>
       <c r="E62" s="10">
-        <v>187.66</v>
+        <v>186.62</v>
       </c>
       <c r="F62" s="10">
-        <v>197.66</v>
+        <v>196.62</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>200.32</v>
+        <v>199.74</v>
       </c>
       <c r="E63" s="13">
-        <v>179.79</v>
+        <v>178.87</v>
       </c>
       <c r="F63" s="13">
-        <v>189.79</v>
+        <v>188.87</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>200.44</v>
+        <v>199.86</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>199.6</v>
+        <v>199.06</v>
       </c>
       <c r="E65" s="13">
-        <v>174.18</v>
+        <v>173.26</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>195.42</v>
+        <v>194.87</v>
       </c>
       <c r="E66" s="10">
-        <v>170.11</v>
+        <v>169.19</v>
       </c>
       <c r="F66" s="10">
-        <v>180.11</v>
+        <v>179.19</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46155</v>
+        <v>46156</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>201.93</v>
+        <v>201.39</v>
       </c>
       <c r="E67" s="13">
-        <v>184.44</v>
+        <v>183.44</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -2152,6 +2152,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
@@ -2160,15 +2169,6 @@
     <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2192,6 +2192,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2202,14 +2210,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Fri May 15 05:02:15 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{1ECC6180-8E92-4F27-89BF-D8171BBDD964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{2BBE064A-7F7A-4961-B3D0-F015C138E4F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,16 +715,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125"/>
-    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.453125"/>
+    <col min="3" max="3" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="6.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -735,7 +735,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -744,7 +744,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -755,7 +755,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -766,7 +766,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -775,7 +775,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -786,7 +786,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -807,133 +807,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>196.57</v>
+        <v>198.85</v>
       </c>
       <c r="E8" s="10">
-        <v>167.98</v>
+        <v>169.53</v>
       </c>
       <c r="F8" s="10">
-        <v>177.98</v>
+        <v>179.53</v>
       </c>
       <c r="G8" s="10">
-        <v>168.56</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>170.11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>196.57</v>
+        <v>198.85</v>
       </c>
       <c r="E9" s="13">
-        <v>167.98</v>
+        <v>169.53</v>
       </c>
       <c r="F9" s="13">
-        <v>177.98</v>
+        <v>179.53</v>
       </c>
       <c r="G9" s="13">
-        <v>168.56</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>170.11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>197.64</v>
+        <v>199.92</v>
       </c>
       <c r="E10" s="10">
-        <v>168.85</v>
+        <v>170.41</v>
       </c>
       <c r="F10" s="10">
-        <v>178.85</v>
+        <v>180.41</v>
       </c>
       <c r="G10" s="10">
-        <v>169.87</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>171.43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>195.04</v>
+        <v>196.57</v>
       </c>
       <c r="E11" s="13">
-        <v>167.54</v>
+        <v>167.98</v>
       </c>
       <c r="F11" s="13">
-        <v>177.54</v>
+        <v>177.98</v>
       </c>
       <c r="G11" s="13">
-        <v>168.12</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>168.56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>195.04</v>
+        <v>196.57</v>
       </c>
       <c r="E12" s="10">
-        <v>167.54</v>
+        <v>167.98</v>
       </c>
       <c r="F12" s="10">
-        <v>177.54</v>
+        <v>177.98</v>
       </c>
       <c r="G12" s="10">
-        <v>168.12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>168.56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>196.06</v>
+        <v>197.64</v>
       </c>
       <c r="E13" s="13">
-        <v>168.38</v>
+        <v>168.85</v>
       </c>
       <c r="F13" s="13">
-        <v>178.38</v>
+        <v>178.85</v>
       </c>
       <c r="G13" s="13">
-        <v>169.4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>169.87</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -942,7 +942,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -953,7 +953,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -972,45 +972,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>202.32</v>
+        <v>204.64</v>
       </c>
       <c r="E17" s="10">
-        <v>174.62</v>
+        <v>176.76</v>
       </c>
       <c r="F17" s="10">
-        <v>184.62</v>
+        <v>186.76</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>200.72</v>
+        <v>202.32</v>
       </c>
       <c r="E18" s="13">
-        <v>174.12</v>
+        <v>174.62</v>
       </c>
       <c r="F18" s="13">
-        <v>184.12</v>
+        <v>184.62</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1019,7 +1019,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1030,7 +1030,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1051,217 +1051,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>197.7</v>
+        <v>199.97</v>
       </c>
       <c r="E22" s="10">
-        <v>168.11</v>
+        <v>170.2</v>
       </c>
       <c r="F22" s="10">
-        <v>177.71</v>
+        <v>179.8</v>
       </c>
       <c r="G22" s="10">
-        <v>167.36</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>169.46</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>203.77</v>
+        <v>204.95</v>
       </c>
       <c r="E23" s="13">
-        <v>174.39</v>
+        <v>175.96</v>
       </c>
       <c r="F23" s="13">
-        <v>184.39</v>
+        <v>185.96</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>203.82</v>
+        <v>205.01</v>
       </c>
       <c r="E24" s="10">
-        <v>175.25</v>
+        <v>176.8</v>
       </c>
       <c r="F24" s="10">
-        <v>185.25</v>
+        <v>186.8</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>203.81</v>
+        <v>205</v>
       </c>
       <c r="E25" s="13">
-        <v>174.97</v>
+        <v>176.53</v>
       </c>
       <c r="F25" s="13">
-        <v>184.97</v>
+        <v>186.53</v>
       </c>
       <c r="G25" s="13">
-        <v>173.47</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>175.02</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>203.2</v>
+        <v>204.39</v>
       </c>
       <c r="E26" s="10">
-        <v>176.96</v>
+        <v>178.53</v>
       </c>
       <c r="F26" s="10">
-        <v>186.96</v>
+        <v>188.53</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>196.16</v>
+        <v>197.7</v>
       </c>
       <c r="E27" s="13">
-        <v>167.67</v>
+        <v>168.11</v>
       </c>
       <c r="F27" s="13">
-        <v>177.27</v>
+        <v>177.71</v>
       </c>
       <c r="G27" s="13">
-        <v>166.92</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>167.36</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>202.19</v>
+        <v>203.77</v>
       </c>
       <c r="E28" s="22">
-        <v>173.92</v>
+        <v>174.39</v>
       </c>
       <c r="F28" s="22">
-        <v>183.92</v>
+        <v>184.39</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>202.24</v>
+        <v>203.82</v>
       </c>
       <c r="E29" s="13">
-        <v>174.79</v>
+        <v>175.25</v>
       </c>
       <c r="F29" s="13">
-        <v>184.79</v>
+        <v>185.25</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>202.24</v>
+        <v>203.81</v>
       </c>
       <c r="E30" s="22">
-        <v>174.51</v>
+        <v>174.97</v>
       </c>
       <c r="F30" s="22">
-        <v>184.51</v>
+        <v>184.97</v>
       </c>
       <c r="G30" s="22">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>173.47</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>201.62</v>
+        <v>203.2</v>
       </c>
       <c r="E31" s="13">
-        <v>176.49</v>
+        <v>176.96</v>
       </c>
       <c r="F31" s="13">
-        <v>186.49</v>
+        <v>186.96</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1270,7 +1270,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1281,7 +1281,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1300,54 +1300,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>195.84</v>
+        <v>198.12</v>
       </c>
       <c r="E35" s="10">
-        <v>167.28</v>
+        <v>169.38</v>
       </c>
       <c r="F35" s="10">
-        <v>176.28</v>
+        <v>178.38</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>194.27</v>
+        <v>195.84</v>
       </c>
       <c r="E36" s="13">
-        <v>166.81</v>
+        <v>167.28</v>
       </c>
       <c r="F36" s="13">
-        <v>175.81</v>
+        <v>176.28</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>211.46</v>
+        <v>213.74</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1357,16 +1357,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>209.89</v>
+        <v>211.46</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1385,7 +1385,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1396,7 +1396,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1415,83 +1415,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>207.28</v>
+        <v>207.89</v>
       </c>
       <c r="E42" s="10">
-        <v>175.97</v>
+        <v>177.51</v>
       </c>
       <c r="F42" s="10">
-        <v>185.97</v>
+        <v>187.51</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>206.92</v>
+        <v>207.53</v>
       </c>
       <c r="E43" s="13">
-        <v>176.39</v>
+        <v>177.92</v>
       </c>
       <c r="F43" s="13">
-        <v>186.39</v>
+        <v>187.92</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>205.72</v>
+        <v>207.28</v>
       </c>
       <c r="E44" s="10">
-        <v>175.76</v>
+        <v>175.97</v>
       </c>
       <c r="F44" s="10">
-        <v>185.76</v>
+        <v>185.97</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>205.37</v>
+        <v>206.92</v>
       </c>
       <c r="E45" s="13">
-        <v>176.18</v>
+        <v>176.39</v>
       </c>
       <c r="F45" s="13">
-        <v>186.18</v>
+        <v>186.39</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1500,7 +1500,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1511,7 +1511,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1530,83 +1530,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>198.98</v>
+        <v>198.66</v>
       </c>
       <c r="E49" s="10">
-        <v>170.3</v>
+        <v>170.1</v>
       </c>
       <c r="F49" s="10">
-        <v>180.3</v>
+        <v>180.1</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>198.43</v>
+        <v>198.12</v>
       </c>
       <c r="E50" s="13">
-        <v>170.2</v>
+        <v>170.01</v>
       </c>
       <c r="F50" s="13">
-        <v>180.2</v>
+        <v>180.01</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A51" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>198.54</v>
+        <v>198.98</v>
       </c>
       <c r="E51" s="10">
-        <v>169.97</v>
+        <v>170.3</v>
       </c>
       <c r="F51" s="10">
-        <v>179.97</v>
+        <v>180.3</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>197.98</v>
+        <v>198.43</v>
       </c>
       <c r="E52" s="13">
-        <v>169.87</v>
+        <v>170.2</v>
       </c>
       <c r="F52" s="13">
-        <v>179.87</v>
+        <v>180.2</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1615,7 +1615,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1626,7 +1626,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1645,54 +1645,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A56" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>211.04</v>
+        <v>213.34</v>
       </c>
       <c r="E56" s="10">
-        <v>186.99</v>
+        <v>188.97</v>
       </c>
       <c r="F56" s="10">
-        <v>196.99</v>
+        <v>198.97</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A57" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>201.31</v>
+        <v>203.6</v>
       </c>
       <c r="E57" s="13">
-        <v>178.81</v>
+        <v>180.95</v>
       </c>
       <c r="F57" s="13">
-        <v>188.82</v>
+        <v>190.95</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A58" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>201.43</v>
+        <v>203.71</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1702,111 +1702,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A59" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>200.66</v>
+        <v>202.98</v>
       </c>
       <c r="E59" s="13">
-        <v>173.2</v>
+        <v>175.34</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A60" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>196.47</v>
+        <v>198.79</v>
       </c>
       <c r="E60" s="10">
-        <v>169.13</v>
+        <v>171.27</v>
       </c>
       <c r="F60" s="10">
-        <v>179.14</v>
+        <v>181.27</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A61" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>202.99</v>
+        <v>205.31</v>
       </c>
       <c r="E61" s="13">
-        <v>183.85</v>
+        <v>185.89</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A62" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>209.45</v>
+        <v>211.04</v>
       </c>
       <c r="E62" s="10">
-        <v>186.62</v>
+        <v>186.99</v>
       </c>
       <c r="F62" s="10">
-        <v>196.62</v>
+        <v>196.99</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A63" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>199.74</v>
+        <v>201.31</v>
       </c>
       <c r="E63" s="13">
-        <v>178.87</v>
+        <v>178.81</v>
       </c>
       <c r="F63" s="13">
-        <v>188.87</v>
+        <v>188.82</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A64" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>199.86</v>
+        <v>201.43</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1816,55 +1816,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>199.06</v>
+        <v>200.66</v>
       </c>
       <c r="E65" s="13">
-        <v>173.26</v>
+        <v>173.2</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="7">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>194.87</v>
+        <v>196.47</v>
       </c>
       <c r="E66" s="10">
-        <v>169.19</v>
+        <v>169.13</v>
       </c>
       <c r="F66" s="10">
-        <v>179.19</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <v>179.14</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="11">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>201.39</v>
+        <v>202.99</v>
       </c>
       <c r="E67" s="13">
-        <v>183.44</v>
+        <v>183.85</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,6 +1892,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2151,27 +2171,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2191,25 +2210,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Mon May 18 05:34:51 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{2BBE064A-7F7A-4961-B3D0-F015C138E4F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{40E21959-5EFA-4AFD-A31C-E44DC07D56B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" concurrentManualCount="12"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -715,16 +715,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.453125"/>
-    <col min="3" max="3" width="18.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125"/>
+    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="6.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -735,7 +735,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -744,7 +744,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -755,7 +755,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -766,7 +766,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -775,7 +775,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -786,7 +786,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -807,133 +807,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>198.85</v>
+        <v>200.96</v>
       </c>
       <c r="E8" s="10">
-        <v>169.53</v>
+        <v>172.46</v>
       </c>
       <c r="F8" s="10">
-        <v>179.53</v>
+        <v>182.46</v>
       </c>
       <c r="G8" s="10">
-        <v>170.11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+        <v>173.04</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>198.85</v>
+        <v>200.96</v>
       </c>
       <c r="E9" s="13">
-        <v>169.53</v>
+        <v>172.46</v>
       </c>
       <c r="F9" s="13">
-        <v>179.53</v>
+        <v>182.46</v>
       </c>
       <c r="G9" s="13">
-        <v>170.11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+        <v>173.04</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>199.92</v>
+        <v>202.05</v>
       </c>
       <c r="E10" s="10">
-        <v>170.41</v>
+        <v>173.36</v>
       </c>
       <c r="F10" s="10">
-        <v>180.41</v>
+        <v>183.36</v>
       </c>
       <c r="G10" s="10">
-        <v>171.43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+        <v>174.38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>196.57</v>
+        <v>198.85</v>
       </c>
       <c r="E11" s="13">
-        <v>167.98</v>
+        <v>169.53</v>
       </c>
       <c r="F11" s="13">
-        <v>177.98</v>
+        <v>179.53</v>
       </c>
       <c r="G11" s="13">
-        <v>168.56</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+        <v>170.11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>196.57</v>
+        <v>198.85</v>
       </c>
       <c r="E12" s="10">
-        <v>167.98</v>
+        <v>169.53</v>
       </c>
       <c r="F12" s="10">
-        <v>177.98</v>
+        <v>179.53</v>
       </c>
       <c r="G12" s="10">
-        <v>168.56</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+        <v>170.11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>197.64</v>
+        <v>199.92</v>
       </c>
       <c r="E13" s="13">
-        <v>168.85</v>
+        <v>170.41</v>
       </c>
       <c r="F13" s="13">
-        <v>178.85</v>
+        <v>180.41</v>
       </c>
       <c r="G13" s="13">
-        <v>169.87</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+        <v>171.43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -942,7 +942,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -953,7 +953,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -972,45 +972,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>204.64</v>
+        <v>206.79</v>
       </c>
       <c r="E17" s="10">
-        <v>176.76</v>
+        <v>179.74</v>
       </c>
       <c r="F17" s="10">
-        <v>186.76</v>
+        <v>189.74</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>202.32</v>
+        <v>204.64</v>
       </c>
       <c r="E18" s="13">
-        <v>174.62</v>
+        <v>176.76</v>
       </c>
       <c r="F18" s="13">
-        <v>184.62</v>
+        <v>186.76</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1019,7 +1019,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1030,7 +1030,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1051,217 +1051,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>199.97</v>
+        <v>202.08</v>
       </c>
       <c r="E22" s="10">
-        <v>170.2</v>
+        <v>173.13</v>
       </c>
       <c r="F22" s="10">
-        <v>179.8</v>
+        <v>182.73</v>
       </c>
       <c r="G22" s="10">
-        <v>169.46</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+        <v>172.39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>204.95</v>
+        <v>207.08</v>
       </c>
       <c r="E23" s="13">
-        <v>175.96</v>
+        <v>178.37</v>
       </c>
       <c r="F23" s="13">
-        <v>185.96</v>
+        <v>188.37</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>205.01</v>
+        <v>206.59</v>
       </c>
       <c r="E24" s="10">
-        <v>176.8</v>
+        <v>179.19</v>
       </c>
       <c r="F24" s="10">
-        <v>186.8</v>
+        <v>189.19</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>205</v>
+        <v>207.13</v>
       </c>
       <c r="E25" s="13">
-        <v>176.53</v>
+        <v>178.92</v>
       </c>
       <c r="F25" s="13">
-        <v>186.53</v>
+        <v>188.92</v>
       </c>
       <c r="G25" s="13">
-        <v>175.02</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+        <v>177.41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>204.39</v>
+        <v>205.99</v>
       </c>
       <c r="E26" s="10">
-        <v>178.53</v>
+        <v>180.94</v>
       </c>
       <c r="F26" s="10">
-        <v>188.53</v>
+        <v>190.94</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>197.7</v>
+        <v>199.97</v>
       </c>
       <c r="E27" s="13">
-        <v>168.11</v>
+        <v>170.2</v>
       </c>
       <c r="F27" s="13">
-        <v>177.71</v>
+        <v>179.8</v>
       </c>
       <c r="G27" s="13">
-        <v>167.36</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+        <v>169.46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>203.77</v>
+        <v>204.95</v>
       </c>
       <c r="E28" s="22">
-        <v>174.39</v>
+        <v>175.96</v>
       </c>
       <c r="F28" s="22">
-        <v>184.39</v>
+        <v>185.96</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>203.82</v>
+        <v>205.01</v>
       </c>
       <c r="E29" s="13">
-        <v>175.25</v>
+        <v>176.8</v>
       </c>
       <c r="F29" s="13">
-        <v>185.25</v>
+        <v>186.8</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>203.81</v>
+        <v>205</v>
       </c>
       <c r="E30" s="22">
-        <v>174.97</v>
+        <v>176.53</v>
       </c>
       <c r="F30" s="22">
-        <v>184.97</v>
+        <v>186.53</v>
       </c>
       <c r="G30" s="22">
-        <v>173.47</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+        <v>175.02</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>203.2</v>
+        <v>204.39</v>
       </c>
       <c r="E31" s="13">
-        <v>176.96</v>
+        <v>178.53</v>
       </c>
       <c r="F31" s="13">
-        <v>186.96</v>
+        <v>188.53</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1270,7 +1270,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1281,7 +1281,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1300,54 +1300,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>198.12</v>
+        <v>200.25</v>
       </c>
       <c r="E35" s="10">
-        <v>169.38</v>
+        <v>172.32</v>
       </c>
       <c r="F35" s="10">
-        <v>178.38</v>
+        <v>181.33</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>195.84</v>
+        <v>198.12</v>
       </c>
       <c r="E36" s="13">
-        <v>167.28</v>
+        <v>169.38</v>
       </c>
       <c r="F36" s="13">
-        <v>176.28</v>
+        <v>178.38</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>213.74</v>
+        <v>215.87</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1357,16 +1357,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>211.46</v>
+        <v>213.74</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1385,7 +1385,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1396,7 +1396,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1415,83 +1415,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>207.89</v>
+        <v>210.01</v>
       </c>
       <c r="E42" s="10">
-        <v>177.51</v>
+        <v>180.1</v>
       </c>
       <c r="F42" s="10">
-        <v>187.51</v>
+        <v>190.1</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>207.53</v>
+        <v>209.65</v>
       </c>
       <c r="E43" s="13">
-        <v>177.92</v>
+        <v>180.52</v>
       </c>
       <c r="F43" s="13">
-        <v>187.92</v>
+        <v>190.52</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>207.28</v>
+        <v>207.89</v>
       </c>
       <c r="E44" s="10">
-        <v>175.97</v>
+        <v>177.51</v>
       </c>
       <c r="F44" s="10">
-        <v>185.97</v>
+        <v>187.51</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>206.92</v>
+        <v>207.53</v>
       </c>
       <c r="E45" s="13">
-        <v>176.39</v>
+        <v>177.92</v>
       </c>
       <c r="F45" s="13">
-        <v>186.39</v>
+        <v>187.92</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1500,7 +1500,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1511,7 +1511,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1530,83 +1530,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>198.66</v>
+        <v>199.75</v>
       </c>
       <c r="E49" s="10">
-        <v>170.1</v>
+        <v>170.95</v>
       </c>
       <c r="F49" s="10">
-        <v>180.1</v>
+        <v>180.95</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>198.12</v>
+        <v>199.22</v>
       </c>
       <c r="E50" s="13">
-        <v>170.01</v>
+        <v>170.87</v>
       </c>
       <c r="F50" s="13">
-        <v>180.01</v>
+        <v>180.87</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>198.98</v>
+        <v>198.66</v>
       </c>
       <c r="E51" s="10">
-        <v>170.3</v>
+        <v>170.1</v>
       </c>
       <c r="F51" s="10">
-        <v>180.3</v>
+        <v>180.1</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>198.43</v>
+        <v>198.12</v>
       </c>
       <c r="E52" s="13">
-        <v>170.2</v>
+        <v>170.01</v>
       </c>
       <c r="F52" s="13">
-        <v>180.2</v>
+        <v>180.01</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1615,7 +1615,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1626,7 +1626,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1645,54 +1645,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>213.34</v>
+        <v>215.49</v>
       </c>
       <c r="E56" s="10">
-        <v>188.97</v>
+        <v>191.81</v>
       </c>
       <c r="F56" s="10">
-        <v>198.97</v>
+        <v>201.81</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>203.6</v>
+        <v>205.73</v>
       </c>
       <c r="E57" s="13">
-        <v>180.95</v>
+        <v>183.37</v>
       </c>
       <c r="F57" s="13">
-        <v>190.95</v>
+        <v>193.37</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>203.71</v>
+        <v>205.83</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1702,111 +1702,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>202.98</v>
+        <v>205.14</v>
       </c>
       <c r="E59" s="13">
-        <v>175.34</v>
+        <v>177.75</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>198.79</v>
+        <v>200.95</v>
       </c>
       <c r="E60" s="10">
-        <v>171.27</v>
+        <v>173.69</v>
       </c>
       <c r="F60" s="10">
-        <v>181.27</v>
+        <v>183.69</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>205.31</v>
+        <v>207.47</v>
       </c>
       <c r="E61" s="13">
-        <v>185.89</v>
+        <v>188.79</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>211.04</v>
+        <v>213.34</v>
       </c>
       <c r="E62" s="10">
-        <v>186.99</v>
+        <v>188.97</v>
       </c>
       <c r="F62" s="10">
-        <v>196.99</v>
+        <v>198.97</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>201.31</v>
+        <v>203.6</v>
       </c>
       <c r="E63" s="13">
-        <v>178.81</v>
+        <v>180.95</v>
       </c>
       <c r="F63" s="13">
-        <v>188.82</v>
+        <v>190.95</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>201.43</v>
+        <v>203.71</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1816,55 +1816,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>200.66</v>
+        <v>202.98</v>
       </c>
       <c r="E65" s="13">
-        <v>173.2</v>
+        <v>175.34</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>196.47</v>
+        <v>198.79</v>
       </c>
       <c r="E66" s="10">
-        <v>169.13</v>
+        <v>171.27</v>
       </c>
       <c r="F66" s="10">
-        <v>179.14</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+        <v>181.27</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46157</v>
+        <v>46158</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>202.99</v>
+        <v>205.31</v>
       </c>
       <c r="E67" s="13">
-        <v>183.85</v>
+        <v>185.89</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Tue May 19 05:14:10 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{40E21959-5EFA-4AFD-A31C-E44DC07D56B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{D8C4612E-152D-40B6-9550-E8DE4E9BD487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>200.96</v>
+        <v>203.21</v>
       </c>
       <c r="E8" s="10">
-        <v>172.46</v>
+        <v>175.11</v>
       </c>
       <c r="F8" s="10">
-        <v>182.46</v>
+        <v>185.11</v>
       </c>
       <c r="G8" s="10">
-        <v>173.04</v>
+        <v>175.69</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>200.96</v>
+        <v>203.21</v>
       </c>
       <c r="E9" s="13">
-        <v>172.46</v>
+        <v>175.11</v>
       </c>
       <c r="F9" s="13">
-        <v>182.46</v>
+        <v>185.11</v>
       </c>
       <c r="G9" s="13">
-        <v>173.04</v>
+        <v>175.69</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>202.05</v>
+        <v>204.31</v>
       </c>
       <c r="E10" s="10">
-        <v>173.36</v>
+        <v>176.03</v>
       </c>
       <c r="F10" s="10">
-        <v>183.36</v>
+        <v>186.03</v>
       </c>
       <c r="G10" s="10">
-        <v>174.38</v>
+        <v>177.05</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>198.85</v>
+        <v>200.96</v>
       </c>
       <c r="E11" s="13">
-        <v>169.53</v>
+        <v>172.46</v>
       </c>
       <c r="F11" s="13">
-        <v>179.53</v>
+        <v>182.46</v>
       </c>
       <c r="G11" s="13">
-        <v>170.11</v>
+        <v>173.04</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>198.85</v>
+        <v>200.96</v>
       </c>
       <c r="E12" s="10">
-        <v>169.53</v>
+        <v>172.46</v>
       </c>
       <c r="F12" s="10">
-        <v>179.53</v>
+        <v>182.46</v>
       </c>
       <c r="G12" s="10">
-        <v>170.11</v>
+        <v>173.04</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>199.92</v>
+        <v>202.05</v>
       </c>
       <c r="E13" s="13">
-        <v>170.41</v>
+        <v>173.36</v>
       </c>
       <c r="F13" s="13">
-        <v>180.41</v>
+        <v>183.36</v>
       </c>
       <c r="G13" s="13">
-        <v>171.43</v>
+        <v>174.38</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>206.79</v>
+        <v>209.07</v>
       </c>
       <c r="E17" s="10">
-        <v>179.74</v>
+        <v>182.44</v>
       </c>
       <c r="F17" s="10">
-        <v>189.74</v>
+        <v>192.44</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>204.64</v>
+        <v>206.79</v>
       </c>
       <c r="E18" s="13">
-        <v>176.76</v>
+        <v>179.74</v>
       </c>
       <c r="F18" s="13">
-        <v>186.76</v>
+        <v>189.74</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>202.08</v>
+        <v>204.32</v>
       </c>
       <c r="E22" s="10">
-        <v>173.13</v>
+        <v>175.78</v>
       </c>
       <c r="F22" s="10">
-        <v>182.73</v>
+        <v>185.38</v>
       </c>
       <c r="G22" s="10">
-        <v>172.39</v>
+        <v>175.04</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>207.08</v>
+        <v>208.24</v>
       </c>
       <c r="E23" s="13">
-        <v>178.37</v>
+        <v>181.05</v>
       </c>
       <c r="F23" s="13">
-        <v>188.37</v>
+        <v>191.05</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>206.59</v>
+        <v>208.3</v>
       </c>
       <c r="E24" s="10">
-        <v>179.19</v>
+        <v>181.86</v>
       </c>
       <c r="F24" s="10">
-        <v>189.19</v>
+        <v>191.86</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>207.13</v>
+        <v>208.29</v>
       </c>
       <c r="E25" s="13">
-        <v>178.92</v>
+        <v>181.59</v>
       </c>
       <c r="F25" s="13">
-        <v>188.92</v>
+        <v>191.59</v>
       </c>
       <c r="G25" s="13">
-        <v>177.41</v>
+        <v>180.08</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>205.99</v>
+        <v>207.7</v>
       </c>
       <c r="E26" s="10">
-        <v>180.94</v>
+        <v>183.63</v>
       </c>
       <c r="F26" s="10">
-        <v>190.94</v>
+        <v>193.63</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>199.97</v>
+        <v>202.08</v>
       </c>
       <c r="E27" s="13">
-        <v>170.2</v>
+        <v>173.13</v>
       </c>
       <c r="F27" s="13">
-        <v>179.8</v>
+        <v>182.73</v>
       </c>
       <c r="G27" s="13">
-        <v>169.46</v>
+        <v>172.39</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>204.95</v>
+        <v>207.08</v>
       </c>
       <c r="E28" s="22">
-        <v>175.96</v>
+        <v>178.37</v>
       </c>
       <c r="F28" s="22">
-        <v>185.96</v>
+        <v>188.37</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>205.01</v>
+        <v>206.59</v>
       </c>
       <c r="E29" s="13">
-        <v>176.8</v>
+        <v>179.19</v>
       </c>
       <c r="F29" s="13">
-        <v>186.8</v>
+        <v>189.19</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>205</v>
+        <v>207.13</v>
       </c>
       <c r="E30" s="22">
-        <v>176.53</v>
+        <v>178.92</v>
       </c>
       <c r="F30" s="22">
-        <v>186.53</v>
+        <v>188.92</v>
       </c>
       <c r="G30" s="22">
-        <v>175.02</v>
+        <v>177.41</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>204.39</v>
+        <v>205.99</v>
       </c>
       <c r="E31" s="13">
-        <v>178.53</v>
+        <v>180.94</v>
       </c>
       <c r="F31" s="13">
-        <v>188.53</v>
+        <v>190.94</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>200.25</v>
+        <v>202.5</v>
       </c>
       <c r="E35" s="10">
-        <v>172.32</v>
+        <v>174.99</v>
       </c>
       <c r="F35" s="10">
-        <v>181.33</v>
+        <v>183.99</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>198.12</v>
+        <v>200.25</v>
       </c>
       <c r="E36" s="13">
-        <v>169.38</v>
+        <v>172.32</v>
       </c>
       <c r="F36" s="13">
-        <v>178.38</v>
+        <v>181.33</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>215.87</v>
+        <v>218.12</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>213.74</v>
+        <v>215.87</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>210.01</v>
+        <v>212.25</v>
       </c>
       <c r="E42" s="10">
-        <v>180.1</v>
+        <v>182.04</v>
       </c>
       <c r="F42" s="10">
-        <v>190.1</v>
+        <v>192.04</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>209.65</v>
+        <v>211.89</v>
       </c>
       <c r="E43" s="13">
-        <v>180.52</v>
+        <v>182.45</v>
       </c>
       <c r="F43" s="13">
-        <v>190.52</v>
+        <v>192.45</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>207.89</v>
+        <v>210.01</v>
       </c>
       <c r="E44" s="10">
-        <v>177.51</v>
+        <v>180.1</v>
       </c>
       <c r="F44" s="10">
-        <v>187.51</v>
+        <v>190.1</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>207.53</v>
+        <v>209.65</v>
       </c>
       <c r="E45" s="13">
-        <v>177.92</v>
+        <v>180.52</v>
       </c>
       <c r="F45" s="13">
-        <v>187.92</v>
+        <v>190.52</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>199.75</v>
+        <v>201.11</v>
       </c>
       <c r="E49" s="10">
-        <v>170.95</v>
+        <v>173.22</v>
       </c>
       <c r="F49" s="10">
-        <v>180.95</v>
+        <v>183.22</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>199.22</v>
+        <v>200.59</v>
       </c>
       <c r="E50" s="13">
-        <v>170.87</v>
+        <v>173.14</v>
       </c>
       <c r="F50" s="13">
-        <v>180.87</v>
+        <v>183.14</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>198.66</v>
+        <v>199.75</v>
       </c>
       <c r="E51" s="10">
-        <v>170.1</v>
+        <v>170.95</v>
       </c>
       <c r="F51" s="10">
-        <v>180.1</v>
+        <v>180.95</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>198.12</v>
+        <v>199.22</v>
       </c>
       <c r="E52" s="13">
-        <v>170.01</v>
+        <v>170.87</v>
       </c>
       <c r="F52" s="13">
-        <v>180.01</v>
+        <v>180.87</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>215.49</v>
+        <v>217.77</v>
       </c>
       <c r="E56" s="10">
-        <v>191.81</v>
+        <v>194.39</v>
       </c>
       <c r="F56" s="10">
-        <v>201.81</v>
+        <v>204.39</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>205.73</v>
+        <v>208</v>
       </c>
       <c r="E57" s="13">
-        <v>183.37</v>
+        <v>186.05</v>
       </c>
       <c r="F57" s="13">
-        <v>193.37</v>
+        <v>196.05</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>205.83</v>
+        <v>208.08</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>205.14</v>
+        <v>207.41</v>
       </c>
       <c r="E59" s="13">
-        <v>177.75</v>
+        <v>180.43</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>200.95</v>
+        <v>203.22</v>
       </c>
       <c r="E60" s="10">
-        <v>173.69</v>
+        <v>176.37</v>
       </c>
       <c r="F60" s="10">
-        <v>183.69</v>
+        <v>186.37</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>207.47</v>
+        <v>209.74</v>
       </c>
       <c r="E61" s="13">
-        <v>188.79</v>
+        <v>191.42</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>213.34</v>
+        <v>215.49</v>
       </c>
       <c r="E62" s="10">
-        <v>188.97</v>
+        <v>191.81</v>
       </c>
       <c r="F62" s="10">
-        <v>198.97</v>
+        <v>201.81</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>203.6</v>
+        <v>205.73</v>
       </c>
       <c r="E63" s="13">
-        <v>180.95</v>
+        <v>183.37</v>
       </c>
       <c r="F63" s="13">
-        <v>190.95</v>
+        <v>193.37</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>203.71</v>
+        <v>205.83</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>202.98</v>
+        <v>205.14</v>
       </c>
       <c r="E65" s="13">
-        <v>175.34</v>
+        <v>177.75</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>198.79</v>
+        <v>200.95</v>
       </c>
       <c r="E66" s="10">
-        <v>171.27</v>
+        <v>173.69</v>
       </c>
       <c r="F66" s="10">
-        <v>181.27</v>
+        <v>183.69</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46158</v>
+        <v>46161</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>205.31</v>
+        <v>207.47</v>
       </c>
       <c r="E67" s="13">
-        <v>185.89</v>
+        <v>188.79</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,26 +1892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2171,26 +2151,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2210,6 +2191,25 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Wed May 20 05:32:55 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{D8C4612E-152D-40B6-9550-E8DE4E9BD487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="14_{A4804B32-B63E-4E0B-8D42-6CA20914FF5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE3EE824-26D7-4FD5-BAAC-855D5E1323B8}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="3294" yWindow="3294" windowWidth="17280" windowHeight="9984" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" concurrentManualCount="12"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -715,16 +715,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125"/>
-    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.41796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.41796875"/>
+    <col min="3" max="3" width="18.26171875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.83984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="6.578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="22.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -735,7 +735,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -744,7 +744,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -755,7 +755,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -766,7 +766,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -775,7 +775,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="19.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -786,7 +786,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -807,133 +807,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>203.21</v>
+        <v>204.8</v>
       </c>
       <c r="E8" s="10">
-        <v>175.11</v>
+        <v>176.71</v>
       </c>
       <c r="F8" s="10">
-        <v>185.11</v>
+        <v>186.71</v>
       </c>
       <c r="G8" s="10">
-        <v>175.69</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>177.29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>203.21</v>
+        <v>204.8</v>
       </c>
       <c r="E9" s="13">
-        <v>175.11</v>
+        <v>176.71</v>
       </c>
       <c r="F9" s="13">
-        <v>185.11</v>
+        <v>186.71</v>
       </c>
       <c r="G9" s="13">
-        <v>175.69</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>177.29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>204.31</v>
+        <v>205.89</v>
       </c>
       <c r="E10" s="10">
-        <v>176.03</v>
+        <v>177.63</v>
       </c>
       <c r="F10" s="10">
-        <v>186.03</v>
+        <v>187.63</v>
       </c>
       <c r="G10" s="10">
-        <v>177.05</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>178.65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>200.96</v>
+        <v>203.21</v>
       </c>
       <c r="E11" s="13">
-        <v>172.46</v>
+        <v>175.11</v>
       </c>
       <c r="F11" s="13">
-        <v>182.46</v>
+        <v>185.11</v>
       </c>
       <c r="G11" s="13">
-        <v>173.04</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>175.69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>200.96</v>
+        <v>203.21</v>
       </c>
       <c r="E12" s="10">
-        <v>172.46</v>
+        <v>175.11</v>
       </c>
       <c r="F12" s="10">
-        <v>182.46</v>
+        <v>185.11</v>
       </c>
       <c r="G12" s="10">
-        <v>173.04</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>175.69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>202.05</v>
+        <v>204.31</v>
       </c>
       <c r="E13" s="13">
-        <v>173.36</v>
+        <v>176.03</v>
       </c>
       <c r="F13" s="13">
-        <v>183.36</v>
+        <v>186.03</v>
       </c>
       <c r="G13" s="13">
-        <v>174.38</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+        <v>177.05</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -942,7 +942,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="19.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -953,7 +953,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -972,45 +972,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>209.07</v>
+        <v>210.13</v>
       </c>
       <c r="E17" s="10">
-        <v>182.44</v>
+        <v>184.06</v>
       </c>
       <c r="F17" s="10">
-        <v>192.44</v>
+        <v>194.06</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>206.79</v>
+        <v>209.07</v>
       </c>
       <c r="E18" s="13">
-        <v>179.74</v>
+        <v>182.44</v>
       </c>
       <c r="F18" s="13">
-        <v>189.74</v>
+        <v>192.44</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1019,7 +1019,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="19.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1030,7 +1030,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1051,217 +1051,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>204.32</v>
+        <v>205.91</v>
       </c>
       <c r="E22" s="10">
-        <v>175.78</v>
+        <v>177.93</v>
       </c>
       <c r="F22" s="10">
-        <v>185.38</v>
+        <v>187.53</v>
       </c>
       <c r="G22" s="10">
-        <v>175.04</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>177.18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>208.24</v>
+        <v>209.82</v>
       </c>
       <c r="E23" s="13">
-        <v>181.05</v>
+        <v>182.65</v>
       </c>
       <c r="F23" s="13">
-        <v>191.05</v>
+        <v>192.65</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>208.3</v>
+        <v>209.88</v>
       </c>
       <c r="E24" s="10">
-        <v>181.86</v>
+        <v>183.44</v>
       </c>
       <c r="F24" s="10">
-        <v>191.86</v>
+        <v>193.44</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>208.29</v>
+        <v>209.87</v>
       </c>
       <c r="E25" s="13">
-        <v>181.59</v>
+        <v>183.17</v>
       </c>
       <c r="F25" s="13">
-        <v>191.59</v>
+        <v>193.17</v>
       </c>
       <c r="G25" s="13">
-        <v>180.08</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+        <v>181.67</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>207.7</v>
+        <v>209.29</v>
       </c>
       <c r="E26" s="10">
-        <v>183.63</v>
+        <v>185.23</v>
       </c>
       <c r="F26" s="10">
-        <v>193.63</v>
+        <v>195.23</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>202.08</v>
+        <v>204.32</v>
       </c>
       <c r="E27" s="13">
-        <v>173.13</v>
+        <v>175.78</v>
       </c>
       <c r="F27" s="13">
-        <v>182.73</v>
+        <v>185.38</v>
       </c>
       <c r="G27" s="13">
-        <v>172.39</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+        <v>175.04</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>207.08</v>
+        <v>208.24</v>
       </c>
       <c r="E28" s="22">
-        <v>178.37</v>
+        <v>181.05</v>
       </c>
       <c r="F28" s="22">
-        <v>188.37</v>
+        <v>191.05</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>206.59</v>
+        <v>208.3</v>
       </c>
       <c r="E29" s="13">
-        <v>179.19</v>
+        <v>181.86</v>
       </c>
       <c r="F29" s="13">
-        <v>189.19</v>
+        <v>191.86</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>207.13</v>
+        <v>208.29</v>
       </c>
       <c r="E30" s="22">
-        <v>178.92</v>
+        <v>181.59</v>
       </c>
       <c r="F30" s="22">
-        <v>188.92</v>
+        <v>191.59</v>
       </c>
       <c r="G30" s="22">
-        <v>177.41</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>180.08</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>205.99</v>
+        <v>207.7</v>
       </c>
       <c r="E31" s="13">
-        <v>180.94</v>
+        <v>183.63</v>
       </c>
       <c r="F31" s="13">
-        <v>190.94</v>
+        <v>193.63</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1270,7 +1270,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" ht="19.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1281,7 +1281,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1300,54 +1300,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>202.5</v>
+        <v>204.08</v>
       </c>
       <c r="E35" s="10">
-        <v>174.99</v>
+        <v>176.58</v>
       </c>
       <c r="F35" s="10">
-        <v>183.99</v>
+        <v>185.58</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>200.25</v>
+        <v>202.5</v>
       </c>
       <c r="E36" s="13">
-        <v>172.32</v>
+        <v>174.99</v>
       </c>
       <c r="F36" s="13">
-        <v>181.33</v>
+        <v>183.99</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>218.12</v>
+        <v>219.7</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1357,16 +1357,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>215.87</v>
+        <v>218.12</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1385,7 +1385,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" ht="19.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1396,7 +1396,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1415,83 +1415,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>212.25</v>
+        <v>212.71</v>
       </c>
       <c r="E42" s="10">
-        <v>182.04</v>
+        <v>183.37</v>
       </c>
       <c r="F42" s="10">
-        <v>192.04</v>
+        <v>193.37</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>211.89</v>
+        <v>212.35</v>
       </c>
       <c r="E43" s="13">
-        <v>182.45</v>
+        <v>183.78</v>
       </c>
       <c r="F43" s="13">
-        <v>192.45</v>
+        <v>193.78</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>210.01</v>
+        <v>212.25</v>
       </c>
       <c r="E44" s="10">
-        <v>180.1</v>
+        <v>182.04</v>
       </c>
       <c r="F44" s="10">
-        <v>190.1</v>
+        <v>192.04</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>209.65</v>
+        <v>211.89</v>
       </c>
       <c r="E45" s="13">
-        <v>180.52</v>
+        <v>182.45</v>
       </c>
       <c r="F45" s="13">
-        <v>190.52</v>
+        <v>192.45</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1500,7 +1500,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" ht="19.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1511,7 +1511,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1530,83 +1530,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>201.11</v>
+        <v>203.13</v>
       </c>
       <c r="E49" s="10">
-        <v>173.22</v>
+        <v>175.67</v>
       </c>
       <c r="F49" s="10">
-        <v>183.22</v>
+        <v>185.67</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>200.59</v>
+        <v>202.63</v>
       </c>
       <c r="E50" s="13">
-        <v>173.14</v>
+        <v>175.6</v>
       </c>
       <c r="F50" s="13">
-        <v>183.14</v>
+        <v>185.6</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>199.75</v>
+        <v>201.11</v>
       </c>
       <c r="E51" s="10">
-        <v>170.95</v>
+        <v>173.22</v>
       </c>
       <c r="F51" s="10">
-        <v>180.95</v>
+        <v>183.22</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>199.22</v>
+        <v>200.59</v>
       </c>
       <c r="E52" s="13">
-        <v>170.87</v>
+        <v>173.14</v>
       </c>
       <c r="F52" s="13">
-        <v>180.87</v>
+        <v>183.14</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1615,7 +1615,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="19.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1626,7 +1626,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1645,54 +1645,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>217.77</v>
+        <v>219.38</v>
       </c>
       <c r="E56" s="10">
-        <v>194.39</v>
+        <v>195.84</v>
       </c>
       <c r="F56" s="10">
-        <v>204.39</v>
+        <v>205.84</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>208</v>
+        <v>209.58</v>
       </c>
       <c r="E57" s="13">
-        <v>186.05</v>
+        <v>188.22</v>
       </c>
       <c r="F57" s="13">
-        <v>196.05</v>
+        <v>198.22</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>208.08</v>
+        <v>209.65</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1702,111 +1702,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>207.41</v>
+        <v>209.02</v>
       </c>
       <c r="E59" s="13">
-        <v>180.43</v>
+        <v>182.6</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>203.22</v>
+        <v>204.84</v>
       </c>
       <c r="E60" s="10">
-        <v>176.37</v>
+        <v>178.54</v>
       </c>
       <c r="F60" s="10">
-        <v>186.37</v>
+        <v>188.54</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>209.74</v>
+        <v>211.36</v>
       </c>
       <c r="E61" s="13">
-        <v>191.42</v>
+        <v>192.94</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>215.49</v>
+        <v>217.77</v>
       </c>
       <c r="E62" s="10">
-        <v>191.81</v>
+        <v>194.39</v>
       </c>
       <c r="F62" s="10">
-        <v>201.81</v>
+        <v>204.39</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>205.73</v>
+        <v>208</v>
       </c>
       <c r="E63" s="13">
-        <v>183.37</v>
+        <v>186.05</v>
       </c>
       <c r="F63" s="13">
-        <v>193.37</v>
+        <v>196.05</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>205.83</v>
+        <v>208.08</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1816,55 +1816,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>205.14</v>
+        <v>207.41</v>
       </c>
       <c r="E65" s="13">
-        <v>177.75</v>
+        <v>180.43</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="7">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>200.95</v>
+        <v>203.22</v>
       </c>
       <c r="E66" s="10">
-        <v>173.69</v>
+        <v>176.37</v>
       </c>
       <c r="F66" s="10">
-        <v>183.69</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <v>186.37</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="11">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>207.47</v>
+        <v>209.74</v>
       </c>
       <c r="E67" s="13">
-        <v>188.79</v>
+        <v>191.42</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1880,7 +1880,7 @@
     <mergeCell ref="A33:B33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C
 # Confidential</oddHeader>

</xml_diff>

<commit_message>
Thu May 21 05:37:24 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="14_{A4804B32-B63E-4E0B-8D42-6CA20914FF5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE3EE824-26D7-4FD5-BAAC-855D5E1323B8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{6B57C10E-24ED-41C9-B4AE-9191EF75F5EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3294" yWindow="3294" windowWidth="17280" windowHeight="9984" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>204.8</v>
+        <v>205.02</v>
       </c>
       <c r="E8" s="10">
-        <v>176.71</v>
+        <v>177.17</v>
       </c>
       <c r="F8" s="10">
-        <v>186.71</v>
+        <v>187.17</v>
       </c>
       <c r="G8" s="10">
-        <v>177.29</v>
+        <v>177.74</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>204.8</v>
+        <v>205.02</v>
       </c>
       <c r="E9" s="13">
-        <v>176.71</v>
+        <v>177.17</v>
       </c>
       <c r="F9" s="13">
-        <v>186.71</v>
+        <v>187.17</v>
       </c>
       <c r="G9" s="13">
-        <v>177.29</v>
+        <v>177.74</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>205.89</v>
+        <v>206.18</v>
       </c>
       <c r="E10" s="10">
-        <v>177.63</v>
+        <v>178.14</v>
       </c>
       <c r="F10" s="10">
-        <v>187.63</v>
+        <v>188.14</v>
       </c>
       <c r="G10" s="10">
-        <v>178.65</v>
+        <v>179.16</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>203.21</v>
+        <v>204.8</v>
       </c>
       <c r="E11" s="13">
-        <v>175.11</v>
+        <v>176.71</v>
       </c>
       <c r="F11" s="13">
-        <v>185.11</v>
+        <v>186.71</v>
       </c>
       <c r="G11" s="13">
-        <v>175.69</v>
+        <v>177.29</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>203.21</v>
+        <v>204.8</v>
       </c>
       <c r="E12" s="10">
-        <v>175.11</v>
+        <v>176.71</v>
       </c>
       <c r="F12" s="10">
-        <v>185.11</v>
+        <v>186.71</v>
       </c>
       <c r="G12" s="10">
-        <v>175.69</v>
+        <v>177.29</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>204.31</v>
+        <v>205.89</v>
       </c>
       <c r="E13" s="13">
-        <v>176.03</v>
+        <v>177.63</v>
       </c>
       <c r="F13" s="13">
-        <v>186.03</v>
+        <v>187.63</v>
       </c>
       <c r="G13" s="13">
-        <v>177.05</v>
+        <v>178.65</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.55000000000000004">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>210.13</v>
+        <v>210.43</v>
       </c>
       <c r="E17" s="10">
-        <v>184.06</v>
+        <v>184.58</v>
       </c>
       <c r="F17" s="10">
-        <v>194.06</v>
+        <v>194.58</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>209.07</v>
+        <v>210.13</v>
       </c>
       <c r="E18" s="13">
-        <v>182.44</v>
+        <v>184.06</v>
       </c>
       <c r="F18" s="13">
-        <v>192.44</v>
+        <v>194.06</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>205.91</v>
+        <v>206.14</v>
       </c>
       <c r="E22" s="10">
-        <v>177.93</v>
+        <v>178.39</v>
       </c>
       <c r="F22" s="10">
-        <v>187.53</v>
+        <v>187.99</v>
       </c>
       <c r="G22" s="10">
-        <v>177.18</v>
+        <v>177.64</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>209.82</v>
+        <v>210.1</v>
       </c>
       <c r="E23" s="13">
-        <v>182.65</v>
+        <v>183.16</v>
       </c>
       <c r="F23" s="13">
-        <v>192.65</v>
+        <v>193.16</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>209.88</v>
+        <v>210.16</v>
       </c>
       <c r="E24" s="10">
-        <v>183.44</v>
+        <v>183.95</v>
       </c>
       <c r="F24" s="10">
-        <v>193.44</v>
+        <v>193.95</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>209.87</v>
+        <v>210.15</v>
       </c>
       <c r="E25" s="13">
-        <v>183.17</v>
+        <v>183.68</v>
       </c>
       <c r="F25" s="13">
-        <v>193.17</v>
+        <v>193.68</v>
       </c>
       <c r="G25" s="13">
-        <v>181.67</v>
+        <v>182.17</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>209.29</v>
+        <v>209.58</v>
       </c>
       <c r="E26" s="10">
-        <v>185.23</v>
+        <v>185.74</v>
       </c>
       <c r="F26" s="10">
-        <v>195.23</v>
+        <v>195.74</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>204.32</v>
+        <v>205.91</v>
       </c>
       <c r="E27" s="13">
-        <v>175.78</v>
+        <v>177.93</v>
       </c>
       <c r="F27" s="13">
-        <v>185.38</v>
+        <v>187.53</v>
       </c>
       <c r="G27" s="13">
-        <v>175.04</v>
+        <v>177.18</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>208.24</v>
+        <v>209.82</v>
       </c>
       <c r="E28" s="22">
-        <v>181.05</v>
+        <v>182.65</v>
       </c>
       <c r="F28" s="22">
-        <v>191.05</v>
+        <v>192.65</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>208.3</v>
+        <v>209.88</v>
       </c>
       <c r="E29" s="13">
-        <v>181.86</v>
+        <v>183.44</v>
       </c>
       <c r="F29" s="13">
-        <v>191.86</v>
+        <v>193.44</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>208.29</v>
+        <v>209.87</v>
       </c>
       <c r="E30" s="22">
-        <v>181.59</v>
+        <v>183.17</v>
       </c>
       <c r="F30" s="22">
-        <v>191.59</v>
+        <v>193.17</v>
       </c>
       <c r="G30" s="22">
-        <v>180.08</v>
+        <v>181.67</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>207.7</v>
+        <v>209.29</v>
       </c>
       <c r="E31" s="13">
-        <v>183.63</v>
+        <v>185.23</v>
       </c>
       <c r="F31" s="13">
-        <v>193.63</v>
+        <v>195.23</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>204.08</v>
+        <v>204.36</v>
       </c>
       <c r="E35" s="10">
-        <v>176.58</v>
+        <v>177.08</v>
       </c>
       <c r="F35" s="10">
-        <v>185.58</v>
+        <v>186.08</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>202.5</v>
+        <v>204.08</v>
       </c>
       <c r="E36" s="13">
-        <v>174.99</v>
+        <v>176.58</v>
       </c>
       <c r="F36" s="13">
-        <v>183.99</v>
+        <v>185.58</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>219.7</v>
+        <v>219.98</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>218.12</v>
+        <v>219.7</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>212.71</v>
+        <v>212.98</v>
       </c>
       <c r="E42" s="10">
-        <v>183.37</v>
+        <v>183.94</v>
       </c>
       <c r="F42" s="10">
-        <v>193.37</v>
+        <v>193.94</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>212.35</v>
+        <v>212.62</v>
       </c>
       <c r="E43" s="13">
-        <v>183.78</v>
+        <v>184.35</v>
       </c>
       <c r="F43" s="13">
-        <v>193.78</v>
+        <v>194.35</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>212.25</v>
+        <v>212.71</v>
       </c>
       <c r="E44" s="10">
-        <v>182.04</v>
+        <v>183.37</v>
       </c>
       <c r="F44" s="10">
-        <v>192.04</v>
+        <v>193.37</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>211.89</v>
+        <v>212.35</v>
       </c>
       <c r="E45" s="13">
-        <v>182.45</v>
+        <v>183.78</v>
       </c>
       <c r="F45" s="13">
-        <v>192.45</v>
+        <v>193.78</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>203.13</v>
+        <v>204.66</v>
       </c>
       <c r="E49" s="10">
-        <v>175.67</v>
+        <v>176.94</v>
       </c>
       <c r="F49" s="10">
-        <v>185.67</v>
+        <v>186.94</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>202.63</v>
+        <v>204.16</v>
       </c>
       <c r="E50" s="13">
-        <v>175.6</v>
+        <v>176.87</v>
       </c>
       <c r="F50" s="13">
-        <v>185.6</v>
+        <v>186.87</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>201.11</v>
+        <v>203.13</v>
       </c>
       <c r="E51" s="10">
-        <v>173.22</v>
+        <v>175.67</v>
       </c>
       <c r="F51" s="10">
-        <v>183.22</v>
+        <v>185.67</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>200.59</v>
+        <v>202.63</v>
       </c>
       <c r="E52" s="13">
-        <v>173.14</v>
+        <v>175.6</v>
       </c>
       <c r="F52" s="13">
-        <v>183.14</v>
+        <v>185.6</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>219.38</v>
+        <v>219.69</v>
       </c>
       <c r="E56" s="10">
-        <v>195.84</v>
+        <v>196.27</v>
       </c>
       <c r="F56" s="10">
-        <v>205.84</v>
+        <v>206.27</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>209.58</v>
+        <v>209.87</v>
       </c>
       <c r="E57" s="13">
-        <v>188.22</v>
+        <v>188.75</v>
       </c>
       <c r="F57" s="13">
-        <v>198.22</v>
+        <v>198.75</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>209.65</v>
+        <v>209.93</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>209.02</v>
+        <v>209.33</v>
       </c>
       <c r="E59" s="13">
-        <v>182.6</v>
+        <v>183.13</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>204.84</v>
+        <v>205.14</v>
       </c>
       <c r="E60" s="10">
-        <v>178.54</v>
+        <v>179.07</v>
       </c>
       <c r="F60" s="10">
-        <v>188.54</v>
+        <v>189.07</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>211.36</v>
+        <v>211.66</v>
       </c>
       <c r="E61" s="13">
-        <v>192.94</v>
+        <v>193.41</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>217.77</v>
+        <v>219.38</v>
       </c>
       <c r="E62" s="10">
-        <v>194.39</v>
+        <v>195.84</v>
       </c>
       <c r="F62" s="10">
-        <v>204.39</v>
+        <v>205.84</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>208</v>
+        <v>209.58</v>
       </c>
       <c r="E63" s="13">
-        <v>186.05</v>
+        <v>188.22</v>
       </c>
       <c r="F63" s="13">
-        <v>196.05</v>
+        <v>198.22</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>208.08</v>
+        <v>209.65</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>207.41</v>
+        <v>209.02</v>
       </c>
       <c r="E65" s="13">
-        <v>180.43</v>
+        <v>182.6</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" s="7">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>203.22</v>
+        <v>204.84</v>
       </c>
       <c r="E66" s="10">
-        <v>176.37</v>
+        <v>178.54</v>
       </c>
       <c r="F66" s="10">
-        <v>186.37</v>
+        <v>188.54</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" s="11">
-        <v>46162</v>
+        <v>46163</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>209.74</v>
+        <v>211.36</v>
       </c>
       <c r="E67" s="13">
-        <v>191.42</v>
+        <v>192.94</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,6 +1892,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2151,17 +2162,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2172,6 +2172,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2191,17 +2202,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Fri May 22 05:14:23 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{6B57C10E-24ED-41C9-B4AE-9191EF75F5EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{9F9B62C5-C0D6-451C-8BB9-204229C7EDBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="28815" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -715,16 +715,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="76.41796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.41796875"/>
-    <col min="3" max="3" width="18.26171875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.83984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="6.578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.42578125"/>
+    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="6.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="22.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:7" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
@@ -735,7 +735,7 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -744,7 +744,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -755,7 +755,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -766,7 +766,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="1"/>
@@ -775,7 +775,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="19.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
@@ -786,7 +786,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -807,133 +807,133 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>205.02</v>
+        <v>204.51</v>
       </c>
       <c r="E8" s="10">
-        <v>177.17</v>
+        <v>175.85</v>
       </c>
       <c r="F8" s="10">
-        <v>187.17</v>
+        <v>185.85</v>
       </c>
       <c r="G8" s="10">
-        <v>177.74</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>176.43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>205.02</v>
+        <v>204.51</v>
       </c>
       <c r="E9" s="13">
-        <v>177.17</v>
+        <v>175.85</v>
       </c>
       <c r="F9" s="13">
-        <v>187.17</v>
+        <v>185.85</v>
       </c>
       <c r="G9" s="13">
-        <v>177.74</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>176.43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>206.18</v>
+        <v>205.74</v>
       </c>
       <c r="E10" s="10">
-        <v>178.14</v>
+        <v>176.89</v>
       </c>
       <c r="F10" s="10">
-        <v>188.14</v>
+        <v>186.89</v>
       </c>
       <c r="G10" s="10">
-        <v>179.16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>177.91</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>204.8</v>
+        <v>205.02</v>
       </c>
       <c r="E11" s="13">
-        <v>176.71</v>
+        <v>177.17</v>
       </c>
       <c r="F11" s="13">
-        <v>186.71</v>
+        <v>187.17</v>
       </c>
       <c r="G11" s="13">
-        <v>177.29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>177.74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>204.8</v>
+        <v>205.02</v>
       </c>
       <c r="E12" s="10">
-        <v>176.71</v>
+        <v>177.17</v>
       </c>
       <c r="F12" s="10">
-        <v>186.71</v>
+        <v>187.17</v>
       </c>
       <c r="G12" s="10">
-        <v>177.29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>177.74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>205.89</v>
+        <v>206.18</v>
       </c>
       <c r="E13" s="13">
-        <v>177.63</v>
+        <v>178.14</v>
       </c>
       <c r="F13" s="13">
-        <v>187.63</v>
+        <v>188.14</v>
       </c>
       <c r="G13" s="13">
-        <v>178.65</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>179.16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
@@ -942,7 +942,7 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="1:7" ht="19.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A15" s="29" t="s">
         <v>13</v>
       </c>
@@ -953,7 +953,7 @@
       <c r="F15" s="17"/>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>4</v>
       </c>
@@ -972,45 +972,45 @@
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>210.43</v>
+        <v>210</v>
       </c>
       <c r="E17" s="10">
-        <v>184.58</v>
+        <v>183.34</v>
       </c>
       <c r="F17" s="10">
-        <v>194.58</v>
+        <v>193.34</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>210.13</v>
+        <v>210.43</v>
       </c>
       <c r="E18" s="13">
-        <v>184.06</v>
+        <v>184.58</v>
       </c>
       <c r="F18" s="13">
-        <v>194.06</v>
+        <v>194.58</v>
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="15"/>
@@ -1019,7 +1019,7 @@
       <c r="F19" s="16"/>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" spans="1:7" ht="19.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
         <v>15</v>
       </c>
@@ -1030,7 +1030,7 @@
       <c r="F20" s="17"/>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>4</v>
       </c>
@@ -1051,217 +1051,217 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>206.14</v>
+        <v>205.63</v>
       </c>
       <c r="E22" s="10">
-        <v>178.39</v>
+        <v>177.07</v>
       </c>
       <c r="F22" s="10">
-        <v>187.99</v>
+        <v>186.67</v>
       </c>
       <c r="G22" s="10">
-        <v>177.64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>176.32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>210.1</v>
+        <v>209.66</v>
       </c>
       <c r="E23" s="13">
-        <v>183.16</v>
+        <v>181.91</v>
       </c>
       <c r="F23" s="13">
-        <v>193.16</v>
+        <v>191.91</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>210.16</v>
+        <v>209.73</v>
       </c>
       <c r="E24" s="10">
-        <v>183.95</v>
+        <v>182.7</v>
       </c>
       <c r="F24" s="10">
-        <v>193.95</v>
+        <v>192.7</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>210.15</v>
+        <v>209.71</v>
       </c>
       <c r="E25" s="13">
-        <v>183.68</v>
+        <v>182.42</v>
       </c>
       <c r="F25" s="13">
-        <v>193.68</v>
+        <v>192.42</v>
       </c>
       <c r="G25" s="13">
-        <v>182.17</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>180.91</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>209.58</v>
+        <v>209.15</v>
       </c>
       <c r="E26" s="10">
-        <v>185.74</v>
+        <v>184.47</v>
       </c>
       <c r="F26" s="10">
-        <v>195.74</v>
+        <v>194.47</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>205.91</v>
+        <v>206.14</v>
       </c>
       <c r="E27" s="13">
-        <v>177.93</v>
+        <v>178.39</v>
       </c>
       <c r="F27" s="13">
-        <v>187.53</v>
+        <v>187.99</v>
       </c>
       <c r="G27" s="13">
-        <v>177.18</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>177.64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>209.82</v>
+        <v>210.1</v>
       </c>
       <c r="E28" s="22">
-        <v>182.65</v>
+        <v>183.16</v>
       </c>
       <c r="F28" s="22">
-        <v>192.65</v>
+        <v>193.16</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>209.88</v>
+        <v>210.16</v>
       </c>
       <c r="E29" s="13">
-        <v>183.44</v>
+        <v>183.95</v>
       </c>
       <c r="F29" s="13">
-        <v>193.44</v>
+        <v>193.95</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>209.87</v>
+        <v>210.15</v>
       </c>
       <c r="E30" s="22">
-        <v>183.17</v>
+        <v>183.68</v>
       </c>
       <c r="F30" s="22">
-        <v>193.17</v>
+        <v>193.68</v>
       </c>
       <c r="G30" s="22">
-        <v>181.67</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+        <v>182.17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>209.29</v>
+        <v>209.58</v>
       </c>
       <c r="E31" s="13">
-        <v>185.23</v>
+        <v>185.74</v>
       </c>
       <c r="F31" s="13">
-        <v>195.23</v>
+        <v>195.74</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
@@ -1270,7 +1270,7 @@
       <c r="F32" s="17"/>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" spans="1:7" ht="19.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A33" s="29" t="s">
         <v>22</v>
       </c>
@@ -1281,7 +1281,7 @@
       <c r="F33" s="17"/>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="23" t="s">
         <v>4</v>
       </c>
@@ -1300,54 +1300,54 @@
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>204.36</v>
+        <v>203.92</v>
       </c>
       <c r="E35" s="10">
-        <v>177.08</v>
+        <v>175.83</v>
       </c>
       <c r="F35" s="10">
-        <v>186.08</v>
+        <v>184.83</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>204.08</v>
+        <v>204.36</v>
       </c>
       <c r="E36" s="13">
-        <v>176.58</v>
+        <v>177.08</v>
       </c>
       <c r="F36" s="13">
-        <v>185.58</v>
+        <v>186.08</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>219.98</v>
+        <v>219.54</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1357,16 +1357,16 @@
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>219.7</v>
+        <v>219.98</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="G38" s="17"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="24"/>
       <c r="B39" s="24"/>
       <c r="C39" s="15"/>
@@ -1385,7 +1385,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
     </row>
-    <row r="40" spans="1:7" ht="19.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="40" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
         <v>25</v>
       </c>
@@ -1396,7 +1396,7 @@
       <c r="F40" s="17"/>
       <c r="G40" s="17"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="23" t="s">
         <v>4</v>
       </c>
@@ -1415,83 +1415,83 @@
       </c>
       <c r="G41" s="17"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>212.98</v>
+        <v>212.53</v>
       </c>
       <c r="E42" s="10">
-        <v>183.94</v>
+        <v>183.38</v>
       </c>
       <c r="F42" s="10">
-        <v>193.94</v>
+        <v>193.38</v>
       </c>
       <c r="G42" s="17"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>212.62</v>
+        <v>212.17</v>
       </c>
       <c r="E43" s="13">
-        <v>184.35</v>
+        <v>183.79</v>
       </c>
       <c r="F43" s="13">
-        <v>194.35</v>
+        <v>193.79</v>
       </c>
       <c r="G43" s="17"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>212.71</v>
+        <v>212.98</v>
       </c>
       <c r="E44" s="10">
-        <v>183.37</v>
+        <v>183.94</v>
       </c>
       <c r="F44" s="10">
-        <v>193.37</v>
+        <v>193.94</v>
       </c>
       <c r="G44" s="17"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>212.35</v>
+        <v>212.62</v>
       </c>
       <c r="E45" s="13">
-        <v>183.78</v>
+        <v>184.35</v>
       </c>
       <c r="F45" s="13">
-        <v>193.78</v>
+        <v>194.35</v>
       </c>
       <c r="G45" s="17"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="24"/>
       <c r="C46" s="15"/>
@@ -1500,7 +1500,7 @@
       <c r="F46" s="16"/>
       <c r="G46" s="17"/>
     </row>
-    <row r="47" spans="1:7" ht="19.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="47" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
         <v>28</v>
       </c>
@@ -1511,7 +1511,7 @@
       <c r="F47" s="17"/>
       <c r="G47" s="17"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
         <v>4</v>
       </c>
@@ -1530,83 +1530,83 @@
       </c>
       <c r="G48" s="17"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>204.66</v>
+        <v>204.44</v>
       </c>
       <c r="E49" s="10">
-        <v>176.94</v>
+        <v>176.54</v>
       </c>
       <c r="F49" s="10">
-        <v>186.94</v>
+        <v>186.54</v>
       </c>
       <c r="G49" s="28"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>204.16</v>
+        <v>203.95</v>
       </c>
       <c r="E50" s="13">
-        <v>176.87</v>
+        <v>176.47</v>
       </c>
       <c r="F50" s="13">
-        <v>186.87</v>
+        <v>186.47</v>
       </c>
       <c r="G50" s="28"/>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>203.13</v>
+        <v>204.66</v>
       </c>
       <c r="E51" s="10">
-        <v>175.67</v>
+        <v>176.94</v>
       </c>
       <c r="F51" s="10">
-        <v>185.67</v>
+        <v>186.94</v>
       </c>
       <c r="G51" s="17"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>202.63</v>
+        <v>204.16</v>
       </c>
       <c r="E52" s="13">
-        <v>175.6</v>
+        <v>176.87</v>
       </c>
       <c r="F52" s="13">
-        <v>185.6</v>
+        <v>186.87</v>
       </c>
       <c r="G52" s="17"/>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="14"/>
       <c r="B53" s="14"/>
       <c r="C53" s="15"/>
@@ -1615,7 +1615,7 @@
       <c r="F53" s="16"/>
       <c r="G53" s="17"/>
     </row>
-    <row r="54" spans="1:7" ht="19.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="54" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A54" s="27" t="s">
         <v>31</v>
       </c>
@@ -1626,7 +1626,7 @@
       <c r="F54" s="17"/>
       <c r="G54" s="17"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="23" t="s">
         <v>4</v>
       </c>
@@ -1645,54 +1645,54 @@
       </c>
       <c r="G55" s="17"/>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>219.69</v>
+        <v>219.28</v>
       </c>
       <c r="E56" s="10">
-        <v>196.27</v>
+        <v>194.95</v>
       </c>
       <c r="F56" s="10">
-        <v>206.27</v>
+        <v>204.95</v>
       </c>
       <c r="G56" s="17"/>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>209.87</v>
+        <v>209.44</v>
       </c>
       <c r="E57" s="13">
-        <v>188.75</v>
+        <v>188.07</v>
       </c>
       <c r="F57" s="13">
-        <v>198.75</v>
+        <v>198.07</v>
       </c>
       <c r="G57" s="17"/>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>209.93</v>
+        <v>209.49</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1702,111 +1702,111 @@
       </c>
       <c r="G58" s="17"/>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>209.33</v>
+        <v>208.91</v>
       </c>
       <c r="E59" s="13">
-        <v>183.13</v>
+        <v>182.45</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G59" s="17"/>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>205.14</v>
+        <v>204.72</v>
       </c>
       <c r="E60" s="10">
-        <v>179.07</v>
+        <v>178.39</v>
       </c>
       <c r="F60" s="10">
-        <v>189.07</v>
+        <v>188.39</v>
       </c>
       <c r="G60" s="17"/>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>211.66</v>
+        <v>211.23</v>
       </c>
       <c r="E61" s="13">
-        <v>193.41</v>
+        <v>192.12</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
       </c>
       <c r="G61" s="17"/>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>219.38</v>
+        <v>219.69</v>
       </c>
       <c r="E62" s="10">
-        <v>195.84</v>
+        <v>196.27</v>
       </c>
       <c r="F62" s="10">
-        <v>205.84</v>
+        <v>206.27</v>
       </c>
       <c r="G62" s="17"/>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>209.58</v>
+        <v>209.87</v>
       </c>
       <c r="E63" s="13">
-        <v>188.22</v>
+        <v>188.75</v>
       </c>
       <c r="F63" s="13">
-        <v>198.22</v>
+        <v>198.75</v>
       </c>
       <c r="G63" s="17"/>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>209.65</v>
+        <v>209.93</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1816,55 +1816,55 @@
       </c>
       <c r="G64" s="17"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>209.02</v>
+        <v>209.33</v>
       </c>
       <c r="E65" s="13">
-        <v>182.6</v>
+        <v>183.13</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>204.84</v>
+        <v>205.14</v>
       </c>
       <c r="E66" s="10">
-        <v>178.54</v>
+        <v>179.07</v>
       </c>
       <c r="F66" s="10">
-        <v>188.54</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.55000000000000004">
+        <v>189.07</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>211.36</v>
+        <v>211.66</v>
       </c>
       <c r="E67" s="13">
-        <v>192.94</v>
+        <v>193.41</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,17 +1892,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2162,6 +2151,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2172,17 +2172,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2202,6 +2191,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Mon May 25 05:50:36 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{9F9B62C5-C0D6-451C-8BB9-204229C7EDBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{3E2CC018-2B8B-4229-AE8B-6239F654F082}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28815" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>204.51</v>
+        <v>202.52</v>
       </c>
       <c r="E8" s="10">
-        <v>175.85</v>
+        <v>173.59</v>
       </c>
       <c r="F8" s="10">
-        <v>185.85</v>
+        <v>183.59</v>
       </c>
       <c r="G8" s="10">
-        <v>176.43</v>
+        <v>174.16</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>204.51</v>
+        <v>202.52</v>
       </c>
       <c r="E9" s="13">
-        <v>175.85</v>
+        <v>173.59</v>
       </c>
       <c r="F9" s="13">
-        <v>185.85</v>
+        <v>183.59</v>
       </c>
       <c r="G9" s="13">
-        <v>176.43</v>
+        <v>174.16</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>205.74</v>
+        <v>203.28</v>
       </c>
       <c r="E10" s="10">
-        <v>176.89</v>
+        <v>174.69</v>
       </c>
       <c r="F10" s="10">
-        <v>186.89</v>
+        <v>184.69</v>
       </c>
       <c r="G10" s="10">
-        <v>177.91</v>
+        <v>175.71</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>205.02</v>
+        <v>204.51</v>
       </c>
       <c r="E11" s="13">
-        <v>177.17</v>
+        <v>175.85</v>
       </c>
       <c r="F11" s="13">
-        <v>187.17</v>
+        <v>185.85</v>
       </c>
       <c r="G11" s="13">
-        <v>177.74</v>
+        <v>176.43</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>205.02</v>
+        <v>204.51</v>
       </c>
       <c r="E12" s="10">
-        <v>177.17</v>
+        <v>175.85</v>
       </c>
       <c r="F12" s="10">
-        <v>187.17</v>
+        <v>185.85</v>
       </c>
       <c r="G12" s="10">
-        <v>177.74</v>
+        <v>176.43</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>206.18</v>
+        <v>205.74</v>
       </c>
       <c r="E13" s="13">
-        <v>178.14</v>
+        <v>176.89</v>
       </c>
       <c r="F13" s="13">
-        <v>188.14</v>
+        <v>186.89</v>
       </c>
       <c r="G13" s="13">
-        <v>179.16</v>
+        <v>177.91</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>210</v>
+        <v>208.11</v>
       </c>
       <c r="E17" s="10">
-        <v>183.34</v>
+        <v>181.15</v>
       </c>
       <c r="F17" s="10">
-        <v>193.34</v>
+        <v>191.15</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>210.43</v>
+        <v>210</v>
       </c>
       <c r="E18" s="13">
-        <v>184.58</v>
+        <v>183.34</v>
       </c>
       <c r="F18" s="13">
-        <v>194.58</v>
+        <v>193.34</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>205.63</v>
+        <v>203.09</v>
       </c>
       <c r="E22" s="10">
-        <v>177.07</v>
+        <v>174.81</v>
       </c>
       <c r="F22" s="10">
-        <v>186.67</v>
+        <v>184.41</v>
       </c>
       <c r="G22" s="10">
-        <v>176.32</v>
+        <v>174.06</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>209.66</v>
+        <v>207.74</v>
       </c>
       <c r="E23" s="13">
-        <v>181.91</v>
+        <v>179.71</v>
       </c>
       <c r="F23" s="13">
-        <v>191.91</v>
+        <v>189.71</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>209.73</v>
+        <v>207.81</v>
       </c>
       <c r="E24" s="10">
-        <v>182.7</v>
+        <v>180.49</v>
       </c>
       <c r="F24" s="10">
-        <v>192.7</v>
+        <v>190.49</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>209.71</v>
+        <v>207.8</v>
       </c>
       <c r="E25" s="13">
-        <v>182.42</v>
+        <v>180.2</v>
       </c>
       <c r="F25" s="13">
-        <v>192.42</v>
+        <v>190.2</v>
       </c>
       <c r="G25" s="13">
-        <v>180.91</v>
+        <v>178.69</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>209.15</v>
+        <v>207.24</v>
       </c>
       <c r="E26" s="10">
-        <v>184.47</v>
+        <v>182.24</v>
       </c>
       <c r="F26" s="10">
-        <v>194.47</v>
+        <v>192.24</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>206.14</v>
+        <v>205.63</v>
       </c>
       <c r="E27" s="13">
-        <v>178.39</v>
+        <v>177.07</v>
       </c>
       <c r="F27" s="13">
-        <v>187.99</v>
+        <v>186.67</v>
       </c>
       <c r="G27" s="13">
-        <v>177.64</v>
+        <v>176.32</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>210.1</v>
+        <v>209.66</v>
       </c>
       <c r="E28" s="22">
-        <v>183.16</v>
+        <v>181.91</v>
       </c>
       <c r="F28" s="22">
-        <v>193.16</v>
+        <v>191.91</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>210.16</v>
+        <v>209.73</v>
       </c>
       <c r="E29" s="13">
-        <v>183.95</v>
+        <v>182.7</v>
       </c>
       <c r="F29" s="13">
-        <v>193.95</v>
+        <v>192.7</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>210.15</v>
+        <v>209.71</v>
       </c>
       <c r="E30" s="22">
-        <v>183.68</v>
+        <v>182.42</v>
       </c>
       <c r="F30" s="22">
-        <v>193.68</v>
+        <v>192.42</v>
       </c>
       <c r="G30" s="22">
-        <v>182.17</v>
+        <v>180.91</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>209.58</v>
+        <v>209.15</v>
       </c>
       <c r="E31" s="13">
-        <v>185.74</v>
+        <v>184.47</v>
       </c>
       <c r="F31" s="13">
-        <v>195.74</v>
+        <v>194.47</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>203.92</v>
+        <v>202</v>
       </c>
       <c r="E35" s="10">
-        <v>175.83</v>
+        <v>173.63</v>
       </c>
       <c r="F35" s="10">
-        <v>184.83</v>
+        <v>182.63</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>204.36</v>
+        <v>203.92</v>
       </c>
       <c r="E36" s="13">
-        <v>177.08</v>
+        <v>175.83</v>
       </c>
       <c r="F36" s="13">
-        <v>186.08</v>
+        <v>184.83</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>219.54</v>
+        <v>217.62</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>219.98</v>
+        <v>219.54</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>212.53</v>
+        <v>210.05</v>
       </c>
       <c r="E42" s="10">
-        <v>183.38</v>
+        <v>181.74</v>
       </c>
       <c r="F42" s="10">
-        <v>193.38</v>
+        <v>191.74</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>212.17</v>
+        <v>209.69</v>
       </c>
       <c r="E43" s="13">
-        <v>183.79</v>
+        <v>182.15</v>
       </c>
       <c r="F43" s="13">
-        <v>193.79</v>
+        <v>192.15</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>212.98</v>
+        <v>212.53</v>
       </c>
       <c r="E44" s="10">
-        <v>183.94</v>
+        <v>183.38</v>
       </c>
       <c r="F44" s="10">
-        <v>193.94</v>
+        <v>193.38</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>212.62</v>
+        <v>212.17</v>
       </c>
       <c r="E45" s="13">
-        <v>184.35</v>
+        <v>183.79</v>
       </c>
       <c r="F45" s="13">
-        <v>194.35</v>
+        <v>193.79</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>204.44</v>
+        <v>203.06</v>
       </c>
       <c r="E49" s="10">
-        <v>176.54</v>
+        <v>175.5</v>
       </c>
       <c r="F49" s="10">
-        <v>186.54</v>
+        <v>185.5</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>203.95</v>
+        <v>202.57</v>
       </c>
       <c r="E50" s="13">
-        <v>176.47</v>
+        <v>175.44</v>
       </c>
       <c r="F50" s="13">
-        <v>186.47</v>
+        <v>185.44</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>204.66</v>
+        <v>204.44</v>
       </c>
       <c r="E51" s="10">
-        <v>176.94</v>
+        <v>176.54</v>
       </c>
       <c r="F51" s="10">
-        <v>186.94</v>
+        <v>186.54</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>204.16</v>
+        <v>203.95</v>
       </c>
       <c r="E52" s="13">
-        <v>176.87</v>
+        <v>176.47</v>
       </c>
       <c r="F52" s="13">
-        <v>186.87</v>
+        <v>186.47</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>219.28</v>
+        <v>217.37</v>
       </c>
       <c r="E56" s="10">
-        <v>194.95</v>
+        <v>192.65</v>
       </c>
       <c r="F56" s="10">
-        <v>204.95</v>
+        <v>202.65</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>209.44</v>
+        <v>207.52</v>
       </c>
       <c r="E57" s="13">
-        <v>188.07</v>
+        <v>184.8</v>
       </c>
       <c r="F57" s="13">
-        <v>198.07</v>
+        <v>194.8</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>209.49</v>
+        <v>207.57</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>208.91</v>
+        <v>207.03</v>
       </c>
       <c r="E59" s="13">
-        <v>182.45</v>
+        <v>179.19</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>204.72</v>
+        <v>202.84</v>
       </c>
       <c r="E60" s="10">
-        <v>178.39</v>
+        <v>175.12</v>
       </c>
       <c r="F60" s="10">
-        <v>188.39</v>
+        <v>185.12</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>211.23</v>
+        <v>209.35</v>
       </c>
       <c r="E61" s="13">
-        <v>192.12</v>
+        <v>189.86</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>219.69</v>
+        <v>219.28</v>
       </c>
       <c r="E62" s="10">
-        <v>196.27</v>
+        <v>194.95</v>
       </c>
       <c r="F62" s="10">
-        <v>206.27</v>
+        <v>204.95</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>209.87</v>
+        <v>209.44</v>
       </c>
       <c r="E63" s="13">
-        <v>188.75</v>
+        <v>188.07</v>
       </c>
       <c r="F63" s="13">
-        <v>198.75</v>
+        <v>198.07</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>209.93</v>
+        <v>209.49</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>209.33</v>
+        <v>208.91</v>
       </c>
       <c r="E65" s="13">
-        <v>183.13</v>
+        <v>182.45</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>205.14</v>
+        <v>204.72</v>
       </c>
       <c r="E66" s="10">
-        <v>179.07</v>
+        <v>178.39</v>
       </c>
       <c r="F66" s="10">
-        <v>189.07</v>
+        <v>188.39</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46164</v>
+        <v>46165</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>211.66</v>
+        <v>211.23</v>
       </c>
       <c r="E67" s="13">
-        <v>193.41</v>
+        <v>192.12</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>
@@ -1892,6 +1892,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D3632DF5622958439304627C030B0427" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c2ecbce386d6bac497f8eb2d8f0fb7a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="87276d81-85f4-4ef2-9e6e-55066304288f" xmlns:ns3="39e1dda6-d1d8-4c88-a3b9-f1abc1284bad" xmlns:ns4="b23b8984-eafa-4e79-985e-54f52f3da58e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cfd0c2f651c1ce156ad4fcb44ea61dd" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="87276d81-85f4-4ef2-9e6e-55066304288f"/>
@@ -2151,27 +2171,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="87276d81-85f4-4ef2-9e6e-55066304288f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="b23b8984-eafa-4e79-985e-54f52f3da58e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
+    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B44E1863-2778-41F9-ACBA-48420F931671}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2191,25 +2210,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57A83D98-2BAE-4D83-823A-D31C464B620C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="87276d81-85f4-4ef2-9e6e-55066304288f"/>
-    <ds:schemaRef ds:uri="b23b8984-eafa-4e79-985e-54f52f3da58e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60519E9-FD90-4339-869C-BC2F85719BB8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{569bf4a9-87bd-4dbf-a36c-1db5158e5def}" enabled="1" method="Privileged" siteId="{ea80952e-a476-42d4-aaf4-5457852b0f7e}" removed="0"/>

</xml_diff>

<commit_message>
Tue May 26 05:14:21 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{3E2CC018-2B8B-4229-AE8B-6239F654F082}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{A6B7D494-4C10-49AB-BC97-348EEC42832D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>202.52</v>
+        <v>198.55</v>
       </c>
       <c r="E8" s="10">
-        <v>173.59</v>
+        <v>170.51</v>
       </c>
       <c r="F8" s="10">
-        <v>183.59</v>
+        <v>180.51</v>
       </c>
       <c r="G8" s="10">
-        <v>174.16</v>
+        <v>171.08</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>202.52</v>
+        <v>198.55</v>
       </c>
       <c r="E9" s="13">
-        <v>173.59</v>
+        <v>170.51</v>
       </c>
       <c r="F9" s="13">
-        <v>183.59</v>
+        <v>180.51</v>
       </c>
       <c r="G9" s="13">
-        <v>174.16</v>
+        <v>171.08</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>203.28</v>
+        <v>198.83</v>
       </c>
       <c r="E10" s="10">
-        <v>174.69</v>
+        <v>171.11</v>
       </c>
       <c r="F10" s="10">
-        <v>184.69</v>
+        <v>181.11</v>
       </c>
       <c r="G10" s="10">
-        <v>175.71</v>
+        <v>172.13</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>204.51</v>
+        <v>202.52</v>
       </c>
       <c r="E11" s="13">
-        <v>175.85</v>
+        <v>173.59</v>
       </c>
       <c r="F11" s="13">
-        <v>185.85</v>
+        <v>183.59</v>
       </c>
       <c r="G11" s="13">
-        <v>176.43</v>
+        <v>174.16</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>204.51</v>
+        <v>202.52</v>
       </c>
       <c r="E12" s="10">
-        <v>175.85</v>
+        <v>173.59</v>
       </c>
       <c r="F12" s="10">
-        <v>185.85</v>
+        <v>183.59</v>
       </c>
       <c r="G12" s="10">
-        <v>176.43</v>
+        <v>174.16</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>205.74</v>
+        <v>203.28</v>
       </c>
       <c r="E13" s="13">
-        <v>176.89</v>
+        <v>174.69</v>
       </c>
       <c r="F13" s="13">
-        <v>186.89</v>
+        <v>184.69</v>
       </c>
       <c r="G13" s="13">
-        <v>177.91</v>
+        <v>175.71</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,39 +974,39 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="7">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D17" s="10">
-        <v>208.11</v>
+        <v>203.68</v>
       </c>
       <c r="E17" s="10">
-        <v>181.15</v>
+        <v>177.59</v>
       </c>
       <c r="F17" s="10">
-        <v>191.15</v>
+        <v>187.59</v>
       </c>
       <c r="G17" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D18" s="13">
-        <v>210</v>
+        <v>208.11</v>
       </c>
       <c r="E18" s="13">
-        <v>183.34</v>
+        <v>181.15</v>
       </c>
       <c r="F18" s="13">
-        <v>193.34</v>
+        <v>191.15</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -1053,41 +1053,41 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B22" s="8"/>
       <c r="C22" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D22" s="10">
-        <v>203.09</v>
+        <v>199.68</v>
       </c>
       <c r="E22" s="10">
-        <v>174.81</v>
+        <v>171.18</v>
       </c>
       <c r="F22" s="10">
-        <v>184.41</v>
+        <v>180.78</v>
       </c>
       <c r="G22" s="10">
-        <v>174.06</v>
+        <v>170.43</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="21" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="13">
-        <v>207.74</v>
+        <v>203.28</v>
       </c>
       <c r="E23" s="13">
-        <v>179.71</v>
+        <v>176.67</v>
       </c>
       <c r="F23" s="13">
-        <v>189.71</v>
+        <v>186.67</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>18</v>
@@ -1095,20 +1095,20 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B24" s="8"/>
       <c r="C24" s="20" t="s">
         <v>19</v>
       </c>
       <c r="D24" s="10">
-        <v>207.81</v>
+        <v>203.36</v>
       </c>
       <c r="E24" s="10">
-        <v>180.49</v>
+        <v>176.9</v>
       </c>
       <c r="F24" s="10">
-        <v>190.49</v>
+        <v>186.9</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>18</v>
@@ -1116,41 +1116,41 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="11">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B25" s="12"/>
       <c r="C25" s="21" t="s">
         <v>20</v>
       </c>
       <c r="D25" s="13">
-        <v>207.8</v>
+        <v>203.34</v>
       </c>
       <c r="E25" s="13">
-        <v>180.2</v>
+        <v>177.15</v>
       </c>
       <c r="F25" s="13">
-        <v>190.2</v>
+        <v>187.15</v>
       </c>
       <c r="G25" s="13">
-        <v>178.69</v>
+        <v>175.64</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B26" s="8"/>
       <c r="C26" s="20" t="s">
         <v>21</v>
       </c>
       <c r="D26" s="10">
-        <v>207.24</v>
+        <v>202.79</v>
       </c>
       <c r="E26" s="10">
-        <v>182.24</v>
+        <v>179.16</v>
       </c>
       <c r="F26" s="10">
-        <v>192.24</v>
+        <v>189.16</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>18</v>
@@ -1158,41 +1158,41 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="13">
-        <v>205.63</v>
+        <v>203.09</v>
       </c>
       <c r="E27" s="13">
-        <v>177.07</v>
+        <v>174.81</v>
       </c>
       <c r="F27" s="13">
-        <v>186.67</v>
+        <v>184.41</v>
       </c>
       <c r="G27" s="13">
-        <v>176.32</v>
+        <v>174.06</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B28" s="8"/>
       <c r="C28" s="20" t="s">
         <v>17</v>
       </c>
       <c r="D28" s="10">
-        <v>209.66</v>
+        <v>207.74</v>
       </c>
       <c r="E28" s="22">
-        <v>181.91</v>
+        <v>179.71</v>
       </c>
       <c r="F28" s="22">
-        <v>191.91</v>
+        <v>189.71</v>
       </c>
       <c r="G28" s="22" t="s">
         <v>18</v>
@@ -1200,20 +1200,20 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B29" s="12"/>
       <c r="C29" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="13">
-        <v>209.73</v>
+        <v>207.81</v>
       </c>
       <c r="E29" s="13">
-        <v>182.7</v>
+        <v>180.49</v>
       </c>
       <c r="F29" s="13">
-        <v>192.7</v>
+        <v>190.49</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>18</v>
@@ -1221,41 +1221,41 @@
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B30" s="8"/>
       <c r="C30" s="20" t="s">
         <v>20</v>
       </c>
       <c r="D30" s="10">
-        <v>209.71</v>
+        <v>207.8</v>
       </c>
       <c r="E30" s="22">
-        <v>182.42</v>
+        <v>180.2</v>
       </c>
       <c r="F30" s="22">
-        <v>192.42</v>
+        <v>190.2</v>
       </c>
       <c r="G30" s="22">
-        <v>180.91</v>
+        <v>178.69</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D31" s="13">
-        <v>209.15</v>
+        <v>207.24</v>
       </c>
       <c r="E31" s="13">
-        <v>184.47</v>
+        <v>182.24</v>
       </c>
       <c r="F31" s="13">
-        <v>194.47</v>
+        <v>192.24</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>18</v>
@@ -1302,52 +1302,52 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="7">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="20" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="10">
-        <v>202</v>
+        <v>197.55</v>
       </c>
       <c r="E35" s="10">
-        <v>173.63</v>
+        <v>170.06</v>
       </c>
       <c r="F35" s="10">
-        <v>182.63</v>
+        <v>179.06</v>
       </c>
       <c r="G35" s="17"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B36" s="12"/>
       <c r="C36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="13">
-        <v>203.92</v>
+        <v>202</v>
       </c>
       <c r="E36" s="13">
-        <v>175.83</v>
+        <v>173.63</v>
       </c>
       <c r="F36" s="13">
-        <v>184.83</v>
+        <v>182.63</v>
       </c>
       <c r="G36" s="17"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="7">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="20" t="s">
         <v>24</v>
       </c>
       <c r="D37" s="10">
-        <v>217.62</v>
+        <v>213.17</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>18</v>
@@ -1359,14 +1359,14 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="13">
-        <v>219.54</v>
+        <v>217.62</v>
       </c>
       <c r="E38" s="13" t="s">
         <v>18</v>
@@ -1417,77 +1417,77 @@
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="7">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B42" s="8"/>
       <c r="C42" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D42" s="10">
-        <v>210.05</v>
+        <v>205.57</v>
       </c>
       <c r="E42" s="10">
-        <v>181.74</v>
+        <v>179.26</v>
       </c>
       <c r="F42" s="10">
-        <v>191.74</v>
+        <v>189.26</v>
       </c>
       <c r="G42" s="17"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B43" s="12"/>
       <c r="C43" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D43" s="13">
-        <v>209.69</v>
+        <v>205.22</v>
       </c>
       <c r="E43" s="13">
-        <v>182.15</v>
+        <v>179.67</v>
       </c>
       <c r="F43" s="13">
-        <v>192.15</v>
+        <v>189.67</v>
       </c>
       <c r="G43" s="17"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B44" s="8"/>
       <c r="C44" s="20" t="s">
         <v>26</v>
       </c>
       <c r="D44" s="10">
-        <v>212.53</v>
+        <v>210.05</v>
       </c>
       <c r="E44" s="10">
-        <v>183.38</v>
+        <v>181.74</v>
       </c>
       <c r="F44" s="10">
-        <v>193.38</v>
+        <v>191.74</v>
       </c>
       <c r="G44" s="17"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="21" t="s">
         <v>27</v>
       </c>
       <c r="D45" s="13">
-        <v>212.17</v>
+        <v>209.69</v>
       </c>
       <c r="E45" s="13">
-        <v>183.79</v>
+        <v>182.15</v>
       </c>
       <c r="F45" s="13">
-        <v>193.79</v>
+        <v>192.15</v>
       </c>
       <c r="G45" s="17"/>
     </row>
@@ -1532,77 +1532,77 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="7">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B49" s="8"/>
       <c r="C49" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D49" s="10">
-        <v>203.06</v>
+        <v>201.28</v>
       </c>
       <c r="E49" s="10">
-        <v>175.5</v>
+        <v>174.29</v>
       </c>
       <c r="F49" s="10">
-        <v>185.5</v>
+        <v>184.29</v>
       </c>
       <c r="G49" s="28"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="11">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="13">
-        <v>202.57</v>
+        <v>200.8</v>
       </c>
       <c r="E50" s="13">
-        <v>175.44</v>
+        <v>174.22</v>
       </c>
       <c r="F50" s="13">
-        <v>185.44</v>
+        <v>184.22</v>
       </c>
       <c r="G50" s="28"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B51" s="8"/>
       <c r="C51" s="20" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="10">
-        <v>204.44</v>
+        <v>203.06</v>
       </c>
       <c r="E51" s="10">
-        <v>176.54</v>
+        <v>175.5</v>
       </c>
       <c r="F51" s="10">
-        <v>186.54</v>
+        <v>185.5</v>
       </c>
       <c r="G51" s="17"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B52" s="12"/>
       <c r="C52" s="21" t="s">
         <v>30</v>
       </c>
       <c r="D52" s="13">
-        <v>203.95</v>
+        <v>202.57</v>
       </c>
       <c r="E52" s="13">
-        <v>176.47</v>
+        <v>175.44</v>
       </c>
       <c r="F52" s="13">
-        <v>186.47</v>
+        <v>185.44</v>
       </c>
       <c r="G52" s="17"/>
     </row>
@@ -1647,52 +1647,52 @@
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="7">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B56" s="8"/>
       <c r="C56" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D56" s="10">
-        <v>217.37</v>
+        <v>212.91</v>
       </c>
       <c r="E56" s="10">
-        <v>192.65</v>
+        <v>188.96</v>
       </c>
       <c r="F56" s="10">
-        <v>202.65</v>
+        <v>198.96</v>
       </c>
       <c r="G56" s="17"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D57" s="13">
-        <v>207.52</v>
+        <v>203.06</v>
       </c>
       <c r="E57" s="13">
-        <v>184.8</v>
+        <v>182.91</v>
       </c>
       <c r="F57" s="13">
-        <v>194.8</v>
+        <v>192.91</v>
       </c>
       <c r="G57" s="17"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="7">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B58" s="8"/>
       <c r="C58" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D58" s="10">
-        <v>207.57</v>
+        <v>203.12</v>
       </c>
       <c r="E58" s="10" t="s">
         <v>18</v>
@@ -1704,17 +1704,17 @@
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="11">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D59" s="13">
-        <v>207.03</v>
+        <v>203.72</v>
       </c>
       <c r="E59" s="13">
-        <v>179.19</v>
+        <v>177.3</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>18</v>
@@ -1723,36 +1723,36 @@
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="7">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B60" s="8"/>
       <c r="C60" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D60" s="10">
-        <v>202.84</v>
+        <v>199.53</v>
       </c>
       <c r="E60" s="10">
-        <v>175.12</v>
+        <v>173.23</v>
       </c>
       <c r="F60" s="10">
-        <v>185.12</v>
+        <v>183.23</v>
       </c>
       <c r="G60" s="17"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="11">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B61" s="12"/>
       <c r="C61" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D61" s="13">
-        <v>209.35</v>
+        <v>204.93</v>
       </c>
       <c r="E61" s="13">
-        <v>189.86</v>
+        <v>186.22</v>
       </c>
       <c r="F61" s="13" t="s">
         <v>18</v>
@@ -1761,52 +1761,52 @@
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="20" t="s">
         <v>32</v>
       </c>
       <c r="D62" s="10">
-        <v>219.28</v>
+        <v>217.37</v>
       </c>
       <c r="E62" s="10">
-        <v>194.95</v>
+        <v>192.65</v>
       </c>
       <c r="F62" s="10">
-        <v>204.95</v>
+        <v>202.65</v>
       </c>
       <c r="G62" s="17"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B63" s="12"/>
       <c r="C63" s="21" t="s">
         <v>33</v>
       </c>
       <c r="D63" s="13">
-        <v>209.44</v>
+        <v>207.52</v>
       </c>
       <c r="E63" s="13">
-        <v>188.07</v>
+        <v>184.8</v>
       </c>
       <c r="F63" s="13">
-        <v>198.07</v>
+        <v>194.8</v>
       </c>
       <c r="G63" s="17"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="20" t="s">
         <v>34</v>
       </c>
       <c r="D64" s="10">
-        <v>209.49</v>
+        <v>207.57</v>
       </c>
       <c r="E64" s="10" t="s">
         <v>18</v>
@@ -1818,17 +1818,17 @@
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="21" t="s">
         <v>35</v>
       </c>
       <c r="D65" s="13">
-        <v>208.91</v>
+        <v>207.03</v>
       </c>
       <c r="E65" s="13">
-        <v>182.45</v>
+        <v>179.19</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>18</v>
@@ -1836,35 +1836,35 @@
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="20" t="s">
         <v>36</v>
       </c>
       <c r="D66" s="10">
-        <v>204.72</v>
+        <v>202.84</v>
       </c>
       <c r="E66" s="10">
-        <v>178.39</v>
+        <v>175.12</v>
       </c>
       <c r="F66" s="10">
-        <v>188.39</v>
+        <v>185.12</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="11">
-        <v>46165</v>
+        <v>46168</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="21" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="13">
-        <v>211.23</v>
+        <v>209.35</v>
       </c>
       <c r="E67" s="13">
-        <v>192.12</v>
+        <v>189.86</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Wed May 27 05:42:52 UTC 2026
</commit_message>
<xml_diff>
--- a/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
+++ b/bp.com-content-dam-bp-country-sites-en_au-australia-home-products-services-pricing-tgp-excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bp365.sharepoint.com/sites/WholesalePricing/Shared Documents/B2C/TGP/Daily TGP/Web TGP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{A6B7D494-4C10-49AB-BC97-348EEC42832D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{7AECB0AB-AF10-43E3-92DF-4CB9751D51CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{1B412EEF-F96D-4DF4-A4E9-C7F0F183C2FB}"/>
   </bookViews>
@@ -809,128 +809,128 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="9" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="10">
-        <v>198.55</v>
+        <v>193.99</v>
       </c>
       <c r="E8" s="10">
-        <v>170.51</v>
+        <v>167.1</v>
       </c>
       <c r="F8" s="10">
-        <v>180.51</v>
+        <v>177.1</v>
       </c>
       <c r="G8" s="10">
-        <v>171.08</v>
+        <v>167.68</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="13">
-        <v>198.55</v>
+        <v>193.99</v>
       </c>
       <c r="E9" s="13">
-        <v>170.51</v>
+        <v>167.1</v>
       </c>
       <c r="F9" s="13">
-        <v>180.51</v>
+        <v>177.1</v>
       </c>
       <c r="G9" s="13">
-        <v>171.08</v>
+        <v>167.68</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
-        <v>46169</v>
+        <v>46170</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="10">
-        <v>198.83</v>
+        <v>194.31</v>
       </c>
       <c r="E10" s="10">
-        <v>171.11</v>
+        <v>167.74</v>
       </c>
       <c r="F10" s="10">
-        <v>181.11</v>
+        <v>177.74</v>
       </c>
       <c r="G10" s="10">
-        <v>172.13</v>
+        <v>168.76</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="13">
-        <v>202.52</v>
+        <v>198.55</v>
       </c>
       <c r="E11" s="13">
-        <v>173.59</v>
+        <v>170.51</v>
       </c>
       <c r="F11" s="13">
-        <v>183.59</v>
+        <v>180.51</v>
       </c>
       <c r="G11" s="13">
-        <v>174.16</v>
+        <v>171.08</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="9" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="10">
-        <v>202.52</v>
+        <v>198.55</v>
       </c>
       <c r="E12" s="10">
-        <v>173.59</v>
+        <v>170.51</v>
       </c>
       <c r="F12" s="10">
-        <v>183.59</v>
+        <v>180.51</v>
       </c>
       <c r="G12" s="10">
-        <v>174.16</v>
+        <v>171.08</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46168</v>
+        <v>46169</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="13">
-        <v>